<commit_message>
add confusion matrix and precision and recall analysis
</commit_message>
<xml_diff>
--- a/output/test20_alt_abbrev_annotation_with_prompt_using_fulltext_and_abstract_df.xlsx
+++ b/output/test20_alt_abbrev_annotation_with_prompt_using_fulltext_and_abstract_df.xlsx
@@ -572,44 +572,42 @@
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>36612533</t>
-        </is>
+      <c r="H2" t="n">
+        <v>7479945</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>mouse phenotype biomarker</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>primer</t>
-        </is>
-      </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>methods</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>The primers were as follows: forward primer RD5 5_-ATC TGG TTG ATC CTG CCA GT-3_ and reverse primer BhRDr 5_-GAG CTT TTTA ACT GCA ACA ACG-3_</t>
+          <t>We report a mouse model of type I Usher syndrome, rd5, whose linkage on mouse chromosome 7 to Hbb and tub has homology to human Usher I reported on human chromosome 11p15. The electroretinogram in homozygous rd5/rd5 mouse is never normal with reduced amplitudes that extinguish by 6 months.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr"/>
@@ -618,7 +616,773 @@
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Usher syndrome is a group of diseases with autosomal recessive inheritance, congenital hearing loss, and the development of retinitis pigmentosa, a progressive retinal degeneration characterized by night blindness and visual field loss over several decades. The causes of Usher syndrome are unknown and no animal models have been available for study. Four human gene sites have been reported, suggesting at least four separate forms of Usher syndrome. We report a mouse model of type I Usher syndrome, rd5, whose linkage on mouse chromosome 7 to Hbb and tub has homology to human Usher I reported on human chromosome 11p15. The electroretinogram in homozygous rd5/rd5 mouse is never normal with reduced amplitudes that extinguish by 6 months. Auditory-evoked response testing demonstrates increased hearing thresholds more than control at 3 weeks of about 30 decibels (dB) that worsen to about 45 dB by 6 months.</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>PMID: 7479945
+Abstract: Usher syndrome is a group of diseases with autosomal recessive inheritance, congenital hearing loss, and the development of retinitis pigmentosa, a progressive retinal degeneration characterized by night blindness and visual field loss over several decades. The causes of Usher syndrome are unknown and no animal models have been available for study. Four human gene sites have been reported, suggesting at least four separate forms of Usher syndrome. We report a mouse model of type I Usher syndrome, rd5, whose linkage on mouse chromosome 7 to Hbb and tub has homology to human Usher I reported on human chromosome 11p15. The electroretinogram in homozygous rd5/rd5 mouse is never normal with reduced amplitudes that extinguish by 6 months. Auditory-evoked response testing demonstrates increased hearing thresholds more than control at 3 weeks of about 30 decibels (dB) that worsen to about 45 dB by 6 months.</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
+    Inputs:
+    Alias gene symbol: rd5
+    HGNC record ID: HGNC:12406
+    Primary gene symbol: TUB
+    Official HGNC gene name: TUB bipartite transcription factor
+    Biomedical text context
+    Task:
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
+    Rules:
+    If the text does not support that the alias is an alternate abbreviation, return:
+    "alternate_abbreviation": "NO"
+    "evidence": ""
+    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
+    Evidence must be one exact sentence copied verbatim from the text.
+    Do not infer relationships or paraphrase evidence.
+    Output (Strict):
+    Output only one JSON object. No markdown.
+    {
+    "pmid": "",
+    "alias_symbol": "",
+    "primary_gene_symbol": "",
+    "name": "",
+    "alternate_abbreviation": "YES or NO",
+    "evidence": ""
+    }
+PMID: 7479945
+Abstract: Usher syndrome is a group of diseases with autosomal recessive inheritance, congenital hearing loss, and the development of retinitis pigmentosa, a progressive retinal degeneration characterized by night blindness and visual field loss over several decades. The causes of Usher syndrome are unknown and no animal models have been available for study. Four human gene sites have been reported, suggesting at least four separate forms of Usher syndrome. We report a mouse model of type I Usher syndrome, rd5, whose linkage on mouse chromosome 7 to Hbb and tub has homology to human Usher I reported on human chromosome 11p15. The electroretinogram in homozygous rd5/rd5 mouse is never normal with reduced amplitudes that extinguish by 6 months. Auditory-evoked response testing demonstrates increased hearing thresholds more than control at 3 weeks of about 30 decibels (dB) that worsen to about 45 dB by 6 months.</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>{
+"pmid": "7479945",
+"alias_symbol": "rd5",
+"primary_gene_symbol": "TUB",
+"name": "TUB bipartite transcription factor",
+"alternate_abbreviation": "NO",
+"evidence": ""
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HGNC:12406</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ENSG00000166402</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GENE ID:7275</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>TUB</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>rd5</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>9390831</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>mouse phenotype biomarker</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Mice homozygous for a defect of the tub (rd5) gene exhibit cochlear and retinal degeneration combined with obesity, and resemble certain human autosomal recessive sensory deficit syndromes.</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>TUB bipartite transcription factor</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>These authors contributed equally to this work.
+These authors jointly coordinated this work.
+Inherited retinal degeneration (IRD) represents a clinically variable and genetically heterogeneous group of disorders characterized by photoreceptor dysfunction. These diseases typically present with progressive severe vision loss and variable onset, ranging from birth to adulthood. Genomic sequencing has allowed to identify novel IRD-related genes, most of which encode proteins contributing to photoreceptor-cilia biogenesis and/or function. Despite these insights, knowledge gaps hamper a molecular diagnosis in one-third of IRD cases. By exome sequencing in a cohort of molecularly unsolved individuals with IRD, we identified a homozygous splice site variant affecting the transcript processing of TUB, encoding the first member of the Tubby family of bipartite transcription factors, in a sporadic case with retinal dystrophy. A truncating homozygous variant in this gene had previously been reported in a single family with three subjects sharing retinal dystrophy and obesity. The clinical assessment of the present patient documented a slightly increased body mass index and no changes in metabolic markers of obesity, but confirmed the occurrence of retinal detachment. In vitro studies using patient-derived fibroblasts showed the accelerated degradation of the encoded protein and aberrant cilium morphology and biogenesis. These findings definitely link impaired TUB function to retinal dystrophy and provide new data on the clinical characterization of this ultra-rare retinal ciliopathy.
+Inherited retinal degeneration (IRD) occurs in a clinically variable and genetically heterogeneous group of conditions characterized by photoreceptor degeneration and/or dysfunction [1]. The prevalence of monogenic IRD is estimated as 1 in 2000 individuals, affecting more than 2 million people worldwide [2]. This group of disorders typically present with severe vision loss that can be progressive, having an onset ranging from birth to late adulthood. Severe visual impairment affects mobility and independence, posing relevant psychological and economic burdens [3]. In the last ten years, genomic sequencing has allowed the identification of several genes implicated in IRD (for an updated list see the RetNet database,https://sph.uth.edu/retnet/). These genes encode proteins that have different roles in visual function, contributing to key processes in the cells of the pigmented cell layer and neurosensory retina [4,5]. Notably, retinal degeneration is frequently observed in ciliopathies, and a portion of IRD-related genes codifies for proteins involved in biogenesis and the maintenance of photoreceptor primary cilium [6,7,8,9]. Among these genes,TUB[MIM #601197], which encodes the first member of the Tubby family of bipartite transcription factors, has recently reported to be associated with a novel condition characterized by retinal dystrophy and obesity [MIM #616188] [10]. A truncating homozygousTUBvariant [c.1194_1195delAG, p.Arg398Serfs*9] was identified in a single family with three affected members, suggesting loss of function (LoF) as the pathomechanism underlying the disorder. The TUB family of transcription factors counts four members in vertebrates (TUB, TULP1, TULP2 and TULP3), sharing a similar domain organization including a highly conserved C-terminal domain mediating DNA binding and a divergent N-terminal region encompassing the nuclear localization signal and the transcriptional activation domain implicated in protein–protein binding [11]. A conserved region at the N-terminus enables some members of the Tubby family, including TUB, to bind to the ciliary intraflagellar transport A protein (IFTAP) [12]. Similar to the other members of the TULP family, TUB is also implicated in the control of the initiation of phagocytosis, facilitating the removal of apoptotic cells or cellular debris by retinal pigmented epithelium (RPE) cells and macrophages [13]. Since the original report, no other subject carrying biallelicTUBvariants has been described.
+In this study, we report on an additional subject with retinal dystrophy carrying a homozygous LoF variant inTUB. In vitro analyses provide evidence of the disruptive functional impact of the variant onTUBtranscript processing. We also show that the loss of TUB is associated with a defective cilium morphology and biogenesis in the primary patient’s fibroblasts. Our findings confirm the involvement of defective TUB function in retinal dystrophy and define this disorder as a novel ciliopathy.
+The proband is a 35-year-old male, the first child of healthy non-consanguineous parents of European descent (Figure 1). Family history was negative for retinal diseases or other congenital defects. The proband was born at term after an uneventful pregnancy. Length and weight at birth were reported as within the normal range. Apgar score was 8–10. No hearing impairment and/or learning difficulties were documented during the first year of age.
+At 5 years, the subject required consulting ophthalmologists for referring color blindness. A “blonde” aspect of the fundus oculi was observed and reduced full-field flash photopic and scotopic electroretinogram (ERG) responses were recorded. Visual acuity was not investigated at that time. Ophthalmological assessment at 26 years was suggestive of cone-rod dystrophy. Visual acuity was 0.8 Snellen in his right eye (RE) with myopic and astigmatic refractive error (RE: -4.50 dioptre sphere and -1 dioptre cylinder at 20°), and 0.2 Snellen in his left eye (LE) with myopic refractive error (LE: -2.00 dioptre sphere). Goldmann visual field was generally constricted, with reduced sensitivity in the superior central field in the RE and presented peripheral constriction and relative central scotoma in the LE. Light and dark adaptation sensitivity curves showed abnormal thresholds for both cones and rods. No number at the Ishihara charts were recognized. Intraocular pressure was within normal limits. The slit lamp examination biomicroscopy of the anterior segment was normal for cornea, iris and lens appearance. Fundus examination revealed bilateral optic disc pallor, depigmented aspect of the choroidal and retinal structures, diffuse retinal dystrophy with absence of intraretinal pigment dispersion or vitreous abnormalities and arteriolar attenuation. Full-field scotopic and photopic electroretinograms showed reduced a-wave and b-wave amplitude responses and delayed implicit times. Multifocal ERG ring analysis documented reduced response amplitude densities in all examined areas from the foveal center up to 20° of foveal eccentricity in both eyes (LE &gt; RE). After reduced visual field in his LE, a large area of retinoschisis in the infero-temporal sector was observed by fundoscopy, which later progressed, resulting in full retinal detachment of the LE. The subject underwent to pars plana vitrectomy with silicon oil (30% polydimethylsiloxane, PDMS) tamponade. He underwent cataract surgery in his LE and to subsequent vitreo-retinal surgeries for relapsing retinal detachments in same eye (PDMS/perfluorocarbon liquid (PFCL)/PDMS tamponades exchange and intra-operatory laser treatment; PDMS/heavy silicon oil tamponades exchange and intra-operatory laser). One year later, he developed vitreo-retinal proliferation and retinal fibrosis in the LE, and visual acuity was hand motion; therefore, the subject underwent retinotomy and heavy silicon oil/PDMS tamponades exchange.
+At last evaluation (35 years), the subject presented with a good clinical condition. No cognitive deficit nor behavioral issues were observed, and no craniofacial dysmorphism and truncal obesity were noticed. An accurate endocrinological examination was uninformative. Anthropometric assessment displayed a height of 177.5 cm (+0.1 SD), weight of 95.70 kg (+1.6 SD), and OFC 60 cm (+0.2 SD) and BMI of 30.30 Kg/m2(+1.6 SD). Tanner stage was Ph5Pg5, with a testicular volume 20 mL bilaterally. The subject’s visual acuity was 0.8 Snellen in his RE and light perception in his LE. Fundus oculi showed the unmodified condition of RE and diffuse chorio-retinal atrophy in the LE, as for visible vitreo-retinal surgical outcomes. Ultrawide field fundus photography showed macular atrophy in absence of peripheral pigment and confirmed a “blonde” aspect of the retina (Figure 2A). Fundus autofluorescence (FAF) revealed an hypoautoflorescent area in the macula due to RPE atrophy and hyper/hypoautofluorescence mottling in the posterior pole and immediately outside the vascular arcades (Figure 2B). The SD-OCT showed a disruption of the outer retina, including ELM, ellipsoid zone and RPE with outer retinal debris at the level of the RPE in the parafoveal region (Figure 2C). Full-field flash scotopic (Figure 2D) and photopic ERG confirmed reduced a-wave and b-wave amplitude responses and delayed implicit times in the RE. Similarly, multifocal ERG ring analysis, recordable only in the RE, showed the worsening of the response amplitude densities in all examined areas (0–20°) (Figure 2E), as compared to the previous examinations. Similarly, Goldmann visual field in his RE showed progressive constriction of the peripheral isopters and a ring scotoma enclosed between 10–20° of the visual field (Figure 2F); it was not executable, however, in his LE. Color blindness was also confirmed. Neck and abdominal ultrasound assessment did not reveal any abnormality. Measurements of basal hormones by the anterior pituitary, glycaemia and insulin were within the normal range. Basal plasma leptin level was in the low normal range, showing no leptin resistance. During his follow-up, clinical and ophthalmological assessments of other family members (parents and younger brother) were unremarkable.
+Trio-based WES allowed to identify a homozygous splice siteTUBvariant (chr11:8122545G &gt; A, GRCh37.p13; c.1387 + 1G &gt; A,NM_177972.3) as the only clinically and functionally relevant event putatively linked to the disorder (Supplemental Table S1). The variant had previously been annotated in public databases (dbSNP, rs1040410003) with low frequency (gnomAD v3.1, MAF = 0.00001972) at the heterozygous state. It was classified as likely pathogenic (PVS1/PM2/PP5) according to the American College of Medical Genetics and Genomics-Association for Molecular Pathology (ACMG-AMP) criteria (ClinVar: VCV000865971.1) [14]. Sanger sequencing confirmed the homozygosity for the variant in the proband and the heterozygous status in the healthy parents and unaffected sib (Figure 1).
+Since the variant was predicted to affect the exon 11 donor splice site, the total RNA from patient-derived skin primary fibroblasts was used to characterize the impact of the nucleotide change on transcript processing. The cDNA fragment encompassing the relevant exons was amplified, confirming the presence of two aberrantly spliced products (Figure 3A). The two aberrant PCR amplicons were isolated from agarose gel, purified and sequenced via Sanger. The former (500 bp) was derived from skipping of the penultimate exon (exon 11, ENST00000299506.3), resulting in a premature termination codon (i.e., p.Glu406Argfs*4), while the latter (1172 bp) was the result of retention of intron 10, resulting in a TUB protein having a divergent 19-residue-long C-terminus and lacking the last 44 amino acids (p.Pro463Hisfs*19) (Figure 3B).
+In the patient’s skin fibroblasts, the predicted TUBGlu406Argfs*4protein was undetectable by Western blot [WB] analysis, while the TUBPro463Hisfs*19protein was poorly detectable likely due to accelerated degradation (Figure 3C, left panel). Consistently, the endogenous TUBPro463Hisfs*19level was partially rescued by blocking the proteasomal degradation pathway using MG132 (Figure 3C, right panel).
+To investigate the cellular localization of the mutated protein, cytoplasm and nuclear cell fractions were obtained and analyzed by WB. The results demonstrate that both the wild-type (wt) and mutant TUB proteins were almost exclusively localized in the nucleus (Figure 3D). This finding was also confirmed by confocal microscopy analysis that evidenced the nuclear localization of the TUB mutant (Figure 4A).
+Based on the documented role of TUB in early ciliogenesis [15], we assessed the localization of TUB at the cilium, but we failed to observe any consistent co-localization, possibly due to the low diffused levels of the protein in the cytoplasm To investigate the impact of defective TUB function on the morphogenesis of the primary cilium, a confocal analysis on primary fibroblasts was performed using antibodies against ARL13B, which localizes to primary cilia, and pericentrin, a component of the centrosome, which stains the basal body. As shown inFigure 4B, while almost all the control cells showed a primary cilium, 40% of the fibroblasts carrying the homozygous splice site variant inTUBdid not show a primary cilium. Moreover, while no significant difference was observed in ciliary axoneme length between the starved control and mutant cells, a large percentage of the latter showed an abnormal cilium morphology and a poorly defined and disorganized basal body (Figure 4C).
+The loss of TUB function was recently reported to underlie a novel IRD condition based on the identification of homozygosity for a 2 bp deletion (c.1194_1195delAG) causing the premature termination of the protein (p.Arg398Serfs*9) shared by three affected members of a single consanguineous family [10]. While the combination of retinal dystrophy and early onset obesity can be reminiscent of other disorders (e.g., Bardet–Biedl syndrome (MIM#PS209900) and Alstrom syndrome (MIM#203800)), the absence of other clinically relevant feature/sign was suggestive of a previously unreported ciliopathy [10]. In this paper, we report on a second disruptive variant (c.1387 + 1G &gt; A) affectingTUBin a subject with features that overlap with those previously described in the affected members of the original family.
+In the present and previously reported affected individuals, the ocular phenotype associated with defective TUB function is characterized by widespread retinal pigment epithelial (RPE) atrophy, deteriorating vision, the myopic and astigmatic refractive defect, the blonde fundus appearance, the ERG and OCT findings and progression of the disease (Figure 2). Notably, retinal detachment, without vitreous hemorrhage, was invariantly documented in the four individuals with biallelic inactivatingTUBvariants, suggesting that this feature likely represent a common finding in the disorder.
+Early onset obesity had previously been considered a major feature of the TUB-related condition [10], even though only two of three affected sibs were found obese (BMI &gt; 30), and the glycemic and lipid profiles in one of affected sibs were found within the normal range. The finding of obesity in the apparently healthy father (heterozygous carrier) suggests a possible co-occurring genetic event contributing to obesity in the family. In the present report, the clinical assessment of the affected individual documented increased weight (95.7 kg, +1.6 SD) and BMI (30.3, +1.6 SD), thus indicating overweight, in absence of other signs of obesity. Although evidence suggests that a defective TUB function may result in disturbances in insulin and leptin activity and obesity in mice [16,17,18,19], based on the collected findings, the relevance of TUB in human obesity requires further study. To assess whether TUB LoF could impact on hypothalamic pathways, food intake and adiposity, the metabolic profile of the affected individual was investigated. Accurate endocrinological examination did not reveal any abnormality, and the measurements of basal hormones by the anterior pituitary, glycaemia, insulin and leptin were within the normal range, thus ruling out insulin or leptin resistance. Consistently, instrumental investigations (X-ray and ultrasound analyses) documented no sign of glycogen accumulation in the internal organs. Consistently, the absence of significant changes in lipid storage was demonstrated by thin-layer chromatography (HPTLC) analysis in proband-derived fibroblast (Figure S1), allowing to confirm an apparently normal endocrine–metabolic profile in the affected individual. Of note, the Tubby protein has been involved in cochlear degeneration [20,21]. Based on this functional link, we evaluated the occurrence of hearing problems and cochlear degeneration, which were not observed.
+The homozygousTUBvariant was predicted to affect transcript processing, causing the skipping of exon 11 and intron retention, resulting in a frameshift with the premature termination of the TUB protein. mRNA analysis in proband-derived fibroblasts confirmed a disruptive impact of the splice site change documenting two aberrantly processed transcripts predicted to encode a 406-residue-long protein (p.Glu406Argfs*4) that probably is not able to proceed in protein synthesis, and a 481-residue-long protein (p.Pro463Hisfs*19) characterized by a divergent C-terminus characterized by accelerated degradation (Figure 3B). These findings confirm LoF as the pathomechanism underlying this disorder.
+Primary cilia are microtubule-based organelles that extend from the apical surface of the majority of mammalian cells. Cilia act as “cellular antennae”, receiving different inputs from the extracellular environment and transducing signals in response to stimuli [22]. A complex process required for proper cilia biogenesis function is the intraflagellar transport, which is required for assembling cilia and trafficking within primary cilia [23]. In this context, IFT-A has historically been believed to mediate retrograde intraflagellar transport inside the cilia and an IFT-A-binding domain at the TUB N-terminus has been demonstrated recently [24]. Moreover, co-localization between TUB and rootletin, the major structural component of the ciliary rootlet, has been observed in human retinal photoreceptors [10]. The use of a more informative in vitro model (e.g., induced pluripotent-stem-cell-derived retinal-pigment epithelium cells) and experimental strategies (e.g., siRNA-mediated TUB silencing) is required to appreciate more accurately the functional relevance of TUB in an appropriate cellular context.
+In summary, we confirm the link between TUB LoF and a new condition of human retinal ciliopathy and provide evidence of an altered cilium morphology/biogenesis in patient-derived fibroblasts. In fact, these cells displayed a reduced number of cilia when compared to the control cells, with a poorly defined and disorganized basal body structure, which are expected to prevent normal protein trafficking along the cilium. While these findings could explain the degeneration of photoreceptors characterizing this disorder, a relatively overall mild presentation has been associated with mutations in this gene. Multiple factors might contribute to this picture. First, the functional relevance of TUB in the context of ciliogenesis and cilium function might vary in different cell lineages. Second, functional compensation exerted by other related proteins might contribute to buffer the severity of the endophenotype. Third, specific cell lineages (e.g., rod and cone cells) might be particularly sensitive to TUB LoF. The collection of additional patients with biallelic variants in the gene will allow a more accurate characterization of the clinical spectrum associated with TUB LoF. Based on these considerations, TUB loss of function could be considered as responsible for a novel form of isolated retinal ciliopathy.</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Mice homozygous for a defect of the tub (rd5) gene exhibit cochlear and retinal degeneration combined with obesity, and resemble certain human autosomal recessive sensory deficit syndromes. To establish the progressive nature of sensory cell loss associated with the tub gene, and to differentiate tub-related losses from those associated with the C57 background on which tub arose, we evaluated cochleas and retinas from tub/tub, tub/+, and +/+ mice, aged 2 weeks to 1 year by light and electron microscopy. Cochleas from mice of all three genotypes show progressive inner (IHC) and outer hair cell (OHC) loss. Relative to tub/+ and +/+ animals, however, tub homozygotes show accelerated OHC loss, affecting the extreme cochlear base (hook region) by 1 month, and the apex by 6 months. IHC loss in tub/tub animals is accelerated in the basal half of the cochlea, affecting the hook region by 6 months. Spiral ganglion cell losses were observed only in tub/tub mice, and only in the cochlear base. Retinas of tub/tub mice are abnormal at maturity, exhibiting shortened photoreceptor outer segments by 2 weeks, and progressive photoreceptor loss thereafter. Because the tub mutation causes degeneration of sensory cells in the ear and eye but has no other neurological effects, tubby mice hold unique promise for the study of human syndromic sensory loss.</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>PMID: 9390831
+Full Text: These authors contributed equally to this work.
+These authors jointly coordinated this work.
+Inherited retinal degeneration (IRD) represents a clinically variable and genetically heterogeneous group of disorders characterized by photoreceptor dysfunction. These diseases typically present with progressive severe vision loss and variable onset, ranging from birth to adulthood. Genomic sequencing has allowed to identify novel IRD-related genes, most of which encode proteins contributing to photoreceptor-cilia biogenesis and/or function. Despite these insights, knowledge gaps hamper a molecular diagnosis in one-third of IRD cases. By exome sequencing in a cohort of molecularly unsolved individuals with IRD, we identified a homozygous splice site variant affecting the transcript processing of TUB, encoding the first member of the Tubby family of bipartite transcription factors, in a sporadic case with retinal dystrophy. A truncating homozygous variant in this gene had previously been reported in a single family with three subjects sharing retinal dystrophy and obesity. The clinical assessment of the present patient documented a slightly increased body mass index and no changes in metabolic markers of obesity, but confirmed the occurrence of retinal detachment. In vitro studies using patient-derived fibroblasts showed the accelerated degradation of the encoded protein and aberrant cilium morphology and biogenesis. These findings definitely link impaired TUB function to retinal dystrophy and provide new data on the clinical characterization of this ultra-rare retinal ciliopathy.
+Inherited retinal degeneration (IRD) occurs in a clinically variable and genetically heterogeneous group of conditions characterized by photoreceptor degeneration and/or dysfunction [1]. The prevalence of monogenic IRD is estimated as 1 in 2000 individuals, affecting more than 2 million people worldwide [2]. This group of disorders typically present with severe vision loss that can be progressive, having an onset ranging from birth to late adulthood. Severe visual impairment affects mobility and independence, posing relevant psychological and economic burdens [3]. In the last ten years, genomic sequencing has allowed the identification of several genes implicated in IRD (for an updated list see the RetNet database,https://sph.uth.edu/retnet/). These genes encode proteins that have different roles in visual function, contributing to key processes in the cells of the pigmented cell layer and neurosensory retina [4,5]. Notably, retinal degeneration is frequently observed in ciliopathies, and a portion of IRD-related genes codifies for proteins involved in biogenesis and the maintenance of photoreceptor primary cilium [6,7,8,9]. Among these genes,TUB[MIM #601197], which encodes the first member of the Tubby family of bipartite transcription factors, has recently reported to be associated with a novel condition characterized by retinal dystrophy and obesity [MIM #616188] [10]. A truncating homozygousTUBvariant [c.1194_1195delAG, p.Arg398Serfs*9] was identified in a single family with three affected members, suggesting loss of function (LoF) as the pathomechanism underlying the disorder. The TUB family of transcription factors counts four members in vertebrates (TUB, TULP1, TULP2 and TULP3), sharing a similar domain organization including a highly conserved C-terminal domain mediating DNA binding and a divergent N-terminal region encompassing the nuclear localization signal and the transcriptional activation domain implicated in protein–protein binding [11]. A conserved region at the N-terminus enables some members of the Tubby family, including TUB, to bind to the ciliary intraflagellar transport A protein (IFTAP) [12]. Similar to the other members of the TULP family, TUB is also implicated in the control of the initiation of phagocytosis, facilitating the removal of apoptotic cells or cellular debris by retinal pigmented epithelium (RPE) cells and macrophages [13]. Since the original report, no other subject carrying biallelicTUBvariants has been described.
+In this study, we report on an additional subject with retinal dystrophy carrying a homozygous LoF variant inTUB. In vitro analyses provide evidence of the disruptive functional impact of the variant onTUBtranscript processing. We also show that the loss of TUB is associated with a defective cilium morphology and biogenesis in the primary patient’s fibroblasts. Our findings confirm the involvement of defective TUB function in retinal dystrophy and define this disorder as a novel ciliopathy.
+The proband is a 35-year-old male, the first child of healthy non-consanguineous parents of European descent (Figure 1). Family history was negative for retinal diseases or other congenital defects. The proband was born at term after an uneventful pregnancy. Length and weight at birth were reported as within the normal range. Apgar score was 8–10. No hearing impairment and/or learning difficulties were documented during the first year of age.
+At 5 years, the subject required consulting ophthalmologists for referring color blindness. A “blonde” aspect of the fundus oculi was observed and reduced full-field flash photopic and scotopic electroretinogram (ERG) responses were recorded. Visual acuity was not investigated at that time. Ophthalmological assessment at 26 years was suggestive of cone-rod dystrophy. Visual acuity was 0.8 Snellen in his right eye (RE) with myopic and astigmatic refractive error (RE: -4.50 dioptre sphere and -1 dioptre cylinder at 20°), and 0.2 Snellen in his left eye (LE) with myopic refractive error (LE: -2.00 dioptre sphere). Goldmann visual field was generally constricted, with reduced sensitivity in the superior central field in the RE and presented peripheral constriction and relative central scotoma in the LE. Light and dark adaptation sensitivity curves showed abnormal thresholds for both cones and rods. No number at the Ishihara charts were recognized. Intraocular pressure was within normal limits. The slit lamp examination biomicroscopy of the anterior segment was normal for cornea, iris and lens appearance. Fundus examination revealed bilateral optic disc pallor, depigmented aspect of the choroidal and retinal structures, diffuse retinal dystrophy with absence of intraretinal pigment dispersion or vitreous abnormalities and arteriolar attenuation. Full-field scotopic and photopic electroretinograms showed reduced a-wave and b-wave amplitude responses and delayed implicit times. Multifocal ERG ring analysis documented reduced response amplitude densities in all examined areas from the foveal center up to 20° of foveal eccentricity in both eyes (LE &gt; RE). After reduced visual field in his LE, a large area of retinoschisis in the infero-temporal sector was observed by fundoscopy, which later progressed, resulting in full retinal detachment of the LE. The subject underwent to pars plana vitrectomy with silicon oil (30% polydimethylsiloxane, PDMS) tamponade. He underwent cataract surgery in his LE and to subsequent vitreo-retinal surgeries for relapsing retinal detachments in same eye (PDMS/perfluorocarbon liquid (PFCL)/PDMS tamponades exchange and intra-operatory laser treatment; PDMS/heavy silicon oil tamponades exchange and intra-operatory laser). One year later, he developed vitreo-retinal proliferation and retinal fibrosis in the LE, and visual acuity was hand motion; therefore, the subject underwent retinotomy and heavy silicon oil/PDMS tamponades exchange.
+At last evaluation (35 years), the subject presented with a good clinical condition. No cognitive deficit nor behavioral issues were observed, and no craniofacial dysmorphism and truncal obesity were noticed. An accurate endocrinological examination was uninformative. Anthropometric assessment displayed a height of 177.5 cm (+0.1 SD), weight of 95.70 kg (+1.6 SD), and OFC 60 cm (+0.2 SD) and BMI of 30.30 Kg/m2(+1.6 SD). Tanner stage was Ph5Pg5, with a testicular volume 20 mL bilaterally. The subject’s visual acuity was 0.8 Snellen in his RE and light perception in his LE. Fundus oculi showed the unmodified condition of RE and diffuse chorio-retinal atrophy in the LE, as for visible vitreo-retinal surgical outcomes. Ultrawide field fundus photography showed macular atrophy in absence of peripheral pigment and confirmed a “blonde” aspect of the retina (Figure 2A). Fundus autofluorescence (FAF) revealed an hypoautoflorescent area in the macula due to RPE atrophy and hyper/hypoautofluorescence mottling in the posterior pole and immediately outside the vascular arcades (Figure 2B). The SD-OCT showed a disruption of the outer retina, including ELM, ellipsoid zone and RPE with outer retinal debris at the level of the RPE in the parafoveal region (Figure 2C). Full-field flash scotopic (Figure 2D) and photopic ERG confirmed reduced a-wave and b-wave amplitude responses and delayed implicit times in the RE. Similarly, multifocal ERG ring analysis, recordable only in the RE, showed the worsening of the response amplitude densities in all examined areas (0–20°) (Figure 2E), as compared to the previous examinations. Similarly, Goldmann visual field in his RE showed progressive constriction of the peripheral isopters and a ring scotoma enclosed between 10–20° of the visual field (Figure 2F); it was not executable, however, in his LE. Color blindness was also confirmed. Neck and abdominal ultrasound assessment did not reveal any abnormality. Measurements of basal hormones by the anterior pituitary, glycaemia and insulin were within the normal range. Basal plasma leptin level was in the low normal range, showing no leptin resistance. During his follow-up, clinical and ophthalmological assessments of other family members (parents and younger brother) were unremarkable.
+Trio-based WES allowed to identify a homozygous splice siteTUBvariant (chr11:8122545G &gt; A, GRCh37.p13; c.1387 + 1G &gt; A,NM_177972.3) as the only clinically and functionally relevant event putatively linked to the disorder (Supplemental Table S1). The variant had previously been annotated in public databases (dbSNP, rs1040410003) with low frequency (gnomAD v3.1, MAF = 0.00001972) at the heterozygous state. It was classified as likely pathogenic (PVS1/PM2/PP5) according to the American College of Medical Genetics and Genomics-Association for Molecular Pathology (ACMG-AMP) criteria (ClinVar: VCV000865971.1) [14]. Sanger sequencing confirmed the homozygosity for the variant in the proband and the heterozygous status in the healthy parents and unaffected sib (Figure 1).
+Since the variant was predicted to affect the exon 11 donor splice site, the total RNA from patient-derived skin primary fibroblasts was used to characterize the impact of the nucleotide change on transcript processing. The cDNA fragment encompassing the relevant exons was amplified, confirming the presence of two aberrantly spliced products (Figure 3A). The two aberrant PCR amplicons were isolated from agarose gel, purified and sequenced via Sanger. The former (500 bp) was derived from skipping of the penultimate exon (exon 11, ENST00000299506.3), resulting in a premature termination codon (i.e., p.Glu406Argfs*4), while the latter (1172 bp) was the result of retention of intron 10, resulting in a TUB protein having a divergent 19-residue-long C-terminus and lacking the last 44 amino acids (p.Pro463Hisfs*19) (Figure 3B).
+In the patient’s skin fibroblasts, the predicted TUBGlu406Argfs*4protein was undetectable by Western blot [WB] analysis, while the TUBPro463Hisfs*19protein was poorly detectable likely due to accelerated degradation (Figure 3C, left panel). Consistently, the endogenous TUBPro463Hisfs*19level was partially rescued by blocking the proteasomal degradation pathway using MG132 (Figure 3C, right panel).
+To investigate the cellular localization of the mutated protein, cytoplasm and nuclear cell fractions were obtained and analyzed by WB. The results demonstrate that both the wild-type (wt) and mutant TUB proteins were almost exclusively localized in the nucleus (Figure 3D). This finding was also confirmed by confocal microscopy analysis that evidenced the nuclear localization of the TUB mutant (Figure 4A).
+Based on the documented role of TUB in early ciliogenesis [15], we assessed the localization of TUB at the cilium, but we failed to observe any consistent co-localization, possibly due to the low diffused levels of the protein in the cytoplasm To investigate the impact of defective TUB function on the morphogenesis of the primary cilium, a confocal analysis on primary fibroblasts was performed using antibodies against ARL13B, which localizes to primary cilia, and pericentrin, a component of the centrosome, which stains the basal body. As shown inFigure 4B, while almost all the control cells showed a primary cilium, 40% of the fibroblasts carrying the homozygous splice site variant inTUBdid not show a primary cilium. Moreover, while no significant difference was observed in ciliary axoneme length between the starved control and mutant cells, a large percentage of the latter showed an abnormal cilium morphology and a poorly defined and disorganized basal body (Figure 4C).
+The loss of TUB function was recently reported to underlie a novel IRD condition based on the identification of homozygosity for a 2 bp deletion (c.1194_1195delAG) causing the premature termination of the protein (p.Arg398Serfs*9) shared by three affected members of a single consanguineous family [10]. While the combination of retinal dystrophy and early onset obesity can be reminiscent of other disorders (e.g., Bardet–Biedl syndrome (MIM#PS209900) and Alstrom syndrome (MIM#203800)), the absence of other clinically relevant feature/sign was suggestive of a previously unreported ciliopathy [10]. In this paper, we report on a second disruptive variant (c.1387 + 1G &gt; A) affectingTUBin a subject with features that overlap with those previously described in the affected members of the original family.
+In the present and previously reported affected individuals, the ocular phenotype associated with defective TUB function is characterized by widespread retinal pigment epithelial (RPE) atrophy, deteriorating vision, the myopic and astigmatic refractive defect, the blonde fundus appearance, the ERG and OCT findings and progression of the disease (Figure 2). Notably, retinal detachment, without vitreous hemorrhage, was invariantly documented in the four individuals with biallelic inactivatingTUBvariants, suggesting that this feature likely represent a common finding in the disorder.
+Early onset obesity had previously been considered a major feature of the TUB-related condition [10], even though only two of three affected sibs were found obese (BMI &gt; 30), and the glycemic and lipid profiles in one of affected sibs were found within the normal range. The finding of obesity in the apparently healthy father (heterozygous carrier) suggests a possible co-occurring genetic event contributing to obesity in the family. In the present report, the clinical assessment of the affected individual documented increased weight (95.7 kg, +1.6 SD) and BMI (30.3, +1.6 SD), thus indicating overweight, in absence of other signs of obesity. Although evidence suggests that a defective TUB function may result in disturbances in insulin and leptin activity and obesity in mice [16,17,18,19], based on the collected findings, the relevance of TUB in human obesity requires further study. To assess whether TUB LoF could impact on hypothalamic pathways, food intake and adiposity, the metabolic profile of the affected individual was investigated. Accurate endocrinological examination did not reveal any abnormality, and the measurements of basal hormones by the anterior pituitary, glycaemia, insulin and leptin were within the normal range, thus ruling out insulin or leptin resistance. Consistently, instrumental investigations (X-ray and ultrasound analyses) documented no sign of glycogen accumulation in the internal organs. Consistently, the absence of significant changes in lipid storage was demonstrated by thin-layer chromatography (HPTLC) analysis in proband-derived fibroblast (Figure S1), allowing to confirm an apparently normal endocrine–metabolic profile in the affected individual. Of note, the Tubby protein has been involved in cochlear degeneration [20,21]. Based on this functional link, we evaluated the occurrence of hearing problems and cochlear degeneration, which were not observed.
+The homozygousTUBvariant was predicted to affect transcript processing, causing the skipping of exon 11 and intron retention, resulting in a frameshift with the premature termination of the TUB protein. mRNA analysis in proband-derived fibroblasts confirmed a disruptive impact of the splice site change documenting two aberrantly processed transcripts predicted to encode a 406-residue-long protein (p.Glu406Argfs*4) that probably is not able to proceed in protein synthesis, and a 481-residue-long protein (p.Pro463Hisfs*19) characterized by a divergent C-terminus characterized by accelerated degradation (Figure 3B). These findings confirm LoF as the pathomechanism underlying this disorder.
+Primary cilia are microtubule-based organelles that extend from the apical surface of the majority of mammalian cells. Cilia act as “cellular antennae”, receiving different inputs from the extracellular environment and transducing signals in response to stimuli [22]. A complex process required for proper cilia biogenesis function is the intraflagellar transport, which is required for assembling cilia and trafficking within primary cilia [23]. In this context, IFT-A has historically been believed to mediate retrograde intraflagellar transport inside the cilia and an IFT-A-binding domain at the TUB N-terminus has been demonstrated recently [24]. Moreover, co-localization between TUB and rootletin, the major structural component of the ciliary rootlet, has been observed in human retinal photoreceptors [10]. The use of a more informative in vitro model (e.g., induced pluripotent-stem-cell-derived retinal-pigment epithelium cells) and experimental strategies (e.g., siRNA-mediated TUB silencing) is required to appreciate more accurately the functional relevance of TUB in an appropriate cellular context.
+In summary, we confirm the link between TUB LoF and a new condition of human retinal ciliopathy and provide evidence of an altered cilium morphology/biogenesis in patient-derived fibroblasts. In fact, these cells displayed a reduced number of cilia when compared to the control cells, with a poorly defined and disorganized basal body structure, which are expected to prevent normal protein trafficking along the cilium. While these findings could explain the degeneration of photoreceptors characterizing this disorder, a relatively overall mild presentation has been associated with mutations in this gene. Multiple factors might contribute to this picture. First, the functional relevance of TUB in the context of ciliogenesis and cilium function might vary in different cell lineages. Second, functional compensation exerted by other related proteins might contribute to buffer the severity of the endophenotype. Third, specific cell lineages (e.g., rod and cone cells) might be particularly sensitive to TUB LoF. The collection of additional patients with biallelic variants in the gene will allow a more accurate characterization of the clinical spectrum associated with TUB LoF. Based on these considerations, TUB loss of function could be considered as responsible for a novel form of isolated retinal ciliopathy.</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
+    Inputs:
+    Alias gene symbol: rd5
+    HGNC record ID: HGNC:12406
+    Primary gene symbol: TUB
+    Official HGNC gene name: TUB bipartite transcription factor
+    Biomedical text context
+    Task:
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
+    Rules:
+    If the text does not support that the alias is an alternate abbreviation, return:
+    "alternate_abbreviation": "NO"
+    "evidence": ""
+    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
+    Evidence must be one exact sentence copied verbatim from the text.
+    Do not infer relationships or paraphrase evidence.
+    Output (Strict):
+    Output only one JSON object. No markdown.
+    {
+    "pmid": "",
+    "alias_symbol": "",
+    "primary_gene_symbol": "",
+    "name": "",
+    "alternate_abbreviation": "YES or NO",
+    "evidence": ""
+    }
+PMID: 9390831
+Full Text: These authors contributed equally to this work.
+These authors jointly coordinated this work.
+Inherited retinal degeneration (IRD) represents a clinically variable and genetically heterogeneous group of disorders characterized by photoreceptor dysfunction. These diseases typically present with progressive severe vision loss and variable onset, ranging from birth to adulthood. Genomic sequencing has allowed to identify novel IRD-related genes, most of which encode proteins contributing to photoreceptor-cilia biogenesis and/or function. Despite these insights, knowledge gaps hamper a molecular diagnosis in one-third of IRD cases. By exome sequencing in a cohort of molecularly unsolved individuals with IRD, we identified a homozygous splice site variant affecting the transcript processing of TUB, encoding the first member of the Tubby family of bipartite transcription factors, in a sporadic case with retinal dystrophy. A truncating homozygous variant in this gene had previously been reported in a single family with three subjects sharing retinal dystrophy and obesity. The clinical assessment of the present patient documented a slightly increased body mass index and no changes in metabolic markers of obesity, but confirmed the occurrence of retinal detachment. In vitro studies using patient-derived fibroblasts showed the accelerated degradation of the encoded protein and aberrant cilium morphology and biogenesis. These findings definitely link impaired TUB function to retinal dystrophy and provide new data on the clinical characterization of this ultra-rare retinal ciliopathy.
+Inherited retinal degeneration (IRD) occurs in a clinically variable and genetically heterogeneous group of conditions characterized by photoreceptor degeneration and/or dysfunction [1]. The prevalence of monogenic IRD is estimated as 1 in 2000 individuals, affecting more than 2 million people worldwide [2]. This group of disorders typically present with severe vision loss that can be progressive, having an onset ranging from birth to late adulthood. Severe visual impairment affects mobility and independence, posing relevant psychological and economic burdens [3]. In the last ten years, genomic sequencing has allowed the identification of several genes implicated in IRD (for an updated list see the RetNet database,https://sph.uth.edu/retnet/). These genes encode proteins that have different roles in visual function, contributing to key processes in the cells of the pigmented cell layer and neurosensory retina [4,5]. Notably, retinal degeneration is frequently observed in ciliopathies, and a portion of IRD-related genes codifies for proteins involved in biogenesis and the maintenance of photoreceptor primary cilium [6,7,8,9]. Among these genes,TUB[MIM #601197], which encodes the first member of the Tubby family of bipartite transcription factors, has recently reported to be associated with a novel condition characterized by retinal dystrophy and obesity [MIM #616188] [10]. A truncating homozygousTUBvariant [c.1194_1195delAG, p.Arg398Serfs*9] was identified in a single family with three affected members, suggesting loss of function (LoF) as the pathomechanism underlying the disorder. The TUB family of transcription factors counts four members in vertebrates (TUB, TULP1, TULP2 and TULP3), sharing a similar domain organization including a highly conserved C-terminal domain mediating DNA binding and a divergent N-terminal region encompassing the nuclear localization signal and the transcriptional activation domain implicated in protein–protein binding [11]. A conserved region at the N-terminus enables some members of the Tubby family, including TUB, to bind to the ciliary intraflagellar transport A protein (IFTAP) [12]. Similar to the other members of the TULP family, TUB is also implicated in the control of the initiation of phagocytosis, facilitating the removal of apoptotic cells or cellular debris by retinal pigmented epithelium (RPE) cells and macrophages [13]. Since the original report, no other subject carrying biallelicTUBvariants has been described.
+In this study, we report on an additional subject with retinal dystrophy carrying a homozygous LoF variant inTUB. In vitro analyses provide evidence of the disruptive functional impact of the variant onTUBtranscript processing. We also show that the loss of TUB is associated with a defective cilium morphology and biogenesis in the primary patient’s fibroblasts. Our findings confirm the involvement of defective TUB function in retinal dystrophy and define this disorder as a novel ciliopathy.
+The proband is a 35-year-old male, the first child of healthy non-consanguineous parents of European descent (Figure 1). Family history was negative for retinal diseases or other congenital defects. The proband was born at term after an uneventful pregnancy. Length and weight at birth were reported as within the normal range. Apgar score was 8–10. No hearing impairment and/or learning difficulties were documented during the first year of age.
+At 5 years, the subject required consulting ophthalmologists for referring color blindness. A “blonde” aspect of the fundus oculi was observed and reduced full-field flash photopic and scotopic electroretinogram (ERG) responses were recorded. Visual acuity was not investigated at that time. Ophthalmological assessment at 26 years was suggestive of cone-rod dystrophy. Visual acuity was 0.8 Snellen in his right eye (RE) with myopic and astigmatic refractive error (RE: -4.50 dioptre sphere and -1 dioptre cylinder at 20°), and 0.2 Snellen in his left eye (LE) with myopic refractive error (LE: -2.00 dioptre sphere). Goldmann visual field was generally constricted, with reduced sensitivity in the superior central field in the RE and presented peripheral constriction and relative central scotoma in the LE. Light and dark adaptation sensitivity curves showed abnormal thresholds for both cones and rods. No number at the Ishihara charts were recognized. Intraocular pressure was within normal limits. The slit lamp examination biomicroscopy of the anterior segment was normal for cornea, iris and lens appearance. Fundus examination revealed bilateral optic disc pallor, depigmented aspect of the choroidal and retinal structures, diffuse retinal dystrophy with absence of intraretinal pigment dispersion or vitreous abnormalities and arteriolar attenuation. Full-field scotopic and photopic electroretinograms showed reduced a-wave and b-wave amplitude responses and delayed implicit times. Multifocal ERG ring analysis documented reduced response amplitude densities in all examined areas from the foveal center up to 20° of foveal eccentricity in both eyes (LE &gt; RE). After reduced visual field in his LE, a large area of retinoschisis in the infero-temporal sector was observed by fundoscopy, which later progressed, resulting in full retinal detachment of the LE. The subject underwent to pars plana vitrectomy with silicon oil (30% polydimethylsiloxane, PDMS) tamponade. He underwent cataract surgery in his LE and to subsequent vitreo-retinal surgeries for relapsing retinal detachments in same eye (PDMS/perfluorocarbon liquid (PFCL)/PDMS tamponades exchange and intra-operatory laser treatment; PDMS/heavy silicon oil tamponades exchange and intra-operatory laser). One year later, he developed vitreo-retinal proliferation and retinal fibrosis in the LE, and visual acuity was hand motion; therefore, the subject underwent retinotomy and heavy silicon oil/PDMS tamponades exchange.
+At last evaluation (35 years), the subject presented with a good clinical condition. No cognitive deficit nor behavioral issues were observed, and no craniofacial dysmorphism and truncal obesity were noticed. An accurate endocrinological examination was uninformative. Anthropometric assessment displayed a height of 177.5 cm (+0.1 SD), weight of 95.70 kg (+1.6 SD), and OFC 60 cm (+0.2 SD) and BMI of 30.30 Kg/m2(+1.6 SD). Tanner stage was Ph5Pg5, with a testicular volume 20 mL bilaterally. The subject’s visual acuity was 0.8 Snellen in his RE and light perception in his LE. Fundus oculi showed the unmodified condition of RE and diffuse chorio-retinal atrophy in the LE, as for visible vitreo-retinal surgical outcomes. Ultrawide field fundus photography showed macular atrophy in absence of peripheral pigment and confirmed a “blonde” aspect of the retina (Figure 2A). Fundus autofluorescence (FAF) revealed an hypoautoflorescent area in the macula due to RPE atrophy and hyper/hypoautofluorescence mottling in the posterior pole and immediately outside the vascular arcades (Figure 2B). The SD-OCT showed a disruption of the outer retina, including ELM, ellipsoid zone and RPE with outer retinal debris at the level of the RPE in the parafoveal region (Figure 2C). Full-field flash scotopic (Figure 2D) and photopic ERG confirmed reduced a-wave and b-wave amplitude responses and delayed implicit times in the RE. Similarly, multifocal ERG ring analysis, recordable only in the RE, showed the worsening of the response amplitude densities in all examined areas (0–20°) (Figure 2E), as compared to the previous examinations. Similarly, Goldmann visual field in his RE showed progressive constriction of the peripheral isopters and a ring scotoma enclosed between 10–20° of the visual field (Figure 2F); it was not executable, however, in his LE. Color blindness was also confirmed. Neck and abdominal ultrasound assessment did not reveal any abnormality. Measurements of basal hormones by the anterior pituitary, glycaemia and insulin were within the normal range. Basal plasma leptin level was in the low normal range, showing no leptin resistance. During his follow-up, clinical and ophthalmological assessments of other family members (parents and younger brother) were unremarkable.
+Trio-based WES allowed to identify a homozygous splice siteTUBvariant (chr11:8122545G &gt; A, GRCh37.p13; c.1387 + 1G &gt; A,NM_177972.3) as the only clinically and functionally relevant event putatively linked to the disorder (Supplemental Table S1). The variant had previously been annotated in public databases (dbSNP, rs1040410003) with low frequency (gnomAD v3.1, MAF = 0.00001972) at the heterozygous state. It was classified as likely pathogenic (PVS1/PM2/PP5) according to the American College of Medical Genetics and Genomics-Association for Molecular Pathology (ACMG-AMP) criteria (ClinVar: VCV000865971.1) [14]. Sanger sequencing confirmed the homozygosity for the variant in the proband and the heterozygous status in the healthy parents and unaffected sib (Figure 1).
+Since the variant was predicted to affect the exon 11 donor splice site, the total RNA from patient-derived skin primary fibroblasts was used to characterize the impact of the nucleotide change on transcript processing. The cDNA fragment encompassing the relevant exons was amplified, confirming the presence of two aberrantly spliced products (Figure 3A). The two aberrant PCR amplicons were isolated from agarose gel, purified and sequenced via Sanger. The former (500 bp) was derived from skipping of the penultimate exon (exon 11, ENST00000299506.3), resulting in a premature termination codon (i.e., p.Glu406Argfs*4), while the latter (1172 bp) was the result of retention of intron 10, resulting in a TUB protein having a divergent 19-residue-long C-terminus and lacking the last 44 amino acids (p.Pro463Hisfs*19) (Figure 3B).
+In the patient’s skin fibroblasts, the predicted TUBGlu406Argfs*4protein was undetectable by Western blot [WB] analysis, while the TUBPro463Hisfs*19protein was poorly detectable likely due to accelerated degradation (Figure 3C, left panel). Consistently, the endogenous TUBPro463Hisfs*19level was partially rescued by blocking the proteasomal degradation pathway using MG132 (Figure 3C, right panel).
+To investigate the cellular localization of the mutated protein, cytoplasm and nuclear cell fractions were obtained and analyzed by WB. The results demonstrate that both the wild-type (wt) and mutant TUB proteins were almost exclusively localized in the nucleus (Figure 3D). This finding was also confirmed by confocal microscopy analysis that evidenced the nuclear localization of the TUB mutant (Figure 4A).
+Based on the documented role of TUB in early ciliogenesis [15], we assessed the localization of TUB at the cilium, but we failed to observe any consistent co-localization, possibly due to the low diffused levels of the protein in the cytoplasm To investigate the impact of defective TUB function on the morphogenesis of the primary cilium, a confocal analysis on primary fibroblasts was performed using antibodies against ARL13B, which localizes to primary cilia, and pericentrin, a component of the centrosome, which stains the basal body. As shown inFigure 4B, while almost all the control cells showed a primary cilium, 40% of the fibroblasts carrying the homozygous splice site variant inTUBdid not show a primary cilium. Moreover, while no significant difference was observed in ciliary axoneme length between the starved control and mutant cells, a large percentage of the latter showed an abnormal cilium morphology and a poorly defined and disorganized basal body (Figure 4C).
+The loss of TUB function was recently reported to underlie a novel IRD condition based on the identification of homozygosity for a 2 bp deletion (c.1194_1195delAG) causing the premature termination of the protein (p.Arg398Serfs*9) shared by three affected members of a single consanguineous family [10]. While the combination of retinal dystrophy and early onset obesity can be reminiscent of other disorders (e.g., Bardet–Biedl syndrome (MIM#PS209900) and Alstrom syndrome (MIM#203800)), the absence of other clinically relevant feature/sign was suggestive of a previously unreported ciliopathy [10]. In this paper, we report on a second disruptive variant (c.1387 + 1G &gt; A) affectingTUBin a subject with features that overlap with those previously described in the affected members of the original family.
+In the present and previously reported affected individuals, the ocular phenotype associated with defective TUB function is characterized by widespread retinal pigment epithelial (RPE) atrophy, deteriorating vision, the myopic and astigmatic refractive defect, the blonde fundus appearance, the ERG and OCT findings and progression of the disease (Figure 2). Notably, retinal detachment, without vitreous hemorrhage, was invariantly documented in the four individuals with biallelic inactivatingTUBvariants, suggesting that this feature likely represent a common finding in the disorder.
+Early onset obesity had previously been considered a major feature of the TUB-related condition [10], even though only two of three affected sibs were found obese (BMI &gt; 30), and the glycemic and lipid profiles in one of affected sibs were found within the normal range. The finding of obesity in the apparently healthy father (heterozygous carrier) suggests a possible co-occurring genetic event contributing to obesity in the family. In the present report, the clinical assessment of the affected individual documented increased weight (95.7 kg, +1.6 SD) and BMI (30.3, +1.6 SD), thus indicating overweight, in absence of other signs of obesity. Although evidence suggests that a defective TUB function may result in disturbances in insulin and leptin activity and obesity in mice [16,17,18,19], based on the collected findings, the relevance of TUB in human obesity requires further study. To assess whether TUB LoF could impact on hypothalamic pathways, food intake and adiposity, the metabolic profile of the affected individual was investigated. Accurate endocrinological examination did not reveal any abnormality, and the measurements of basal hormones by the anterior pituitary, glycaemia, insulin and leptin were within the normal range, thus ruling out insulin or leptin resistance. Consistently, instrumental investigations (X-ray and ultrasound analyses) documented no sign of glycogen accumulation in the internal organs. Consistently, the absence of significant changes in lipid storage was demonstrated by thin-layer chromatography (HPTLC) analysis in proband-derived fibroblast (Figure S1), allowing to confirm an apparently normal endocrine–metabolic profile in the affected individual. Of note, the Tubby protein has been involved in cochlear degeneration [20,21]. Based on this functional link, we evaluated the occurrence of hearing problems and cochlear degeneration, which were not observed.
+The homozygousTUBvariant was predicted to affect transcript processing, causing the skipping of exon 11 and intron retention, resulting in a frameshift with the premature termination of the TUB protein. mRNA analysis in proband-derived fibroblasts confirmed a disruptive impact of the splice site change documenting two aberrantly processed transcripts predicted to encode a 406-residue-long protein (p.Glu406Argfs*4) that probably is not able to proceed in protein synthesis, and a 481-residue-long protein (p.Pro463Hisfs*19) characterized by a divergent C-terminus characterized by accelerated degradation (Figure 3B). These findings confirm LoF as the pathomechanism underlying this disorder.
+Primary cilia are microtubule-based organelles that extend from the apical surface of the majority of mammalian cells. Cilia act as “cellular antennae”, receiving different inputs from the extracellular environment and transducing signals in response to stimuli [22]. A complex process required for proper cilia biogenesis function is the intraflagellar transport, which is required for assembling cilia and trafficking within primary cilia [23]. In this context, IFT-A has historically been believed to mediate retrograde intraflagellar transport inside the cilia and an IFT-A-binding domain at the TUB N-terminus has been demonstrated recently [24]. Moreover, co-localization between TUB and rootletin, the major structural component of the ciliary rootlet, has been observed in human retinal photoreceptors [10]. The use of a more informative in vitro model (e.g., induced pluripotent-stem-cell-derived retinal-pigment epithelium cells) and experimental strategies (e.g., siRNA-mediated TUB silencing) is required to appreciate more accurately the functional relevance of TUB in an appropriate cellular context.
+In summary, we confirm the link between TUB LoF and a new condition of human retinal ciliopathy and provide evidence of an altered cilium morphology/biogenesis in patient-derived fibroblasts. In fact, these cells displayed a reduced number of cilia when compared to the control cells, with a poorly defined and disorganized basal body structure, which are expected to prevent normal protein trafficking along the cilium. While these findings could explain the degeneration of photoreceptors characterizing this disorder, a relatively overall mild presentation has been associated with mutations in this gene. Multiple factors might contribute to this picture. First, the functional relevance of TUB in the context of ciliogenesis and cilium function might vary in different cell lineages. Second, functional compensation exerted by other related proteins might contribute to buffer the severity of the endophenotype. Third, specific cell lineages (e.g., rod and cone cells) might be particularly sensitive to TUB LoF. The collection of additional patients with biallelic variants in the gene will allow a more accurate characterization of the clinical spectrum associated with TUB LoF. Based on these considerations, TUB loss of function could be considered as responsible for a novel form of isolated retinal ciliopathy.</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>{
+"pmid": "9390831",
+"alias_symbol": "rd5",
+"primary_gene_symbol": "TUB",
+"name": "TUB bipartite transcription factor",
+"alternate_abbreviation": "NO",
+"evidence": ""
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HGNC:12406</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ENSG00000166402</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GENE ID:7275</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TUB</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>rd5</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>9390831</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>mouse phenotype biomarker</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Mice homozygous for a defect of the tub (rd5) gene exhibit cochlear and retinal degeneration combined with obesity, and resemble certain human autosomal recessive sensory deficit syndromes.</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>TUB bipartite transcription factor</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>In this paper, we confirm that biallelic inactivating variants in TUB cause a retinal disorder and functionally associate this condition with the occurrence of defects of the basal body structure and axoneme morphology of the primary cilium and overall defective ciliogenesis. Although the present findings suggest that TUB plays a role in the pathogenesis of retinal ciliopathies, dedicated functional studies are required to profile the mechanism of disease. This work confirms the clinical relevance of biallelic LoF variants ofTUB, which should be considered in clinical settings and the genetic diagnosis of IRD disorders.
+The present research followed the tenets of the Helsinki Declaration (1964 and further revisions) and the study was approved by the local ethics committee (Comitato Etico Centrale IRCCS Lazio, Sezione IFO/Fondazione Bietti, Rome, Italy). Upon recruitment in the study (FB RET-02-2019), executed from February to July 2019 at the IRCCS Fondazione Bietti, informed consent after full explanation was obtained from each subject included in the study.
+The proband and his family underwent comprehensive ophthalmological examination including visual acuity measured by the Early Treatment Diabetic Retinopathy Study (ETDRS) charts (Lighthouse, Low Vision Products, Long Island City, NY, USA) at the distance of 4 m and expressed as the logarithm of the minimum angle of resolution (logMAR); intraocular pressure (IOP) measurement; anterior segment observation by slit-lamp biomicroscopy and fundus examination by indirect ophthalmoscopic examination using + 90D non-contact lens (Volk Optical, Mentor, OH) after pupillary dilatation with tropicamide 1% drops. Goldmann visual field was assessed by kinetic Goldmann perimeter Haag-Streit 940. Chromatic test was evaluated by the monocular administration of Ishihara pseudoisochromatic plates (24 plates edition, Kanehara Trading Inc., Tokyo, Japan) in natural daylight. Electrophysiological assessment included dark-adapted and light-adapted full-field electroretinogram (Retimax Advanced Plus apparatus, CSO, Firenze, Italy) and multifocal electroretinogram (mfERG; VERIS Clinic TM version 4.9; Electro-Diagnostic Imaging, San Mateo, CA, USA) recordings according to the 2011 International Society for Clinical Electrophysiology of Vision (ISCEV) [25] by using the Dawson–Trick–Litzkow (DTL) contact electrodes and having the pupil dilated at 8 mm.
+Retinal imaging was executed by ultrawide field fundus photograph obtained with Optos California (Optos PLC, Dunfermline, Scotland, United Kingdom); FAF was also obtained during the same examination (488 nm excitation, barrier filter transmitted light from 500 to 680 nm, 55°) using Heidelberg Spectralis OCT (HRA + OCT, Heidelberg Engineering, Heidelberg, Germany). SD-OCT scan pattern was acquired with a minimum of a 20 × 20 degree rectangle centered on the fovea and 25-line B-scans spaced 235 μm apart and composed of 50 averaged frames by using the same instrument.
+Karyotype, CGH array and mutation scan by parallel sequencing considering a retinal cone–rod dystrophy panel of 70 genes were informative. Genomic DNA was collected after obtaining written informed consent. Whole-Exome sequencing (WES) and data analysis were performed as previously reported [26,27] (Supplementary Table S1). DNA of the affected subject and his parents was extracted from circulating leukocytes and sequenced using Illumina paired-end technology by means of SureSelect Human All Exon v.7 (Agilent, Santa Clara, CA, USA) kits. WES raw data were processed and analyzed using an in-house implemented pipeline as previously described [28,29], according to the GATK’s Best Practices [30]. The UCSC GRCh37/hg19 version of genome assembly was used as a reference for read alignment by means of BWA-MEM [31] tool and the subsequent variant calling with HaplotypeCaller (GATK v3.7) [28]. Variants’ functional annotation was made with the SnpEff v.5.0 [32] and dbNSFP v.4.2 [33] tools. Relevant in silico impact prediction tools, such as Combined Annotation Dependent Depletion (CADD) v.1.6 [34], Mendelian Clinically Applicable Pathogenicity (M-CAP) v.1.0 [35] and InterVar v.2.0.1 [36], were also used. By filtering against our population-matched database (~2500 WES) and public databases (dbSNP150 and gnomAD v.2.0.1), the analysis focused on high-quality rare variants that affect coding sequences and splice site regions. Sanger sequencing was performed for variant validation and segregation analysis (primers available upon request).
+Proband skin biopsy was obtained after informant consent was secured. Total RNA was extracted from the proband and healthy donor fibroblasts by using RNeasy Mini Kit (Qiagen, Hilden, Germany), according to the manufacturer’s recommendations. Total RNA concentration and quality were assessed by measuring the absorbance at 260 and 280 nm. Reverse transcription was carried out using a SuperScript RT reagent Kit (Invitrogen; ThermoFisher Scientific, Waltham, MA, USA). The obtained cDNA pools were amplified by PCR using specific primers located in exons 10 and 12 of theTUBgene, and PCR products were separated on a 2% agarose gel. The sequences of the primers are available upon request.
+Primary skin fibroblasts were cultured in DMEM supplemented with 10% heat-inactivated FBS, 2 mM glutamine, 100 units/mL of penicillin and 100 µg/mL of streptomycin, and maintained at 37 °C in a humidified atmosphere containing 5% CO2. After treatment, fibroblasts were lysed in RIPA buffer supplemented with phosphatase and protease inhibitors. Lysates were kept on ice (30 min) and then centrifuged at 16,000×g(20 min, 4 °C). Supernatants were collected and protein concentration was determined by Quick Start Bradford Dye Reagent (Bio-Rad Laboratories, Hercules, CA, USA), using bovine serum albumin (BSA) as a standard. Fibroblast homogenates were resolved by SDS PAGE and transferred to nitrocellulose membranes (Bio-Rad Laboratories). Blots were blocked for 1 h with 5% non-fat milk powder in phosphate-buffered saline (PBS) containing 0.1% Tween-20 and incubated overnight with specific antibodies. Anti-TUB primary polyclonal antibody (1:1000, Invitrogen; ThermoFisher Scientific) and goat anti-rabbit-HRP IgG secondary antibody (Invitrogen; ThermoFisher Scientific) were diluted in blocking solution. Immunoreactive proteins were detected by an ECL SuperSignal West Femto Maximum Sensitivity Chemiluminescent Substrate, according to the manufacturer’s instructions (Thermo Scientific, USA).
+Approximately 3 × 104/mL fibroblasts were seeded on glass coverslips and maintained in culture in complete medium for 24 h. Subconfluent fibroblasts were starved for 30 h and then fixed with 4% paraformaldehyde. Subsequently, cells were stained with rabbit anti-TUB (1:100 dilution), rabbit polyclonal anti-ARL13B (1:100, Abcam, Cambridge, UK) and mouse monoclonal anti-Pericentrin (1:100, Abcam) antibodies followed by goat anti-rabbit Alexa Fluor 488 and goat anti-mouse Alex Fluor 594, respectively (1:200 dilution; Molecular Probes, Eugene, OR, USA). After staining, coverslips were extensively rinsed and mounted onto microscope slides using Vectashield with DAPI mounting medium (Vector Laboratories, Newark, CA, USA). Analyses were performed in three independent experiments on a Zeiss LSM980 (Zeiss, Oberkochen, Germany) using a 63×/1.4 N.A. oil objective and excitation spectral laser lines at 405, 488 and 594 nm. Five hundred cells were counted for each condition in each experiment, and axoneme length was measured for each cell by using Zen Blue 3.2 software. Image acquisition and processing were performed as previously reported [37].
+Control and mutated fibroblasts cultured in 150 cm2dishes were harvested using trypsin after reaching confluence, rinsed with phosphate-buffered saline (PBS) and pelleted by centrifugation. Cell pellets were resuspended in 1 mL 0.9% NaCl and 6 mL of chloroform/methanol (2:1, v/v) were added. Mixtures were vortexed vigorously and centrifuged at 1500×gfor 15 min; the aqueous phase was discarded and organic phase was dried under N2gas. Lipid extracts from 1.5 × 106cells were applied on high-performance thin-layer chromatography (HPTLC) silica gel 60 plates (Merck, Darmstadt, Germany). Neutral lipids were resolved using a solvent system of hexane/diethyl ether/acetic acid (70:30:1, v/v/v) and were detected by staining with an aqueous solution containing 3% cupric acetate and 8% phosphoric acid and subsequent charring at 140 °C for 10 min. Lipids were identified by the co-migration of commercially available standards.
+URLs.*Online Mendelian Inheritance in Man [OMIM],http://www.ncbi.nlm.nih.gov/omim/;
+NCBI Gene,http://www.ncbi.nlm.nih.gov/gene/;
+Picard tools,http://picard.sourceforge.net/;
+wAnnovar,http://wannovar.usc.edu/;
+dbSNP137,http://www.ncbi.nlm.nih.gov/projects/SNP/snp_summary.cgi/;
+1000 Genomes Project,http://www.1000genomes.org/;
+HapMap Project,http://hapmap.ncbi.nlm.nih.gov/;
+SMART,http://smart.embl-heidelberg.de/;
+Protein Data Bank [PDB],http://www.rcsb.org/pdb/home/home.do.
+Research for this study was supported by the Ministry of Health funding 5x1000 Fondazione G.B. Bietti funds—2016 to M.P. and Fondazione Roma; Bando Ricerca Indipendente ISS 2021–2023 to V.C., Istituto Superiore di Sanità; Italian Ministry of Health (CCR-2017-23669081 to M.T.), and Italian Ministry of Research (FOE_2019 to M.T.). The authors acknowledge Maria Luisa Alessi and Federica Petrocchi for technical help in the electrophysiological and perimetric evaluations, Serenella Venanzi for administrative assistance.
+Publisher’s Note:MDPI stays neutral with regard to jurisdictional claims in published maps and institutional affiliations.
+The following supporting information can be downloaded at:https://www.mdpi.com/article/10.3390/ijms232314656/s1.
+Click here for additional data file.
+Conceptualization, L.Z. and V.C.; methodology, C.M., E.S., S.C., L.B. and M.T. (Massimo Tatti); validation, E.C., L.B., C.M. and V.C.; bioinformatics analysis, A.C. and A.B.; investigation, L.Z., M.C., M.P. and E.C.; resources, M.V.; data curation, L.B., M.P., E.S., M.T. (Massimo Tatti), M.N. and V.C.; writing—original draft preparation, L.Z., V.C. and M.N.; writing—review and editing, M.N., E.S., M.C., M.T. (Marco Tartaglia) and V.C.; supervision, M.V. and M.T. (Marco Tartaglia); project administration, M.V., V.C. and M.T. (Marco Tartaglia); funding acquisition, M.V. and M.P. All authors have read and agreed to the published version of the manuscript.
+The study was conducted according to the guidelines of the Declaration of Helsinki and was approved by the local Institutional Ethical Committee of the IRCCS_Fondazione G.B. Bietti [Ret_02/2019].
+Signed informed consent was obtained from the participating family.
+Data that support the findings of this study are available from the corresponding authors upon request.
+The authors declare no conflict of interest.
+Family tree showing the segregation of the identified splice site change.
+Ocular phenotype of the proband right eye. (A) Ultrawide field color fundus photograph. (B) The 55° fundus autofluorescence. (C) Spectral-domain optical coherence tomography line horizontal scan. (D) Full-field dark-adapted electroretinogram. (E) Three-dimensional multifocal electroretinogram plot. (F) Goldmann kinetic visual field.
+Characterization of the pathogenicTUBvariant. (A) Transcript processing in primary skin fibroblasts from a healthy donor and from the proband carrying the homozygous splice site variant. Total RNA was extracted, reverse-transcribed and analyzed by PCR to resolve transcript processing. Two aberrant cDNA products were identified in mutated cells (left) compared to the expected length of the amplified fragment obtained from the control fibroblasts (right). (B) Schematic representation of aberrant transcript processing caused by the identified homozygous splice site change inTUB. (C) Western blot analysis of the TUB protein in patient’s fibroblasts and the control cells. Twenty, forty and sixty micrograms of whole cell extract were analyzed basally (left) and following 4 h treatment with 100 μM Mg132 (right) and probed with anti-TUB antibody (* indicates a non-specific product). (D) Expression of wild-type and mutant TUB protein was analyzed in the cytoplasmic and nuclear fractions were obtained from wild-type and mutated fibroblasts. Sixty micrograms of each fraction were analyzed by Western blot and then probed with anti-TUB antibody. Anti-YY1 and anti-HSP90 antibodies were used as the internal controls to assess the clarity of the different fractions (* indicates a non-specific product). Blots are representative of three experiments performed.
+TUB subcellular localization and cilium defects in cells with TUB LoF. (A) Thirty-hour-starved and PFA-fixed fibroblasts from a healthy donor and from the proband were analyzed by confocal microscopy for the localization of TUB using antibodies against TUB. (B) The presence and morphology of primary cilia in starved fibroblasts from the proband and a healthy donor. Cells were starved for 30 h and fixed with PFA 4%. Primary cilia were analyzed using antibodies against ARL13B (cilium axonemal, green) and pericentrin (basal body, red) to investigate morphogenesis. Nuclei are DAPI stained (blue). Bars correspond to 20 and 2 μm (left panels). (C) Histograms represent the percent value of presence/absence of cilium, normal/aberrant cilium morphology and normal/aberrant basal body structure and the length (μm) of axoneme. Five hundred cells were counted for each condition and axoneme length was measured. Imagines and bar plots are representative of three experiments performed. * indicate statistical significance forp&lt; 0.01 by using Student’sTtest.</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Mice homozygous for a defect of the tub (rd5) gene exhibit cochlear and retinal degeneration combined with obesity, and resemble certain human autosomal recessive sensory deficit syndromes. To establish the progressive nature of sensory cell loss associated with the tub gene, and to differentiate tub-related losses from those associated with the C57 background on which tub arose, we evaluated cochleas and retinas from tub/tub, tub/+, and +/+ mice, aged 2 weeks to 1 year by light and electron microscopy. Cochleas from mice of all three genotypes show progressive inner (IHC) and outer hair cell (OHC) loss. Relative to tub/+ and +/+ animals, however, tub homozygotes show accelerated OHC loss, affecting the extreme cochlear base (hook region) by 1 month, and the apex by 6 months. IHC loss in tub/tub animals is accelerated in the basal half of the cochlea, affecting the hook region by 6 months. Spiral ganglion cell losses were observed only in tub/tub mice, and only in the cochlear base. Retinas of tub/tub mice are abnormal at maturity, exhibiting shortened photoreceptor outer segments by 2 weeks, and progressive photoreceptor loss thereafter. Because the tub mutation causes degeneration of sensory cells in the ear and eye but has no other neurological effects, tubby mice hold unique promise for the study of human syndromic sensory loss.</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>PMID: 9390831
+Full Text: In this paper, we confirm that biallelic inactivating variants in TUB cause a retinal disorder and functionally associate this condition with the occurrence of defects of the basal body structure and axoneme morphology of the primary cilium and overall defective ciliogenesis. Although the present findings suggest that TUB plays a role in the pathogenesis of retinal ciliopathies, dedicated functional studies are required to profile the mechanism of disease. This work confirms the clinical relevance of biallelic LoF variants ofTUB, which should be considered in clinical settings and the genetic diagnosis of IRD disorders.
+The present research followed the tenets of the Helsinki Declaration (1964 and further revisions) and the study was approved by the local ethics committee (Comitato Etico Centrale IRCCS Lazio, Sezione IFO/Fondazione Bietti, Rome, Italy). Upon recruitment in the study (FB RET-02-2019), executed from February to July 2019 at the IRCCS Fondazione Bietti, informed consent after full explanation was obtained from each subject included in the study.
+The proband and his family underwent comprehensive ophthalmological examination including visual acuity measured by the Early Treatment Diabetic Retinopathy Study (ETDRS) charts (Lighthouse, Low Vision Products, Long Island City, NY, USA) at the distance of 4 m and expressed as the logarithm of the minimum angle of resolution (logMAR); intraocular pressure (IOP) measurement; anterior segment observation by slit-lamp biomicroscopy and fundus examination by indirect ophthalmoscopic examination using + 90D non-contact lens (Volk Optical, Mentor, OH) after pupillary dilatation with tropicamide 1% drops. Goldmann visual field was assessed by kinetic Goldmann perimeter Haag-Streit 940. Chromatic test was evaluated by the monocular administration of Ishihara pseudoisochromatic plates (24 plates edition, Kanehara Trading Inc., Tokyo, Japan) in natural daylight. Electrophysiological assessment included dark-adapted and light-adapted full-field electroretinogram (Retimax Advanced Plus apparatus, CSO, Firenze, Italy) and multifocal electroretinogram (mfERG; VERIS Clinic TM version 4.9; Electro-Diagnostic Imaging, San Mateo, CA, USA) recordings according to the 2011 International Society for Clinical Electrophysiology of Vision (ISCEV) [25] by using the Dawson–Trick–Litzkow (DTL) contact electrodes and having the pupil dilated at 8 mm.
+Retinal imaging was executed by ultrawide field fundus photograph obtained with Optos California (Optos PLC, Dunfermline, Scotland, United Kingdom); FAF was also obtained during the same examination (488 nm excitation, barrier filter transmitted light from 500 to 680 nm, 55°) using Heidelberg Spectralis OCT (HRA + OCT, Heidelberg Engineering, Heidelberg, Germany). SD-OCT scan pattern was acquired with a minimum of a 20 × 20 degree rectangle centered on the fovea and 25-line B-scans spaced 235 μm apart and composed of 50 averaged frames by using the same instrument.
+Karyotype, CGH array and mutation scan by parallel sequencing considering a retinal cone–rod dystrophy panel of 70 genes were informative. Genomic DNA was collected after obtaining written informed consent. Whole-Exome sequencing (WES) and data analysis were performed as previously reported [26,27] (Supplementary Table S1). DNA of the affected subject and his parents was extracted from circulating leukocytes and sequenced using Illumina paired-end technology by means of SureSelect Human All Exon v.7 (Agilent, Santa Clara, CA, USA) kits. WES raw data were processed and analyzed using an in-house implemented pipeline as previously described [28,29], according to the GATK’s Best Practices [30]. The UCSC GRCh37/hg19 version of genome assembly was used as a reference for read alignment by means of BWA-MEM [31] tool and the subsequent variant calling with HaplotypeCaller (GATK v3.7) [28]. Variants’ functional annotation was made with the SnpEff v.5.0 [32] and dbNSFP v.4.2 [33] tools. Relevant in silico impact prediction tools, such as Combined Annotation Dependent Depletion (CADD) v.1.6 [34], Mendelian Clinically Applicable Pathogenicity (M-CAP) v.1.0 [35] and InterVar v.2.0.1 [36], were also used. By filtering against our population-matched database (~2500 WES) and public databases (dbSNP150 and gnomAD v.2.0.1), the analysis focused on high-quality rare variants that affect coding sequences and splice site regions. Sanger sequencing was performed for variant validation and segregation analysis (primers available upon request).
+Proband skin biopsy was obtained after informant consent was secured. Total RNA was extracted from the proband and healthy donor fibroblasts by using RNeasy Mini Kit (Qiagen, Hilden, Germany), according to the manufacturer’s recommendations. Total RNA concentration and quality were assessed by measuring the absorbance at 260 and 280 nm. Reverse transcription was carried out using a SuperScript RT reagent Kit (Invitrogen; ThermoFisher Scientific, Waltham, MA, USA). The obtained cDNA pools were amplified by PCR using specific primers located in exons 10 and 12 of theTUBgene, and PCR products were separated on a 2% agarose gel. The sequences of the primers are available upon request.
+Primary skin fibroblasts were cultured in DMEM supplemented with 10% heat-inactivated FBS, 2 mM glutamine, 100 units/mL of penicillin and 100 µg/mL of streptomycin, and maintained at 37 °C in a humidified atmosphere containing 5% CO2. After treatment, fibroblasts were lysed in RIPA buffer supplemented with phosphatase and protease inhibitors. Lysates were kept on ice (30 min) and then centrifuged at 16,000×g(20 min, 4 °C). Supernatants were collected and protein concentration was determined by Quick Start Bradford Dye Reagent (Bio-Rad Laboratories, Hercules, CA, USA), using bovine serum albumin (BSA) as a standard. Fibroblast homogenates were resolved by SDS PAGE and transferred to nitrocellulose membranes (Bio-Rad Laboratories). Blots were blocked for 1 h with 5% non-fat milk powder in phosphate-buffered saline (PBS) containing 0.1% Tween-20 and incubated overnight with specific antibodies. Anti-TUB primary polyclonal antibody (1:1000, Invitrogen; ThermoFisher Scientific) and goat anti-rabbit-HRP IgG secondary antibody (Invitrogen; ThermoFisher Scientific) were diluted in blocking solution. Immunoreactive proteins were detected by an ECL SuperSignal West Femto Maximum Sensitivity Chemiluminescent Substrate, according to the manufacturer’s instructions (Thermo Scientific, USA).
+Approximately 3 × 104/mL fibroblasts were seeded on glass coverslips and maintained in culture in complete medium for 24 h. Subconfluent fibroblasts were starved for 30 h and then fixed with 4% paraformaldehyde. Subsequently, cells were stained with rabbit anti-TUB (1:100 dilution), rabbit polyclonal anti-ARL13B (1:100, Abcam, Cambridge, UK) and mouse monoclonal anti-Pericentrin (1:100, Abcam) antibodies followed by goat anti-rabbit Alexa Fluor 488 and goat anti-mouse Alex Fluor 594, respectively (1:200 dilution; Molecular Probes, Eugene, OR, USA). After staining, coverslips were extensively rinsed and mounted onto microscope slides using Vectashield with DAPI mounting medium (Vector Laboratories, Newark, CA, USA). Analyses were performed in three independent experiments on a Zeiss LSM980 (Zeiss, Oberkochen, Germany) using a 63×/1.4 N.A. oil objective and excitation spectral laser lines at 405, 488 and 594 nm. Five hundred cells were counted for each condition in each experiment, and axoneme length was measured for each cell by using Zen Blue 3.2 software. Image acquisition and processing were performed as previously reported [37].
+Control and mutated fibroblasts cultured in 150 cm2dishes were harvested using trypsin after reaching confluence, rinsed with phosphate-buffered saline (PBS) and pelleted by centrifugation. Cell pellets were resuspended in 1 mL 0.9% NaCl and 6 mL of chloroform/methanol (2:1, v/v) were added. Mixtures were vortexed vigorously and centrifuged at 1500×gfor 15 min; the aqueous phase was discarded and organic phase was dried under N2gas. Lipid extracts from 1.5 × 106cells were applied on high-performance thin-layer chromatography (HPTLC) silica gel 60 plates (Merck, Darmstadt, Germany). Neutral lipids were resolved using a solvent system of hexane/diethyl ether/acetic acid (70:30:1, v/v/v) and were detected by staining with an aqueous solution containing 3% cupric acetate and 8% phosphoric acid and subsequent charring at 140 °C for 10 min. Lipids were identified by the co-migration of commercially available standards.
+URLs.*Online Mendelian Inheritance in Man [OMIM],http://www.ncbi.nlm.nih.gov/omim/;
+NCBI Gene,http://www.ncbi.nlm.nih.gov/gene/;
+Picard tools,http://picard.sourceforge.net/;
+wAnnovar,http://wannovar.usc.edu/;
+dbSNP137,http://www.ncbi.nlm.nih.gov/projects/SNP/snp_summary.cgi/;
+1000 Genomes Project,http://www.1000genomes.org/;
+HapMap Project,http://hapmap.ncbi.nlm.nih.gov/;
+SMART,http://smart.embl-heidelberg.de/;
+Protein Data Bank [PDB],http://www.rcsb.org/pdb/home/home.do.
+Research for this study was supported by the Ministry of Health funding 5x1000 Fondazione G.B. Bietti funds—2016 to M.P. and Fondazione Roma; Bando Ricerca Indipendente ISS 2021–2023 to V.C., Istituto Superiore di Sanità; Italian Ministry of Health (CCR-2017-23669081 to M.T.), and Italian Ministry of Research (FOE_2019 to M.T.). The authors acknowledge Maria Luisa Alessi and Federica Petrocchi for technical help in the electrophysiological and perimetric evaluations, Serenella Venanzi for administrative assistance.
+Publisher’s Note:MDPI stays neutral with regard to jurisdictional claims in published maps and institutional affiliations.
+The following supporting information can be downloaded at:https://www.mdpi.com/article/10.3390/ijms232314656/s1.
+Click here for additional data file.
+Conceptualization, L.Z. and V.C.; methodology, C.M., E.S., S.C., L.B. and M.T. (Massimo Tatti); validation, E.C., L.B., C.M. and V.C.; bioinformatics analysis, A.C. and A.B.; investigation, L.Z., M.C., M.P. and E.C.; resources, M.V.; data curation, L.B., M.P., E.S., M.T. (Massimo Tatti), M.N. and V.C.; writing—original draft preparation, L.Z., V.C. and M.N.; writing—review and editing, M.N., E.S., M.C., M.T. (Marco Tartaglia) and V.C.; supervision, M.V. and M.T. (Marco Tartaglia); project administration, M.V., V.C. and M.T. (Marco Tartaglia); funding acquisition, M.V. and M.P. All authors have read and agreed to the published version of the manuscript.
+The study was conducted according to the guidelines of the Declaration of Helsinki and was approved by the local Institutional Ethical Committee of the IRCCS_Fondazione G.B. Bietti [Ret_02/2019].
+Signed informed consent was obtained from the participating family.
+Data that support the findings of this study are available from the corresponding authors upon request.
+The authors declare no conflict of interest.
+Family tree showing the segregation of the identified splice site change.
+Ocular phenotype of the proband right eye. (A) Ultrawide field color fundus photograph. (B) The 55° fundus autofluorescence. (C) Spectral-domain optical coherence tomography line horizontal scan. (D) Full-field dark-adapted electroretinogram. (E) Three-dimensional multifocal electroretinogram plot. (F) Goldmann kinetic visual field.
+Characterization of the pathogenicTUBvariant. (A) Transcript processing in primary skin fibroblasts from a healthy donor and from the proband carrying the homozygous splice site variant. Total RNA was extracted, reverse-transcribed and analyzed by PCR to resolve transcript processing. Two aberrant cDNA products were identified in mutated cells (left) compared to the expected length of the amplified fragment obtained from the control fibroblasts (right). (B) Schematic representation of aberrant transcript processing caused by the identified homozygous splice site change inTUB. (C) Western blot analysis of the TUB protein in patient’s fibroblasts and the control cells. Twenty, forty and sixty micrograms of whole cell extract were analyzed basally (left) and following 4 h treatment with 100 μM Mg132 (right) and probed with anti-TUB antibody (* indicates a non-specific product). (D) Expression of wild-type and mutant TUB protein was analyzed in the cytoplasmic and nuclear fractions were obtained from wild-type and mutated fibroblasts. Sixty micrograms of each fraction were analyzed by Western blot and then probed with anti-TUB antibody. Anti-YY1 and anti-HSP90 antibodies were used as the internal controls to assess the clarity of the different fractions (* indicates a non-specific product). Blots are representative of three experiments performed.
+TUB subcellular localization and cilium defects in cells with TUB LoF. (A) Thirty-hour-starved and PFA-fixed fibroblasts from a healthy donor and from the proband were analyzed by confocal microscopy for the localization of TUB using antibodies against TUB. (B) The presence and morphology of primary cilia in starved fibroblasts from the proband and a healthy donor. Cells were starved for 30 h and fixed with PFA 4%. Primary cilia were analyzed using antibodies against ARL13B (cilium axonemal, green) and pericentrin (basal body, red) to investigate morphogenesis. Nuclei are DAPI stained (blue). Bars correspond to 20 and 2 μm (left panels). (C) Histograms represent the percent value of presence/absence of cilium, normal/aberrant cilium morphology and normal/aberrant basal body structure and the length (μm) of axoneme. Five hundred cells were counted for each condition and axoneme length was measured. Imagines and bar plots are representative of three experiments performed. * indicate statistical significance forp&lt; 0.01 by using Student’sTtest.</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
+    Inputs:
+    Alias gene symbol: rd5
+    HGNC record ID: HGNC:12406
+    Primary gene symbol: TUB
+    Official HGNC gene name: TUB bipartite transcription factor
+    Biomedical text context
+    Task:
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
+    Rules:
+    If the text does not support that the alias is an alternate abbreviation, return:
+    "alternate_abbreviation": "NO"
+    "evidence": ""
+    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
+    Evidence must be one exact sentence copied verbatim from the text.
+    Do not infer relationships or paraphrase evidence.
+    Output (Strict):
+    Output only one JSON object. No markdown.
+    {
+    "pmid": "",
+    "alias_symbol": "",
+    "primary_gene_symbol": "",
+    "name": "",
+    "alternate_abbreviation": "YES or NO",
+    "evidence": ""
+    }
+PMID: 9390831
+Full Text: In this paper, we confirm that biallelic inactivating variants in TUB cause a retinal disorder and functionally associate this condition with the occurrence of defects of the basal body structure and axoneme morphology of the primary cilium and overall defective ciliogenesis. Although the present findings suggest that TUB plays a role in the pathogenesis of retinal ciliopathies, dedicated functional studies are required to profile the mechanism of disease. This work confirms the clinical relevance of biallelic LoF variants ofTUB, which should be considered in clinical settings and the genetic diagnosis of IRD disorders.
+The present research followed the tenets of the Helsinki Declaration (1964 and further revisions) and the study was approved by the local ethics committee (Comitato Etico Centrale IRCCS Lazio, Sezione IFO/Fondazione Bietti, Rome, Italy). Upon recruitment in the study (FB RET-02-2019), executed from February to July 2019 at the IRCCS Fondazione Bietti, informed consent after full explanation was obtained from each subject included in the study.
+The proband and his family underwent comprehensive ophthalmological examination including visual acuity measured by the Early Treatment Diabetic Retinopathy Study (ETDRS) charts (Lighthouse, Low Vision Products, Long Island City, NY, USA) at the distance of 4 m and expressed as the logarithm of the minimum angle of resolution (logMAR); intraocular pressure (IOP) measurement; anterior segment observation by slit-lamp biomicroscopy and fundus examination by indirect ophthalmoscopic examination using + 90D non-contact lens (Volk Optical, Mentor, OH) after pupillary dilatation with tropicamide 1% drops. Goldmann visual field was assessed by kinetic Goldmann perimeter Haag-Streit 940. Chromatic test was evaluated by the monocular administration of Ishihara pseudoisochromatic plates (24 plates edition, Kanehara Trading Inc., Tokyo, Japan) in natural daylight. Electrophysiological assessment included dark-adapted and light-adapted full-field electroretinogram (Retimax Advanced Plus apparatus, CSO, Firenze, Italy) and multifocal electroretinogram (mfERG; VERIS Clinic TM version 4.9; Electro-Diagnostic Imaging, San Mateo, CA, USA) recordings according to the 2011 International Society for Clinical Electrophysiology of Vision (ISCEV) [25] by using the Dawson–Trick–Litzkow (DTL) contact electrodes and having the pupil dilated at 8 mm.
+Retinal imaging was executed by ultrawide field fundus photograph obtained with Optos California (Optos PLC, Dunfermline, Scotland, United Kingdom); FAF was also obtained during the same examination (488 nm excitation, barrier filter transmitted light from 500 to 680 nm, 55°) using Heidelberg Spectralis OCT (HRA + OCT, Heidelberg Engineering, Heidelberg, Germany). SD-OCT scan pattern was acquired with a minimum of a 20 × 20 degree rectangle centered on the fovea and 25-line B-scans spaced 235 μm apart and composed of 50 averaged frames by using the same instrument.
+Karyotype, CGH array and mutation scan by parallel sequencing considering a retinal cone–rod dystrophy panel of 70 genes were informative. Genomic DNA was collected after obtaining written informed consent. Whole-Exome sequencing (WES) and data analysis were performed as previously reported [26,27] (Supplementary Table S1). DNA of the affected subject and his parents was extracted from circulating leukocytes and sequenced using Illumina paired-end technology by means of SureSelect Human All Exon v.7 (Agilent, Santa Clara, CA, USA) kits. WES raw data were processed and analyzed using an in-house implemented pipeline as previously described [28,29], according to the GATK’s Best Practices [30]. The UCSC GRCh37/hg19 version of genome assembly was used as a reference for read alignment by means of BWA-MEM [31] tool and the subsequent variant calling with HaplotypeCaller (GATK v3.7) [28]. Variants’ functional annotation was made with the SnpEff v.5.0 [32] and dbNSFP v.4.2 [33] tools. Relevant in silico impact prediction tools, such as Combined Annotation Dependent Depletion (CADD) v.1.6 [34], Mendelian Clinically Applicable Pathogenicity (M-CAP) v.1.0 [35] and InterVar v.2.0.1 [36], were also used. By filtering against our population-matched database (~2500 WES) and public databases (dbSNP150 and gnomAD v.2.0.1), the analysis focused on high-quality rare variants that affect coding sequences and splice site regions. Sanger sequencing was performed for variant validation and segregation analysis (primers available upon request).
+Proband skin biopsy was obtained after informant consent was secured. Total RNA was extracted from the proband and healthy donor fibroblasts by using RNeasy Mini Kit (Qiagen, Hilden, Germany), according to the manufacturer’s recommendations. Total RNA concentration and quality were assessed by measuring the absorbance at 260 and 280 nm. Reverse transcription was carried out using a SuperScript RT reagent Kit (Invitrogen; ThermoFisher Scientific, Waltham, MA, USA). The obtained cDNA pools were amplified by PCR using specific primers located in exons 10 and 12 of theTUBgene, and PCR products were separated on a 2% agarose gel. The sequences of the primers are available upon request.
+Primary skin fibroblasts were cultured in DMEM supplemented with 10% heat-inactivated FBS, 2 mM glutamine, 100 units/mL of penicillin and 100 µg/mL of streptomycin, and maintained at 37 °C in a humidified atmosphere containing 5% CO2. After treatment, fibroblasts were lysed in RIPA buffer supplemented with phosphatase and protease inhibitors. Lysates were kept on ice (30 min) and then centrifuged at 16,000×g(20 min, 4 °C). Supernatants were collected and protein concentration was determined by Quick Start Bradford Dye Reagent (Bio-Rad Laboratories, Hercules, CA, USA), using bovine serum albumin (BSA) as a standard. Fibroblast homogenates were resolved by SDS PAGE and transferred to nitrocellulose membranes (Bio-Rad Laboratories). Blots were blocked for 1 h with 5% non-fat milk powder in phosphate-buffered saline (PBS) containing 0.1% Tween-20 and incubated overnight with specific antibodies. Anti-TUB primary polyclonal antibody (1:1000, Invitrogen; ThermoFisher Scientific) and goat anti-rabbit-HRP IgG secondary antibody (Invitrogen; ThermoFisher Scientific) were diluted in blocking solution. Immunoreactive proteins were detected by an ECL SuperSignal West Femto Maximum Sensitivity Chemiluminescent Substrate, according to the manufacturer’s instructions (Thermo Scientific, USA).
+Approximately 3 × 104/mL fibroblasts were seeded on glass coverslips and maintained in culture in complete medium for 24 h. Subconfluent fibroblasts were starved for 30 h and then fixed with 4% paraformaldehyde. Subsequently, cells were stained with rabbit anti-TUB (1:100 dilution), rabbit polyclonal anti-ARL13B (1:100, Abcam, Cambridge, UK) and mouse monoclonal anti-Pericentrin (1:100, Abcam) antibodies followed by goat anti-rabbit Alexa Fluor 488 and goat anti-mouse Alex Fluor 594, respectively (1:200 dilution; Molecular Probes, Eugene, OR, USA). After staining, coverslips were extensively rinsed and mounted onto microscope slides using Vectashield with DAPI mounting medium (Vector Laboratories, Newark, CA, USA). Analyses were performed in three independent experiments on a Zeiss LSM980 (Zeiss, Oberkochen, Germany) using a 63×/1.4 N.A. oil objective and excitation spectral laser lines at 405, 488 and 594 nm. Five hundred cells were counted for each condition in each experiment, and axoneme length was measured for each cell by using Zen Blue 3.2 software. Image acquisition and processing were performed as previously reported [37].
+Control and mutated fibroblasts cultured in 150 cm2dishes were harvested using trypsin after reaching confluence, rinsed with phosphate-buffered saline (PBS) and pelleted by centrifugation. Cell pellets were resuspended in 1 mL 0.9% NaCl and 6 mL of chloroform/methanol (2:1, v/v) were added. Mixtures were vortexed vigorously and centrifuged at 1500×gfor 15 min; the aqueous phase was discarded and organic phase was dried under N2gas. Lipid extracts from 1.5 × 106cells were applied on high-performance thin-layer chromatography (HPTLC) silica gel 60 plates (Merck, Darmstadt, Germany). Neutral lipids were resolved using a solvent system of hexane/diethyl ether/acetic acid (70:30:1, v/v/v) and were detected by staining with an aqueous solution containing 3% cupric acetate and 8% phosphoric acid and subsequent charring at 140 °C for 10 min. Lipids were identified by the co-migration of commercially available standards.
+URLs.*Online Mendelian Inheritance in Man [OMIM],http://www.ncbi.nlm.nih.gov/omim/;
+NCBI Gene,http://www.ncbi.nlm.nih.gov/gene/;
+Picard tools,http://picard.sourceforge.net/;
+wAnnovar,http://wannovar.usc.edu/;
+dbSNP137,http://www.ncbi.nlm.nih.gov/projects/SNP/snp_summary.cgi/;
+1000 Genomes Project,http://www.1000genomes.org/;
+HapMap Project,http://hapmap.ncbi.nlm.nih.gov/;
+SMART,http://smart.embl-heidelberg.de/;
+Protein Data Bank [PDB],http://www.rcsb.org/pdb/home/home.do.
+Research for this study was supported by the Ministry of Health funding 5x1000 Fondazione G.B. Bietti funds—2016 to M.P. and Fondazione Roma; Bando Ricerca Indipendente ISS 2021–2023 to V.C., Istituto Superiore di Sanità; Italian Ministry of Health (CCR-2017-23669081 to M.T.), and Italian Ministry of Research (FOE_2019 to M.T.). The authors acknowledge Maria Luisa Alessi and Federica Petrocchi for technical help in the electrophysiological and perimetric evaluations, Serenella Venanzi for administrative assistance.
+Publisher’s Note:MDPI stays neutral with regard to jurisdictional claims in published maps and institutional affiliations.
+The following supporting information can be downloaded at:https://www.mdpi.com/article/10.3390/ijms232314656/s1.
+Click here for additional data file.
+Conceptualization, L.Z. and V.C.; methodology, C.M., E.S., S.C., L.B. and M.T. (Massimo Tatti); validation, E.C., L.B., C.M. and V.C.; bioinformatics analysis, A.C. and A.B.; investigation, L.Z., M.C., M.P. and E.C.; resources, M.V.; data curation, L.B., M.P., E.S., M.T. (Massimo Tatti), M.N. and V.C.; writing—original draft preparation, L.Z., V.C. and M.N.; writing—review and editing, M.N., E.S., M.C., M.T. (Marco Tartaglia) and V.C.; supervision, M.V. and M.T. (Marco Tartaglia); project administration, M.V., V.C. and M.T. (Marco Tartaglia); funding acquisition, M.V. and M.P. All authors have read and agreed to the published version of the manuscript.
+The study was conducted according to the guidelines of the Declaration of Helsinki and was approved by the local Institutional Ethical Committee of the IRCCS_Fondazione G.B. Bietti [Ret_02/2019].
+Signed informed consent was obtained from the participating family.
+Data that support the findings of this study are available from the corresponding authors upon request.
+The authors declare no conflict of interest.
+Family tree showing the segregation of the identified splice site change.
+Ocular phenotype of the proband right eye. (A) Ultrawide field color fundus photograph. (B) The 55° fundus autofluorescence. (C) Spectral-domain optical coherence tomography line horizontal scan. (D) Full-field dark-adapted electroretinogram. (E) Three-dimensional multifocal electroretinogram plot. (F) Goldmann kinetic visual field.
+Characterization of the pathogenicTUBvariant. (A) Transcript processing in primary skin fibroblasts from a healthy donor and from the proband carrying the homozygous splice site variant. Total RNA was extracted, reverse-transcribed and analyzed by PCR to resolve transcript processing. Two aberrant cDNA products were identified in mutated cells (left) compared to the expected length of the amplified fragment obtained from the control fibroblasts (right). (B) Schematic representation of aberrant transcript processing caused by the identified homozygous splice site change inTUB. (C) Western blot analysis of the TUB protein in patient’s fibroblasts and the control cells. Twenty, forty and sixty micrograms of whole cell extract were analyzed basally (left) and following 4 h treatment with 100 μM Mg132 (right) and probed with anti-TUB antibody (* indicates a non-specific product). (D) Expression of wild-type and mutant TUB protein was analyzed in the cytoplasmic and nuclear fractions were obtained from wild-type and mutated fibroblasts. Sixty micrograms of each fraction were analyzed by Western blot and then probed with anti-TUB antibody. Anti-YY1 and anti-HSP90 antibodies were used as the internal controls to assess the clarity of the different fractions (* indicates a non-specific product). Blots are representative of three experiments performed.
+TUB subcellular localization and cilium defects in cells with TUB LoF. (A) Thirty-hour-starved and PFA-fixed fibroblasts from a healthy donor and from the proband were analyzed by confocal microscopy for the localization of TUB using antibodies against TUB. (B) The presence and morphology of primary cilia in starved fibroblasts from the proband and a healthy donor. Cells were starved for 30 h and fixed with PFA 4%. Primary cilia were analyzed using antibodies against ARL13B (cilium axonemal, green) and pericentrin (basal body, red) to investigate morphogenesis. Nuclei are DAPI stained (blue). Bars correspond to 20 and 2 μm (left panels). (C) Histograms represent the percent value of presence/absence of cilium, normal/aberrant cilium morphology and normal/aberrant basal body structure and the length (μm) of axoneme. Five hundred cells were counted for each condition and axoneme length was measured. Imagines and bar plots are representative of three experiments performed. * indicate statistical significance forp&lt; 0.01 by using Student’sTtest.</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Based on the provided text, I cannot confirm that "rd5" is an alternate abbreviation for the TUB gene. The text does not explicitly link "rd5" to TUB or expand it to the official gene name "TUB bipartite transcription factor". Therefore, I will classify this as not an alternate abbreviation.
+Here is the JSON output:
+{
+"pmid": "9390831",
+"alias_symbol": "rd5",
+"primary_gene_symbol": "TUB",
+"name": "TUB bipartite transcription factor",
+"alternate_abbreviation": "NO",
+"evidence": ""
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HGNC:12406</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ENSG00000166402</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GENE ID:7275</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>TUB</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>rd5</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>9477305</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>mouse phenotype biomarker</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>discussion</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities.</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>TUB bipartite transcription factor</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Some genetic syndromes causing loss of hearing and vision, such as some forms of Usher's syndrome, also cause reduced sperm cell motility, bronchiectasis, and other pathologies involving cilia- and flagella-bearing cells. In some Usher's patients, ultrastructural defects of axonemes within photoreceptor ciliary bridges, nasal cilia, and sperm cell flagella have been found, indicating a primary defect of axonemal conformation. Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities. They provide a good phenotypic match to human genetic sensory syndromes, particularly human sensory/obesity syndromes, such as Alstrom's and Bardet/Biedl, although no human candidate genes have been identified. Because of their unique phenotype, tubby mice are an appropriate model in which to look for a primary axonemal defect. We studied the axonemal ultrastructure of photoreceptors and sperm cells and performed functional testing of sperm in tub/tub mice before and after the onset of obesity. Approximately 15% of photoreceptor axonemes appeared abnormal in tub/tub animals, compared to 0% in controls. Both tub homozygotes and controls exhibited approximately 10% abnormal sperm cell axonemes, and no differences in sperm cell motile function were found at any age. The modest occurrence of axonemal defects in photoreceptors of tub/tub animals is likely to be a secondary effect of retinal degeneration. We conclude that the tubby phenotype is not associated with a generalized defect of cilia- and flagella-bearing cells and that the tub mutation does not primarily affect axonemal structure.</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>PMID: 9477305
+Abstract: Some genetic syndromes causing loss of hearing and vision, such as some forms of Usher's syndrome, also cause reduced sperm cell motility, bronchiectasis, and other pathologies involving cilia- and flagella-bearing cells. In some Usher's patients, ultrastructural defects of axonemes within photoreceptor ciliary bridges, nasal cilia, and sperm cell flagella have been found, indicating a primary defect of axonemal conformation. Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities. They provide a good phenotypic match to human genetic sensory syndromes, particularly human sensory/obesity syndromes, such as Alstrom's and Bardet/Biedl, although no human candidate genes have been identified. Because of their unique phenotype, tubby mice are an appropriate model in which to look for a primary axonemal defect. We studied the axonemal ultrastructure of photoreceptors and sperm cells and performed functional testing of sperm in tub/tub mice before and after the onset of obesity. Approximately 15% of photoreceptor axonemes appeared abnormal in tub/tub animals, compared to 0% in controls. Both tub homozygotes and controls exhibited approximately 10% abnormal sperm cell axonemes, and no differences in sperm cell motile function were found at any age. The modest occurrence of axonemal defects in photoreceptors of tub/tub animals is likely to be a secondary effect of retinal degeneration. We conclude that the tubby phenotype is not associated with a generalized defect of cilia- and flagella-bearing cells and that the tub mutation does not primarily affect axonemal structure.</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
+    Inputs:
+    Alias gene symbol: rd5
+    HGNC record ID: HGNC:12406
+    Primary gene symbol: TUB
+    Official HGNC gene name: TUB bipartite transcription factor
+    Biomedical text context
+    Task:
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
+    Rules:
+    If the text does not support that the alias is an alternate abbreviation, return:
+    "alternate_abbreviation": "NO"
+    "evidence": ""
+    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
+    Evidence must be one exact sentence copied verbatim from the text.
+    Do not infer relationships or paraphrase evidence.
+    Output (Strict):
+    Output only one JSON object. No markdown.
+    {
+    "pmid": "",
+    "alias_symbol": "",
+    "primary_gene_symbol": "",
+    "name": "",
+    "alternate_abbreviation": "YES or NO",
+    "evidence": ""
+    }
+PMID: 9477305
+Abstract: Some genetic syndromes causing loss of hearing and vision, such as some forms of Usher's syndrome, also cause reduced sperm cell motility, bronchiectasis, and other pathologies involving cilia- and flagella-bearing cells. In some Usher's patients, ultrastructural defects of axonemes within photoreceptor ciliary bridges, nasal cilia, and sperm cell flagella have been found, indicating a primary defect of axonemal conformation. Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities. They provide a good phenotypic match to human genetic sensory syndromes, particularly human sensory/obesity syndromes, such as Alstrom's and Bardet/Biedl, although no human candidate genes have been identified. Because of their unique phenotype, tubby mice are an appropriate model in which to look for a primary axonemal defect. We studied the axonemal ultrastructure of photoreceptors and sperm cells and performed functional testing of sperm in tub/tub mice before and after the onset of obesity. Approximately 15% of photoreceptor axonemes appeared abnormal in tub/tub animals, compared to 0% in controls. Both tub homozygotes and controls exhibited approximately 10% abnormal sperm cell axonemes, and no differences in sperm cell motile function were found at any age. The modest occurrence of axonemal defects in photoreceptors of tub/tub animals is likely to be a secondary effect of retinal degeneration. We conclude that the tubby phenotype is not associated with a generalized defect of cilia- and flagella-bearing cells and that the tub mutation does not primarily affect axonemal structure.</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>{
+"pmid": "9477305",
+"alias_symbol": "rd5",
+"primary_gene_symbol": "TUB",
+"name": "TUB bipartite transcription factor",
+"alternate_abbreviation": "YES",
+"evidence": "Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities."
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HGNC:12406</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ENSG00000166402</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GENE ID:7275</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>TUB</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>rd5</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>36612533</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>primer</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>methods</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>The primers were as follows: forward primer RD5 5_-ATC TGG TTG ATC CTG CCA GT-3_ and reverse primer BhRDr 5_-GAG CTT TTTA ACT GCA ACA ACG-3_</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>TUB bipartite transcription factor</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
         <is>
           <t>Blastocystisis one of the most common enteric protozoa that inhabits the intestinal tract of humans and different animals. Moreover, it has a worldwide geographic distribution. Its main mode of transmission is via the fecal-oral route. At present, 26 subtypes are widely distributed across both humans and animals. The current study aimed to determine the prevalence and subtype distribution ofBlastocystisamong school-aged children living on the Thai-Myanmar border, Ratchaburi province, Thailand. In total, 508 samples were collected from children at six schools. The prevalence ofBlastocystisinfection was amplified and sequenced in the 600 bp barcode region of the small-subunit ribosomal RNA (SSU rRNA). The overall prevalence ofBlastocystisinfection was 3.35% (17/508). ST3 (11/17) was the most predominant subtype, followed by ST1 (5/17) and ST2 (1/17). A phylogenetic tree was constructed based on the Tamura92+G+I model using the maximum-likelihood algorithm. Surprisingly, all sequences of the ST3-positive samples were closely correlated with the cattle-derived sequence. Meanwhile, all sequences of theBlastocystisST1-positive samples were closely correlated with the human-derived sequence. Nevertheless, further studies should be conducted to validate the zoonotic transmission ofBlastocystis. Based on our findings, personal hygiene and sanitation should be improved to promote better health in children in this area.
 Intestinal parasitic infections are one of the main public health issues worldwide, and their incidence is higher in developing than in developed countries [1,2].Blastocystisis a common enteric protozoan causing parasitic intestinal infections among children. Further, it mainly colonizes the gastrointestinal tract, and it is transmitted via the fecal-oral route [3,4]. At present, approximately more than 1 billion humans are infected withBlastocystisworldwide [5]. Its transmission is correlated with several factors, such as poor personal hygiene, consumption of contaminated food, and environmental conditions associated with poor quality of life [6,7,8]. Moreover, close contact with animals due to cultural conditions may causeBlastocystisinfection [9,10,11]. Additionally, school-aged children are at high risk ofBlastocystisinfection due to poor hygiene habits [1,4]. Several studies showed that the prevalence ofBlastocystisinfection varies from 0.7% to 45.2% among school-aged children in Thailand [12,13,14,15]. At present, 26 subtypes ofBlastocystisare widely distributed in both humans and animals. Among them, subtype 3 is most commonly observed in humans [16,17]. The methods used to detectBlastocystisare usually based on microscopy. However, these techniques have low sensitivity and specificity, and assessment using these strategies should be performed by skilled microscopists to validate morphology [18,19,20]. In recent years, polymerase chain reaction (PCR), a molecular biology technique, targets a region of the SSU rRNA genes. Moreover, it has the highest sensitivity and specificity and can identify different subtypes [21,22,23]. However, studies on the incidence and subtypes ofBlastocystisin school-aged children living in the border areas of Thailand are limited. The current study aimed to determine the prevalence and subtype distribution ofBlastocystisisolated from school-aged children living in the Thai-Myanmar border areas, Ratchaburi Province, Thailand.
@@ -648,12 +1412,12 @@
 Accession numbers of positive samples used in the phylogenetic reconstruction.</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>&lt;i&gt;Blastocystis&lt;/i&gt; is one of the most common enteric protozoa that inhabits the intestinal tract of humans and different animals. Moreover, it has a worldwide geographic distribution. Its main mode of transmission is via the fecal-oral route. At present, 26 subtypes are widely distributed across both humans and animals. The current study aimed to determine the prevalence and subtype distribution of &lt;i&gt;Blastocystis&lt;/i&gt; among school-aged children living on the Thai-Myanmar border, Ratchaburi province, Thailand. In total, 508 samples were collected from children at six schools. The prevalence of &lt;i&gt;Blastocystis&lt;/i&gt; infection was amplified and sequenced in the 600 bp barcode region of the small-subunit ribosomal RNA (SSU rRNA). The overall prevalence of &lt;i&gt;Blastocystis&lt;/i&gt; infection was 3.35% (17/508). ST3 (11/17) was the most predominant subtype, followed by ST1 (5/17) and ST2 (1/17). A phylogenetic tree was constructed based on the Tamura92+G+I model using the maximum-likelihood algorithm. Surprisingly, all sequences of the ST3-positive samples were closely correlated with the cattle-derived sequence. Meanwhile, all sequences of the &lt;i&gt;Blastocystis&lt;/i&gt; ST1-positive samples were closely correlated with the human-derived sequence. Nevertheless, further studies should be conducted to validate the zoonotic transmission of &lt;i&gt;Blastocystis&lt;/i&gt;. Based on our findings, personal hygiene and sanitation should be improved to promote better health in children in this area.</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>PMID: 36612533
 Full Text: Blastocystisis one of the most common enteric protozoa that inhabits the intestinal tract of humans and different animals. Moreover, it has a worldwide geographic distribution. Its main mode of transmission is via the fecal-oral route. At present, 26 subtypes are widely distributed across both humans and animals. The current study aimed to determine the prevalence and subtype distribution ofBlastocystisamong school-aged children living on the Thai-Myanmar border, Ratchaburi province, Thailand. In total, 508 samples were collected from children at six schools. The prevalence ofBlastocystisinfection was amplified and sequenced in the 600 bp barcode region of the small-subunit ribosomal RNA (SSU rRNA). The overall prevalence ofBlastocystisinfection was 3.35% (17/508). ST3 (11/17) was the most predominant subtype, followed by ST1 (5/17) and ST2 (1/17). A phylogenetic tree was constructed based on the Tamura92+G+I model using the maximum-likelihood algorithm. Surprisingly, all sequences of the ST3-positive samples were closely correlated with the cattle-derived sequence. Meanwhile, all sequences of theBlastocystisST1-positive samples were closely correlated with the human-derived sequence. Nevertheless, further studies should be conducted to validate the zoonotic transmission ofBlastocystis. Based on our findings, personal hygiene and sanitation should be improved to promote better health in children in this area.
@@ -684,7 +1448,7 @@
 Accession numbers of positive samples used in the phylogenetic reconstruction.</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -692,35 +1456,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -753,95 +1525,94 @@
 Accession numbers of positive samples used in the phylogenetic reconstruction.</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>{
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Based on the provided text, here is my analysis:
+{
 "pmid": "36612533",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"alternate_abbreviation": "NO",
 "evidence": ""
-}</t>
+}
+The text does not provide any evidence that "rd5" is an alternate abbreviation for the TUB gene. The symbol "RD5" appears in the text, but it is used as a primer name for PCR amplification of Blastocystis DNA, not as a gene symbol. There is no explicit link or expansion connecting "rd5" to the official gene name "TUB bipartite transcription factor" or the primary symbol "TUB". Therefore, I have classified this as not an alternate abbreviation and provided no evidence.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>36650547</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>36650547</v>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
         <is>
           <t>alias</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>alias</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>intro</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>TUB (MIM #601197), also known as rd5 or RDOB, maps to 11p15.4 and encodes the tubby-bipartite transcription regulator</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr">
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>Retinitis pigmentosa (RP) is the most common type of inherited retinopathy. At least 69 genes for RP have been identified. A significant proportion of RP, however, remains genetically unsolved. In this study, the genetic basis of a Chinese consanguineous family with presumed autosomal recessive retinitis pigmentosa (arRP) was investigated.
 Overall ophthalmic examinations, including funduscopy, decimal best-corrected visual acuity, axial length and electroretinography (ERG) were performed for the family. Genomic DNA from peripheral blood of the proband was subjected to whole exome sequencing. In silico predictions, structural modelling, and minigene assays were conducted to evaluate the pathogenicity of the variant.
@@ -871,7 +1642,7 @@
 In the current study, we examined a consanguineous family with arRP from central south China and detected a novel homozygous variant (c.1379 G &gt; A: p.Asn460Ser) inTUB. This variant co-segregated with the disease in an autosomal recessive manner and was absent in 118 ethnically matched healthy controls. This homozygous variant has not been reported in the literature or deposited in existing databases including gnomAD, 1000G phase3, ExAC, or dbSNP, indicating that this variant is rare. Multiple bioinformatic algorithms predicted that this variant was deleterious or damaging. Conservative analysis showed the codon Asn460 fallen within a highly conserved region across diverse species (Fig.3B). Further structural modeling showed that amino acid substitution (Ser) of the variant at residue Asn460 could affect the protein conformation, the binding ability of the tubby domain [26], as well as the solubility and stabilization of the mutant protein [27]. Taken together, these data strongly supported the hypothesis that this novelTUBvariant (c.1379 A &gt; G: p. Asn460Ser) might be the genetic basis of arRP in this Chinese consanguineous family.</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>Retinitis pigmentosa (RP) is the most common type of inherited retinopathy. At least 69 genes for RP have been identified. A significant proportion of RP, however, remains genetically unsolved. In this study, the genetic basis of a Chinese consanguineous family with presumed autosomal recessive retinitis pigmentosa (arRP) was investigated.
 Overall ophthalmic examinations, including funduscopy, decimal best-corrected visual acuity, axial length and electroretinography (ERG) were performed for the family. Genomic DNA from peripheral blood of the proband was subjected to whole exome sequencing. In silico predictions, structural modelling, and minigene assays were conducted to evaluate the pathogenicity of the variant.
@@ -879,7 +1650,7 @@
 A novel missense variant in TUB was identified, which was probably the pathogenic basis for arRP in this consanguineous family. This is the first report of a homozygous missense variant in TUB for RP.</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>PMID: 36650547
 Full Text: Retinitis pigmentosa (RP) is the most common type of inherited retinopathy. At least 69 genes for RP have been identified. A significant proportion of RP, however, remains genetically unsolved. In this study, the genetic basis of a Chinese consanguineous family with presumed autosomal recessive retinitis pigmentosa (arRP) was investigated.
@@ -910,7 +1681,7 @@
 In the current study, we examined a consanguineous family with arRP from central south China and detected a novel homozygous variant (c.1379 G &gt; A: p.Asn460Ser) inTUB. This variant co-segregated with the disease in an autosomal recessive manner and was absent in 118 ethnically matched healthy controls. This homozygous variant has not been reported in the literature or deposited in existing databases including gnomAD, 1000G phase3, ExAC, or dbSNP, indicating that this variant is rare. Multiple bioinformatic algorithms predicted that this variant was deleterious or damaging. Conservative analysis showed the codon Asn460 fallen within a highly conserved region across diverse species (Fig.3B). Further structural modeling showed that amino acid substitution (Ser) of the variant at residue Asn460 could affect the protein conformation, the binding ability of the tubby domain [26], as well as the solubility and stabilization of the mutant protein [27]. Taken together, these data strongly supported the hypothesis that this novelTUBvariant (c.1379 A &gt; G: p. Asn460Ser) might be the genetic basis of arRP in this Chinese consanguineous family.</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -918,35 +1689,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -979,95 +1758,94 @@
 In the current study, we examined a consanguineous family with arRP from central south China and detected a novel homozygous variant (c.1379 G &gt; A: p.Asn460Ser) inTUB. This variant co-segregated with the disease in an autosomal recessive manner and was absent in 118 ethnically matched healthy controls. This homozygous variant has not been reported in the literature or deposited in existing databases including gnomAD, 1000G phase3, ExAC, or dbSNP, indicating that this variant is rare. Multiple bioinformatic algorithms predicted that this variant was deleterious or damaging. Conservative analysis showed the codon Asn460 fallen within a highly conserved region across diverse species (Fig.3B). Further structural modeling showed that amino acid substitution (Ser) of the variant at residue Asn460 could affect the protein conformation, the binding ability of the tubby domain [26], as well as the solubility and stabilization of the mutant protein [27]. Taken together, these data strongly supported the hypothesis that this novelTUBvariant (c.1379 A &gt; G: p. Asn460Ser) might be the genetic basis of arRP in this Chinese consanguineous family.</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>{
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Based on the provided text, here is my analysis:
+{
 "pmid": "36650547",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "YES",
-"alternate_abbreviation": "NO",
+"alternate_abbreviation": "YES",
 "evidence": "TUB (MIM #601197), also known as rd5 or RDOB, maps to 11p15.4 and encodes the tubby-bipartite transcription regulator [10,11]."
-}</t>
+}
+The text explicitly links the alias symbol "rd5" to the TUB gene, stating that TUB is "also known as rd5". This provides clear evidence that rd5 is an alternate abbreviation for the TUB gene.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>36650547</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>36650547</v>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
         <is>
           <t>alias</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>alias</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>intro</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>TUB (MIM #601197), also known as rd5 or RDOB, maps to 11p15.4 and encodes the tubby-bipartite transcription regulator</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr">
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>For RP-associated diseases in humans, variants inTUBare extremely rare. Till now, only one arRP-associated mutation inTUBfor has been reported in the literature, in which a homozygous frameshift variant resulted in retinal dystrophy, hearing loss, and obesity in a consanguineous UK Caucasian family [12]. Even so, a total of 354TUBvariants have been deposited in the ClinVar database with 25 items marked of “pathogenic” or “likely pathogenic” clinical significance, among which at least 3 “pathogenic” or “likely pathogenic” variants have been reported in more than 6 patients with arRP (Additional file1: Table S3). Interestingly, all these cases mentioned above are generated either by splice-site or protein-truncating mutations inTUB.Although the variant found in this study was a single base-substitution, which resulted in a substitution of Asn to Ser at codon 460 in exon 11. According to the ACMG Standards/Guidelines, it’s important to assess the possibility that the variant may act through splicing disruption instead of amino acid change [24]. Considering loss of function is a common mechanism of genetic disease, this homozygous variant coincidently resides on the last but one base of exon 11 of theTUBgene, which is classified as a type II splice variant [28]. We first investigate the splicing effect of the variant by RNA analysis from the peripheral blood of the proband as well as healthy controls. But no mRNA ofTUBwas detected in available somatic cells (data not shown), which is consistent with the records in GTEx that the mRNA ofTUBin peripheral blood is extremely low (Additional file1: Fig. S1). Considering the unavailability of specific tissues, we further tried to explore the splicing effect of this variant via minigene assay, a powerful way for evaluating the role of novel variants on splicing [29]. The splicing assay in this study, however, showed no differences between theTUB/WTandTUB/MTminigenes in two different cell lines, indicating the possible impact of this variant on splicing could be basically ruled out. A mutant TUB protein induced by the homozygous missense variant instead of loss of function from splicing-error or protein-truncating was probably the pathogenic basis for the simple arRP in this consanguineous family.
 To date, five mammalian tubby-like proteins (TULPs) family members (TUB and TULP1 to 4) have been identified with an important role in maintenance of the central nervous system [17]. The TULPs are characterized by a unique “tubby domain” of ~ 260 amino acid residues in the C-terminal [30], which forms a central hydrophobic α-helix traversing the β-barrel structure [11]. The ‘tubby domain’ contains a phosphatidylinositol-binding region specifically binding to phosphatidylinositol 4,5-bisphosphate (PIP2) functioning as membrane-bound transcription regulators [10] and a DNA-binding domain (DBD) that selectively binding to double-stranded DNA [11]. Although the N-terminal motifs of the TULPs are poorly conserved [31], the C-terminal “tubby domains” of the TULPs are remarkedly conserved with 55–95% identity across species from plants to humans [17], implying an evolutionarily conserved function [11]. Structure–function analysis by Sunshin Kim et al. demonstrated that the tubby domain inTUBplays a crucial role in its subcellular localization and solubility [26]. In addition, mutations in anotherTULPs family member,TULP1(also known as RP14), is known to cause retinal degeneration in both humans and mice [32–35]. Previous studies demonstrated that bothTUBandTULP1are essential for G protein-coupled receptors (GPCRs) mediated trafficking of photoreceptors [30,36] and MerTK-dependent phagocytosis in retinal pigment epithelium (RPE) and apoptotic cells [37]. Caspase mediated apoptosis and MerTK-dependent phagocytosis are the underlying mechanism of photoreceptor cell death in retinal degeneration [37–40]. Therefore, we presume that the pathogenic missense variant inTUBreported here may influence TUB functions through disruption of the ‘tubby domain’, affecting GPCR trafficking, as well as the normal physiology of the photoreceptor cells, and ultimately lead to arRP. Further functional studies, however, are required to elucidate the exact role ofTUBin arRP. Genetically modified animal models are being developed in the lab to address these points.
@@ -1095,7 +1873,7 @@
 All authors declared no conflict of interest.</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>Retinitis pigmentosa (RP) is the most common type of inherited retinopathy. At least 69 genes for RP have been identified. A significant proportion of RP, however, remains genetically unsolved. In this study, the genetic basis of a Chinese consanguineous family with presumed autosomal recessive retinitis pigmentosa (arRP) was investigated.
 Overall ophthalmic examinations, including funduscopy, decimal best-corrected visual acuity, axial length and electroretinography (ERG) were performed for the family. Genomic DNA from peripheral blood of the proband was subjected to whole exome sequencing. In silico predictions, structural modelling, and minigene assays were conducted to evaluate the pathogenicity of the variant.
@@ -1103,7 +1881,7 @@
 A novel missense variant in TUB was identified, which was probably the pathogenic basis for arRP in this consanguineous family. This is the first report of a homozygous missense variant in TUB for RP.</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>PMID: 36650547
 Full Text: For RP-associated diseases in humans, variants inTUBare extremely rare. Till now, only one arRP-associated mutation inTUBfor has been reported in the literature, in which a homozygous frameshift variant resulted in retinal dystrophy, hearing loss, and obesity in a consanguineous UK Caucasian family [12]. Even so, a total of 354TUBvariants have been deposited in the ClinVar database with 25 items marked of “pathogenic” or “likely pathogenic” clinical significance, among which at least 3 “pathogenic” or “likely pathogenic” variants have been reported in more than 6 patients with arRP (Additional file1: Table S3). Interestingly, all these cases mentioned above are generated either by splice-site or protein-truncating mutations inTUB.Although the variant found in this study was a single base-substitution, which resulted in a substitution of Asn to Ser at codon 460 in exon 11. According to the ACMG Standards/Guidelines, it’s important to assess the possibility that the variant may act through splicing disruption instead of amino acid change [24]. Considering loss of function is a common mechanism of genetic disease, this homozygous variant coincidently resides on the last but one base of exon 11 of theTUBgene, which is classified as a type II splice variant [28]. We first investigate the splicing effect of the variant by RNA analysis from the peripheral blood of the proband as well as healthy controls. But no mRNA ofTUBwas detected in available somatic cells (data not shown), which is consistent with the records in GTEx that the mRNA ofTUBin peripheral blood is extremely low (Additional file1: Fig. S1). Considering the unavailability of specific tissues, we further tried to explore the splicing effect of this variant via minigene assay, a powerful way for evaluating the role of novel variants on splicing [29]. The splicing assay in this study, however, showed no differences between theTUB/WTandTUB/MTminigenes in two different cell lines, indicating the possible impact of this variant on splicing could be basically ruled out. A mutant TUB protein induced by the homozygous missense variant instead of loss of function from splicing-error or protein-truncating was probably the pathogenic basis for the simple arRP in this consanguineous family.
@@ -1132,7 +1910,7 @@
 All authors declared no conflict of interest.</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -1140,35 +1918,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -1199,99 +1985,96 @@
 All authors declared no conflict of interest.</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>{
 "pmid": "36650547",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"alternate_abbreviation": "NO",
 "evidence": ""
 }</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>37185159</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>37185159</v>
+      </c>
+      <c r="I9" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>primer</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>In the first reaction, the broadly specific oligonucleotide primers RD5 (5Õ-GGAAGCTTATCTGGTTGATCCTGCCAGTA-3Õ) and RD3 (5Õ-GGGATCCTGATCCTTCCGCAGGTTCACCTAC-3Õ) were used</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr">
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>Blastocystisis a protist of controversial pathogenicity inhabiting the gut of humans and other animals. Despite a century of intense study, understanding of the epidemiology ofBlastocystisremains fragmentary. Here, we aimed to explore its prevalence, stability of colonisation and association with various factors in a rural elementary school in northern Thailand. One hundred and forty faecal samples were collected from 104 children at two time points (tp) 105 days apart. For tp2, samples were also obtained from 15 animals residing on campus and seven water locations. Prevalence in children was 67% at tp1 and 89% at tp2, 63% in chickens, 86% in pigs, and 57% in water. Ten STs were identified, two of which were shared between humans and animals, one between animals and water, and three between humans and water. Eighteen children (out of 36) carried the same ST over both time points, indicating stable colonisation. Presence ofBlastocystis(or ST) was not associated with body mass index, ethnicity, birth delivery mode, or milk source as an infant. This study advances understanding ofBlastocystisprevalence in an understudied age group, the role of the environment in transmission, and the ability of specific STs to stably colonise children.
 Blastocystisis a unicellular eukaryote inhabiting the gastrointestinal tract of vertebrates [1–3] and invertebrates [4,5]. The organism comprises the most common protist identified in human stool samples [6]. The genetic heterogeneity ofBlastocystisis extremely high based on the small subunit ribosomal RNA (SSU rRNA) gene [7–14]. To date, 34 subtypes (STs; ST1–ST17, ST21, and ST23–ST38) have been identified in avian and mammalian hosts. Of these, 14 have been recorded in humans (ST1–ST10, ST12, ST14, ST16, and ST23) [13,15–20], with ST1–ST3 accounting for the majority of human carriage [21,22]. The remaining STs mostly colonise non-human endothermic hosts [1,6].
@@ -1320,12 +2103,12 @@
 This analysis involved only sequences from tp2. ST sharing was noted among all three categories herein: humans, animals, and water (Figure 2). ST5 and ST7 were shared between humans and animals, ST1, ST3, and ST7 between humans and water, and ST7 between animals and water. ST7 was shared by all three. The ST5 sequences from humans and pigs were not identical. Similarly, ST1 sequences from water and children differed. ST3 sequences from the water creek, and 16 children were identical. ST7 sequences from two children samples and a water sample obtained from the tap outside the school bathroom were also identical.Figure 2.Blastocystissubtypes (STs) present in humans, animals, and water in a rural elementary school in northern Thailand. STs on arrows indicate overlap. Shaded STs indicate the presence in all sources considered in this study.</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>&lt;i&gt;Blastocystis&lt;/i&gt; is a protist of controversial pathogenicity inhabiting the gut of humans and other animals. Despite a century of intense study, understanding of the epidemiology of &lt;i&gt;Blastocystis&lt;/i&gt; remains fragmentary. Here, we aimed to explore its prevalence, stability of colonisation and association with various factors in a rural elementary school in northern Thailand. One hundred and forty faecal samples were collected from 104 children at two time points (tp) 105 days apart. For tp2, samples were also obtained from 15 animals residing on campus and seven water locations. Prevalence in children was 67% at tp1 and 89% at tp2, 63% in chickens, 86% in pigs, and 57% in water. Ten STs were identified, two of which were shared between humans and animals, one between animals and water, and three between humans and water. Eighteen children (out of 36) carried the same ST over both time points, indicating stable colonisation. Presence of &lt;i&gt;Blastocystis&lt;/i&gt; (or ST) was not associated with body mass index, ethnicity, birth delivery mode, or milk source as an infant. This study advances understanding of &lt;i&gt;Blastocystis&lt;/i&gt; prevalence in an understudied age group, the role of the environment in transmission, and the ability of specific STs to stably colonise children.</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>PMID: 37185159
 Full Text: Blastocystisis a protist of controversial pathogenicity inhabiting the gut of humans and other animals. Despite a century of intense study, understanding of the epidemiology ofBlastocystisremains fragmentary. Here, we aimed to explore its prevalence, stability of colonisation and association with various factors in a rural elementary school in northern Thailand. One hundred and forty faecal samples were collected from 104 children at two time points (tp) 105 days apart. For tp2, samples were also obtained from 15 animals residing on campus and seven water locations. Prevalence in children was 67% at tp1 and 89% at tp2, 63% in chickens, 86% in pigs, and 57% in water. Ten STs were identified, two of which were shared between humans and animals, one between animals and water, and three between humans and water. Eighteen children (out of 36) carried the same ST over both time points, indicating stable colonisation. Presence ofBlastocystis(or ST) was not associated with body mass index, ethnicity, birth delivery mode, or milk source as an infant. This study advances understanding ofBlastocystisprevalence in an understudied age group, the role of the environment in transmission, and the ability of specific STs to stably colonise children.
@@ -1355,7 +2138,7 @@
 This analysis involved only sequences from tp2. ST sharing was noted among all three categories herein: humans, animals, and water (Figure 2). ST5 and ST7 were shared between humans and animals, ST1, ST3, and ST7 between humans and water, and ST7 between animals and water. ST7 was shared by all three. The ST5 sequences from humans and pigs were not identical. Similarly, ST1 sequences from water and children differed. ST3 sequences from the water creek, and 16 children were identical. ST7 sequences from two children samples and a water sample obtained from the tap outside the school bathroom were also identical.Figure 2.Blastocystissubtypes (STs) present in humans, animals, and water in a rural elementary school in northern Thailand. STs on arrows indicate overlap. Shaded STs indicate the presence in all sources considered in this study.</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -1363,35 +2146,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -1423,100 +2214,98 @@
 This analysis involved only sequences from tp2. ST sharing was noted among all three categories herein: humans, animals, and water (Figure 2). ST5 and ST7 were shared between humans and animals, ST1, ST3, and ST7 between humans and water, and ST7 between animals and water. ST7 was shared by all three. The ST5 sequences from humans and pigs were not identical. Similarly, ST1 sequences from water and children differed. ST3 sequences from the water creek, and 16 children were identical. ST7 sequences from two children samples and a water sample obtained from the tap outside the school bathroom were also identical.Figure 2.Blastocystissubtypes (STs) present in humans, animals, and water in a rural elementary school in northern Thailand. STs on arrows indicate overlap. Shaded STs indicate the presence in all sources considered in this study.</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>Based on the provided text, here is the JSON output:
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Based on the provided text, here is the analysis for the alias symbol "rd5":
 {
 "pmid": "37185159",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"alternate_abbreviation": "NO",
 "evidence": ""
-}</t>
+}
+The text does not provide any evidence that "rd5" is an alternate abbreviation for the TUB gene. The symbol "RD5" appears to be used as a primer name in the PCR methodology section, but it is not explicitly linked to or expanded as the TUB gene name. Therefore, there is insufficient evidence to classify "rd5" as an alternate abbreviation for TUB in this context.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>37185159</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>37185159</v>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>primer</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>In the first reaction, the broadly specific oligonucleotide primers RD5 (5Õ-GGAAGCTTATCTGGTTGATCCTGCCAGTA-3Õ) and RD3 (5Õ-GGGATCCTGATCCTTCCGCAGGTTCACCTAC-3Õ) were used</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr">
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>Blastocystissubtypes (STs) present in humans, animals, and water in a rural elementary school in northern Thailand. STs on arrows indicate overlap. Shaded STs indicate the presence in all sources considered in this study.
 For the phylogenetic analysis, 23 sequences were chosen to represent the different STs present in the sample cohort (Figure 3). ST15 found in the pig sample grouped with previously published ST15 sequences and together with ST28 and sequences from ectothermic hosts placed at the base of the tree. Newly generated sequences placed within clades consisting of known STs. Sequences identified as ST10 and ST23 were grouped with similar sequences from our previous One Health study [15].Figure 3.Maximum likelihood phylogeny inferred from 175Blastocystissequences and 1,392 sites of theSSUrRNA gene. Newly generated sequences are in bold font. Numerical values indicate bootstrap support. Only values above 70 are shown.
@@ -1542,12 +2331,12 @@
 The authors declare none.</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>&lt;i&gt;Blastocystis&lt;/i&gt; is a protist of controversial pathogenicity inhabiting the gut of humans and other animals. Despite a century of intense study, understanding of the epidemiology of &lt;i&gt;Blastocystis&lt;/i&gt; remains fragmentary. Here, we aimed to explore its prevalence, stability of colonisation and association with various factors in a rural elementary school in northern Thailand. One hundred and forty faecal samples were collected from 104 children at two time points (tp) 105 days apart. For tp2, samples were also obtained from 15 animals residing on campus and seven water locations. Prevalence in children was 67% at tp1 and 89% at tp2, 63% in chickens, 86% in pigs, and 57% in water. Ten STs were identified, two of which were shared between humans and animals, one between animals and water, and three between humans and water. Eighteen children (out of 36) carried the same ST over both time points, indicating stable colonisation. Presence of &lt;i&gt;Blastocystis&lt;/i&gt; (or ST) was not associated with body mass index, ethnicity, birth delivery mode, or milk source as an infant. This study advances understanding of &lt;i&gt;Blastocystis&lt;/i&gt; prevalence in an understudied age group, the role of the environment in transmission, and the ability of specific STs to stably colonise children.</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>PMID: 37185159
 Full Text: Blastocystissubtypes (STs) present in humans, animals, and water in a rural elementary school in northern Thailand. STs on arrows indicate overlap. Shaded STs indicate the presence in all sources considered in this study.
@@ -1574,7 +2363,7 @@
 The authors declare none.</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -1582,35 +2371,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -1639,99 +2436,96 @@
 The authors declare none.</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="V10" t="inlineStr">
         <is>
           <t>{
 "pmid": "37185159",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"alternate_abbreviation": "NO",
 "evidence": ""
 }</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>38543574</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>38543574</v>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>primer</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>PCR amplification of Blastocystis sp. was carried out using barcoding region primers BhRDr (5_-GAGCTTTTTAACTGCAACAACG-3_) and RD5 (5_-ATCTGGTTGATCCTGCCAGT-3_) for SSU rRNA</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr">
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>Blastocystissp. is the most common intestinal protozoan affecting human health worldwide. Several studies have reported the prevalence ofBlastocystissp. in various regions of the Republic of Korea. However, limited data are available on the prevalence and subtype (ST) distribution of this parasite among regions. Therefore, we investigated the prevalence and ST distributions of this parasite in the Republic of Korea. For this purpose, 894 stool specimens were collected from patients with diarrhea and tested for the presence ofBlastocystissp. using PCR analysis. The isolates were subsequently subtyped. The overall prevalence was 11.6%. Of the 104 isolates, ST3 was the most prevalent, followed by ST1. Additionally, a single case of the rare subtype ST8 was identified, representing the first reported case in the Republic of Korea. The results suggested that the predominance of ST3 observed in this study reflects human-to-human transmission with low genetic diversity within the ST, while ST1 transmission is likely correlated with animals. In the future, to better understandBlastocystissp. transmission dynamics, human, animal, and environmental factors should be studied from a “One Health” perspective.
 Blastocystissp. is a protozoan parasite that resides within the gastrointestinal tract of a wide range of hosts, including mammals, birds, fish, reptiles, insects, and humans [1,2]. This enteric microorganism is a causative agent of waterborne and foodborne diseases. The infective cysts are transmitted through the fecal–oral route [3,4]. An estimated more than 1 billion people are infected with this parasite worldwide, with a prevalence of 10–15% in developed countries and &gt;50% in developing nations [5]. Although most infected people are asymptomatic carriers, some vulnerable individuals develop symptoms, including diarrhea, abdominal pain, gas, and nausea, as well as extraintestinal symptoms such as urticaria and rash [6,7,8,9,10].Blastocystissp. colonization is reportedly associated with a healthy gut microbiome rather than intestinal dysbacteriosis [6]. However, in vitro and in vivo studies combined with genomic analyses have identified various virulence factors that may be related to the genetic variation inBlastocystisisolates [2,11].
@@ -1768,12 +2562,12 @@
 Distribution ofBlastocystissp. infection among patients with diarrhea in the Republic of Korea.</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>&lt;i&gt;Blastocystis&lt;/i&gt; sp. is the most common intestinal protozoan affecting human health worldwide. Several studies have reported the prevalence of &lt;i&gt;Blastocystis&lt;/i&gt; sp. in various regions of the Republic of Korea. However, limited data are available on the prevalence and subtype (ST) distribution of this parasite among regions. Therefore, we investigated the prevalence and ST distributions of this parasite in the Republic of Korea. For this purpose, 894 stool specimens were collected from patients with diarrhea and tested for the presence of &lt;i&gt;Blastocystis&lt;/i&gt; sp. using PCR analysis. The isolates were subsequently subtyped. The overall prevalence was 11.6%. Of the 104 isolates, ST3 was the most prevalent, followed by ST1. Additionally, a single case of the rare subtype ST8 was identified, representing the first reported case in the Republic of Korea. The results suggested that the predominance of ST3 observed in this study reflects human-to-human transmission with low genetic diversity within the ST, while ST1 transmission is likely correlated with animals. In the future, to better understand &lt;i&gt;Blastocystis&lt;/i&gt; sp. transmission dynamics, human, animal, and environmental factors should be studied from a "One Health" perspective.</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>PMID: 38543574
 Full Text: Blastocystissp. is the most common intestinal protozoan affecting human health worldwide. Several studies have reported the prevalence ofBlastocystissp. in various regions of the Republic of Korea. However, limited data are available on the prevalence and subtype (ST) distribution of this parasite among regions. Therefore, we investigated the prevalence and ST distributions of this parasite in the Republic of Korea. For this purpose, 894 stool specimens were collected from patients with diarrhea and tested for the presence ofBlastocystissp. using PCR analysis. The isolates were subsequently subtyped. The overall prevalence was 11.6%. Of the 104 isolates, ST3 was the most prevalent, followed by ST1. Additionally, a single case of the rare subtype ST8 was identified, representing the first reported case in the Republic of Korea. The results suggested that the predominance of ST3 observed in this study reflects human-to-human transmission with low genetic diversity within the ST, while ST1 transmission is likely correlated with animals. In the future, to better understandBlastocystissp. transmission dynamics, human, animal, and environmental factors should be studied from a “One Health” perspective.
@@ -1811,7 +2605,7 @@
 Distribution ofBlastocystissp. infection among patients with diarrhea in the Republic of Korea.</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -1819,35 +2613,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -1887,99 +2689,98 @@
 Distribution ofBlastocystissp. infection among patients with diarrhea in the Republic of Korea.</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>{
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Based on the provided text, here is my analysis:
+{
 "pmid": "38543574",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"alternate_abbreviation": "NO",
 "evidence": ""
-}</t>
+}
+The text does not provide any evidence that "rd5" is an alternate abbreviation for the TUB gene. The symbol "RD5" appears in the text, but it is used as a primer name for PCR amplification of Blastocystis sp., not as an alias for the TUB gene. There is no explicit link or expansion connecting "rd5" to the official gene name "TUB bipartite transcription factor". Therefore, I have classified this as not an alternate abbreviation and provided no evidence.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>38578271</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>38578271</v>
+      </c>
+      <c r="I12" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>primer</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>The gDNA samples were analysed by PCR amplification of _600 bp of the SSU rRNA gene of Blastocystis sp. using the primers RD5 (5__ATCTGGTTGATCCTGCCAGT_3_) and BhRDr (5_GAGCTTTTTAACTGCAACAACG_3_) to identify the presence of Blastocystis sp. Infection</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr">
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>Blastocystissp. is a zoonotic protozoan parasite, and there is limited information about its molecular prevalence and subtypes (STs) distribution in camels globally, especially in Iran.
 This study aimed to examine the prevalence, STs distribution, and zoonotic potential ofBlastocystissp. in one‐humped and two‐humped camels in Ardabil province, northwestern Iran.
@@ -2022,7 +2823,7 @@
 The datasets used and/or analysed during the current study are available in the online version.</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>Blastocystis sp. is a zoonotic protozoan parasite, and there is limited information about its molecular prevalence and subtypes (STs) distribution in camels globally, especially in Iran.
 This study aimed to examine the prevalence, STs distribution, and zoonotic potential of Blastocystis sp. in one-humped and two-humped camels in Ardabil province, northwestern Iran.
@@ -2031,7 +2832,7 @@
 These findings indicate that camels serve as a proper reservoir for a diverse array of Blastocystis STs and thereby can play a significant role in the transmission of this protozoan infection to humans, animals, and water reservoirs.</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>PMID: 38578271
 Full Text: Blastocystissp. is a zoonotic protozoan parasite, and there is limited information about its molecular prevalence and subtypes (STs) distribution in camels globally, especially in Iran.
@@ -2075,7 +2876,7 @@
 The datasets used and/or analysed during the current study are available in the online version.</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -2083,35 +2884,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -2157,99 +2966,96 @@
 The datasets used and/or analysed during the current study are available in the online version.</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>{
 "pmid": "38578271",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"alternate_abbreviation": "NO",
 "evidence": ""
 }</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>38980911</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>38980911</v>
+      </c>
+      <c r="I13" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>primer</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>PCR amplification of DNA was performed using a nested PCR reaction. Briefly, the first PCR used the broad-specificity eukaryotic primer RD5 (5Õ-GGAAGCTTATCTGGTTGA TCCTGCCAGTA-3Õ) and RD3 (5Õ-GGGATCCTGATCCTTC CGCAGGTTCACCTAC-3Õ), which amplifies a ~1,800 bp fragment of the SSU rDNA</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr">
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="R13" t="inlineStr">
         <is>
           <t>The authors have declared that no competing interests exist.
 Blastocystisis a unicellular eukaryote commonly found in the intestinal tract of humans and other animals. The prevalence ofBlastocystishas been investigated in both developed and developing countries, yet its occurrence and distribution in rural locations has been less studied. Herein, we aimed to examine the distribution ofBlastocystiscolonization in Thai adults representing background populations along a rural/peri-urban gradient, as well as associations between colonization and personal characteristics.
@@ -2290,7 +3096,7 @@
 Altogether, we detected a single subtype in 88.8% (142/160) ofBlastocystis-positive individuals, whereas a mixed-subtype (mixST) infection was detected in 3.8% (6/160). Nine subtypes were identified. The most abundant subtype was ST3 (n = 63), followed by ST7 (n = 37), ST1 (n = 23), ST23 (n = 9), ST10 (n = 4), ST2 (n = 2), ST5 (n = 2), ST4 (n = 1) and ST6 (n = 1). In 7.5% (12/160) of the cases, the subtype could not be identified precisely either due to short length and/or presence of ambiguous chromatogram peaks (unk).</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="S13" t="inlineStr">
         <is>
           <t>Blastocystis is a unicellular eukaryote commonly found in the intestinal tract of humans and other animals. The prevalence of Blastocystis has been investigated in both developed and developing countries, yet its occurrence and distribution in rural locations has been less studied. Herein, we aimed to examine the distribution of Blastocystis colonization in Thai adults representing background populations along a rural/peri-urban gradient, as well as associations between colonization and personal characteristics.
 A total of 238 participants were recruited from rural and peri-urban areas situated in three provinces. The presence of Blastocystis in feces was evaluated using PCR and qPCR. Information on gender, age, region (province), rural/peri-urban location, and body mass index (BMI) was collected.
@@ -2298,7 +3104,7 @@
 This study increases the understanding of the epidemiology of Blastocystis colonization and its association with population parameters and characteristics in middle-income countries.</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>PMID: 38980911
 Full Text: The authors have declared that no competing interests exist.
@@ -2340,7 +3146,7 @@
 Altogether, we detected a single subtype in 88.8% (142/160) ofBlastocystis-positive individuals, whereas a mixed-subtype (mixST) infection was detected in 3.8% (6/160). Nine subtypes were identified. The most abundant subtype was ST3 (n = 63), followed by ST7 (n = 37), ST1 (n = 23), ST23 (n = 9), ST10 (n = 4), ST2 (n = 2), ST5 (n = 2), ST4 (n = 1) and ST6 (n = 1). In 7.5% (12/160) of the cases, the subtype could not be identified precisely either due to short length and/or presence of ambiguous chromatogram peaks (unk).</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -2348,35 +3154,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -2420,100 +3234,98 @@
 Altogether, we detected a single subtype in 88.8% (142/160) ofBlastocystis-positive individuals, whereas a mixed-subtype (mixST) infection was detected in 3.8% (6/160). Nine subtypes were identified. The most abundant subtype was ST3 (n = 63), followed by ST7 (n = 37), ST1 (n = 23), ST23 (n = 9), ST10 (n = 4), ST2 (n = 2), ST5 (n = 2), ST4 (n = 1) and ST6 (n = 1). In 7.5% (12/160) of the cases, the subtype could not be identified precisely either due to short length and/or presence of ambiguous chromatogram peaks (unk).</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>Based on the provided text, here is the JSON output:
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Based on the provided text, I do not see any evidence that the alias symbol "rd5" is explicitly expanded or linked to the official HGNC gene name "TUB bipartite transcription factor" or the primary gene symbol "TUB". The text appears to be about Blastocystis epidemiology and does not mention the TUB gene. Therefore, I cannot classify "rd5" as an alternate abbreviation for TUB in this context.
+Here is the output in the requested JSON format:
 {
 "pmid": "38980911",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"alternate_abbreviation": "NO",
 "evidence": ""
 }</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>38980911</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>38980911</v>
+      </c>
+      <c r="I14" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>primer</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>PCR amplification of DNA was performed using a nested PCR reaction. Briefly, the first PCR used the broad-specificity eukaryotic primer RD5 (5Õ-GGAAGCTTATCTGGTTGA TCCTGCCAGTA-3Õ) and RD3 (5Õ-GGGATCCTGATCCTTC CGCAGGTTCACCTAC-3Õ), which amplifies a ~1,800 bp fragment of the SSU rDNA</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr">
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="R14" t="inlineStr">
         <is>
           <t>According to gender,BlastocystisST3, ST1, and ST7 were the most frequently found in males, while ST3, ST7 and ST1 were the most frequently found subtypes in females in that order.BlastocystisST1-ST7, ST10 and ST23 were identified in lean and overweight, whereas in obese participants carriage was limited to ST1, ST3 and ST7 (Table 5). Finally,BlastocystisST1, ST3 and ST7 were the most common subtypes across all age groups. The middle-aged (45–64 years) individuals exhibited the highest diversity of subtypes. Regarding region,BlastocystisST1-ST7, ST10 and ST23 were observed in CR province, ST1-ST3 and ST7 in PY province and ST1, ST3, ST5, ST7 and ST10 in CH province (Fig 3). The top threeBlastocystissubtypes in CR were ST3, ST1 and ST23, while ST3, ST7 and ST1 were the most abundant in PY and CH province, in this order.
 (A) Chiang Rai (CR). (B) Phayao (PY). (C) Chachoengsao (CH).
@@ -2620,7 +3432,7 @@
 • DNA extraction and purification</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="S14" t="inlineStr">
         <is>
           <t>Blastocystis is a unicellular eukaryote commonly found in the intestinal tract of humans and other animals. The prevalence of Blastocystis has been investigated in both developed and developing countries, yet its occurrence and distribution in rural locations has been less studied. Herein, we aimed to examine the distribution of Blastocystis colonization in Thai adults representing background populations along a rural/peri-urban gradient, as well as associations between colonization and personal characteristics.
 A total of 238 participants were recruited from rural and peri-urban areas situated in three provinces. The presence of Blastocystis in feces was evaluated using PCR and qPCR. Information on gender, age, region (province), rural/peri-urban location, and body mass index (BMI) was collected.
@@ -2628,7 +3440,7 @@
 This study increases the understanding of the epidemiology of Blastocystis colonization and its association with population parameters and characteristics in middle-income countries.</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="T14" t="inlineStr">
         <is>
           <t>PMID: 38980911
 Full Text: According to gender,BlastocystisST3, ST1, and ST7 were the most frequently found in males, while ST3, ST7 and ST1 were the most frequently found subtypes in females in that order.BlastocystisST1-ST7, ST10 and ST23 were identified in lean and overweight, whereas in obese participants carriage was limited to ST1, ST3 and ST7 (Table 5). Finally,BlastocystisST1, ST3 and ST7 were the most common subtypes across all age groups. The middle-aged (45–64 years) individuals exhibited the highest diversity of subtypes. Regarding region,BlastocystisST1-ST7, ST10 and ST23 were observed in CR province, ST1-ST3 and ST7 in PY province and ST1, ST3, ST5, ST7 and ST10 in CH province (Fig 3). The top threeBlastocystissubtypes in CR were ST3, ST1 and ST23, while ST3, ST7 and ST1 were the most abundant in PY and CH province, in this order.
@@ -2736,7 +3548,7 @@
 • DNA extraction and purification</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="U14" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -2744,35 +3556,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -2882,112 +3702,106 @@
 • DNA extraction and purification</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>Based on my review of the manuscript, here are the key points regarding the methodology and limitations:
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Based on my review of the manuscript, here are some key points regarding the methodology and limitations:
 1. The inclusion/exclusion criteria for participant recruitment are not clearly stated. This is an important limitation that should be acknowledged.
 2. The authors did not check for the presence of other enteric parasites that could act as confounders. This is another limitation that should be noted. 
 3. BMI data was unavailable for 36% of participants, which may have compromised the robustness of the results related to BMI associations. This limitation should be discussed.
-4. The study was restricted to adults, potentially missing effects of primary colonization in younger ages. The authors should discuss this limitation and potential impacts.
-5. The diagnostic algorithm using both nested PCR and qPCR is unclear. The rationale for using both methods should be explained.
-6. The molecular methods section needs better structure and more details on DNA extraction, PCR protocols, sequencing, etc.
-7. Information on mixed infections and how they were detected/analyzed is lacking. 
-8. Some statistical analyses need clarification, particularly regarding the logistic regression model.
-9. Certain figures and tables need improvements in clarity and labeling.
-10. The discussion should be expanded to address these limitations and put the results in broader context with recent literature.
-To address these issues, the authors should:
-- Clearly state inclusion/exclusion criteria 
-- Acknowledge limitations regarding lack of data on other parasites and incomplete BMI data
-- Discuss potential impacts of focusing only on adults
-- Clarify and justify the PCR methodology used
-- Restructure and expand the molecular methods section
-- Provide details on detection of mixed infections
-- Clarify statistical analyses 
-- Improve figures/tables as suggested
-- Expand the discussion to address limitations and compare to recent literature
-Addressing these points would strengthen the manuscript and provide important context for interpreting the results. The core data on Blastocystis prevalence and subtypes is valuable, but needs to be presented with appropriate caveats.</t>
+4. The study was restricted to adults only, potentially missing effects of primary colonization at younger ages. The authors should discuss this limitation and consider citing some of the suggested longitudinal studies in humans and animals.
+5. The diagnostic algorithm using both nested PCR and qPCR is unclear. The rationale for using both methods should be better explained.
+6. The molecular methods section needs to be restructured and described in more detail, with separate subsections for DNA extraction, PCR methods, sequencing, etc.
+7. The sample size is relatively modest, which may limit the strength of some conclusions. This should be acknowledged as a limitation.
+8. More details are needed on how mixed infections were detected and resolved.
+To address these issues, I would recommend:
+- Clearly stating inclusion/exclusion criteria 
+- Acknowledging limitations related to lack of data on other parasites and missing BMI data
+- Discussing potential impacts of focusing only on adults
+- Clarifying and justifying the PCR methodology used
+- Restructuring the molecular methods section
+- Acknowledging sample size limitations
+- Providing more details on detection of mixed infections
+Addressing these points would strengthen the methodology and discussion of limitations in the manuscript. The authors should carefully consider how these factors may impact their results and conclusions.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>38980911</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>38980911</v>
+      </c>
+      <c r="I15" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>primer</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>PCR amplification of DNA was performed using a nested PCR reaction. Briefly, the first PCR used the broad-specificity eukaryotic primer RD5 (5Õ-GGAAGCTTATCTGGTTGA TCCTGCCAGTA-3Õ) and RD3 (5Õ-GGGATCCTGATCCTTC CGCAGGTTCACCTAC-3Õ), which amplifies a ~1,800 bp fragment of the SSU rDNA</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr">
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="R15" t="inlineStr">
         <is>
           <t>• qPCR protocol
 • nested-PCR protocol, including gel electrophoresis and imaging
@@ -3100,7 +3914,7 @@
 PLOS Neglected Tropical Diseases</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="S15" t="inlineStr">
         <is>
           <t>Blastocystis is a unicellular eukaryote commonly found in the intestinal tract of humans and other animals. The prevalence of Blastocystis has been investigated in both developed and developing countries, yet its occurrence and distribution in rural locations has been less studied. Herein, we aimed to examine the distribution of Blastocystis colonization in Thai adults representing background populations along a rural/peri-urban gradient, as well as associations between colonization and personal characteristics.
 A total of 238 participants were recruited from rural and peri-urban areas situated in three provinces. The presence of Blastocystis in feces was evaluated using PCR and qPCR. Information on gender, age, region (province), rural/peri-urban location, and body mass index (BMI) was collected.
@@ -3108,7 +3922,7 @@
 This study increases the understanding of the epidemiology of Blastocystis colonization and its association with population parameters and characteristics in middle-income countries.</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>PMID: 38980911
 Full Text: • qPCR protocol
@@ -3222,7 +4036,7 @@
 PLOS Neglected Tropical Diseases</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="U15" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -3230,35 +4044,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -3374,99 +4196,97 @@
 PLOS Neglected Tropical Diseases</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>Based on the reviewer comments and editorial decision, it appears that:
-1. The manuscript "Blastocystis colonization and associations with population parameters in Thai adults" has been provisionally accepted for publication in PLOS Neglected Tropical Diseases.
-2. The authors have adequately addressed the previous reviewer comments and made the requested revisions.
-3. The study design, methods, analysis, and conclusions are considered appropriate and supported by the data.
-4. Only minor formatting changes are still needed before final acceptance.
-5. The manuscript has been deemed suitable for publication after the latest round of revisions.
-6. The corresponding author will receive typeset proofs to review for any final corrections before publication.
-7. The manuscript will be published open access in PLOS Neglected Tropical Diseases once the final production steps are completed.
-Overall, it seems the peer review and revision process has been completed successfully, and the manuscript is now on track for publication pending only minor final formatting changes. The editors and reviewers appear satisfied with the scientific content and quality of the revised manuscript.</t>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Congratulations on the acceptance of your manuscript "Blastocystis colonization and associations with population parameters in Thai adults" for publication in PLOS Neglected Tropical Diseases! Here are the key points from the acceptance letter:
+- Your manuscript has been formally accepted for publication.
+- It has been passed to the PLOS Production Department to complete the publication process. 
+- All authors will receive a confirmation email upon publication.
+- The corresponding author will soon receive a typeset proof to review for any errors introduced during production.
+- You should carefully review the PDF proof, as this is the last chance to correct any scientific or typesetting errors. Major changes may delay publication.
+- An early version will be published online soon unless you opted out of this process. The final version will be published to the same URL later.
+- The editors thanked you for supporting open-access publishing and look forward to publishing your work.
+The next steps are to watch for the typeset proof to review, make any final minor corrections needed, and then await publication of the early version online. Congratulations again on reaching this milestone with your research!</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>39961042</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>39961042</v>
+      </c>
+      <c r="I16" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>primer</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>The primers used in this study were: RD5: 5_ÐATCTGGTTGATCCTGCCAGTÐ3Õ; BhRDr: 5_ÐGAGCTTTTTAACTGCAACAACGÐ3_.</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr">
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="R16" t="inlineStr">
         <is>
           <t>Blastocystissp. is a zoonotic intestinal protozoan that is ubiquitous globally, residing in the gastrointestinal tracts of both humans and various animals. In the present study, a PCR-sequencing tool based on the SSU rRNA gene was employed to investigate the prevalence and subtypes ofBlastocystisspp. in 204 fresh fecal samples collected from 20 captive wildlife species from a bird park in Henan Province, Central China. Overall,Blastocystiswas present in 13.73% (28 out of 204) of the samples and 25% (5 out of 20) of the species. A total of four zoonotic subtypes ofBlastocystissp. were found: ST1, ST3, ST5, and ST27, with the latter being the most prevalent, accounting for 35.71% (10 out of 28) of the 5 species positive forBlastocystissp. To the best of our knowledge, this is the first report ofBlastocystisST27 in birds in China, namely bar-headed goose (Anser indicus)and peafowl (Pavo muticus). The data suggest that captive wildlife, particularly those in bird parks, may frequently be infected with this zoonotic pathogen. Consequently, these animals may serve as potential reservoirs for zoonotic infections in humans.
 Blastocystissp. est un protozoaire intestinal zoonotique omniprésent dans le monde entier, résidant dans le tractus gastro-intestinal des humains et de divers animaux. Dans la présente étude, un outil de séquençage par PCR basé sur le gène SSU rRNA a été utilisé pour étudier la prévalence et les sous-types deBlastocystisspp. dans 204 échantillons de matières fécales fraîches prélevés sur 20 espèces sauvages en captivité dans un parc ornithologique de la province du Henan, en Chine centrale. Dans l’ensemble,Blastocystisétait présent dans 13,73 % (28 sur 204) des échantillons et dans 25 % (5 sur 20) des espèces. Au total, quatre sous-types zoonotiques deBlastocystissp. ont été trouvés : ST1, ST3, ST5 et ST27, ce dernier étant le plus répandu, représentant 35,71% (10 sur 28) des 5 espèces positives pourBlastocystissp. À notre connaissance, il s’agit du premier signalement deBlastocystisST27 chez des oiseaux en Chine, à savoir l’oie à tête barrée (Anser indicus) et le paon (Pavo muticus). Les données suggèrent que la faune en captivité, en particulier celle des parcs ornithologiques, peut être fréquemment infectée par ce pathogène zoonotique. Par conséquent, ces animaux peuvent servir de réservoirs potentiels d’infections zoonotiques pour l’homme.
@@ -3501,12 +4321,12 @@
 Cite this article as: Cui Z, Huang X, Zhang S, Li K, Zhang A, Li Q, Zhang Y, Li J &amp; Qi M. 2025. Molecular characterization and subtype analysis ofBlastocystissp. in captive wildlife in Henan, China. Parasite32, 11.https://doi.org/10.1051/parasite/2025006.</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="S16" t="inlineStr">
         <is>
           <t>Blastocystis sp. is a zoonotic intestinal protozoan that is ubiquitous globally, residing in the gastrointestinal tracts of both humans and various animals. In the present study, a PCR-sequencing tool based on the SSU rRNA gene was employed to investigate the prevalence and subtypes of Blastocystis spp. in 204 fresh fecal samples collected from 20 captive wildlife species from a bird park in Henan Province, Central China. Overall, Blastocystis was present in 13.73% (28 out of 204) of the samples and 25% (5 out of 20) of the species. A total of four zoonotic subtypes of Blastocystis sp. were found: ST1, ST3, ST5, and ST27, with the latter being the most prevalent, accounting for 35.71% (10 out of 28) of the 5 species positive for Blastocystis sp. To the best of our knowledge, this is the first report of Blastocystis ST27 in birds in China, namely bar-headed goose (Anser indicus) and peafowl (Pavo muticus). The data suggest that captive wildlife, particularly those in bird parks, may frequently be infected with this zoonotic pathogen. Consequently, these animals may serve as potential reservoirs for zoonotic infections in humans.</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="T16" t="inlineStr">
         <is>
           <t>PMID: 39961042
 Full Text: Blastocystissp. is a zoonotic intestinal protozoan that is ubiquitous globally, residing in the gastrointestinal tracts of both humans and various animals. In the present study, a PCR-sequencing tool based on the SSU rRNA gene was employed to investigate the prevalence and subtypes ofBlastocystisspp. in 204 fresh fecal samples collected from 20 captive wildlife species from a bird park in Henan Province, Central China. Overall,Blastocystiswas present in 13.73% (28 out of 204) of the samples and 25% (5 out of 20) of the species. A total of four zoonotic subtypes ofBlastocystissp. were found: ST1, ST3, ST5, and ST27, with the latter being the most prevalent, accounting for 35.71% (10 out of 28) of the 5 species positive forBlastocystissp. To the best of our knowledge, this is the first report ofBlastocystisST27 in birds in China, namely bar-headed goose (Anser indicus)and peafowl (Pavo muticus). The data suggest that captive wildlife, particularly those in bird parks, may frequently be infected with this zoonotic pathogen. Consequently, these animals may serve as potential reservoirs for zoonotic infections in humans.
@@ -3542,7 +4362,7 @@
 Cite this article as: Cui Z, Huang X, Zhang S, Li K, Zhang A, Li Q, Zhang Y, Li J &amp; Qi M. 2025. Molecular characterization and subtype analysis ofBlastocystissp. in captive wildlife in Henan, China. Parasite32, 11.https://doi.org/10.1051/parasite/2025006.</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="U16" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -3550,35 +4370,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -3616,843 +4444,249 @@
 Cite this article as: Cui Z, Huang X, Zhang S, Li K, Zhang A, Li Q, Zhang Y, Li J &amp; Qi M. 2025. Molecular characterization and subtype analysis ofBlastocystissp. in captive wildlife in Henan, China. Parasite32, 11.https://doi.org/10.1051/parasite/2025006.</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="V16" t="inlineStr">
         <is>
           <t>{
 "pmid": "39961042",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"alternate_abbreviation": "NO",
 "evidence": ""
 }</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>HGNC:12406</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>ENSG00000166402</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>GENE ID:7275</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>TUB</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>rd5</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>HGNC:13919</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ENSG00000234651, ENSG00000096155, ENSG00000233348, ENSG00000204463, ENSG00000228760, ENSG00000229524, ENSG00000227761</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>GENE ID:7917</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>BAG6</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SCYTHE</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>7479945</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>9799223</v>
+      </c>
+      <c r="I17" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>mouse phenotype biomarker</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>literature defined (uniprot alternative protein name)</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>abstract</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>We report a mouse model of type I Usher syndrome, rd5, whose linkage on mouse chromosome 7 to Hbb and tub has homology to human Usher I reported on human chromosome 11p15. The electroretinogram in homozygous rd5/rd5 mouse is never normal with reduced amplitudes that extinguish by 6 months.</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>TUB bipartite transcription factor</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>Usher syndrome is a group of diseases with autosomal recessive inheritance, congenital hearing loss, and the development of retinitis pigmentosa, a progressive retinal degeneration characterized by night blindness and visual field loss over several decades. The causes of Usher syndrome are unknown and no animal models have been available for study. Four human gene sites have been reported, suggesting at least four separate forms of Usher syndrome. We report a mouse model of type I Usher syndrome, rd5, whose linkage on mouse chromosome 7 to Hbb and tub has homology to human Usher I reported on human chromosome 11p15. The electroretinogram in homozygous rd5/rd5 mouse is never normal with reduced amplitudes that extinguish by 6 months. Auditory-evoked response testing demonstrates increased hearing thresholds more than control at 3 weeks of about 30 decibels (dB) that worsen to about 45 dB by 6 months.</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>PMID: 7479945
-Abstract: Usher syndrome is a group of diseases with autosomal recessive inheritance, congenital hearing loss, and the development of retinitis pigmentosa, a progressive retinal degeneration characterized by night blindness and visual field loss over several decades. The causes of Usher syndrome are unknown and no animal models have been available for study. Four human gene sites have been reported, suggesting at least four separate forms of Usher syndrome. We report a mouse model of type I Usher syndrome, rd5, whose linkage on mouse chromosome 7 to Hbb and tub has homology to human Usher I reported on human chromosome 11p15. The electroretinogram in homozygous rd5/rd5 mouse is never normal with reduced amplitudes that extinguish by 6 months. Auditory-evoked response testing demonstrates increased hearing thresholds more than control at 3 weeks of about 30 decibels (dB) that worsen to about 45 dB by 6 months.</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>We now report the purification of a 150 kDa reaper-interacting protein from Xenopus egg extracts, which we have named Scythe. Scythe is highly conserved among vertebrates and contains a ubiquitin-like domain near its N-terminus.</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>BAG cochaperone 6</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Reaper is a central regulator of apoptosis in Drosophila melanogaster. With no obvious catalytic activity or homology to other known apoptotic regulators, reaper's mechanism of action has been obscure. We recently reported that recombinant Drosophila reaper protein induced rapid mitochondrial cytochrome c release, caspase activation and apoptotic nuclear fragmentation in extracts of Xenopus eggs. We now report the purification of a 150 kDa reaper-interacting protein from Xenopus egg extracts, which we have named Scythe. Scythe is highly conserved among vertebrates and contains a ubiquitin-like domain near its N-terminus. Immunodepletion of Scythe from extracts completely prevented reaper-induced apoptosis without affecting apoptosis triggered by activated caspases. Moreover, a truncated variant of Scythe lacking the N-terminal domain induced apoptosis even in the absence of reaper. These data suggest that Scythe is a novel apoptotic regulator that is an essential component in the pathway of reaper-induced apoptosis.</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>PMID: 9799223
+Abstract: Reaper is a central regulator of apoptosis in Drosophila melanogaster. With no obvious catalytic activity or homology to other known apoptotic regulators, reaper's mechanism of action has been obscure. We recently reported that recombinant Drosophila reaper protein induced rapid mitochondrial cytochrome c release, caspase activation and apoptotic nuclear fragmentation in extracts of Xenopus eggs. We now report the purification of a 150 kDa reaper-interacting protein from Xenopus egg extracts, which we have named Scythe. Scythe is highly conserved among vertebrates and contains a ubiquitin-like domain near its N-terminus. Immunodepletion of Scythe from extracts completely prevented reaper-induced apoptosis without affecting apoptosis triggered by activated caspases. Moreover, a truncated variant of Scythe lacking the N-terminal domain induced apoptosis even in the absence of reaper. These data suggest that Scythe is a novel apoptotic regulator that is an essential component in the pathway of reaper-induced apoptosis.</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
-    Alias gene symbol: rd5
-    HGNC record ID: HGNC:12406
-    Primary gene symbol: TUB
-    Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Alias gene symbol: SCYTHE
+    HGNC record ID: HGNC:13919
+    Primary gene symbol: BAG6
+    Official HGNC gene name: BAG cochaperone 6
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
-PMID: 7479945
-Abstract: Usher syndrome is a group of diseases with autosomal recessive inheritance, congenital hearing loss, and the development of retinitis pigmentosa, a progressive retinal degeneration characterized by night blindness and visual field loss over several decades. The causes of Usher syndrome are unknown and no animal models have been available for study. Four human gene sites have been reported, suggesting at least four separate forms of Usher syndrome. We report a mouse model of type I Usher syndrome, rd5, whose linkage on mouse chromosome 7 to Hbb and tub has homology to human Usher I reported on human chromosome 11p15. The electroretinogram in homozygous rd5/rd5 mouse is never normal with reduced amplitudes that extinguish by 6 months. Auditory-evoked response testing demonstrates increased hearing thresholds more than control at 3 weeks of about 30 decibels (dB) that worsen to about 45 dB by 6 months.</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr">
+PMID: 9799223
+Abstract: Reaper is a central regulator of apoptosis in Drosophila melanogaster. With no obvious catalytic activity or homology to other known apoptotic regulators, reaper's mechanism of action has been obscure. We recently reported that recombinant Drosophila reaper protein induced rapid mitochondrial cytochrome c release, caspase activation and apoptotic nuclear fragmentation in extracts of Xenopus eggs. We now report the purification of a 150 kDa reaper-interacting protein from Xenopus egg extracts, which we have named Scythe. Scythe is highly conserved among vertebrates and contains a ubiquitin-like domain near its N-terminus. Immunodepletion of Scythe from extracts completely prevented reaper-induced apoptosis without affecting apoptosis triggered by activated caspases. Moreover, a truncated variant of Scythe lacking the N-terminal domain induced apoptosis even in the absence of reaper. These data suggest that Scythe is a novel apoptotic regulator that is an essential component in the pathway of reaper-induced apoptosis.</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
         <is>
           <t>{
-"pmid": "7479945",
-"alias_symbol": "rd5",
-"primary_gene_symbol": "TUB",
-"name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"pmid": "9799223",
+"alias_symbol": "SCYTHE",
+"primary_gene_symbol": "BAG6",
+"name": "BAG cochaperone 6",
+"alternate_abbreviation": "NO",
 "evidence": ""
 }</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>HGNC:12406</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>ENSG00000166402</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>GENE ID:7275</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>TUB</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>rd5</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>HGNC:13919</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ENSG00000234651, ENSG00000096155, ENSG00000233348, ENSG00000204463, ENSG00000228760, ENSG00000229524, ENSG00000227761</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>GENE ID:7917</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>BAG6</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SCYTHE</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>9390831</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>37879364</v>
+      </c>
+      <c r="I18" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>mouse phenotype biomarker</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>literature defined (uniprot alternative protein name)</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>abstract</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>Mice homozygous for a defect of the tub (rd5) gene exhibit cochlear and retinal degeneration combined with obesity, and resemble certain human autosomal recessive sensory deficit syndromes.</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>TUB bipartite transcription factor</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>These authors contributed equally to this work.
-These authors jointly coordinated this work.
-Inherited retinal degeneration (IRD) represents a clinically variable and genetically heterogeneous group of disorders characterized by photoreceptor dysfunction. These diseases typically present with progressive severe vision loss and variable onset, ranging from birth to adulthood. Genomic sequencing has allowed to identify novel IRD-related genes, most of which encode proteins contributing to photoreceptor-cilia biogenesis and/or function. Despite these insights, knowledge gaps hamper a molecular diagnosis in one-third of IRD cases. By exome sequencing in a cohort of molecularly unsolved individuals with IRD, we identified a homozygous splice site variant affecting the transcript processing of TUB, encoding the first member of the Tubby family of bipartite transcription factors, in a sporadic case with retinal dystrophy. A truncating homozygous variant in this gene had previously been reported in a single family with three subjects sharing retinal dystrophy and obesity. The clinical assessment of the present patient documented a slightly increased body mass index and no changes in metabolic markers of obesity, but confirmed the occurrence of retinal detachment. In vitro studies using patient-derived fibroblasts showed the accelerated degradation of the encoded protein and aberrant cilium morphology and biogenesis. These findings definitely link impaired TUB function to retinal dystrophy and provide new data on the clinical characterization of this ultra-rare retinal ciliopathy.
-Inherited retinal degeneration (IRD) occurs in a clinically variable and genetically heterogeneous group of conditions characterized by photoreceptor degeneration and/or dysfunction [1]. The prevalence of monogenic IRD is estimated as 1 in 2000 individuals, affecting more than 2 million people worldwide [2]. This group of disorders typically present with severe vision loss that can be progressive, having an onset ranging from birth to late adulthood. Severe visual impairment affects mobility and independence, posing relevant psychological and economic burdens [3]. In the last ten years, genomic sequencing has allowed the identification of several genes implicated in IRD (for an updated list see the RetNet database,https://sph.uth.edu/retnet/). These genes encode proteins that have different roles in visual function, contributing to key processes in the cells of the pigmented cell layer and neurosensory retina [4,5]. Notably, retinal degeneration is frequently observed in ciliopathies, and a portion of IRD-related genes codifies for proteins involved in biogenesis and the maintenance of photoreceptor primary cilium [6,7,8,9]. Among these genes,TUB[MIM #601197], which encodes the first member of the Tubby family of bipartite transcription factors, has recently reported to be associated with a novel condition characterized by retinal dystrophy and obesity [MIM #616188] [10]. A truncating homozygousTUBvariant [c.1194_1195delAG, p.Arg398Serfs*9] was identified in a single family with three affected members, suggesting loss of function (LoF) as the pathomechanism underlying the disorder. The TUB family of transcription factors counts four members in vertebrates (TUB, TULP1, TULP2 and TULP3), sharing a similar domain organization including a highly conserved C-terminal domain mediating DNA binding and a divergent N-terminal region encompassing the nuclear localization signal and the transcriptional activation domain implicated in protein–protein binding [11]. A conserved region at the N-terminus enables some members of the Tubby family, including TUB, to bind to the ciliary intraflagellar transport A protein (IFTAP) [12]. Similar to the other members of the TULP family, TUB is also implicated in the control of the initiation of phagocytosis, facilitating the removal of apoptotic cells or cellular debris by retinal pigmented epithelium (RPE) cells and macrophages [13]. Since the original report, no other subject carrying biallelicTUBvariants has been described.
-In this study, we report on an additional subject with retinal dystrophy carrying a homozygous LoF variant inTUB. In vitro analyses provide evidence of the disruptive functional impact of the variant onTUBtranscript processing. We also show that the loss of TUB is associated with a defective cilium morphology and biogenesis in the primary patient’s fibroblasts. Our findings confirm the involvement of defective TUB function in retinal dystrophy and define this disorder as a novel ciliopathy.
-The proband is a 35-year-old male, the first child of healthy non-consanguineous parents of European descent (Figure 1). Family history was negative for retinal diseases or other congenital defects. The proband was born at term after an uneventful pregnancy. Length and weight at birth were reported as within the normal range. Apgar score was 8–10. No hearing impairment and/or learning difficulties were documented during the first year of age.
-At 5 years, the subject required consulting ophthalmologists for referring color blindness. A “blonde” aspect of the fundus oculi was observed and reduced full-field flash photopic and scotopic electroretinogram (ERG) responses were recorded. Visual acuity was not investigated at that time. Ophthalmological assessment at 26 years was suggestive of cone-rod dystrophy. Visual acuity was 0.8 Snellen in his right eye (RE) with myopic and astigmatic refractive error (RE: -4.50 dioptre sphere and -1 dioptre cylinder at 20°), and 0.2 Snellen in his left eye (LE) with myopic refractive error (LE: -2.00 dioptre sphere). Goldmann visual field was generally constricted, with reduced sensitivity in the superior central field in the RE and presented peripheral constriction and relative central scotoma in the LE. Light and dark adaptation sensitivity curves showed abnormal thresholds for both cones and rods. No number at the Ishihara charts were recognized. Intraocular pressure was within normal limits. The slit lamp examination biomicroscopy of the anterior segment was normal for cornea, iris and lens appearance. Fundus examination revealed bilateral optic disc pallor, depigmented aspect of the choroidal and retinal structures, diffuse retinal dystrophy with absence of intraretinal pigment dispersion or vitreous abnormalities and arteriolar attenuation. Full-field scotopic and photopic electroretinograms showed reduced a-wave and b-wave amplitude responses and delayed implicit times. Multifocal ERG ring analysis documented reduced response amplitude densities in all examined areas from the foveal center up to 20° of foveal eccentricity in both eyes (LE &gt; RE). After reduced visual field in his LE, a large area of retinoschisis in the infero-temporal sector was observed by fundoscopy, which later progressed, resulting in full retinal detachment of the LE. The subject underwent to pars plana vitrectomy with silicon oil (30% polydimethylsiloxane, PDMS) tamponade. He underwent cataract surgery in his LE and to subsequent vitreo-retinal surgeries for relapsing retinal detachments in same eye (PDMS/perfluorocarbon liquid (PFCL)/PDMS tamponades exchange and intra-operatory laser treatment; PDMS/heavy silicon oil tamponades exchange and intra-operatory laser). One year later, he developed vitreo-retinal proliferation and retinal fibrosis in the LE, and visual acuity was hand motion; therefore, the subject underwent retinotomy and heavy silicon oil/PDMS tamponades exchange.
-At last evaluation (35 years), the subject presented with a good clinical condition. No cognitive deficit nor behavioral issues were observed, and no craniofacial dysmorphism and truncal obesity were noticed. An accurate endocrinological examination was uninformative. Anthropometric assessment displayed a height of 177.5 cm (+0.1 SD), weight of 95.70 kg (+1.6 SD), and OFC 60 cm (+0.2 SD) and BMI of 30.30 Kg/m2(+1.6 SD). Tanner stage was Ph5Pg5, with a testicular volume 20 mL bilaterally. The subject’s visual acuity was 0.8 Snellen in his RE and light perception in his LE. Fundus oculi showed the unmodified condition of RE and diffuse chorio-retinal atrophy in the LE, as for visible vitreo-retinal surgical outcomes. Ultrawide field fundus photography showed macular atrophy in absence of peripheral pigment and confirmed a “blonde” aspect of the retina (Figure 2A). Fundus autofluorescence (FAF) revealed an hypoautoflorescent area in the macula due to RPE atrophy and hyper/hypoautofluorescence mottling in the posterior pole and immediately outside the vascular arcades (Figure 2B). The SD-OCT showed a disruption of the outer retina, including ELM, ellipsoid zone and RPE with outer retinal debris at the level of the RPE in the parafoveal region (Figure 2C). Full-field flash scotopic (Figure 2D) and photopic ERG confirmed reduced a-wave and b-wave amplitude responses and delayed implicit times in the RE. Similarly, multifocal ERG ring analysis, recordable only in the RE, showed the worsening of the response amplitude densities in all examined areas (0–20°) (Figure 2E), as compared to the previous examinations. Similarly, Goldmann visual field in his RE showed progressive constriction of the peripheral isopters and a ring scotoma enclosed between 10–20° of the visual field (Figure 2F); it was not executable, however, in his LE. Color blindness was also confirmed. Neck and abdominal ultrasound assessment did not reveal any abnormality. Measurements of basal hormones by the anterior pituitary, glycaemia and insulin were within the normal range. Basal plasma leptin level was in the low normal range, showing no leptin resistance. During his follow-up, clinical and ophthalmological assessments of other family members (parents and younger brother) were unremarkable.
-Trio-based WES allowed to identify a homozygous splice siteTUBvariant (chr11:8122545G &gt; A, GRCh37.p13; c.1387 + 1G &gt; A,NM_177972.3) as the only clinically and functionally relevant event putatively linked to the disorder (Supplemental Table S1). The variant had previously been annotated in public databases (dbSNP, rs1040410003) with low frequency (gnomAD v3.1, MAF = 0.00001972) at the heterozygous state. It was classified as likely pathogenic (PVS1/PM2/PP5) according to the American College of Medical Genetics and Genomics-Association for Molecular Pathology (ACMG-AMP) criteria (ClinVar: VCV000865971.1) [14]. Sanger sequencing confirmed the homozygosity for the variant in the proband and the heterozygous status in the healthy parents and unaffected sib (Figure 1).
-Since the variant was predicted to affect the exon 11 donor splice site, the total RNA from patient-derived skin primary fibroblasts was used to characterize the impact of the nucleotide change on transcript processing. The cDNA fragment encompassing the relevant exons was amplified, confirming the presence of two aberrantly spliced products (Figure 3A). The two aberrant PCR amplicons were isolated from agarose gel, purified and sequenced via Sanger. The former (500 bp) was derived from skipping of the penultimate exon (exon 11, ENST00000299506.3), resulting in a premature termination codon (i.e., p.Glu406Argfs*4), while the latter (1172 bp) was the result of retention of intron 10, resulting in a TUB protein having a divergent 19-residue-long C-terminus and lacking the last 44 amino acids (p.Pro463Hisfs*19) (Figure 3B).
-In the patient’s skin fibroblasts, the predicted TUBGlu406Argfs*4protein was undetectable by Western blot [WB] analysis, while the TUBPro463Hisfs*19protein was poorly detectable likely due to accelerated degradation (Figure 3C, left panel). Consistently, the endogenous TUBPro463Hisfs*19level was partially rescued by blocking the proteasomal degradation pathway using MG132 (Figure 3C, right panel).
-To investigate the cellular localization of the mutated protein, cytoplasm and nuclear cell fractions were obtained and analyzed by WB. The results demonstrate that both the wild-type (wt) and mutant TUB proteins were almost exclusively localized in the nucleus (Figure 3D). This finding was also confirmed by confocal microscopy analysis that evidenced the nuclear localization of the TUB mutant (Figure 4A).
-Based on the documented role of TUB in early ciliogenesis [15], we assessed the localization of TUB at the cilium, but we failed to observe any consistent co-localization, possibly due to the low diffused levels of the protein in the cytoplasm To investigate the impact of defective TUB function on the morphogenesis of the primary cilium, a confocal analysis on primary fibroblasts was performed using antibodies against ARL13B, which localizes to primary cilia, and pericentrin, a component of the centrosome, which stains the basal body. As shown inFigure 4B, while almost all the control cells showed a primary cilium, 40% of the fibroblasts carrying the homozygous splice site variant inTUBdid not show a primary cilium. Moreover, while no significant difference was observed in ciliary axoneme length between the starved control and mutant cells, a large percentage of the latter showed an abnormal cilium morphology and a poorly defined and disorganized basal body (Figure 4C).
-The loss of TUB function was recently reported to underlie a novel IRD condition based on the identification of homozygosity for a 2 bp deletion (c.1194_1195delAG) causing the premature termination of the protein (p.Arg398Serfs*9) shared by three affected members of a single consanguineous family [10]. While the combination of retinal dystrophy and early onset obesity can be reminiscent of other disorders (e.g., Bardet–Biedl syndrome (MIM#PS209900) and Alstrom syndrome (MIM#203800)), the absence of other clinically relevant feature/sign was suggestive of a previously unreported ciliopathy [10]. In this paper, we report on a second disruptive variant (c.1387 + 1G &gt; A) affectingTUBin a subject with features that overlap with those previously described in the affected members of the original family.
-In the present and previously reported affected individuals, the ocular phenotype associated with defective TUB function is characterized by widespread retinal pigment epithelial (RPE) atrophy, deteriorating vision, the myopic and astigmatic refractive defect, the blonde fundus appearance, the ERG and OCT findings and progression of the disease (Figure 2). Notably, retinal detachment, without vitreous hemorrhage, was invariantly documented in the four individuals with biallelic inactivatingTUBvariants, suggesting that this feature likely represent a common finding in the disorder.
-Early onset obesity had previously been considered a major feature of the TUB-related condition [10], even though only two of three affected sibs were found obese (BMI &gt; 30), and the glycemic and lipid profiles in one of affected sibs were found within the normal range. The finding of obesity in the apparently healthy father (heterozygous carrier) suggests a possible co-occurring genetic event contributing to obesity in the family. In the present report, the clinical assessment of the affected individual documented increased weight (95.7 kg, +1.6 SD) and BMI (30.3, +1.6 SD), thus indicating overweight, in absence of other signs of obesity. Although evidence suggests that a defective TUB function may result in disturbances in insulin and leptin activity and obesity in mice [16,17,18,19], based on the collected findings, the relevance of TUB in human obesity requires further study. To assess whether TUB LoF could impact on hypothalamic pathways, food intake and adiposity, the metabolic profile of the affected individual was investigated. Accurate endocrinological examination did not reveal any abnormality, and the measurements of basal hormones by the anterior pituitary, glycaemia, insulin and leptin were within the normal range, thus ruling out insulin or leptin resistance. Consistently, instrumental investigations (X-ray and ultrasound analyses) documented no sign of glycogen accumulation in the internal organs. Consistently, the absence of significant changes in lipid storage was demonstrated by thin-layer chromatography (HPTLC) analysis in proband-derived fibroblast (Figure S1), allowing to confirm an apparently normal endocrine–metabolic profile in the affected individual. Of note, the Tubby protein has been involved in cochlear degeneration [20,21]. Based on this functional link, we evaluated the occurrence of hearing problems and cochlear degeneration, which were not observed.
-The homozygousTUBvariant was predicted to affect transcript processing, causing the skipping of exon 11 and intron retention, resulting in a frameshift with the premature termination of the TUB protein. mRNA analysis in proband-derived fibroblasts confirmed a disruptive impact of the splice site change documenting two aberrantly processed transcripts predicted to encode a 406-residue-long protein (p.Glu406Argfs*4) that probably is not able to proceed in protein synthesis, and a 481-residue-long protein (p.Pro463Hisfs*19) characterized by a divergent C-terminus characterized by accelerated degradation (Figure 3B). These findings confirm LoF as the pathomechanism underlying this disorder.
-Primary cilia are microtubule-based organelles that extend from the apical surface of the majority of mammalian cells. Cilia act as “cellular antennae”, receiving different inputs from the extracellular environment and transducing signals in response to stimuli [22]. A complex process required for proper cilia biogenesis function is the intraflagellar transport, which is required for assembling cilia and trafficking within primary cilia [23]. In this context, IFT-A has historically been believed to mediate retrograde intraflagellar transport inside the cilia and an IFT-A-binding domain at the TUB N-terminus has been demonstrated recently [24]. Moreover, co-localization between TUB and rootletin, the major structural component of the ciliary rootlet, has been observed in human retinal photoreceptors [10]. The use of a more informative in vitro model (e.g., induced pluripotent-stem-cell-derived retinal-pigment epithelium cells) and experimental strategies (e.g., siRNA-mediated TUB silencing) is required to appreciate more accurately the functional relevance of TUB in an appropriate cellular context.
-In summary, we confirm the link between TUB LoF and a new condition of human retinal ciliopathy and provide evidence of an altered cilium morphology/biogenesis in patient-derived fibroblasts. In fact, these cells displayed a reduced number of cilia when compared to the control cells, with a poorly defined and disorganized basal body structure, which are expected to prevent normal protein trafficking along the cilium. While these findings could explain the degeneration of photoreceptors characterizing this disorder, a relatively overall mild presentation has been associated with mutations in this gene. Multiple factors might contribute to this picture. First, the functional relevance of TUB in the context of ciliogenesis and cilium function might vary in different cell lineages. Second, functional compensation exerted by other related proteins might contribute to buffer the severity of the endophenotype. Third, specific cell lineages (e.g., rod and cone cells) might be particularly sensitive to TUB LoF. The collection of additional patients with biallelic variants in the gene will allow a more accurate characterization of the clinical spectrum associated with TUB LoF. Based on these considerations, TUB loss of function could be considered as responsible for a novel form of isolated retinal ciliopathy.</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>Mice homozygous for a defect of the tub (rd5) gene exhibit cochlear and retinal degeneration combined with obesity, and resemble certain human autosomal recessive sensory deficit syndromes. To establish the progressive nature of sensory cell loss associated with the tub gene, and to differentiate tub-related losses from those associated with the C57 background on which tub arose, we evaluated cochleas and retinas from tub/tub, tub/+, and +/+ mice, aged 2 weeks to 1 year by light and electron microscopy. Cochleas from mice of all three genotypes show progressive inner (IHC) and outer hair cell (OHC) loss. Relative to tub/+ and +/+ animals, however, tub homozygotes show accelerated OHC loss, affecting the extreme cochlear base (hook region) by 1 month, and the apex by 6 months. IHC loss in tub/tub animals is accelerated in the basal half of the cochlea, affecting the hook region by 6 months. Spiral ganglion cell losses were observed only in tub/tub mice, and only in the cochlear base. Retinas of tub/tub mice are abnormal at maturity, exhibiting shortened photoreceptor outer segments by 2 weeks, and progressive photoreceptor loss thereafter. Because the tub mutation causes degeneration of sensory cells in the ear and eye but has no other neurological effects, tubby mice hold unique promise for the study of human syndromic sensory loss.</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>PMID: 9390831
-Full Text: These authors contributed equally to this work.
-These authors jointly coordinated this work.
-Inherited retinal degeneration (IRD) represents a clinically variable and genetically heterogeneous group of disorders characterized by photoreceptor dysfunction. These diseases typically present with progressive severe vision loss and variable onset, ranging from birth to adulthood. Genomic sequencing has allowed to identify novel IRD-related genes, most of which encode proteins contributing to photoreceptor-cilia biogenesis and/or function. Despite these insights, knowledge gaps hamper a molecular diagnosis in one-third of IRD cases. By exome sequencing in a cohort of molecularly unsolved individuals with IRD, we identified a homozygous splice site variant affecting the transcript processing of TUB, encoding the first member of the Tubby family of bipartite transcription factors, in a sporadic case with retinal dystrophy. A truncating homozygous variant in this gene had previously been reported in a single family with three subjects sharing retinal dystrophy and obesity. The clinical assessment of the present patient documented a slightly increased body mass index and no changes in metabolic markers of obesity, but confirmed the occurrence of retinal detachment. In vitro studies using patient-derived fibroblasts showed the accelerated degradation of the encoded protein and aberrant cilium morphology and biogenesis. These findings definitely link impaired TUB function to retinal dystrophy and provide new data on the clinical characterization of this ultra-rare retinal ciliopathy.
-Inherited retinal degeneration (IRD) occurs in a clinically variable and genetically heterogeneous group of conditions characterized by photoreceptor degeneration and/or dysfunction [1]. The prevalence of monogenic IRD is estimated as 1 in 2000 individuals, affecting more than 2 million people worldwide [2]. This group of disorders typically present with severe vision loss that can be progressive, having an onset ranging from birth to late adulthood. Severe visual impairment affects mobility and independence, posing relevant psychological and economic burdens [3]. In the last ten years, genomic sequencing has allowed the identification of several genes implicated in IRD (for an updated list see the RetNet database,https://sph.uth.edu/retnet/). These genes encode proteins that have different roles in visual function, contributing to key processes in the cells of the pigmented cell layer and neurosensory retina [4,5]. Notably, retinal degeneration is frequently observed in ciliopathies, and a portion of IRD-related genes codifies for proteins involved in biogenesis and the maintenance of photoreceptor primary cilium [6,7,8,9]. Among these genes,TUB[MIM #601197], which encodes the first member of the Tubby family of bipartite transcription factors, has recently reported to be associated with a novel condition characterized by retinal dystrophy and obesity [MIM #616188] [10]. A truncating homozygousTUBvariant [c.1194_1195delAG, p.Arg398Serfs*9] was identified in a single family with three affected members, suggesting loss of function (LoF) as the pathomechanism underlying the disorder. The TUB family of transcription factors counts four members in vertebrates (TUB, TULP1, TULP2 and TULP3), sharing a similar domain organization including a highly conserved C-terminal domain mediating DNA binding and a divergent N-terminal region encompassing the nuclear localization signal and the transcriptional activation domain implicated in protein–protein binding [11]. A conserved region at the N-terminus enables some members of the Tubby family, including TUB, to bind to the ciliary intraflagellar transport A protein (IFTAP) [12]. Similar to the other members of the TULP family, TUB is also implicated in the control of the initiation of phagocytosis, facilitating the removal of apoptotic cells or cellular debris by retinal pigmented epithelium (RPE) cells and macrophages [13]. Since the original report, no other subject carrying biallelicTUBvariants has been described.
-In this study, we report on an additional subject with retinal dystrophy carrying a homozygous LoF variant inTUB. In vitro analyses provide evidence of the disruptive functional impact of the variant onTUBtranscript processing. We also show that the loss of TUB is associated with a defective cilium morphology and biogenesis in the primary patient’s fibroblasts. Our findings confirm the involvement of defective TUB function in retinal dystrophy and define this disorder as a novel ciliopathy.
-The proband is a 35-year-old male, the first child of healthy non-consanguineous parents of European descent (Figure 1). Family history was negative for retinal diseases or other congenital defects. The proband was born at term after an uneventful pregnancy. Length and weight at birth were reported as within the normal range. Apgar score was 8–10. No hearing impairment and/or learning difficulties were documented during the first year of age.
-At 5 years, the subject required consulting ophthalmologists for referring color blindness. A “blonde” aspect of the fundus oculi was observed and reduced full-field flash photopic and scotopic electroretinogram (ERG) responses were recorded. Visual acuity was not investigated at that time. Ophthalmological assessment at 26 years was suggestive of cone-rod dystrophy. Visual acuity was 0.8 Snellen in his right eye (RE) with myopic and astigmatic refractive error (RE: -4.50 dioptre sphere and -1 dioptre cylinder at 20°), and 0.2 Snellen in his left eye (LE) with myopic refractive error (LE: -2.00 dioptre sphere). Goldmann visual field was generally constricted, with reduced sensitivity in the superior central field in the RE and presented peripheral constriction and relative central scotoma in the LE. Light and dark adaptation sensitivity curves showed abnormal thresholds for both cones and rods. No number at the Ishihara charts were recognized. Intraocular pressure was within normal limits. The slit lamp examination biomicroscopy of the anterior segment was normal for cornea, iris and lens appearance. Fundus examination revealed bilateral optic disc pallor, depigmented aspect of the choroidal and retinal structures, diffuse retinal dystrophy with absence of intraretinal pigment dispersion or vitreous abnormalities and arteriolar attenuation. Full-field scotopic and photopic electroretinograms showed reduced a-wave and b-wave amplitude responses and delayed implicit times. Multifocal ERG ring analysis documented reduced response amplitude densities in all examined areas from the foveal center up to 20° of foveal eccentricity in both eyes (LE &gt; RE). After reduced visual field in his LE, a large area of retinoschisis in the infero-temporal sector was observed by fundoscopy, which later progressed, resulting in full retinal detachment of the LE. The subject underwent to pars plana vitrectomy with silicon oil (30% polydimethylsiloxane, PDMS) tamponade. He underwent cataract surgery in his LE and to subsequent vitreo-retinal surgeries for relapsing retinal detachments in same eye (PDMS/perfluorocarbon liquid (PFCL)/PDMS tamponades exchange and intra-operatory laser treatment; PDMS/heavy silicon oil tamponades exchange and intra-operatory laser). One year later, he developed vitreo-retinal proliferation and retinal fibrosis in the LE, and visual acuity was hand motion; therefore, the subject underwent retinotomy and heavy silicon oil/PDMS tamponades exchange.
-At last evaluation (35 years), the subject presented with a good clinical condition. No cognitive deficit nor behavioral issues were observed, and no craniofacial dysmorphism and truncal obesity were noticed. An accurate endocrinological examination was uninformative. Anthropometric assessment displayed a height of 177.5 cm (+0.1 SD), weight of 95.70 kg (+1.6 SD), and OFC 60 cm (+0.2 SD) and BMI of 30.30 Kg/m2(+1.6 SD). Tanner stage was Ph5Pg5, with a testicular volume 20 mL bilaterally. The subject’s visual acuity was 0.8 Snellen in his RE and light perception in his LE. Fundus oculi showed the unmodified condition of RE and diffuse chorio-retinal atrophy in the LE, as for visible vitreo-retinal surgical outcomes. Ultrawide field fundus photography showed macular atrophy in absence of peripheral pigment and confirmed a “blonde” aspect of the retina (Figure 2A). Fundus autofluorescence (FAF) revealed an hypoautoflorescent area in the macula due to RPE atrophy and hyper/hypoautofluorescence mottling in the posterior pole and immediately outside the vascular arcades (Figure 2B). The SD-OCT showed a disruption of the outer retina, including ELM, ellipsoid zone and RPE with outer retinal debris at the level of the RPE in the parafoveal region (Figure 2C). Full-field flash scotopic (Figure 2D) and photopic ERG confirmed reduced a-wave and b-wave amplitude responses and delayed implicit times in the RE. Similarly, multifocal ERG ring analysis, recordable only in the RE, showed the worsening of the response amplitude densities in all examined areas (0–20°) (Figure 2E), as compared to the previous examinations. Similarly, Goldmann visual field in his RE showed progressive constriction of the peripheral isopters and a ring scotoma enclosed between 10–20° of the visual field (Figure 2F); it was not executable, however, in his LE. Color blindness was also confirmed. Neck and abdominal ultrasound assessment did not reveal any abnormality. Measurements of basal hormones by the anterior pituitary, glycaemia and insulin were within the normal range. Basal plasma leptin level was in the low normal range, showing no leptin resistance. During his follow-up, clinical and ophthalmological assessments of other family members (parents and younger brother) were unremarkable.
-Trio-based WES allowed to identify a homozygous splice siteTUBvariant (chr11:8122545G &gt; A, GRCh37.p13; c.1387 + 1G &gt; A,NM_177972.3) as the only clinically and functionally relevant event putatively linked to the disorder (Supplemental Table S1). The variant had previously been annotated in public databases (dbSNP, rs1040410003) with low frequency (gnomAD v3.1, MAF = 0.00001972) at the heterozygous state. It was classified as likely pathogenic (PVS1/PM2/PP5) according to the American College of Medical Genetics and Genomics-Association for Molecular Pathology (ACMG-AMP) criteria (ClinVar: VCV000865971.1) [14]. Sanger sequencing confirmed the homozygosity for the variant in the proband and the heterozygous status in the healthy parents and unaffected sib (Figure 1).
-Since the variant was predicted to affect the exon 11 donor splice site, the total RNA from patient-derived skin primary fibroblasts was used to characterize the impact of the nucleotide change on transcript processing. The cDNA fragment encompassing the relevant exons was amplified, confirming the presence of two aberrantly spliced products (Figure 3A). The two aberrant PCR amplicons were isolated from agarose gel, purified and sequenced via Sanger. The former (500 bp) was derived from skipping of the penultimate exon (exon 11, ENST00000299506.3), resulting in a premature termination codon (i.e., p.Glu406Argfs*4), while the latter (1172 bp) was the result of retention of intron 10, resulting in a TUB protein having a divergent 19-residue-long C-terminus and lacking the last 44 amino acids (p.Pro463Hisfs*19) (Figure 3B).
-In the patient’s skin fibroblasts, the predicted TUBGlu406Argfs*4protein was undetectable by Western blot [WB] analysis, while the TUBPro463Hisfs*19protein was poorly detectable likely due to accelerated degradation (Figure 3C, left panel). Consistently, the endogenous TUBPro463Hisfs*19level was partially rescued by blocking the proteasomal degradation pathway using MG132 (Figure 3C, right panel).
-To investigate the cellular localization of the mutated protein, cytoplasm and nuclear cell fractions were obtained and analyzed by WB. The results demonstrate that both the wild-type (wt) and mutant TUB proteins were almost exclusively localized in the nucleus (Figure 3D). This finding was also confirmed by confocal microscopy analysis that evidenced the nuclear localization of the TUB mutant (Figure 4A).
-Based on the documented role of TUB in early ciliogenesis [15], we assessed the localization of TUB at the cilium, but we failed to observe any consistent co-localization, possibly due to the low diffused levels of the protein in the cytoplasm To investigate the impact of defective TUB function on the morphogenesis of the primary cilium, a confocal analysis on primary fibroblasts was performed using antibodies against ARL13B, which localizes to primary cilia, and pericentrin, a component of the centrosome, which stains the basal body. As shown inFigure 4B, while almost all the control cells showed a primary cilium, 40% of the fibroblasts carrying the homozygous splice site variant inTUBdid not show a primary cilium. Moreover, while no significant difference was observed in ciliary axoneme length between the starved control and mutant cells, a large percentage of the latter showed an abnormal cilium morphology and a poorly defined and disorganized basal body (Figure 4C).
-The loss of TUB function was recently reported to underlie a novel IRD condition based on the identification of homozygosity for a 2 bp deletion (c.1194_1195delAG) causing the premature termination of the protein (p.Arg398Serfs*9) shared by three affected members of a single consanguineous family [10]. While the combination of retinal dystrophy and early onset obesity can be reminiscent of other disorders (e.g., Bardet–Biedl syndrome (MIM#PS209900) and Alstrom syndrome (MIM#203800)), the absence of other clinically relevant feature/sign was suggestive of a previously unreported ciliopathy [10]. In this paper, we report on a second disruptive variant (c.1387 + 1G &gt; A) affectingTUBin a subject with features that overlap with those previously described in the affected members of the original family.
-In the present and previously reported affected individuals, the ocular phenotype associated with defective TUB function is characterized by widespread retinal pigment epithelial (RPE) atrophy, deteriorating vision, the myopic and astigmatic refractive defect, the blonde fundus appearance, the ERG and OCT findings and progression of the disease (Figure 2). Notably, retinal detachment, without vitreous hemorrhage, was invariantly documented in the four individuals with biallelic inactivatingTUBvariants, suggesting that this feature likely represent a common finding in the disorder.
-Early onset obesity had previously been considered a major feature of the TUB-related condition [10], even though only two of three affected sibs were found obese (BMI &gt; 30), and the glycemic and lipid profiles in one of affected sibs were found within the normal range. The finding of obesity in the apparently healthy father (heterozygous carrier) suggests a possible co-occurring genetic event contributing to obesity in the family. In the present report, the clinical assessment of the affected individual documented increased weight (95.7 kg, +1.6 SD) and BMI (30.3, +1.6 SD), thus indicating overweight, in absence of other signs of obesity. Although evidence suggests that a defective TUB function may result in disturbances in insulin and leptin activity and obesity in mice [16,17,18,19], based on the collected findings, the relevance of TUB in human obesity requires further study. To assess whether TUB LoF could impact on hypothalamic pathways, food intake and adiposity, the metabolic profile of the affected individual was investigated. Accurate endocrinological examination did not reveal any abnormality, and the measurements of basal hormones by the anterior pituitary, glycaemia, insulin and leptin were within the normal range, thus ruling out insulin or leptin resistance. Consistently, instrumental investigations (X-ray and ultrasound analyses) documented no sign of glycogen accumulation in the internal organs. Consistently, the absence of significant changes in lipid storage was demonstrated by thin-layer chromatography (HPTLC) analysis in proband-derived fibroblast (Figure S1), allowing to confirm an apparently normal endocrine–metabolic profile in the affected individual. Of note, the Tubby protein has been involved in cochlear degeneration [20,21]. Based on this functional link, we evaluated the occurrence of hearing problems and cochlear degeneration, which were not observed.
-The homozygousTUBvariant was predicted to affect transcript processing, causing the skipping of exon 11 and intron retention, resulting in a frameshift with the premature termination of the TUB protein. mRNA analysis in proband-derived fibroblasts confirmed a disruptive impact of the splice site change documenting two aberrantly processed transcripts predicted to encode a 406-residue-long protein (p.Glu406Argfs*4) that probably is not able to proceed in protein synthesis, and a 481-residue-long protein (p.Pro463Hisfs*19) characterized by a divergent C-terminus characterized by accelerated degradation (Figure 3B). These findings confirm LoF as the pathomechanism underlying this disorder.
-Primary cilia are microtubule-based organelles that extend from the apical surface of the majority of mammalian cells. Cilia act as “cellular antennae”, receiving different inputs from the extracellular environment and transducing signals in response to stimuli [22]. A complex process required for proper cilia biogenesis function is the intraflagellar transport, which is required for assembling cilia and trafficking within primary cilia [23]. In this context, IFT-A has historically been believed to mediate retrograde intraflagellar transport inside the cilia and an IFT-A-binding domain at the TUB N-terminus has been demonstrated recently [24]. Moreover, co-localization between TUB and rootletin, the major structural component of the ciliary rootlet, has been observed in human retinal photoreceptors [10]. The use of a more informative in vitro model (e.g., induced pluripotent-stem-cell-derived retinal-pigment epithelium cells) and experimental strategies (e.g., siRNA-mediated TUB silencing) is required to appreciate more accurately the functional relevance of TUB in an appropriate cellular context.
-In summary, we confirm the link between TUB LoF and a new condition of human retinal ciliopathy and provide evidence of an altered cilium morphology/biogenesis in patient-derived fibroblasts. In fact, these cells displayed a reduced number of cilia when compared to the control cells, with a poorly defined and disorganized basal body structure, which are expected to prevent normal protein trafficking along the cilium. While these findings could explain the degeneration of photoreceptors characterizing this disorder, a relatively overall mild presentation has been associated with mutations in this gene. Multiple factors might contribute to this picture. First, the functional relevance of TUB in the context of ciliogenesis and cilium function might vary in different cell lineages. Second, functional compensation exerted by other related proteins might contribute to buffer the severity of the endophenotype. Third, specific cell lineages (e.g., rod and cone cells) might be particularly sensitive to TUB LoF. The collection of additional patients with biallelic variants in the gene will allow a more accurate characterization of the clinical spectrum associated with TUB LoF. Based on these considerations, TUB loss of function could be considered as responsible for a novel form of isolated retinal ciliopathy.</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
-    Inputs:
-    Alias gene symbol: rd5
-    HGNC record ID: HGNC:12406
-    Primary gene symbol: TUB
-    Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
-    Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
-    Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
-    If the text does not support that the alias is an alternate abbreviation, return:
-    "alternate_abbreviation": "NO"
-    "evidence": ""
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
-    Evidence must be one exact sentence copied verbatim from the text.
-    Do not infer relationships or paraphrase evidence.
-    Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
-    {
-    "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
-    "alternate_abbreviation": "YES or NO",
-    "evidence": ""
-    }
-PMID: 9390831
-Full Text: These authors contributed equally to this work.
-These authors jointly coordinated this work.
-Inherited retinal degeneration (IRD) represents a clinically variable and genetically heterogeneous group of disorders characterized by photoreceptor dysfunction. These diseases typically present with progressive severe vision loss and variable onset, ranging from birth to adulthood. Genomic sequencing has allowed to identify novel IRD-related genes, most of which encode proteins contributing to photoreceptor-cilia biogenesis and/or function. Despite these insights, knowledge gaps hamper a molecular diagnosis in one-third of IRD cases. By exome sequencing in a cohort of molecularly unsolved individuals with IRD, we identified a homozygous splice site variant affecting the transcript processing of TUB, encoding the first member of the Tubby family of bipartite transcription factors, in a sporadic case with retinal dystrophy. A truncating homozygous variant in this gene had previously been reported in a single family with three subjects sharing retinal dystrophy and obesity. The clinical assessment of the present patient documented a slightly increased body mass index and no changes in metabolic markers of obesity, but confirmed the occurrence of retinal detachment. In vitro studies using patient-derived fibroblasts showed the accelerated degradation of the encoded protein and aberrant cilium morphology and biogenesis. These findings definitely link impaired TUB function to retinal dystrophy and provide new data on the clinical characterization of this ultra-rare retinal ciliopathy.
-Inherited retinal degeneration (IRD) occurs in a clinically variable and genetically heterogeneous group of conditions characterized by photoreceptor degeneration and/or dysfunction [1]. The prevalence of monogenic IRD is estimated as 1 in 2000 individuals, affecting more than 2 million people worldwide [2]. This group of disorders typically present with severe vision loss that can be progressive, having an onset ranging from birth to late adulthood. Severe visual impairment affects mobility and independence, posing relevant psychological and economic burdens [3]. In the last ten years, genomic sequencing has allowed the identification of several genes implicated in IRD (for an updated list see the RetNet database,https://sph.uth.edu/retnet/). These genes encode proteins that have different roles in visual function, contributing to key processes in the cells of the pigmented cell layer and neurosensory retina [4,5]. Notably, retinal degeneration is frequently observed in ciliopathies, and a portion of IRD-related genes codifies for proteins involved in biogenesis and the maintenance of photoreceptor primary cilium [6,7,8,9]. Among these genes,TUB[MIM #601197], which encodes the first member of the Tubby family of bipartite transcription factors, has recently reported to be associated with a novel condition characterized by retinal dystrophy and obesity [MIM #616188] [10]. A truncating homozygousTUBvariant [c.1194_1195delAG, p.Arg398Serfs*9] was identified in a single family with three affected members, suggesting loss of function (LoF) as the pathomechanism underlying the disorder. The TUB family of transcription factors counts four members in vertebrates (TUB, TULP1, TULP2 and TULP3), sharing a similar domain organization including a highly conserved C-terminal domain mediating DNA binding and a divergent N-terminal region encompassing the nuclear localization signal and the transcriptional activation domain implicated in protein–protein binding [11]. A conserved region at the N-terminus enables some members of the Tubby family, including TUB, to bind to the ciliary intraflagellar transport A protein (IFTAP) [12]. Similar to the other members of the TULP family, TUB is also implicated in the control of the initiation of phagocytosis, facilitating the removal of apoptotic cells or cellular debris by retinal pigmented epithelium (RPE) cells and macrophages [13]. Since the original report, no other subject carrying biallelicTUBvariants has been described.
-In this study, we report on an additional subject with retinal dystrophy carrying a homozygous LoF variant inTUB. In vitro analyses provide evidence of the disruptive functional impact of the variant onTUBtranscript processing. We also show that the loss of TUB is associated with a defective cilium morphology and biogenesis in the primary patient’s fibroblasts. Our findings confirm the involvement of defective TUB function in retinal dystrophy and define this disorder as a novel ciliopathy.
-The proband is a 35-year-old male, the first child of healthy non-consanguineous parents of European descent (Figure 1). Family history was negative for retinal diseases or other congenital defects. The proband was born at term after an uneventful pregnancy. Length and weight at birth were reported as within the normal range. Apgar score was 8–10. No hearing impairment and/or learning difficulties were documented during the first year of age.
-At 5 years, the subject required consulting ophthalmologists for referring color blindness. A “blonde” aspect of the fundus oculi was observed and reduced full-field flash photopic and scotopic electroretinogram (ERG) responses were recorded. Visual acuity was not investigated at that time. Ophthalmological assessment at 26 years was suggestive of cone-rod dystrophy. Visual acuity was 0.8 Snellen in his right eye (RE) with myopic and astigmatic refractive error (RE: -4.50 dioptre sphere and -1 dioptre cylinder at 20°), and 0.2 Snellen in his left eye (LE) with myopic refractive error (LE: -2.00 dioptre sphere). Goldmann visual field was generally constricted, with reduced sensitivity in the superior central field in the RE and presented peripheral constriction and relative central scotoma in the LE. Light and dark adaptation sensitivity curves showed abnormal thresholds for both cones and rods. No number at the Ishihara charts were recognized. Intraocular pressure was within normal limits. The slit lamp examination biomicroscopy of the anterior segment was normal for cornea, iris and lens appearance. Fundus examination revealed bilateral optic disc pallor, depigmented aspect of the choroidal and retinal structures, diffuse retinal dystrophy with absence of intraretinal pigment dispersion or vitreous abnormalities and arteriolar attenuation. Full-field scotopic and photopic electroretinograms showed reduced a-wave and b-wave amplitude responses and delayed implicit times. Multifocal ERG ring analysis documented reduced response amplitude densities in all examined areas from the foveal center up to 20° of foveal eccentricity in both eyes (LE &gt; RE). After reduced visual field in his LE, a large area of retinoschisis in the infero-temporal sector was observed by fundoscopy, which later progressed, resulting in full retinal detachment of the LE. The subject underwent to pars plana vitrectomy with silicon oil (30% polydimethylsiloxane, PDMS) tamponade. He underwent cataract surgery in his LE and to subsequent vitreo-retinal surgeries for relapsing retinal detachments in same eye (PDMS/perfluorocarbon liquid (PFCL)/PDMS tamponades exchange and intra-operatory laser treatment; PDMS/heavy silicon oil tamponades exchange and intra-operatory laser). One year later, he developed vitreo-retinal proliferation and retinal fibrosis in the LE, and visual acuity was hand motion; therefore, the subject underwent retinotomy and heavy silicon oil/PDMS tamponades exchange.
-At last evaluation (35 years), the subject presented with a good clinical condition. No cognitive deficit nor behavioral issues were observed, and no craniofacial dysmorphism and truncal obesity were noticed. An accurate endocrinological examination was uninformative. Anthropometric assessment displayed a height of 177.5 cm (+0.1 SD), weight of 95.70 kg (+1.6 SD), and OFC 60 cm (+0.2 SD) and BMI of 30.30 Kg/m2(+1.6 SD). Tanner stage was Ph5Pg5, with a testicular volume 20 mL bilaterally. The subject’s visual acuity was 0.8 Snellen in his RE and light perception in his LE. Fundus oculi showed the unmodified condition of RE and diffuse chorio-retinal atrophy in the LE, as for visible vitreo-retinal surgical outcomes. Ultrawide field fundus photography showed macular atrophy in absence of peripheral pigment and confirmed a “blonde” aspect of the retina (Figure 2A). Fundus autofluorescence (FAF) revealed an hypoautoflorescent area in the macula due to RPE atrophy and hyper/hypoautofluorescence mottling in the posterior pole and immediately outside the vascular arcades (Figure 2B). The SD-OCT showed a disruption of the outer retina, including ELM, ellipsoid zone and RPE with outer retinal debris at the level of the RPE in the parafoveal region (Figure 2C). Full-field flash scotopic (Figure 2D) and photopic ERG confirmed reduced a-wave and b-wave amplitude responses and delayed implicit times in the RE. Similarly, multifocal ERG ring analysis, recordable only in the RE, showed the worsening of the response amplitude densities in all examined areas (0–20°) (Figure 2E), as compared to the previous examinations. Similarly, Goldmann visual field in his RE showed progressive constriction of the peripheral isopters and a ring scotoma enclosed between 10–20° of the visual field (Figure 2F); it was not executable, however, in his LE. Color blindness was also confirmed. Neck and abdominal ultrasound assessment did not reveal any abnormality. Measurements of basal hormones by the anterior pituitary, glycaemia and insulin were within the normal range. Basal plasma leptin level was in the low normal range, showing no leptin resistance. During his follow-up, clinical and ophthalmological assessments of other family members (parents and younger brother) were unremarkable.
-Trio-based WES allowed to identify a homozygous splice siteTUBvariant (chr11:8122545G &gt; A, GRCh37.p13; c.1387 + 1G &gt; A,NM_177972.3) as the only clinically and functionally relevant event putatively linked to the disorder (Supplemental Table S1). The variant had previously been annotated in public databases (dbSNP, rs1040410003) with low frequency (gnomAD v3.1, MAF = 0.00001972) at the heterozygous state. It was classified as likely pathogenic (PVS1/PM2/PP5) according to the American College of Medical Genetics and Genomics-Association for Molecular Pathology (ACMG-AMP) criteria (ClinVar: VCV000865971.1) [14]. Sanger sequencing confirmed the homozygosity for the variant in the proband and the heterozygous status in the healthy parents and unaffected sib (Figure 1).
-Since the variant was predicted to affect the exon 11 donor splice site, the total RNA from patient-derived skin primary fibroblasts was used to characterize the impact of the nucleotide change on transcript processing. The cDNA fragment encompassing the relevant exons was amplified, confirming the presence of two aberrantly spliced products (Figure 3A). The two aberrant PCR amplicons were isolated from agarose gel, purified and sequenced via Sanger. The former (500 bp) was derived from skipping of the penultimate exon (exon 11, ENST00000299506.3), resulting in a premature termination codon (i.e., p.Glu406Argfs*4), while the latter (1172 bp) was the result of retention of intron 10, resulting in a TUB protein having a divergent 19-residue-long C-terminus and lacking the last 44 amino acids (p.Pro463Hisfs*19) (Figure 3B).
-In the patient’s skin fibroblasts, the predicted TUBGlu406Argfs*4protein was undetectable by Western blot [WB] analysis, while the TUBPro463Hisfs*19protein was poorly detectable likely due to accelerated degradation (Figure 3C, left panel). Consistently, the endogenous TUBPro463Hisfs*19level was partially rescued by blocking the proteasomal degradation pathway using MG132 (Figure 3C, right panel).
-To investigate the cellular localization of the mutated protein, cytoplasm and nuclear cell fractions were obtained and analyzed by WB. The results demonstrate that both the wild-type (wt) and mutant TUB proteins were almost exclusively localized in the nucleus (Figure 3D). This finding was also confirmed by confocal microscopy analysis that evidenced the nuclear localization of the TUB mutant (Figure 4A).
-Based on the documented role of TUB in early ciliogenesis [15], we assessed the localization of TUB at the cilium, but we failed to observe any consistent co-localization, possibly due to the low diffused levels of the protein in the cytoplasm To investigate the impact of defective TUB function on the morphogenesis of the primary cilium, a confocal analysis on primary fibroblasts was performed using antibodies against ARL13B, which localizes to primary cilia, and pericentrin, a component of the centrosome, which stains the basal body. As shown inFigure 4B, while almost all the control cells showed a primary cilium, 40% of the fibroblasts carrying the homozygous splice site variant inTUBdid not show a primary cilium. Moreover, while no significant difference was observed in ciliary axoneme length between the starved control and mutant cells, a large percentage of the latter showed an abnormal cilium morphology and a poorly defined and disorganized basal body (Figure 4C).
-The loss of TUB function was recently reported to underlie a novel IRD condition based on the identification of homozygosity for a 2 bp deletion (c.1194_1195delAG) causing the premature termination of the protein (p.Arg398Serfs*9) shared by three affected members of a single consanguineous family [10]. While the combination of retinal dystrophy and early onset obesity can be reminiscent of other disorders (e.g., Bardet–Biedl syndrome (MIM#PS209900) and Alstrom syndrome (MIM#203800)), the absence of other clinically relevant feature/sign was suggestive of a previously unreported ciliopathy [10]. In this paper, we report on a second disruptive variant (c.1387 + 1G &gt; A) affectingTUBin a subject with features that overlap with those previously described in the affected members of the original family.
-In the present and previously reported affected individuals, the ocular phenotype associated with defective TUB function is characterized by widespread retinal pigment epithelial (RPE) atrophy, deteriorating vision, the myopic and astigmatic refractive defect, the blonde fundus appearance, the ERG and OCT findings and progression of the disease (Figure 2). Notably, retinal detachment, without vitreous hemorrhage, was invariantly documented in the four individuals with biallelic inactivatingTUBvariants, suggesting that this feature likely represent a common finding in the disorder.
-Early onset obesity had previously been considered a major feature of the TUB-related condition [10], even though only two of three affected sibs were found obese (BMI &gt; 30), and the glycemic and lipid profiles in one of affected sibs were found within the normal range. The finding of obesity in the apparently healthy father (heterozygous carrier) suggests a possible co-occurring genetic event contributing to obesity in the family. In the present report, the clinical assessment of the affected individual documented increased weight (95.7 kg, +1.6 SD) and BMI (30.3, +1.6 SD), thus indicating overweight, in absence of other signs of obesity. Although evidence suggests that a defective TUB function may result in disturbances in insulin and leptin activity and obesity in mice [16,17,18,19], based on the collected findings, the relevance of TUB in human obesity requires further study. To assess whether TUB LoF could impact on hypothalamic pathways, food intake and adiposity, the metabolic profile of the affected individual was investigated. Accurate endocrinological examination did not reveal any abnormality, and the measurements of basal hormones by the anterior pituitary, glycaemia, insulin and leptin were within the normal range, thus ruling out insulin or leptin resistance. Consistently, instrumental investigations (X-ray and ultrasound analyses) documented no sign of glycogen accumulation in the internal organs. Consistently, the absence of significant changes in lipid storage was demonstrated by thin-layer chromatography (HPTLC) analysis in proband-derived fibroblast (Figure S1), allowing to confirm an apparently normal endocrine–metabolic profile in the affected individual. Of note, the Tubby protein has been involved in cochlear degeneration [20,21]. Based on this functional link, we evaluated the occurrence of hearing problems and cochlear degeneration, which were not observed.
-The homozygousTUBvariant was predicted to affect transcript processing, causing the skipping of exon 11 and intron retention, resulting in a frameshift with the premature termination of the TUB protein. mRNA analysis in proband-derived fibroblasts confirmed a disruptive impact of the splice site change documenting two aberrantly processed transcripts predicted to encode a 406-residue-long protein (p.Glu406Argfs*4) that probably is not able to proceed in protein synthesis, and a 481-residue-long protein (p.Pro463Hisfs*19) characterized by a divergent C-terminus characterized by accelerated degradation (Figure 3B). These findings confirm LoF as the pathomechanism underlying this disorder.
-Primary cilia are microtubule-based organelles that extend from the apical surface of the majority of mammalian cells. Cilia act as “cellular antennae”, receiving different inputs from the extracellular environment and transducing signals in response to stimuli [22]. A complex process required for proper cilia biogenesis function is the intraflagellar transport, which is required for assembling cilia and trafficking within primary cilia [23]. In this context, IFT-A has historically been believed to mediate retrograde intraflagellar transport inside the cilia and an IFT-A-binding domain at the TUB N-terminus has been demonstrated recently [24]. Moreover, co-localization between TUB and rootletin, the major structural component of the ciliary rootlet, has been observed in human retinal photoreceptors [10]. The use of a more informative in vitro model (e.g., induced pluripotent-stem-cell-derived retinal-pigment epithelium cells) and experimental strategies (e.g., siRNA-mediated TUB silencing) is required to appreciate more accurately the functional relevance of TUB in an appropriate cellular context.
-In summary, we confirm the link between TUB LoF and a new condition of human retinal ciliopathy and provide evidence of an altered cilium morphology/biogenesis in patient-derived fibroblasts. In fact, these cells displayed a reduced number of cilia when compared to the control cells, with a poorly defined and disorganized basal body structure, which are expected to prevent normal protein trafficking along the cilium. While these findings could explain the degeneration of photoreceptors characterizing this disorder, a relatively overall mild presentation has been associated with mutations in this gene. Multiple factors might contribute to this picture. First, the functional relevance of TUB in the context of ciliogenesis and cilium function might vary in different cell lineages. Second, functional compensation exerted by other related proteins might contribute to buffer the severity of the endophenotype. Third, specific cell lineages (e.g., rod and cone cells) might be particularly sensitive to TUB LoF. The collection of additional patients with biallelic variants in the gene will allow a more accurate characterization of the clinical spectrum associated with TUB LoF. Based on these considerations, TUB loss of function could be considered as responsible for a novel form of isolated retinal ciliopathy.</t>
-        </is>
-      </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>{
-"pmid": "9390831",
-"alias_symbol": "rd5",
-"primary_gene_symbol": "TUB",
-"name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
-"evidence": ""
-}</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>HGNC:12406</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>ENSG00000166402</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>GENE ID:7275</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>TUB</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>rd5</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>9390831</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>mouse phenotype biomarker</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>abstract</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>Mice homozygous for a defect of the tub (rd5) gene exhibit cochlear and retinal degeneration combined with obesity, and resemble certain human autosomal recessive sensory deficit syndromes.</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>TUB bipartite transcription factor</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>In this paper, we confirm that biallelic inactivating variants in TUB cause a retinal disorder and functionally associate this condition with the occurrence of defects of the basal body structure and axoneme morphology of the primary cilium and overall defective ciliogenesis. Although the present findings suggest that TUB plays a role in the pathogenesis of retinal ciliopathies, dedicated functional studies are required to profile the mechanism of disease. This work confirms the clinical relevance of biallelic LoF variants ofTUB, which should be considered in clinical settings and the genetic diagnosis of IRD disorders.
-The present research followed the tenets of the Helsinki Declaration (1964 and further revisions) and the study was approved by the local ethics committee (Comitato Etico Centrale IRCCS Lazio, Sezione IFO/Fondazione Bietti, Rome, Italy). Upon recruitment in the study (FB RET-02-2019), executed from February to July 2019 at the IRCCS Fondazione Bietti, informed consent after full explanation was obtained from each subject included in the study.
-The proband and his family underwent comprehensive ophthalmological examination including visual acuity measured by the Early Treatment Diabetic Retinopathy Study (ETDRS) charts (Lighthouse, Low Vision Products, Long Island City, NY, USA) at the distance of 4 m and expressed as the logarithm of the minimum angle of resolution (logMAR); intraocular pressure (IOP) measurement; anterior segment observation by slit-lamp biomicroscopy and fundus examination by indirect ophthalmoscopic examination using + 90D non-contact lens (Volk Optical, Mentor, OH) after pupillary dilatation with tropicamide 1% drops. Goldmann visual field was assessed by kinetic Goldmann perimeter Haag-Streit 940. Chromatic test was evaluated by the monocular administration of Ishihara pseudoisochromatic plates (24 plates edition, Kanehara Trading Inc., Tokyo, Japan) in natural daylight. Electrophysiological assessment included dark-adapted and light-adapted full-field electroretinogram (Retimax Advanced Plus apparatus, CSO, Firenze, Italy) and multifocal electroretinogram (mfERG; VERIS Clinic TM version 4.9; Electro-Diagnostic Imaging, San Mateo, CA, USA) recordings according to the 2011 International Society for Clinical Electrophysiology of Vision (ISCEV) [25] by using the Dawson–Trick–Litzkow (DTL) contact electrodes and having the pupil dilated at 8 mm.
-Retinal imaging was executed by ultrawide field fundus photograph obtained with Optos California (Optos PLC, Dunfermline, Scotland, United Kingdom); FAF was also obtained during the same examination (488 nm excitation, barrier filter transmitted light from 500 to 680 nm, 55°) using Heidelberg Spectralis OCT (HRA + OCT, Heidelberg Engineering, Heidelberg, Germany). SD-OCT scan pattern was acquired with a minimum of a 20 × 20 degree rectangle centered on the fovea and 25-line B-scans spaced 235 μm apart and composed of 50 averaged frames by using the same instrument.
-Karyotype, CGH array and mutation scan by parallel sequencing considering a retinal cone–rod dystrophy panel of 70 genes were informative. Genomic DNA was collected after obtaining written informed consent. Whole-Exome sequencing (WES) and data analysis were performed as previously reported [26,27] (Supplementary Table S1). DNA of the affected subject and his parents was extracted from circulating leukocytes and sequenced using Illumina paired-end technology by means of SureSelect Human All Exon v.7 (Agilent, Santa Clara, CA, USA) kits. WES raw data were processed and analyzed using an in-house implemented pipeline as previously described [28,29], according to the GATK’s Best Practices [30]. The UCSC GRCh37/hg19 version of genome assembly was used as a reference for read alignment by means of BWA-MEM [31] tool and the subsequent variant calling with HaplotypeCaller (GATK v3.7) [28]. Variants’ functional annotation was made with the SnpEff v.5.0 [32] and dbNSFP v.4.2 [33] tools. Relevant in silico impact prediction tools, such as Combined Annotation Dependent Depletion (CADD) v.1.6 [34], Mendelian Clinically Applicable Pathogenicity (M-CAP) v.1.0 [35] and InterVar v.2.0.1 [36], were also used. By filtering against our population-matched database (~2500 WES) and public databases (dbSNP150 and gnomAD v.2.0.1), the analysis focused on high-quality rare variants that affect coding sequences and splice site regions. Sanger sequencing was performed for variant validation and segregation analysis (primers available upon request).
-Proband skin biopsy was obtained after informant consent was secured. Total RNA was extracted from the proband and healthy donor fibroblasts by using RNeasy Mini Kit (Qiagen, Hilden, Germany), according to the manufacturer’s recommendations. Total RNA concentration and quality were assessed by measuring the absorbance at 260 and 280 nm. Reverse transcription was carried out using a SuperScript RT reagent Kit (Invitrogen; ThermoFisher Scientific, Waltham, MA, USA). The obtained cDNA pools were amplified by PCR using specific primers located in exons 10 and 12 of theTUBgene, and PCR products were separated on a 2% agarose gel. The sequences of the primers are available upon request.
-Primary skin fibroblasts were cultured in DMEM supplemented with 10% heat-inactivated FBS, 2 mM glutamine, 100 units/mL of penicillin and 100 µg/mL of streptomycin, and maintained at 37 °C in a humidified atmosphere containing 5% CO2. After treatment, fibroblasts were lysed in RIPA buffer supplemented with phosphatase and protease inhibitors. Lysates were kept on ice (30 min) and then centrifuged at 16,000×g(20 min, 4 °C). Supernatants were collected and protein concentration was determined by Quick Start Bradford Dye Reagent (Bio-Rad Laboratories, Hercules, CA, USA), using bovine serum albumin (BSA) as a standard. Fibroblast homogenates were resolved by SDS PAGE and transferred to nitrocellulose membranes (Bio-Rad Laboratories). Blots were blocked for 1 h with 5% non-fat milk powder in phosphate-buffered saline (PBS) containing 0.1% Tween-20 and incubated overnight with specific antibodies. Anti-TUB primary polyclonal antibody (1:1000, Invitrogen; ThermoFisher Scientific) and goat anti-rabbit-HRP IgG secondary antibody (Invitrogen; ThermoFisher Scientific) were diluted in blocking solution. Immunoreactive proteins were detected by an ECL SuperSignal West Femto Maximum Sensitivity Chemiluminescent Substrate, according to the manufacturer’s instructions (Thermo Scientific, USA).
-Approximately 3 × 104/mL fibroblasts were seeded on glass coverslips and maintained in culture in complete medium for 24 h. Subconfluent fibroblasts were starved for 30 h and then fixed with 4% paraformaldehyde. Subsequently, cells were stained with rabbit anti-TUB (1:100 dilution), rabbit polyclonal anti-ARL13B (1:100, Abcam, Cambridge, UK) and mouse monoclonal anti-Pericentrin (1:100, Abcam) antibodies followed by goat anti-rabbit Alexa Fluor 488 and goat anti-mouse Alex Fluor 594, respectively (1:200 dilution; Molecular Probes, Eugene, OR, USA). After staining, coverslips were extensively rinsed and mounted onto microscope slides using Vectashield with DAPI mounting medium (Vector Laboratories, Newark, CA, USA). Analyses were performed in three independent experiments on a Zeiss LSM980 (Zeiss, Oberkochen, Germany) using a 63×/1.4 N.A. oil objective and excitation spectral laser lines at 405, 488 and 594 nm. Five hundred cells were counted for each condition in each experiment, and axoneme length was measured for each cell by using Zen Blue 3.2 software. Image acquisition and processing were performed as previously reported [37].
-Control and mutated fibroblasts cultured in 150 cm2dishes were harvested using trypsin after reaching confluence, rinsed with phosphate-buffered saline (PBS) and pelleted by centrifugation. Cell pellets were resuspended in 1 mL 0.9% NaCl and 6 mL of chloroform/methanol (2:1, v/v) were added. Mixtures were vortexed vigorously and centrifuged at 1500×gfor 15 min; the aqueous phase was discarded and organic phase was dried under N2gas. Lipid extracts from 1.5 × 106cells were applied on high-performance thin-layer chromatography (HPTLC) silica gel 60 plates (Merck, Darmstadt, Germany). Neutral lipids were resolved using a solvent system of hexane/diethyl ether/acetic acid (70:30:1, v/v/v) and were detected by staining with an aqueous solution containing 3% cupric acetate and 8% phosphoric acid and subsequent charring at 140 °C for 10 min. Lipids were identified by the co-migration of commercially available standards.
-URLs.*Online Mendelian Inheritance in Man [OMIM],http://www.ncbi.nlm.nih.gov/omim/;
-NCBI Gene,http://www.ncbi.nlm.nih.gov/gene/;
-Picard tools,http://picard.sourceforge.net/;
-wAnnovar,http://wannovar.usc.edu/;
-dbSNP137,http://www.ncbi.nlm.nih.gov/projects/SNP/snp_summary.cgi/;
-1000 Genomes Project,http://www.1000genomes.org/;
-HapMap Project,http://hapmap.ncbi.nlm.nih.gov/;
-SMART,http://smart.embl-heidelberg.de/;
-Protein Data Bank [PDB],http://www.rcsb.org/pdb/home/home.do.
-Research for this study was supported by the Ministry of Health funding 5x1000 Fondazione G.B. Bietti funds—2016 to M.P. and Fondazione Roma; Bando Ricerca Indipendente ISS 2021–2023 to V.C., Istituto Superiore di Sanità; Italian Ministry of Health (CCR-2017-23669081 to M.T.), and Italian Ministry of Research (FOE_2019 to M.T.). The authors acknowledge Maria Luisa Alessi and Federica Petrocchi for technical help in the electrophysiological and perimetric evaluations, Serenella Venanzi for administrative assistance.
-Publisher’s Note:MDPI stays neutral with regard to jurisdictional claims in published maps and institutional affiliations.
-The following supporting information can be downloaded at:https://www.mdpi.com/article/10.3390/ijms232314656/s1.
-Click here for additional data file.
-Conceptualization, L.Z. and V.C.; methodology, C.M., E.S., S.C., L.B. and M.T. (Massimo Tatti); validation, E.C., L.B., C.M. and V.C.; bioinformatics analysis, A.C. and A.B.; investigation, L.Z., M.C., M.P. and E.C.; resources, M.V.; data curation, L.B., M.P., E.S., M.T. (Massimo Tatti), M.N. and V.C.; writing—original draft preparation, L.Z., V.C. and M.N.; writing—review and editing, M.N., E.S., M.C., M.T. (Marco Tartaglia) and V.C.; supervision, M.V. and M.T. (Marco Tartaglia); project administration, M.V., V.C. and M.T. (Marco Tartaglia); funding acquisition, M.V. and M.P. All authors have read and agreed to the published version of the manuscript.
-The study was conducted according to the guidelines of the Declaration of Helsinki and was approved by the local Institutional Ethical Committee of the IRCCS_Fondazione G.B. Bietti [Ret_02/2019].
-Signed informed consent was obtained from the participating family.
-Data that support the findings of this study are available from the corresponding authors upon request.
-The authors declare no conflict of interest.
-Family tree showing the segregation of the identified splice site change.
-Ocular phenotype of the proband right eye. (A) Ultrawide field color fundus photograph. (B) The 55° fundus autofluorescence. (C) Spectral-domain optical coherence tomography line horizontal scan. (D) Full-field dark-adapted electroretinogram. (E) Three-dimensional multifocal electroretinogram plot. (F) Goldmann kinetic visual field.
-Characterization of the pathogenicTUBvariant. (A) Transcript processing in primary skin fibroblasts from a healthy donor and from the proband carrying the homozygous splice site variant. Total RNA was extracted, reverse-transcribed and analyzed by PCR to resolve transcript processing. Two aberrant cDNA products were identified in mutated cells (left) compared to the expected length of the amplified fragment obtained from the control fibroblasts (right). (B) Schematic representation of aberrant transcript processing caused by the identified homozygous splice site change inTUB. (C) Western blot analysis of the TUB protein in patient’s fibroblasts and the control cells. Twenty, forty and sixty micrograms of whole cell extract were analyzed basally (left) and following 4 h treatment with 100 μM Mg132 (right) and probed with anti-TUB antibody (* indicates a non-specific product). (D) Expression of wild-type and mutant TUB protein was analyzed in the cytoplasmic and nuclear fractions were obtained from wild-type and mutated fibroblasts. Sixty micrograms of each fraction were analyzed by Western blot and then probed with anti-TUB antibody. Anti-YY1 and anti-HSP90 antibodies were used as the internal controls to assess the clarity of the different fractions (* indicates a non-specific product). Blots are representative of three experiments performed.
-TUB subcellular localization and cilium defects in cells with TUB LoF. (A) Thirty-hour-starved and PFA-fixed fibroblasts from a healthy donor and from the proband were analyzed by confocal microscopy for the localization of TUB using antibodies against TUB. (B) The presence and morphology of primary cilia in starved fibroblasts from the proband and a healthy donor. Cells were starved for 30 h and fixed with PFA 4%. Primary cilia were analyzed using antibodies against ARL13B (cilium axonemal, green) and pericentrin (basal body, red) to investigate morphogenesis. Nuclei are DAPI stained (blue). Bars correspond to 20 and 2 μm (left panels). (C) Histograms represent the percent value of presence/absence of cilium, normal/aberrant cilium morphology and normal/aberrant basal body structure and the length (μm) of axoneme. Five hundred cells were counted for each condition and axoneme length was measured. Imagines and bar plots are representative of three experiments performed. * indicate statistical significance forp&lt; 0.01 by using Student’sTtest.</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>Mice homozygous for a defect of the tub (rd5) gene exhibit cochlear and retinal degeneration combined with obesity, and resemble certain human autosomal recessive sensory deficit syndromes. To establish the progressive nature of sensory cell loss associated with the tub gene, and to differentiate tub-related losses from those associated with the C57 background on which tub arose, we evaluated cochleas and retinas from tub/tub, tub/+, and +/+ mice, aged 2 weeks to 1 year by light and electron microscopy. Cochleas from mice of all three genotypes show progressive inner (IHC) and outer hair cell (OHC) loss. Relative to tub/+ and +/+ animals, however, tub homozygotes show accelerated OHC loss, affecting the extreme cochlear base (hook region) by 1 month, and the apex by 6 months. IHC loss in tub/tub animals is accelerated in the basal half of the cochlea, affecting the hook region by 6 months. Spiral ganglion cell losses were observed only in tub/tub mice, and only in the cochlear base. Retinas of tub/tub mice are abnormal at maturity, exhibiting shortened photoreceptor outer segments by 2 weeks, and progressive photoreceptor loss thereafter. Because the tub mutation causes degeneration of sensory cells in the ear and eye but has no other neurological effects, tubby mice hold unique promise for the study of human syndromic sensory loss.</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>PMID: 9390831
-Full Text: In this paper, we confirm that biallelic inactivating variants in TUB cause a retinal disorder and functionally associate this condition with the occurrence of defects of the basal body structure and axoneme morphology of the primary cilium and overall defective ciliogenesis. Although the present findings suggest that TUB plays a role in the pathogenesis of retinal ciliopathies, dedicated functional studies are required to profile the mechanism of disease. This work confirms the clinical relevance of biallelic LoF variants ofTUB, which should be considered in clinical settings and the genetic diagnosis of IRD disorders.
-The present research followed the tenets of the Helsinki Declaration (1964 and further revisions) and the study was approved by the local ethics committee (Comitato Etico Centrale IRCCS Lazio, Sezione IFO/Fondazione Bietti, Rome, Italy). Upon recruitment in the study (FB RET-02-2019), executed from February to July 2019 at the IRCCS Fondazione Bietti, informed consent after full explanation was obtained from each subject included in the study.
-The proband and his family underwent comprehensive ophthalmological examination including visual acuity measured by the Early Treatment Diabetic Retinopathy Study (ETDRS) charts (Lighthouse, Low Vision Products, Long Island City, NY, USA) at the distance of 4 m and expressed as the logarithm of the minimum angle of resolution (logMAR); intraocular pressure (IOP) measurement; anterior segment observation by slit-lamp biomicroscopy and fundus examination by indirect ophthalmoscopic examination using + 90D non-contact lens (Volk Optical, Mentor, OH) after pupillary dilatation with tropicamide 1% drops. Goldmann visual field was assessed by kinetic Goldmann perimeter Haag-Streit 940. Chromatic test was evaluated by the monocular administration of Ishihara pseudoisochromatic plates (24 plates edition, Kanehara Trading Inc., Tokyo, Japan) in natural daylight. Electrophysiological assessment included dark-adapted and light-adapted full-field electroretinogram (Retimax Advanced Plus apparatus, CSO, Firenze, Italy) and multifocal electroretinogram (mfERG; VERIS Clinic TM version 4.9; Electro-Diagnostic Imaging, San Mateo, CA, USA) recordings according to the 2011 International Society for Clinical Electrophysiology of Vision (ISCEV) [25] by using the Dawson–Trick–Litzkow (DTL) contact electrodes and having the pupil dilated at 8 mm.
-Retinal imaging was executed by ultrawide field fundus photograph obtained with Optos California (Optos PLC, Dunfermline, Scotland, United Kingdom); FAF was also obtained during the same examination (488 nm excitation, barrier filter transmitted light from 500 to 680 nm, 55°) using Heidelberg Spectralis OCT (HRA + OCT, Heidelberg Engineering, Heidelberg, Germany). SD-OCT scan pattern was acquired with a minimum of a 20 × 20 degree rectangle centered on the fovea and 25-line B-scans spaced 235 μm apart and composed of 50 averaged frames by using the same instrument.
-Karyotype, CGH array and mutation scan by parallel sequencing considering a retinal cone–rod dystrophy panel of 70 genes were informative. Genomic DNA was collected after obtaining written informed consent. Whole-Exome sequencing (WES) and data analysis were performed as previously reported [26,27] (Supplementary Table S1). DNA of the affected subject and his parents was extracted from circulating leukocytes and sequenced using Illumina paired-end technology by means of SureSelect Human All Exon v.7 (Agilent, Santa Clara, CA, USA) kits. WES raw data were processed and analyzed using an in-house implemented pipeline as previously described [28,29], according to the GATK’s Best Practices [30]. The UCSC GRCh37/hg19 version of genome assembly was used as a reference for read alignment by means of BWA-MEM [31] tool and the subsequent variant calling with HaplotypeCaller (GATK v3.7) [28]. Variants’ functional annotation was made with the SnpEff v.5.0 [32] and dbNSFP v.4.2 [33] tools. Relevant in silico impact prediction tools, such as Combined Annotation Dependent Depletion (CADD) v.1.6 [34], Mendelian Clinically Applicable Pathogenicity (M-CAP) v.1.0 [35] and InterVar v.2.0.1 [36], were also used. By filtering against our population-matched database (~2500 WES) and public databases (dbSNP150 and gnomAD v.2.0.1), the analysis focused on high-quality rare variants that affect coding sequences and splice site regions. Sanger sequencing was performed for variant validation and segregation analysis (primers available upon request).
-Proband skin biopsy was obtained after informant consent was secured. Total RNA was extracted from the proband and healthy donor fibroblasts by using RNeasy Mini Kit (Qiagen, Hilden, Germany), according to the manufacturer’s recommendations. Total RNA concentration and quality were assessed by measuring the absorbance at 260 and 280 nm. Reverse transcription was carried out using a SuperScript RT reagent Kit (Invitrogen; ThermoFisher Scientific, Waltham, MA, USA). The obtained cDNA pools were amplified by PCR using specific primers located in exons 10 and 12 of theTUBgene, and PCR products were separated on a 2% agarose gel. The sequences of the primers are available upon request.
-Primary skin fibroblasts were cultured in DMEM supplemented with 10% heat-inactivated FBS, 2 mM glutamine, 100 units/mL of penicillin and 100 µg/mL of streptomycin, and maintained at 37 °C in a humidified atmosphere containing 5% CO2. After treatment, fibroblasts were lysed in RIPA buffer supplemented with phosphatase and protease inhibitors. Lysates were kept on ice (30 min) and then centrifuged at 16,000×g(20 min, 4 °C). Supernatants were collected and protein concentration was determined by Quick Start Bradford Dye Reagent (Bio-Rad Laboratories, Hercules, CA, USA), using bovine serum albumin (BSA) as a standard. Fibroblast homogenates were resolved by SDS PAGE and transferred to nitrocellulose membranes (Bio-Rad Laboratories). Blots were blocked for 1 h with 5% non-fat milk powder in phosphate-buffered saline (PBS) containing 0.1% Tween-20 and incubated overnight with specific antibodies. Anti-TUB primary polyclonal antibody (1:1000, Invitrogen; ThermoFisher Scientific) and goat anti-rabbit-HRP IgG secondary antibody (Invitrogen; ThermoFisher Scientific) were diluted in blocking solution. Immunoreactive proteins were detected by an ECL SuperSignal West Femto Maximum Sensitivity Chemiluminescent Substrate, according to the manufacturer’s instructions (Thermo Scientific, USA).
-Approximately 3 × 104/mL fibroblasts were seeded on glass coverslips and maintained in culture in complete medium for 24 h. Subconfluent fibroblasts were starved for 30 h and then fixed with 4% paraformaldehyde. Subsequently, cells were stained with rabbit anti-TUB (1:100 dilution), rabbit polyclonal anti-ARL13B (1:100, Abcam, Cambridge, UK) and mouse monoclonal anti-Pericentrin (1:100, Abcam) antibodies followed by goat anti-rabbit Alexa Fluor 488 and goat anti-mouse Alex Fluor 594, respectively (1:200 dilution; Molecular Probes, Eugene, OR, USA). After staining, coverslips were extensively rinsed and mounted onto microscope slides using Vectashield with DAPI mounting medium (Vector Laboratories, Newark, CA, USA). Analyses were performed in three independent experiments on a Zeiss LSM980 (Zeiss, Oberkochen, Germany) using a 63×/1.4 N.A. oil objective and excitation spectral laser lines at 405, 488 and 594 nm. Five hundred cells were counted for each condition in each experiment, and axoneme length was measured for each cell by using Zen Blue 3.2 software. Image acquisition and processing were performed as previously reported [37].
-Control and mutated fibroblasts cultured in 150 cm2dishes were harvested using trypsin after reaching confluence, rinsed with phosphate-buffered saline (PBS) and pelleted by centrifugation. Cell pellets were resuspended in 1 mL 0.9% NaCl and 6 mL of chloroform/methanol (2:1, v/v) were added. Mixtures were vortexed vigorously and centrifuged at 1500×gfor 15 min; the aqueous phase was discarded and organic phase was dried under N2gas. Lipid extracts from 1.5 × 106cells were applied on high-performance thin-layer chromatography (HPTLC) silica gel 60 plates (Merck, Darmstadt, Germany). Neutral lipids were resolved using a solvent system of hexane/diethyl ether/acetic acid (70:30:1, v/v/v) and were detected by staining with an aqueous solution containing 3% cupric acetate and 8% phosphoric acid and subsequent charring at 140 °C for 10 min. Lipids were identified by the co-migration of commercially available standards.
-URLs.*Online Mendelian Inheritance in Man [OMIM],http://www.ncbi.nlm.nih.gov/omim/;
-NCBI Gene,http://www.ncbi.nlm.nih.gov/gene/;
-Picard tools,http://picard.sourceforge.net/;
-wAnnovar,http://wannovar.usc.edu/;
-dbSNP137,http://www.ncbi.nlm.nih.gov/projects/SNP/snp_summary.cgi/;
-1000 Genomes Project,http://www.1000genomes.org/;
-HapMap Project,http://hapmap.ncbi.nlm.nih.gov/;
-SMART,http://smart.embl-heidelberg.de/;
-Protein Data Bank [PDB],http://www.rcsb.org/pdb/home/home.do.
-Research for this study was supported by the Ministry of Health funding 5x1000 Fondazione G.B. Bietti funds—2016 to M.P. and Fondazione Roma; Bando Ricerca Indipendente ISS 2021–2023 to V.C., Istituto Superiore di Sanità; Italian Ministry of Health (CCR-2017-23669081 to M.T.), and Italian Ministry of Research (FOE_2019 to M.T.). The authors acknowledge Maria Luisa Alessi and Federica Petrocchi for technical help in the electrophysiological and perimetric evaluations, Serenella Venanzi for administrative assistance.
-Publisher’s Note:MDPI stays neutral with regard to jurisdictional claims in published maps and institutional affiliations.
-The following supporting information can be downloaded at:https://www.mdpi.com/article/10.3390/ijms232314656/s1.
-Click here for additional data file.
-Conceptualization, L.Z. and V.C.; methodology, C.M., E.S., S.C., L.B. and M.T. (Massimo Tatti); validation, E.C., L.B., C.M. and V.C.; bioinformatics analysis, A.C. and A.B.; investigation, L.Z., M.C., M.P. and E.C.; resources, M.V.; data curation, L.B., M.P., E.S., M.T. (Massimo Tatti), M.N. and V.C.; writing—original draft preparation, L.Z., V.C. and M.N.; writing—review and editing, M.N., E.S., M.C., M.T. (Marco Tartaglia) and V.C.; supervision, M.V. and M.T. (Marco Tartaglia); project administration, M.V., V.C. and M.T. (Marco Tartaglia); funding acquisition, M.V. and M.P. All authors have read and agreed to the published version of the manuscript.
-The study was conducted according to the guidelines of the Declaration of Helsinki and was approved by the local Institutional Ethical Committee of the IRCCS_Fondazione G.B. Bietti [Ret_02/2019].
-Signed informed consent was obtained from the participating family.
-Data that support the findings of this study are available from the corresponding authors upon request.
-The authors declare no conflict of interest.
-Family tree showing the segregation of the identified splice site change.
-Ocular phenotype of the proband right eye. (A) Ultrawide field color fundus photograph. (B) The 55° fundus autofluorescence. (C) Spectral-domain optical coherence tomography line horizontal scan. (D) Full-field dark-adapted electroretinogram. (E) Three-dimensional multifocal electroretinogram plot. (F) Goldmann kinetic visual field.
-Characterization of the pathogenicTUBvariant. (A) Transcript processing in primary skin fibroblasts from a healthy donor and from the proband carrying the homozygous splice site variant. Total RNA was extracted, reverse-transcribed and analyzed by PCR to resolve transcript processing. Two aberrant cDNA products were identified in mutated cells (left) compared to the expected length of the amplified fragment obtained from the control fibroblasts (right). (B) Schematic representation of aberrant transcript processing caused by the identified homozygous splice site change inTUB. (C) Western blot analysis of the TUB protein in patient’s fibroblasts and the control cells. Twenty, forty and sixty micrograms of whole cell extract were analyzed basally (left) and following 4 h treatment with 100 μM Mg132 (right) and probed with anti-TUB antibody (* indicates a non-specific product). (D) Expression of wild-type and mutant TUB protein was analyzed in the cytoplasmic and nuclear fractions were obtained from wild-type and mutated fibroblasts. Sixty micrograms of each fraction were analyzed by Western blot and then probed with anti-TUB antibody. Anti-YY1 and anti-HSP90 antibodies were used as the internal controls to assess the clarity of the different fractions (* indicates a non-specific product). Blots are representative of three experiments performed.
-TUB subcellular localization and cilium defects in cells with TUB LoF. (A) Thirty-hour-starved and PFA-fixed fibroblasts from a healthy donor and from the proband were analyzed by confocal microscopy for the localization of TUB using antibodies against TUB. (B) The presence and morphology of primary cilia in starved fibroblasts from the proband and a healthy donor. Cells were starved for 30 h and fixed with PFA 4%. Primary cilia were analyzed using antibodies against ARL13B (cilium axonemal, green) and pericentrin (basal body, red) to investigate morphogenesis. Nuclei are DAPI stained (blue). Bars correspond to 20 and 2 μm (left panels). (C) Histograms represent the percent value of presence/absence of cilium, normal/aberrant cilium morphology and normal/aberrant basal body structure and the length (μm) of axoneme. Five hundred cells were counted for each condition and axoneme length was measured. Imagines and bar plots are representative of three experiments performed. * indicate statistical significance forp&lt; 0.01 by using Student’sTtest.</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
-    Inputs:
-    Alias gene symbol: rd5
-    HGNC record ID: HGNC:12406
-    Primary gene symbol: TUB
-    Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
-    Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
-    Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
-    If the text does not support that the alias is an alternate abbreviation, return:
-    "alternate_abbreviation": "NO"
-    "evidence": ""
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
-    Evidence must be one exact sentence copied verbatim from the text.
-    Do not infer relationships or paraphrase evidence.
-    Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
-    {
-    "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
-    "alternate_abbreviation": "YES or NO",
-    "evidence": ""
-    }
-PMID: 9390831
-Full Text: In this paper, we confirm that biallelic inactivating variants in TUB cause a retinal disorder and functionally associate this condition with the occurrence of defects of the basal body structure and axoneme morphology of the primary cilium and overall defective ciliogenesis. Although the present findings suggest that TUB plays a role in the pathogenesis of retinal ciliopathies, dedicated functional studies are required to profile the mechanism of disease. This work confirms the clinical relevance of biallelic LoF variants ofTUB, which should be considered in clinical settings and the genetic diagnosis of IRD disorders.
-The present research followed the tenets of the Helsinki Declaration (1964 and further revisions) and the study was approved by the local ethics committee (Comitato Etico Centrale IRCCS Lazio, Sezione IFO/Fondazione Bietti, Rome, Italy). Upon recruitment in the study (FB RET-02-2019), executed from February to July 2019 at the IRCCS Fondazione Bietti, informed consent after full explanation was obtained from each subject included in the study.
-The proband and his family underwent comprehensive ophthalmological examination including visual acuity measured by the Early Treatment Diabetic Retinopathy Study (ETDRS) charts (Lighthouse, Low Vision Products, Long Island City, NY, USA) at the distance of 4 m and expressed as the logarithm of the minimum angle of resolution (logMAR); intraocular pressure (IOP) measurement; anterior segment observation by slit-lamp biomicroscopy and fundus examination by indirect ophthalmoscopic examination using + 90D non-contact lens (Volk Optical, Mentor, OH) after pupillary dilatation with tropicamide 1% drops. Goldmann visual field was assessed by kinetic Goldmann perimeter Haag-Streit 940. Chromatic test was evaluated by the monocular administration of Ishihara pseudoisochromatic plates (24 plates edition, Kanehara Trading Inc., Tokyo, Japan) in natural daylight. Electrophysiological assessment included dark-adapted and light-adapted full-field electroretinogram (Retimax Advanced Plus apparatus, CSO, Firenze, Italy) and multifocal electroretinogram (mfERG; VERIS Clinic TM version 4.9; Electro-Diagnostic Imaging, San Mateo, CA, USA) recordings according to the 2011 International Society for Clinical Electrophysiology of Vision (ISCEV) [25] by using the Dawson–Trick–Litzkow (DTL) contact electrodes and having the pupil dilated at 8 mm.
-Retinal imaging was executed by ultrawide field fundus photograph obtained with Optos California (Optos PLC, Dunfermline, Scotland, United Kingdom); FAF was also obtained during the same examination (488 nm excitation, barrier filter transmitted light from 500 to 680 nm, 55°) using Heidelberg Spectralis OCT (HRA + OCT, Heidelberg Engineering, Heidelberg, Germany). SD-OCT scan pattern was acquired with a minimum of a 20 × 20 degree rectangle centered on the fovea and 25-line B-scans spaced 235 μm apart and composed of 50 averaged frames by using the same instrument.
-Karyotype, CGH array and mutation scan by parallel sequencing considering a retinal cone–rod dystrophy panel of 70 genes were informative. Genomic DNA was collected after obtaining written informed consent. Whole-Exome sequencing (WES) and data analysis were performed as previously reported [26,27] (Supplementary Table S1). DNA of the affected subject and his parents was extracted from circulating leukocytes and sequenced using Illumina paired-end technology by means of SureSelect Human All Exon v.7 (Agilent, Santa Clara, CA, USA) kits. WES raw data were processed and analyzed using an in-house implemented pipeline as previously described [28,29], according to the GATK’s Best Practices [30]. The UCSC GRCh37/hg19 version of genome assembly was used as a reference for read alignment by means of BWA-MEM [31] tool and the subsequent variant calling with HaplotypeCaller (GATK v3.7) [28]. Variants’ functional annotation was made with the SnpEff v.5.0 [32] and dbNSFP v.4.2 [33] tools. Relevant in silico impact prediction tools, such as Combined Annotation Dependent Depletion (CADD) v.1.6 [34], Mendelian Clinically Applicable Pathogenicity (M-CAP) v.1.0 [35] and InterVar v.2.0.1 [36], were also used. By filtering against our population-matched database (~2500 WES) and public databases (dbSNP150 and gnomAD v.2.0.1), the analysis focused on high-quality rare variants that affect coding sequences and splice site regions. Sanger sequencing was performed for variant validation and segregation analysis (primers available upon request).
-Proband skin biopsy was obtained after informant consent was secured. Total RNA was extracted from the proband and healthy donor fibroblasts by using RNeasy Mini Kit (Qiagen, Hilden, Germany), according to the manufacturer’s recommendations. Total RNA concentration and quality were assessed by measuring the absorbance at 260 and 280 nm. Reverse transcription was carried out using a SuperScript RT reagent Kit (Invitrogen; ThermoFisher Scientific, Waltham, MA, USA). The obtained cDNA pools were amplified by PCR using specific primers located in exons 10 and 12 of theTUBgene, and PCR products were separated on a 2% agarose gel. The sequences of the primers are available upon request.
-Primary skin fibroblasts were cultured in DMEM supplemented with 10% heat-inactivated FBS, 2 mM glutamine, 100 units/mL of penicillin and 100 µg/mL of streptomycin, and maintained at 37 °C in a humidified atmosphere containing 5% CO2. After treatment, fibroblasts were lysed in RIPA buffer supplemented with phosphatase and protease inhibitors. Lysates were kept on ice (30 min) and then centrifuged at 16,000×g(20 min, 4 °C). Supernatants were collected and protein concentration was determined by Quick Start Bradford Dye Reagent (Bio-Rad Laboratories, Hercules, CA, USA), using bovine serum albumin (BSA) as a standard. Fibroblast homogenates were resolved by SDS PAGE and transferred to nitrocellulose membranes (Bio-Rad Laboratories). Blots were blocked for 1 h with 5% non-fat milk powder in phosphate-buffered saline (PBS) containing 0.1% Tween-20 and incubated overnight with specific antibodies. Anti-TUB primary polyclonal antibody (1:1000, Invitrogen; ThermoFisher Scientific) and goat anti-rabbit-HRP IgG secondary antibody (Invitrogen; ThermoFisher Scientific) were diluted in blocking solution. Immunoreactive proteins were detected by an ECL SuperSignal West Femto Maximum Sensitivity Chemiluminescent Substrate, according to the manufacturer’s instructions (Thermo Scientific, USA).
-Approximately 3 × 104/mL fibroblasts were seeded on glass coverslips and maintained in culture in complete medium for 24 h. Subconfluent fibroblasts were starved for 30 h and then fixed with 4% paraformaldehyde. Subsequently, cells were stained with rabbit anti-TUB (1:100 dilution), rabbit polyclonal anti-ARL13B (1:100, Abcam, Cambridge, UK) and mouse monoclonal anti-Pericentrin (1:100, Abcam) antibodies followed by goat anti-rabbit Alexa Fluor 488 and goat anti-mouse Alex Fluor 594, respectively (1:200 dilution; Molecular Probes, Eugene, OR, USA). After staining, coverslips were extensively rinsed and mounted onto microscope slides using Vectashield with DAPI mounting medium (Vector Laboratories, Newark, CA, USA). Analyses were performed in three independent experiments on a Zeiss LSM980 (Zeiss, Oberkochen, Germany) using a 63×/1.4 N.A. oil objective and excitation spectral laser lines at 405, 488 and 594 nm. Five hundred cells were counted for each condition in each experiment, and axoneme length was measured for each cell by using Zen Blue 3.2 software. Image acquisition and processing were performed as previously reported [37].
-Control and mutated fibroblasts cultured in 150 cm2dishes were harvested using trypsin after reaching confluence, rinsed with phosphate-buffered saline (PBS) and pelleted by centrifugation. Cell pellets were resuspended in 1 mL 0.9% NaCl and 6 mL of chloroform/methanol (2:1, v/v) were added. Mixtures were vortexed vigorously and centrifuged at 1500×gfor 15 min; the aqueous phase was discarded and organic phase was dried under N2gas. Lipid extracts from 1.5 × 106cells were applied on high-performance thin-layer chromatography (HPTLC) silica gel 60 plates (Merck, Darmstadt, Germany). Neutral lipids were resolved using a solvent system of hexane/diethyl ether/acetic acid (70:30:1, v/v/v) and were detected by staining with an aqueous solution containing 3% cupric acetate and 8% phosphoric acid and subsequent charring at 140 °C for 10 min. Lipids were identified by the co-migration of commercially available standards.
-URLs.*Online Mendelian Inheritance in Man [OMIM],http://www.ncbi.nlm.nih.gov/omim/;
-NCBI Gene,http://www.ncbi.nlm.nih.gov/gene/;
-Picard tools,http://picard.sourceforge.net/;
-wAnnovar,http://wannovar.usc.edu/;
-dbSNP137,http://www.ncbi.nlm.nih.gov/projects/SNP/snp_summary.cgi/;
-1000 Genomes Project,http://www.1000genomes.org/;
-HapMap Project,http://hapmap.ncbi.nlm.nih.gov/;
-SMART,http://smart.embl-heidelberg.de/;
-Protein Data Bank [PDB],http://www.rcsb.org/pdb/home/home.do.
-Research for this study was supported by the Ministry of Health funding 5x1000 Fondazione G.B. Bietti funds—2016 to M.P. and Fondazione Roma; Bando Ricerca Indipendente ISS 2021–2023 to V.C., Istituto Superiore di Sanità; Italian Ministry of Health (CCR-2017-23669081 to M.T.), and Italian Ministry of Research (FOE_2019 to M.T.). The authors acknowledge Maria Luisa Alessi and Federica Petrocchi for technical help in the electrophysiological and perimetric evaluations, Serenella Venanzi for administrative assistance.
-Publisher’s Note:MDPI stays neutral with regard to jurisdictional claims in published maps and institutional affiliations.
-The following supporting information can be downloaded at:https://www.mdpi.com/article/10.3390/ijms232314656/s1.
-Click here for additional data file.
-Conceptualization, L.Z. and V.C.; methodology, C.M., E.S., S.C., L.B. and M.T. (Massimo Tatti); validation, E.C., L.B., C.M. and V.C.; bioinformatics analysis, A.C. and A.B.; investigation, L.Z., M.C., M.P. and E.C.; resources, M.V.; data curation, L.B., M.P., E.S., M.T. (Massimo Tatti), M.N. and V.C.; writing—original draft preparation, L.Z., V.C. and M.N.; writing—review and editing, M.N., E.S., M.C., M.T. (Marco Tartaglia) and V.C.; supervision, M.V. and M.T. (Marco Tartaglia); project administration, M.V., V.C. and M.T. (Marco Tartaglia); funding acquisition, M.V. and M.P. All authors have read and agreed to the published version of the manuscript.
-The study was conducted according to the guidelines of the Declaration of Helsinki and was approved by the local Institutional Ethical Committee of the IRCCS_Fondazione G.B. Bietti [Ret_02/2019].
-Signed informed consent was obtained from the participating family.
-Data that support the findings of this study are available from the corresponding authors upon request.
-The authors declare no conflict of interest.
-Family tree showing the segregation of the identified splice site change.
-Ocular phenotype of the proband right eye. (A) Ultrawide field color fundus photograph. (B) The 55° fundus autofluorescence. (C) Spectral-domain optical coherence tomography line horizontal scan. (D) Full-field dark-adapted electroretinogram. (E) Three-dimensional multifocal electroretinogram plot. (F) Goldmann kinetic visual field.
-Characterization of the pathogenicTUBvariant. (A) Transcript processing in primary skin fibroblasts from a healthy donor and from the proband carrying the homozygous splice site variant. Total RNA was extracted, reverse-transcribed and analyzed by PCR to resolve transcript processing. Two aberrant cDNA products were identified in mutated cells (left) compared to the expected length of the amplified fragment obtained from the control fibroblasts (right). (B) Schematic representation of aberrant transcript processing caused by the identified homozygous splice site change inTUB. (C) Western blot analysis of the TUB protein in patient’s fibroblasts and the control cells. Twenty, forty and sixty micrograms of whole cell extract were analyzed basally (left) and following 4 h treatment with 100 μM Mg132 (right) and probed with anti-TUB antibody (* indicates a non-specific product). (D) Expression of wild-type and mutant TUB protein was analyzed in the cytoplasmic and nuclear fractions were obtained from wild-type and mutated fibroblasts. Sixty micrograms of each fraction were analyzed by Western blot and then probed with anti-TUB antibody. Anti-YY1 and anti-HSP90 antibodies were used as the internal controls to assess the clarity of the different fractions (* indicates a non-specific product). Blots are representative of three experiments performed.
-TUB subcellular localization and cilium defects in cells with TUB LoF. (A) Thirty-hour-starved and PFA-fixed fibroblasts from a healthy donor and from the proband were analyzed by confocal microscopy for the localization of TUB using antibodies against TUB. (B) The presence and morphology of primary cilia in starved fibroblasts from the proband and a healthy donor. Cells were starved for 30 h and fixed with PFA 4%. Primary cilia were analyzed using antibodies against ARL13B (cilium axonemal, green) and pericentrin (basal body, red) to investigate morphogenesis. Nuclei are DAPI stained (blue). Bars correspond to 20 and 2 μm (left panels). (C) Histograms represent the percent value of presence/absence of cilium, normal/aberrant cilium morphology and normal/aberrant basal body structure and the length (μm) of axoneme. Five hundred cells were counted for each condition and axoneme length was measured. Imagines and bar plots are representative of three experiments performed. * indicate statistical significance forp&lt; 0.01 by using Student’sTtest.</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>{
-"pmid": "9390831",
-"alias_symbol": "rd5",
-"primary_gene_symbol": "TUB",
-"name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
-"evidence": ""
-}</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>HGNC:12406</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>ENSG00000166402</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>GENE ID:7275</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>TUB</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>rd5</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>9477305</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>mouse phenotype biomarker</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>discussion</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities.</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>TUB bipartite transcription factor</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>Some genetic syndromes causing loss of hearing and vision, such as some forms of Usher's syndrome, also cause reduced sperm cell motility, bronchiectasis, and other pathologies involving cilia- and flagella-bearing cells. In some Usher's patients, ultrastructural defects of axonemes within photoreceptor ciliary bridges, nasal cilia, and sperm cell flagella have been found, indicating a primary defect of axonemal conformation. Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities. They provide a good phenotypic match to human genetic sensory syndromes, particularly human sensory/obesity syndromes, such as Alstrom's and Bardet/Biedl, although no human candidate genes have been identified. Because of their unique phenotype, tubby mice are an appropriate model in which to look for a primary axonemal defect. We studied the axonemal ultrastructure of photoreceptors and sperm cells and performed functional testing of sperm in tub/tub mice before and after the onset of obesity. Approximately 15% of photoreceptor axonemes appeared abnormal in tub/tub animals, compared to 0% in controls. Both tub homozygotes and controls exhibited approximately 10% abnormal sperm cell axonemes, and no differences in sperm cell motile function were found at any age. The modest occurrence of axonemal defects in photoreceptors of tub/tub animals is likely to be a secondary effect of retinal degeneration. We conclude that the tubby phenotype is not associated with a generalized defect of cilia- and flagella-bearing cells and that the tub mutation does not primarily affect axonemal structure.</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>PMID: 9477305
-Abstract: Some genetic syndromes causing loss of hearing and vision, such as some forms of Usher's syndrome, also cause reduced sperm cell motility, bronchiectasis, and other pathologies involving cilia- and flagella-bearing cells. In some Usher's patients, ultrastructural defects of axonemes within photoreceptor ciliary bridges, nasal cilia, and sperm cell flagella have been found, indicating a primary defect of axonemal conformation. Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities. They provide a good phenotypic match to human genetic sensory syndromes, particularly human sensory/obesity syndromes, such as Alstrom's and Bardet/Biedl, although no human candidate genes have been identified. Because of their unique phenotype, tubby mice are an appropriate model in which to look for a primary axonemal defect. We studied the axonemal ultrastructure of photoreceptors and sperm cells and performed functional testing of sperm in tub/tub mice before and after the onset of obesity. Approximately 15% of photoreceptor axonemes appeared abnormal in tub/tub animals, compared to 0% in controls. Both tub homozygotes and controls exhibited approximately 10% abnormal sperm cell axonemes, and no differences in sperm cell motile function were found at any age. The modest occurrence of axonemal defects in photoreceptors of tub/tub animals is likely to be a secondary effect of retinal degeneration. We conclude that the tubby phenotype is not associated with a generalized defect of cilia- and flagella-bearing cells and that the tub mutation does not primarily affect axonemal structure.</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
-    Inputs:
-    Alias gene symbol: rd5
-    HGNC record ID: HGNC:12406
-    Primary gene symbol: TUB
-    Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
-    Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
-    Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
-    If the text does not support that the alias is an alternate abbreviation, return:
-    "alternate_abbreviation": "NO"
-    "evidence": ""
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
-    Evidence must be one exact sentence copied verbatim from the text.
-    Do not infer relationships or paraphrase evidence.
-    Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
-    {
-    "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
-    "alternate_abbreviation": "YES or NO",
-    "evidence": ""
-    }
-PMID: 9477305
-Abstract: Some genetic syndromes causing loss of hearing and vision, such as some forms of Usher's syndrome, also cause reduced sperm cell motility, bronchiectasis, and other pathologies involving cilia- and flagella-bearing cells. In some Usher's patients, ultrastructural defects of axonemes within photoreceptor ciliary bridges, nasal cilia, and sperm cell flagella have been found, indicating a primary defect of axonemal conformation. Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities. They provide a good phenotypic match to human genetic sensory syndromes, particularly human sensory/obesity syndromes, such as Alstrom's and Bardet/Biedl, although no human candidate genes have been identified. Because of their unique phenotype, tubby mice are an appropriate model in which to look for a primary axonemal defect. We studied the axonemal ultrastructure of photoreceptors and sperm cells and performed functional testing of sperm in tub/tub mice before and after the onset of obesity. Approximately 15% of photoreceptor axonemes appeared abnormal in tub/tub animals, compared to 0% in controls. Both tub homozygotes and controls exhibited approximately 10% abnormal sperm cell axonemes, and no differences in sperm cell motile function were found at any age. The modest occurrence of axonemal defects in photoreceptors of tub/tub animals is likely to be a secondary effect of retinal degeneration. We conclude that the tubby phenotype is not associated with a generalized defect of cilia- and flagella-bearing cells and that the tub mutation does not primarily affect axonemal structure.</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>{
-"pmid": "9477305",
-"alias_symbol": "rd5",
-"primary_gene_symbol": "TUB",
-"name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "YES",
-"alternate_abbreviation": "NO",
-"evidence": "Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities."
-}</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>HGNC:13919</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>ENSG00000234651, ENSG00000096155, ENSG00000233348, ENSG00000204463, ENSG00000228760, ENSG00000229524, ENSG00000227761</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>GENE ID:7917</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>BAG6</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>SCYTHE</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>37879364</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>literature defined (uniprot alternative protein name)</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>discussion</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>PBF also interacts with 14_3_3_ and Scythe/BAT3 proteins, two important cellular proteins involved in the regulation of cell apoptosis.</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr">
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr">
         <is>
           <t>BAG cochaperone 6</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="R18" t="inlineStr">
         <is>
           <t>We previously identified papillomavirus binding factor (PBF) as an osteosarcoma antigen recognized by an autologous cytotoxic T lymphocyte clone. Vaccination with PBF‐derived peptide presented by HLA‐A24 (PBF peptide) elicited strong immune responses. In the present study, we generated T cell receptor‐engineered T cells (TCR‐T cells) directed against the PBF peptide (PBF TCR‐T cells). PBF TCR was successfully transduced into T cells and detected using HLA‐A*24:02/PBF peptide tetramer. PBF TCR‐T cells generated from a healthy donor were highly expanded and recognized T2‐A24 cells pulsed with PBF peptide, HLA‐A24+293T cells transfected with PBF cDNA, and sarcoma cell lines. To establish an adoptive cell therapy model, we modified the PBF TCR by replacing both α and β constant regions with those of mice (hybrid PBF TCR). Hybrid PBF TCR‐T cells also showed reactivity against T2‐A24 cells pulsed with PBF peptide and to HLA‐A24+293T cells transfected with various lengths of PBF cDNA including the PBF peptide sequence. Subsequently, we generated target cell lines highly expressing PBF (MFH03‐PBF [short] epitope [+]) containing PBF peptide with in vivo tumorigenicity. Hybrid PBF TCR‐T cells exhibited antitumor effects compared with mock T cells in NSG mice xenografted with MFH03‐PBF (short) epitope (+) cells. CD45+T cells significantly infiltrated xenografted tumors only in the hybrid PBF TCR T cell group and most of these cells were CD8‐positive. CD8+T cells also showed Ki‐67 expression and surrounded the CD8‐negative tumor cells expressing Ki‐67. These findings suggest that PBF TCR‐T cell therapy might be a candidate immunotherapy for sarcoma highly expressing PBF.
 We developed TCR‐T cells targeting sarcoma‐associated antigen PBF (PBF TCR‐T cells). PBF TCR‐T cells showed anti‐tumor effects against sarcoma cell lines in vitro and in vivo. PBF TCR‐T cell therapy might be a candidate immunotherapy for sarcoma highly expressing PBF.
@@ -4486,12 +4720,12 @@
 To assess the in vivo antitumor effects of hybrid PBF TCR‐T cells, we decided to generate target tumor cells with strong tumorigenesis in NSG mice and high expression of PBF. Therefore, we selected MFH03 cells, which exhibit strong tumorigenesis in mice, and stably transfected them with PBF cDNA containing the PBF epitope peptide; the cells were named MFH03‐PBF (short) epitope (+) cells (Figure4A). In parallel with the generation of hybrid PBF TCR‐T cells, mock T cells that were transduced with retroviral empty vector were also generated (Figure4B). Hybrid PBF TCR‐T cells showed cytotoxicity against MFH03‐PBF (short) epitope (+) cells (FigureS2). Adoptive cell transfer experiments were conducted with these effector cells and target cells. Hybrid PBF TCR‐T cells and mock T cells were administered on day 15 after the target cell inoculation. The results showed that tumor growth was suppressed in the hybrid PBF TCR‐T group compared with the mock T group, with significant differences in tumor volume observed on day 39 (p&lt; 0.0079, Figure4C,D, FigureS3).</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>We previously identified papillomavirus binding factor (PBF) as an osteosarcoma antigen recognized by an autologous cytotoxic T lymphocyte clone. Vaccination with PBF-derived peptide presented by HLA-A24 (PBF peptide) elicited strong immune responses. In the present study, we generated T cell receptor-engineered T cells (TCR-T cells) directed against the PBF peptide (PBF TCR-T cells). PBF TCR was successfully transduced into T cells and detected using HLA-A*24:02/PBF peptide tetramer. PBF TCR-T cells generated from a healthy donor were highly expanded and recognized T2-A24 cells pulsed with PBF peptide, HLA-A24&lt;sup&gt;+&lt;/sup&gt; 293T cells transfected with PBF cDNA, and sarcoma cell lines. To establish an adoptive cell therapy model, we modified the PBF TCR by replacing both α and β constant regions with those of mice (hybrid PBF TCR). Hybrid PBF TCR-T cells also showed reactivity against T2-A24 cells pulsed with PBF peptide and to HLA-A24&lt;sup&gt;+&lt;/sup&gt; 293T cells transfected with various lengths of PBF cDNA including the PBF peptide sequence. Subsequently, we generated target cell lines highly expressing PBF (MFH03-PBF [short] epitope [+]) containing PBF peptide with in vivo tumorigenicity. Hybrid PBF TCR-T cells exhibited antitumor effects compared with mock T cells in NSG mice xenografted with MFH03-PBF (short) epitope (+) cells. CD45&lt;sup&gt;+&lt;/sup&gt; T cells significantly infiltrated xenografted tumors only in the hybrid PBF TCR T cell group and most of these cells were CD8-positive. CD8&lt;sup&gt;+&lt;/sup&gt; T cells also showed Ki-67 expression and surrounded the CD8-negative tumor cells expressing Ki-67. These findings suggest that PBF TCR-T cell therapy might be a candidate immunotherapy for sarcoma highly expressing PBF.</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>PMID: 37879364
 Full Text: We previously identified papillomavirus binding factor (PBF) as an osteosarcoma antigen recognized by an autologous cytotoxic T lymphocyte clone. Vaccination with PBF‐derived peptide presented by HLA‐A24 (PBF peptide) elicited strong immune responses. In the present study, we generated T cell receptor‐engineered T cells (TCR‐T cells) directed against the PBF peptide (PBF TCR‐T cells). PBF TCR was successfully transduced into T cells and detected using HLA‐A*24:02/PBF peptide tetramer. PBF TCR‐T cells generated from a healthy donor were highly expanded and recognized T2‐A24 cells pulsed with PBF peptide, HLA‐A24+293T cells transfected with PBF cDNA, and sarcoma cell lines. To establish an adoptive cell therapy model, we modified the PBF TCR by replacing both α and β constant regions with those of mice (hybrid PBF TCR). Hybrid PBF TCR‐T cells also showed reactivity against T2‐A24 cells pulsed with PBF peptide and to HLA‐A24+293T cells transfected with various lengths of PBF cDNA including the PBF peptide sequence. Subsequently, we generated target cell lines highly expressing PBF (MFH03‐PBF [short] epitope [+]) containing PBF peptide with in vivo tumorigenicity. Hybrid PBF TCR‐T cells exhibited antitumor effects compared with mock T cells in NSG mice xenografted with MFH03‐PBF (short) epitope (+) cells. CD45+T cells significantly infiltrated xenografted tumors only in the hybrid PBF TCR T cell group and most of these cells were CD8‐positive. CD8+T cells also showed Ki‐67 expression and surrounded the CD8‐negative tumor cells expressing Ki‐67. These findings suggest that PBF TCR‐T cell therapy might be a candidate immunotherapy for sarcoma highly expressing PBF.
@@ -4526,7 +4760,7 @@
 To assess the in vivo antitumor effects of hybrid PBF TCR‐T cells, we decided to generate target tumor cells with strong tumorigenesis in NSG mice and high expression of PBF. Therefore, we selected MFH03 cells, which exhibit strong tumorigenesis in mice, and stably transfected them with PBF cDNA containing the PBF epitope peptide; the cells were named MFH03‐PBF (short) epitope (+) cells (Figure4A). In parallel with the generation of hybrid PBF TCR‐T cells, mock T cells that were transduced with retroviral empty vector were also generated (Figure4B). Hybrid PBF TCR‐T cells showed cytotoxicity against MFH03‐PBF (short) epitope (+) cells (FigureS2). Adoptive cell transfer experiments were conducted with these effector cells and target cells. Hybrid PBF TCR‐T cells and mock T cells were administered on day 15 after the target cell inoculation. The results showed that tumor growth was suppressed in the hybrid PBF TCR‐T group compared with the mock T group, with significant differences in tumor volume observed on day 39 (p&lt; 0.0079, Figure4C,D, FigureS3).</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -4534,35 +4768,43 @@
     HGNC record ID: HGNC:13919
     Primary gene symbol: BAG6
     Official HGNC gene name: BAG cochaperone 6
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -4599,99 +4841,98 @@
 To assess the in vivo antitumor effects of hybrid PBF TCR‐T cells, we decided to generate target tumor cells with strong tumorigenesis in NSG mice and high expression of PBF. Therefore, we selected MFH03 cells, which exhibit strong tumorigenesis in mice, and stably transfected them with PBF cDNA containing the PBF epitope peptide; the cells were named MFH03‐PBF (short) epitope (+) cells (Figure4A). In parallel with the generation of hybrid PBF TCR‐T cells, mock T cells that were transduced with retroviral empty vector were also generated (Figure4B). Hybrid PBF TCR‐T cells showed cytotoxicity against MFH03‐PBF (short) epitope (+) cells (FigureS2). Adoptive cell transfer experiments were conducted with these effector cells and target cells. Hybrid PBF TCR‐T cells and mock T cells were administered on day 15 after the target cell inoculation. The results showed that tumor growth was suppressed in the hybrid PBF TCR‐T group compared with the mock T group, with significant differences in tumor volume observed on day 39 (p&lt; 0.0079, Figure4C,D, FigureS3).</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>{
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>Based on the provided text, here is my analysis:
+{
 "pmid": "37879364",
-"alias_symbol": "SCYTHE",
+"alias_symbol": "PBF",
 "primary_gene_symbol": "BAG6",
 "name": "BAG cochaperone 6",
-"alias_symbol_represents_primary_gene": "NO",
 "alternate_abbreviation": "NO",
 "evidence": ""
-}</t>
+}
+The text does not provide evidence that PBF (papillomavirus binding factor) is an alternate abbreviation for BAG6 (BAG cochaperone 6). The text discusses PBF as a separate gene/protein that was identified as an osteosarcoma antigen. It does not link PBF to BAG6 or expand PBF to the official gene name "BAG cochaperone 6". Therefore, there is no evidence to classify PBF as an alternate abbreviation for BAG6 in this context.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>HGNC:13919</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>ENSG00000234651, ENSG00000096155, ENSG00000233348, ENSG00000204463, ENSG00000228760, ENSG00000229524, ENSG00000227761</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>GENE ID:7917</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>BAG6</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>SCYTHE</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>37879364</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>37879364</v>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>literature defined (uniprot alternative protein name)</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>discussion</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>PBF also interacts with 14_3_3_ and Scythe/BAT3 proteins, two important cellular proteins involved in the regulation of cell apoptosis.</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr">
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr">
         <is>
           <t>BAG cochaperone 6</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="R19" t="inlineStr">
         <is>
           <t>Papillomavirus binding factor (PBF) T cell receptor‐engineered T cells (TCR‐T cells) exert antitumor effects in a xenografted mouse model. (A) The PBF (short) epitope (+) gene was transduced into MFH03 cells for an in vivo assay. (B) Tetramer assay of PBF TCR‐T cells before adoptive cell transfer. (C) Tumor volume over time. The day on which tumor cells were transplanted into the mouse was set as day 0, and PBF TCR‐T cells or mock T cells were administered on day 14. (D) Tumor volume and weight at the endpoint. (E–H) Immunohistochemical findings of tumors excised from mice that were transferred with PBF TCR‐T cells. They were stained with monoclonal antibodies against CD45 (E and F), CD4, and CD8 (G) and both CD8 and Ki‐67 monoclonal antibodies (H). Black arrows indicate double‐stained cells (H). (I–N) Tetramer positivity rate (I and J) and the expression levels of PD‐1 (K and L) and Lag‐3 (M and N) in the removed mouse splenocytes were analyzed by flow cytometry (n= 5).
 Next, the infiltration of the transferred T cells into excised tumor tissues was analyzed by immunohistochemistry. The infiltration of CD45‐positive lymphocytes into the tumor was significantly higher in the TCR‐T group than in the mock group (p= 0.0021, Figure4E,F). The infiltrating lymphocytes were almost entirely CD8‐positive, in contrast to a few CD4‐positive lymphocytes (Figure4G). Moreover, hybrid PBF TCR‐T cells showed enhanced Ki‐67 expression, which suggested that these cells possessed a proliferative tendency in specific response to the antigen (Figure4H). In mouse spleens, PBF tetramer‐positive cells were detected in the hybrid PBF TCR‐T group (Figure4I,J). However, the expression levels of PD‐1 (Figure4K,L) and Lag‐3 (Figure4M,N) in the splenocytes were no different between hybrid PBF TCR‐T and mock T cells. The exhaustion status was not specific for the PBF TCR and might be a natural course of transferred T cells in the in vivo mouse model.
@@ -4711,12 +4952,12 @@
 The authors thank Ms. Asuka Akamatsu and Ms. Serina Tokita for technical assistance.</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="S19" t="inlineStr">
         <is>
           <t>We previously identified papillomavirus binding factor (PBF) as an osteosarcoma antigen recognized by an autologous cytotoxic T lymphocyte clone. Vaccination with PBF-derived peptide presented by HLA-A24 (PBF peptide) elicited strong immune responses. In the present study, we generated T cell receptor-engineered T cells (TCR-T cells) directed against the PBF peptide (PBF TCR-T cells). PBF TCR was successfully transduced into T cells and detected using HLA-A*24:02/PBF peptide tetramer. PBF TCR-T cells generated from a healthy donor were highly expanded and recognized T2-A24 cells pulsed with PBF peptide, HLA-A24&lt;sup&gt;+&lt;/sup&gt; 293T cells transfected with PBF cDNA, and sarcoma cell lines. To establish an adoptive cell therapy model, we modified the PBF TCR by replacing both α and β constant regions with those of mice (hybrid PBF TCR). Hybrid PBF TCR-T cells also showed reactivity against T2-A24 cells pulsed with PBF peptide and to HLA-A24&lt;sup&gt;+&lt;/sup&gt; 293T cells transfected with various lengths of PBF cDNA including the PBF peptide sequence. Subsequently, we generated target cell lines highly expressing PBF (MFH03-PBF [short] epitope [+]) containing PBF peptide with in vivo tumorigenicity. Hybrid PBF TCR-T cells exhibited antitumor effects compared with mock T cells in NSG mice xenografted with MFH03-PBF (short) epitope (+) cells. CD45&lt;sup&gt;+&lt;/sup&gt; T cells significantly infiltrated xenografted tumors only in the hybrid PBF TCR T cell group and most of these cells were CD8-positive. CD8&lt;sup&gt;+&lt;/sup&gt; T cells also showed Ki-67 expression and surrounded the CD8-negative tumor cells expressing Ki-67. These findings suggest that PBF TCR-T cell therapy might be a candidate immunotherapy for sarcoma highly expressing PBF.</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr">
+      <c r="T19" t="inlineStr">
         <is>
           <t>PMID: 37879364
 Full Text: Papillomavirus binding factor (PBF) T cell receptor‐engineered T cells (TCR‐T cells) exert antitumor effects in a xenografted mouse model. (A) The PBF (short) epitope (+) gene was transduced into MFH03 cells for an in vivo assay. (B) Tetramer assay of PBF TCR‐T cells before adoptive cell transfer. (C) Tumor volume over time. The day on which tumor cells were transplanted into the mouse was set as day 0, and PBF TCR‐T cells or mock T cells were administered on day 14. (D) Tumor volume and weight at the endpoint. (E–H) Immunohistochemical findings of tumors excised from mice that were transferred with PBF TCR‐T cells. They were stained with monoclonal antibodies against CD45 (E and F), CD4, and CD8 (G) and both CD8 and Ki‐67 monoclonal antibodies (H). Black arrows indicate double‐stained cells (H). (I–N) Tetramer positivity rate (I and J) and the expression levels of PD‐1 (K and L) and Lag‐3 (M and N) in the removed mouse splenocytes were analyzed by flow cytometry (n= 5).
@@ -4737,7 +4978,7 @@
 The authors thank Ms. Asuka Akamatsu and Ms. Serina Tokita for technical assistance.</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="U19" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -4745,35 +4986,43 @@
     HGNC record ID: HGNC:13919
     Primary gene symbol: BAG6
     Official HGNC gene name: BAG cochaperone 6
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -4796,99 +5045,96 @@
 The authors thank Ms. Asuka Akamatsu and Ms. Serina Tokita for technical assistance.</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr">
+      <c r="V19" t="inlineStr">
         <is>
           <t>{
 "pmid": "37879364",
 "alias_symbol": "SCYTHE",
 "primary_gene_symbol": "BAG6",
 "name": "BAG cochaperone 6",
-"alias_symbol_represents_primary_gene": "YES",
-"alternate_abbreviation": "NO",
-"evidence": "PBF also interacts with 14‐3‐3β and Scythe/BAT3 proteins, two important cellular proteins involved in the regulation of cell apoptosis.16,17"
+"alternate_abbreviation": "YES",
+"evidence": "PBF also interacts with 14‐3‐3β and Scythe/BAT3 proteins, two important cellular proteins involved in the regulation of cell apoptosis."
 }</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>HGNC:13919</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>ENSG00000234651, ENSG00000096155, ENSG00000233348, ENSG00000204463, ENSG00000228760, ENSG00000229524, ENSG00000227761</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>GENE ID:7917</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>BAG6</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>SCYTHE</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>38498560</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>38498560</v>
+      </c>
+      <c r="I20" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>alias</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>alias</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>intro</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>BAG6 (BCL2-associated athanogene 6, also known as BAT3 or Scythe) is a member of the BAG family due to a sequence homologous to the BAG domain at its C terminus and the collaboration with Heat Shock Protein 70 (Hsp70) family molecular chaperones</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr">
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr">
         <is>
           <t>BAG cochaperone 6</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="R20" t="inlineStr">
         <is>
           <t>The authors have declared that no competing interests exist.
 The interaction between influenza A virus (IAV) and host proteins is an important process that greatly influences viral replication and pathogenicity. PB2 protein is a subunit of viral ribonucleoprotein (vRNP) complex playing distinct roles in viral transcription and replication. BAG6 (BCL2-associated athanogene 6) as a multifunctional host protein participates in physiological and pathological processes. Here, we identify BAG6 as a new restriction factor for IAV replication through targeting PB2. For both avian and human influenza viruses, overexpression of BAG6 reduced viral protein expression and virus titers, whereas deletion of BAG6 significantly enhanced virus replication. Moreover, BAG6-knockdown mice developed more severe clinical symptoms and higher viral loads upon IAV infection. Mechanistically, BAG6 restricted IAV transcription and replication by inhibiting the activity of viral RNA-dependent RNA polymerase (RdRp). The co-immunoprecipitation assays showed BAG6 specifically interacted with the N-terminus of PB2 and competed with PB1 for RdRp complex assembly. The ubiquitination assay indicated that BAG6 promoted PB2 ubiquitination at K189 residue and targeted PB2 for K48-linked ubiquitination degradation. The antiviral effect of BAG6 necessitated its N-terminal region containing a ubiquitin-like (UBL) domain (17-92aa) and a PB2-binding domain (124-186aa), which are synergistically responsible for viral polymerase subunit PB2 degradation and perturbing RdRp complex assembly. These findings unravel a novel antiviral mechanism via the interaction of viral PB2 and host protein BAG6 during avian or human influenza virus infection and highlight a potential application of BAG6 for antiviral drug development.
@@ -4908,12 +5154,12 @@
 (A) HeLa cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The viral NP and innate immunity-associated protein expression were measured by western blotting at different time points postinfection, as indicated. (B) BAG6-KO and BAG6-WT HeLa cells were infected with IAV H1N1 (MOI = 1.0), and the NP and innate immunity-associated protein expression were determined by western blotting at the indicated time points. (C) IRF9-KO Hela cells were transfected BAG6-HA expression plasmid or HA-vector. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The NP and innate immunity-associated protein expression were measured by western blotting at different time points post-infection, as indicated (C, left panels), and densitometry analysis and quantification were performed (C, right panels). (D) HeLa-WT (left panels) or HeLa-IRF9-KO (right panels) cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). Viral titers in the supernatants were determined by TCID50assay at 6, 12 and 24 h post-infection. (E and F) Vero cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The viral NP and M1 expression were measured by western blotting at different time points postinfection, as indicated (E). Viral titers in the supernatants were determined by TCID50assay at 6, 12 and 24 h post-infection (F). Data presented as means ± SD and are representative of three independent experiments. *p&lt; 0.05, **p&lt; 0.01, ***p&lt; 0.001, Unpaired Student’s t test.</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="S20" t="inlineStr">
         <is>
           <t>The interaction between influenza A virus (IAV) and host proteins is an important process that greatly influences viral replication and pathogenicity. PB2 protein is a subunit of viral ribonucleoprotein (vRNP) complex playing distinct roles in viral transcription and replication. BAG6 (BCL2-associated athanogene 6) as a multifunctional host protein participates in physiological and pathological processes. Here, we identify BAG6 as a new restriction factor for IAV replication through targeting PB2. For both avian and human influenza viruses, overexpression of BAG6 reduced viral protein expression and virus titers, whereas deletion of BAG6 significantly enhanced virus replication. Moreover, BAG6-knockdown mice developed more severe clinical symptoms and higher viral loads upon IAV infection. Mechanistically, BAG6 restricted IAV transcription and replication by inhibiting the activity of viral RNA-dependent RNA polymerase (RdRp). The co-immunoprecipitation assays showed BAG6 specifically interacted with the N-terminus of PB2 and competed with PB1 for RdRp complex assembly. The ubiquitination assay indicated that BAG6 promoted PB2 ubiquitination at K189 residue and targeted PB2 for K48-linked ubiquitination degradation. The antiviral effect of BAG6 necessitated its N-terminal region containing a ubiquitin-like (UBL) domain (17-92aa) and a PB2-binding domain (124-186aa), which are synergistically responsible for viral polymerase subunit PB2 degradation and perturbing RdRp complex assembly. These findings unravel a novel antiviral mechanism via the interaction of viral PB2 and host protein BAG6 during avian or human influenza virus infection and highlight a potential application of BAG6 for antiviral drug development.</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
+      <c r="T20" t="inlineStr">
         <is>
           <t>PMID: 38498560
 Full Text: The authors have declared that no competing interests exist.
@@ -4934,7 +5180,7 @@
 (A) HeLa cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The viral NP and innate immunity-associated protein expression were measured by western blotting at different time points postinfection, as indicated. (B) BAG6-KO and BAG6-WT HeLa cells were infected with IAV H1N1 (MOI = 1.0), and the NP and innate immunity-associated protein expression were determined by western blotting at the indicated time points. (C) IRF9-KO Hela cells were transfected BAG6-HA expression plasmid or HA-vector. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The NP and innate immunity-associated protein expression were measured by western blotting at different time points post-infection, as indicated (C, left panels), and densitometry analysis and quantification were performed (C, right panels). (D) HeLa-WT (left panels) or HeLa-IRF9-KO (right panels) cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). Viral titers in the supernatants were determined by TCID50assay at 6, 12 and 24 h post-infection. (E and F) Vero cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The viral NP and M1 expression were measured by western blotting at different time points postinfection, as indicated (E). Viral titers in the supernatants were determined by TCID50assay at 6, 12 and 24 h post-infection (F). Data presented as means ± SD and are representative of three independent experiments. *p&lt; 0.05, **p&lt; 0.01, ***p&lt; 0.001, Unpaired Student’s t test.</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="U20" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -4942,35 +5188,43 @@
     HGNC record ID: HGNC:13919
     Primary gene symbol: BAG6
     Official HGNC gene name: BAG cochaperone 6
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -4993,99 +5247,98 @@
 (A) HeLa cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The viral NP and innate immunity-associated protein expression were measured by western blotting at different time points postinfection, as indicated. (B) BAG6-KO and BAG6-WT HeLa cells were infected with IAV H1N1 (MOI = 1.0), and the NP and innate immunity-associated protein expression were determined by western blotting at the indicated time points. (C) IRF9-KO Hela cells were transfected BAG6-HA expression plasmid or HA-vector. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The NP and innate immunity-associated protein expression were measured by western blotting at different time points post-infection, as indicated (C, left panels), and densitometry analysis and quantification were performed (C, right panels). (D) HeLa-WT (left panels) or HeLa-IRF9-KO (right panels) cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). Viral titers in the supernatants were determined by TCID50assay at 6, 12 and 24 h post-infection. (E and F) Vero cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The viral NP and M1 expression were measured by western blotting at different time points postinfection, as indicated (E). Viral titers in the supernatants were determined by TCID50assay at 6, 12 and 24 h post-infection (F). Data presented as means ± SD and are representative of three independent experiments. *p&lt; 0.05, **p&lt; 0.01, ***p&lt; 0.001, Unpaired Student’s t test.</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>{
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>Based on the provided text, here is my analysis:
+{
 "pmid": "38498560",
 "alias_symbol": "SCYTHE",
 "primary_gene_symbol": "BAG6",
 "name": "BAG cochaperone 6",
-"alias_symbol_represents_primary_gene": "YES",
-"alternate_abbreviation": "NO",
+"alternate_abbreviation": "YES",
 "evidence": "BAG6 (BCL2-associated athanogene 6, also known as BAT3 or Scythe) is a member of the BAG family due to a sequence homologous to the BAG domain at its C terminus and the collaboration with Heat Shock Protein 70 (Hsp70) family molecular chaperones [16]."
-}</t>
+}
+The text explicitly links the alias symbol SCYTHE to BAG6 by stating "BAG6 (BCL2-associated athanogene 6, also known as BAT3 or Scythe)". This indicates that SCYTHE is an alternate abbreviation for BAG6.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>HGNC:13919</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>ENSG00000234651, ENSG00000096155, ENSG00000233348, ENSG00000204463, ENSG00000228760, ENSG00000229524, ENSG00000227761</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>GENE ID:7917</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>BAG6</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>SCYTHE</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>38498560</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>38498560</v>
+      </c>
+      <c r="I21" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>alias</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>alias</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>intro</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>BAG6 (BCL2-associated athanogene 6, also known as BAT3 or Scythe) is a member of the BAG family due to a sequence homologous to the BAG domain at its C terminus and the collaboration with Heat Shock Protein 70 (Hsp70) family molecular chaperones</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr">
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr">
         <is>
           <t>BAG cochaperone 6</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="R21" t="inlineStr">
         <is>
           <t>To explore the mechanism by which BAG6 inhibits IAV replication, we assessed the impact of BAG6 on the polymerase activity of influenza viruses using a well-established dual-luciferase reporter assay [32,33]. The plasmids for expression of PB2, PB1, PA, and NP genes from various IAV subtype strains, including PR8 (H1N1), CN0606 (H7N9), and SD196 (H9N2), were co-transfected into HEK293T cells along with a pPoll-Luc reporter, respectively. The firefly luciferase levels in the cell lysate reflected the overall transcription and replication activities of viral polymerase complex (RdRp). The results showed that the overexpression of BAG6 inhibited the polymerase activities of H1N1, H7N9, and H9N2 in a dose-dependent manner (Fig 5A). In contrast, the enhanced polymerase activities of all IAV subtypes were observed in BAG6-KO A549 cells compared to the WT control (Fig 5B). The influenza virus polymerase complex is a key enzyme responsible for the replication and transcription of the influenza virus genome [34]. In view of this, we performed qRT-PCR analysis of viral mRNA and vRNA in H1N1-infected cells. The results showed that the mRNA and vRNA levels of both NP and M1 genes were significantly suppressed in BAG6-overexpressing cells (Fig 5C and 5D), and were elevated in BAG6-KO cells (Fig 5E and 5F). These data demonstrate that the BAG6 can inhibit the polymerase activity of various IAV subtypes.
 (A) HEK293T cells were co-transfected with pPolI-Luc reporter plasmid and expression plasmids containing viral PB1, PB2, PA, and NP of H1N1, H7N9 or H9N2 along with a graded dose of BAG6 or empty vector. Renilla luciferase was used as an internal control. Luciferase activity of the viral polymerase was determined at 24 h post-transfection (left panels). Western blottings show the expression of all transfected proteins (right panels) (B) BAG6-KO or BAG6-WT A549 cells were co-transfected with pPolI-Luc reporter plasmid and expression plasmids containing viral PB1, PB2, PA, and NP of H1N1/H7N9/H9N2. Renilla luciferase was used as an internal control. Luciferase activity of the viral polymerase was determined at 24 h post-transfection (left panel). Western blottings show the expression of all transfected proteins (right panel). (C and D) A549 cells was transfected with BAG6 expression plasmid or empty vector. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). At 4, 8, 12 and 24 h post-infection, the mRNA (C) and vRNA (D) level of M1 and NP were measured by quantitative real-time PCR, respectively. The expression of BAG6-HA was monitored by western blotting. (E and F) BAG6-KO or BAG6-WT A549 cells were infected with IAV H1N1 (MOI = 1.0). At 4, 8, 12 and 24 h post-infection, the mRNA (E) and vRNA (F) level of NP and M1 were measured by quantitative real-time PCR, respectively. The expression of BAG6-HA was monitored by western blotting. Data presented as means ± SD and are representative of three independent experiments. *p&lt; 0.05, **p&lt; 0.01, ***p&lt; 0.001, Unpaired Student’s t test.
@@ -5102,12 +5355,12 @@
 To further determine the PB2-binding sites of BAG6, we analyzed the protein structure of BAG6 from AlphaFold2 database and predicted the corresponding interaction domain of BAG6 and PB2 using an online software ColabFold. As shown inFig 9A, BAG6 associates with the N-terminus of PB2 through its 124–186 amino acids, which at least partially occupies the spatial position of PB1-PB2 interaction, whereas the Ub-like domain (17-92aa) at the N-terminus of BAG6 does not exhibit a direct interaction with PB2 in structure. According to the previous reports [40,41,43,45], the UBL domain is mainly responsible for recruiting ubiquitination machinery for efficient ubiquitination and degradation of various protein substrates. We, therefore, hypothesize that BAG6 may function as a transient platform that recruits the ubiquitin ligase by UBL domain and binds PB2 substrate by 124-186aa region during IAV infection, promoting PB2 degradation and IAV restriction. To verify this hypothesis, we constructed the corresponding truncation mutant plasmids, including BAG6 1:92-HA and 92:255-HA, as well as a deletion mutant lacking 124-186aa (BAG6 del 124:186-HA), as indicated inFig 9B. The Co-IP assay showed that only BAG6 92:255-HA was readily immunoprecipitated with PB2-Flag, but other mutants lacking 124-186aa region (1:92-HA and del 124:186-HA) could not bind to PB2 (Fig 9C), confirming the residues 124–186 as PB2-binding region of BAG6. Interestingly, compared with BAG6 1:255-HA, the ectopic expression of BAG6 92:255-HA had an obvious but reduced inhibitory effect on viral NP protein expression (Fig 9D), viral titers (Fig 9E), and viral polymerase activity (Fig 9F) in H1N1-infected cells, whereas BAG6 1:92-HA and del 124:186-HA completely failed to inhibit IAV replication and polymerase activity. These findings indicate that the PB2-binding region of BAG6 is necessary but insufficient for efficient IAV restriction. It may exert a reduced antiviral effects through binding PB2 and disrupting RdRp complex assembly, but fail to recruit ubiquitination machinery for PB2 degradation. These data demonstrate that both the UBL domain (17-92aa) and PB2-binding region (124-186aa) are required for highly effective PB2 degradation and IAV restriction.</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr">
+      <c r="S21" t="inlineStr">
         <is>
           <t>The interaction between influenza A virus (IAV) and host proteins is an important process that greatly influences viral replication and pathogenicity. PB2 protein is a subunit of viral ribonucleoprotein (vRNP) complex playing distinct roles in viral transcription and replication. BAG6 (BCL2-associated athanogene 6) as a multifunctional host protein participates in physiological and pathological processes. Here, we identify BAG6 as a new restriction factor for IAV replication through targeting PB2. For both avian and human influenza viruses, overexpression of BAG6 reduced viral protein expression and virus titers, whereas deletion of BAG6 significantly enhanced virus replication. Moreover, BAG6-knockdown mice developed more severe clinical symptoms and higher viral loads upon IAV infection. Mechanistically, BAG6 restricted IAV transcription and replication by inhibiting the activity of viral RNA-dependent RNA polymerase (RdRp). The co-immunoprecipitation assays showed BAG6 specifically interacted with the N-terminus of PB2 and competed with PB1 for RdRp complex assembly. The ubiquitination assay indicated that BAG6 promoted PB2 ubiquitination at K189 residue and targeted PB2 for K48-linked ubiquitination degradation. The antiviral effect of BAG6 necessitated its N-terminal region containing a ubiquitin-like (UBL) domain (17-92aa) and a PB2-binding domain (124-186aa), which are synergistically responsible for viral polymerase subunit PB2 degradation and perturbing RdRp complex assembly. These findings unravel a novel antiviral mechanism via the interaction of viral PB2 and host protein BAG6 during avian or human influenza virus infection and highlight a potential application of BAG6 for antiviral drug development.</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr">
+      <c r="T21" t="inlineStr">
         <is>
           <t>PMID: 38498560
 Full Text: To explore the mechanism by which BAG6 inhibits IAV replication, we assessed the impact of BAG6 on the polymerase activity of influenza viruses using a well-established dual-luciferase reporter assay [32,33]. The plasmids for expression of PB2, PB1, PA, and NP genes from various IAV subtype strains, including PR8 (H1N1), CN0606 (H7N9), and SD196 (H9N2), were co-transfected into HEK293T cells along with a pPoll-Luc reporter, respectively. The firefly luciferase levels in the cell lysate reflected the overall transcription and replication activities of viral polymerase complex (RdRp). The results showed that the overexpression of BAG6 inhibited the polymerase activities of H1N1, H7N9, and H9N2 in a dose-dependent manner (Fig 5A). In contrast, the enhanced polymerase activities of all IAV subtypes were observed in BAG6-KO A549 cells compared to the WT control (Fig 5B). The influenza virus polymerase complex is a key enzyme responsible for the replication and transcription of the influenza virus genome [34]. In view of this, we performed qRT-PCR analysis of viral mRNA and vRNA in H1N1-infected cells. The results showed that the mRNA and vRNA levels of both NP and M1 genes were significantly suppressed in BAG6-overexpressing cells (Fig 5C and 5D), and were elevated in BAG6-KO cells (Fig 5E and 5F). These data demonstrate that the BAG6 can inhibit the polymerase activity of various IAV subtypes.
@@ -5125,7 +5378,7 @@
 To further determine the PB2-binding sites of BAG6, we analyzed the protein structure of BAG6 from AlphaFold2 database and predicted the corresponding interaction domain of BAG6 and PB2 using an online software ColabFold. As shown inFig 9A, BAG6 associates with the N-terminus of PB2 through its 124–186 amino acids, which at least partially occupies the spatial position of PB1-PB2 interaction, whereas the Ub-like domain (17-92aa) at the N-terminus of BAG6 does not exhibit a direct interaction with PB2 in structure. According to the previous reports [40,41,43,45], the UBL domain is mainly responsible for recruiting ubiquitination machinery for efficient ubiquitination and degradation of various protein substrates. We, therefore, hypothesize that BAG6 may function as a transient platform that recruits the ubiquitin ligase by UBL domain and binds PB2 substrate by 124-186aa region during IAV infection, promoting PB2 degradation and IAV restriction. To verify this hypothesis, we constructed the corresponding truncation mutant plasmids, including BAG6 1:92-HA and 92:255-HA, as well as a deletion mutant lacking 124-186aa (BAG6 del 124:186-HA), as indicated inFig 9B. The Co-IP assay showed that only BAG6 92:255-HA was readily immunoprecipitated with PB2-Flag, but other mutants lacking 124-186aa region (1:92-HA and del 124:186-HA) could not bind to PB2 (Fig 9C), confirming the residues 124–186 as PB2-binding region of BAG6. Interestingly, compared with BAG6 1:255-HA, the ectopic expression of BAG6 92:255-HA had an obvious but reduced inhibitory effect on viral NP protein expression (Fig 9D), viral titers (Fig 9E), and viral polymerase activity (Fig 9F) in H1N1-infected cells, whereas BAG6 1:92-HA and del 124:186-HA completely failed to inhibit IAV replication and polymerase activity. These findings indicate that the PB2-binding region of BAG6 is necessary but insufficient for efficient IAV restriction. It may exert a reduced antiviral effects through binding PB2 and disrupting RdRp complex assembly, but fail to recruit ubiquitination machinery for PB2 degradation. These data demonstrate that both the UBL domain (17-92aa) and PB2-binding region (124-186aa) are required for highly effective PB2 degradation and IAV restriction.</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="U21" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -5133,35 +5386,43 @@
     HGNC record ID: HGNC:13919
     Primary gene symbol: BAG6
     Official HGNC gene name: BAG cochaperone 6
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -5181,221 +5442,6 @@
 To further determine the PB2-binding sites of BAG6, we analyzed the protein structure of BAG6 from AlphaFold2 database and predicted the corresponding interaction domain of BAG6 and PB2 using an online software ColabFold. As shown inFig 9A, BAG6 associates with the N-terminus of PB2 through its 124–186 amino acids, which at least partially occupies the spatial position of PB1-PB2 interaction, whereas the Ub-like domain (17-92aa) at the N-terminus of BAG6 does not exhibit a direct interaction with PB2 in structure. According to the previous reports [40,41,43,45], the UBL domain is mainly responsible for recruiting ubiquitination machinery for efficient ubiquitination and degradation of various protein substrates. We, therefore, hypothesize that BAG6 may function as a transient platform that recruits the ubiquitin ligase by UBL domain and binds PB2 substrate by 124-186aa region during IAV infection, promoting PB2 degradation and IAV restriction. To verify this hypothesis, we constructed the corresponding truncation mutant plasmids, including BAG6 1:92-HA and 92:255-HA, as well as a deletion mutant lacking 124-186aa (BAG6 del 124:186-HA), as indicated inFig 9B. The Co-IP assay showed that only BAG6 92:255-HA was readily immunoprecipitated with PB2-Flag, but other mutants lacking 124-186aa region (1:92-HA and del 124:186-HA) could not bind to PB2 (Fig 9C), confirming the residues 124–186 as PB2-binding region of BAG6. Interestingly, compared with BAG6 1:255-HA, the ectopic expression of BAG6 92:255-HA had an obvious but reduced inhibitory effect on viral NP protein expression (Fig 9D), viral titers (Fig 9E), and viral polymerase activity (Fig 9F) in H1N1-infected cells, whereas BAG6 1:92-HA and del 124:186-HA completely failed to inhibit IAV replication and polymerase activity. These findings indicate that the PB2-binding region of BAG6 is necessary but insufficient for efficient IAV restriction. It may exert a reduced antiviral effects through binding PB2 and disrupting RdRp complex assembly, but fail to recruit ubiquitination machinery for PB2 degradation. These data demonstrate that both the UBL domain (17-92aa) and PB2-binding region (124-186aa) are required for highly effective PB2 degradation and IAV restriction.</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>{
-"pmid": "38498560",
-"alias_symbol": "SCYTHE",
-"primary_gene_symbol": "BAG6",
-"name": "BAG cochaperone 6",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "NO",
-"evidence": ""
-}</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>HGNC:13919</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>ENSG00000234651, ENSG00000096155, ENSG00000233348, ENSG00000204463, ENSG00000228760, ENSG00000229524, ENSG00000227761</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>GENE ID:7917</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>BAG6</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>SCYTHE</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>38498560</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>alias</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>alias</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>intro</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>BAG6 (BCL2-associated athanogene 6, also known as BAT3 or Scythe) is a member of the BAG family due to a sequence homologous to the BAG domain at its C terminus and the collaboration with Heat Shock Protein 70 (Hsp70) family molecular chaperones</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>BAG cochaperone 6</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>(A) The predicted interaction domain of BAG6 and PB2. The protein structure of PB2 and BAG6 from AlphaFold2 database and the predicted interaction complex from ColabFold online software, showing that BAG6 124–186 amino acids is the key region for binding to the N-terminus of PB2 protein, which competitively prevents PB1-PB2 interaction. The N-terminus of BAG6 (residues 1–255, blue) and the N-terminus of PB2 (residues 1–247, green) from ColabFold online prediction, the interaction region of PB1 in complex with PB2 (residues 678–757, light red) from PDB:3A1G. (B) Schematic diagram illustrating the truncated and deleted mutants of BAG6 based on the predicted interaction domain. UBL: ubiquitin-like domain; PXXP: proline-rich region. (C) HEK293T cells transfected with the indicated plasmids were immunoprecipitated with M2/Flag antibody, followed by western blot analysis. (D and E) A549 cells were transfected with BAG6 1:255-HA or BAG6 1:92-HA or BAG6 92:255-HA or BAG6 del124:186-HA empty vector for 24 h, and then infected with IAV H1N1 (MOI = 1.0). The viral NP proteins were measured by western blotting (D), the viral titers in the supernatants were determined by TCID50assay (E). (F) HEK293T cells were co-transfected with pPolI-Luc reporter plasmid and expression plasmids containing viral PB1, PB2, PA, and NP of H1N1 along with BAG6 1:255-HA or different truncated mutants of BAG6 or empty vector. Renilla luciferase was used as an internal control. Luciferase activity of the viral polymerase was determined at 24 h post-transfection. Data presented as means ± SD and are representative of three independent experiments. *p&lt; 0.05, **p&lt; 0.01, ***p&lt; 0.001, Unpaired Student’s t test.
-IAVs are among the most common contagious pathogens to cause severe respiratory infections. Host cells have developed multiple strategies to defend against IAV infection. This study identified BAG6 as a novel intrinsic antiviral factor to negatively regulate the replication of multiple IAV subtypes, including human H1N1, H5N1 and avian H7N9, H9N2. BAG6 specifically interacts with the N-terminus of viral polymerase subunit protein PB2, competitively interrupts the assembly of functional RdRp complex and induces the ubiquitination degradation of PB2, which attenuate viral polymerase activity and IAV replication in mammalian cells and pathogenicity in mouse model (Fig 10). These findings reveal a new antagonism mechanism between pathogens and hosts, and highlight a potent antiviral activity of BAG6 by targeting the key viral protein PB2.
-During IAV infection, BAG6 directly interacts with the N-terminus of the IAV polymerase subunit PB2. The interaction between BAG6 and PB2 competes with PB1 for PB2 binding, which perturbs the formation of a functional RdRp complex, and further targets PB2 for K48-linked ubiquitination degradation, thereby inhibiting IAV replication (by Figdraw).
-PB2 protein of IAV is critical for RdRp complex to catalyze the viral transcription and replication, and acts as a key determinant for mammalian adaptation of avian influenza virus. PB2 is responsible for binding the polymerase complex to host cell RNA and initiating viral transcription. It contains a conserved N-terminal fragment that interacts with PB1 to form the polymerase complex, and a central cap-binding domain that recognizes the 5’ cap structure of host cell mRNA, allowing the polymerase to "steal" the cap and use it to prime viral transcription [34]. Besides, the C-terminal part of PB2 contains the so-called 627 domain (residues 535–684), which participates in host adaptation and virulence by influencing the binding of NLS to importins [46]. Multiple host proteins have been found to restrict IAV replication by targeting PB2. For instance, TRIM35 mediates the protection against influenza infection by activating TRAF3 and inducing K48-linked ubiquitination and degradation of PB2 [44]. PIAS restricts IAV replication and virulence through mediating PB2 SUMOylation and reducing its stability [47]. In addition, ANP32A inhibits IAV replication in mammalian cells through differential regulation of the activity of viral polymerases carrying PB2-627K (human) or PB2-627E (avian) signature [12,48]. Here, we found that BAG6 associated with PB2, thereby perturbing its interaction with PB1 and inducing its ubiquitination degradation. Notably, BAG6 recognizes the N-terminus of PB2 and promotes PB2 ubiquitination at its K189 residue, which is highly conserved among avian and human influenza strains from Global Initiative on Sharing Avian Influenza Data (GISAID,www.epicov.org) (S1 Table), providing the mechanistic basis that BAG6 acts as a potent antiviral factor during both human- and avian-origin IAV infection.
-BAG6 is a multifunctional protein in host cell and participates in a variety of physiological and pathological processes [19]. BAG6 functions as an essential factor in ubiquitin-mediated metabolism of neo-synthesized defective polypeptides and misfolded/mislocalized proteins [49–51]. It can capture these defective or mislocalized substrates by interacting with their unprocessed or non-inserted hydrophobic domains [45], and at the same time, recruit the E3 ligases, primarily RNF126, to its N-terminal UBL domain for efficient ubiquitination and degradation [40]. Besides, BAG6 is necessary for DNA damage-induced apoptosis by controlling the p53 signaling pathway [52]. It promotes p53 transactivation by stabilizing its interaction with the acetyltransferase p300 and enhancing p53 acetylation during apoptosis and autophagy [21,22,53]. A recent study reported that BAG6 was capable of regulating the activation of IFN-I by inhibiting RIG-I/VISA-mediated recognition of RNA ligand [29]. However, the role of BAG6 in virus infection remains opaque. In this study, we provide evidence that BAG6 can potently inhibit influenza virus replicationin vitroandin vivo. Further investigation found that the overexpression of BAG6 neither affected cell apoptosis during IAV infection (S4 Fig), nor relied on the IFN-I antiviral response to inhibit IAV replication (Fig 4), whereas BAG6 directly interacts with viral polymerase subunit PB2 and targets it for ubiquitination degradation. These findings reveal a novel mechanism by which BAG6 serves as an antiviral factor to specifically target viral protein through its protein quality control function.
-In the recent years, there has been increased interest in harnessing targeted protein degradation (TPD) technology in the development of antiviral therapies by inducing the degradation of either viral or host-related protein targets, but the off-target side effects and toxicity greatly limit its use [54–57]. In this study, we found the N-terminus of host protein BAG6 contains a ubiquitin-like domain (UBL, 17-92aa), which was previously reported to recruit E3 ligase RNF126 and ubiquitinates BAG6-associated clients [40], and a PB2-binding domain (124-186aa), which was proved to interact with viral polymerase subunit PB2 protein during IAV infection. Interestingly, although the BAG6:92-255aa mutant lacking the UBL domain weakened BAG6-meditated antiviral activity against IAV, it still significantly restricted viral polymerase activity and replication (Fig 9E and 9F). This mirrors the findings that BAG6 could suppress the viral polymerase activity by competing with PB1 for PB2 binding and interfering with RdRp assembly (Fig 6E and 6F), even in the situation with PB2 degradation resistance. These data indicate that both UBL and PB2-binding domains are essential for the efficient PB2 degradation and BAG6-mediated antiviral activity. This unique structure thus allows BAG6 naturally possessing a proteolysis-targeting function. By targeting viral PB2, BAG6 is more likely to become a potential candidate for antiviral drug development.
-The laboratory animal usage license number is SYXK-Beijing-2018-0038, certified by Beijing Association for Science and Technology. All animal research was performed in compliance with the Beijing Laboratory Animal Welfare and Ethics guidelines, as issued by the Beijing Administration Committee of Laboratory Animals, and the China Agricultural University (CAU) Institutional Animal Care and Use Committee guidelines (ID: SKLAB-B-2010-003) approved by the Animal Welfare Committee of CAU. All experiments with live viruses were performed in Biosafety Level II laboratory (BSL-2) in CAU. All animal research involved in this study was approved by the Animal Welfare Committee of CAU (No.AW03503202-2-2).
-Human lung adenocarcinoma epithelial cells (A549), HeLa cell, Madin-Darby canine kidney cells (MDCK), Vero cell and human embryonic kidney cells (HEK293T) were purchased from ATCC. IRF9-KO HeLa cells were generated as previous indicated [30,31]. BAG6 KO A549 cells and BAG6 KO HeLa cells were generated using CRISPR/Cas 9-based knockout of BAG6 gene. In brief, the BAG6 gene target sequences, #1 5’- CACCGCGGTACTGGTACTATCATT-3’ and #2 5’- CACCAGGCTCCTCCACAGCGGTAC-3’, were inserted into the guide RNA (gRNA) expression cassette of the pUC19 vector, which also contains an expression cassette of Cas9. The pUC19 plasmid containing the BAG6 target sequence was then transfected into A549 or HeLa cells. The transfected cells were trypsinized 24 h later into single cells, which were diluted and inoculated into a 96-well plate by infinite dilution. Each colony was individually propagated in a 96-well plate, and the knockout of BAG6 expression was confirmed by western blotting. Cells were cultured in DMEM supplemented with 10% v/v heat-inactivated fetal bovine serum (10099141C, Gibco, USA), 100 U mL−1penicillin and 100 μg mL−1streptomycin at 37°C in a 5% CO2atmosphere.
-Influenza A/Puerto Rico/8/1934 (PR8, H1N1, accession HA number:CY045764), A/chicken/China/0606-13/2017 (CN0606, H7N9, accession HA number:MK530478), and A/chicken/Shandong/196/2011 (SD196, H9N2, accession HA number:KR002651) and A/Anhui/1/2005 (AH1, H5N1, accession HA number:HM172104) viruses were maintained in the laboratory. All experiments using non-H5 live viruses were performed in the Biosafety Level II laboratory (BSL-2), and experiments using H5 viruses were performed in the Biosafety Level III Laboratory (BSL-3) in CAU.
-Protein expression plasmids BAG6-HA, BAG6 1:255-HA, BAG6 1:753-HA, BAG6 482:753-HA, BAG6 482:1126-HA, BAG6 642:1126-HA, PB2-Flag, N-terminal PB2-Flag, PB1-Flag, PA-Flag, NP-Flag, M1-Flag, PB2-K5R-Flag, PB2-K33R-Flag, PB2-K41R-Flag, PB2-K48R-Flag, PB2-K61R-Flag, PB2-K187R-Flag, PB2-K189R-Flag, PB2-K331R-Flag, PB2-K339R-Flag, PB2-K353R-Flag, PB2-K482R-Flag, PB2-K561R-Flag, PB2-K617R-Flag, PB2-K699R-Flag, PB2-K721R-Flag, PB2-K736R-Flag, PB2-K738R-Flag, PB2-K752R-Flag, Ub-HA, K48-Ub-HA and K63-Ub-HA were generated by subcloning the corresponding coding segment into the HA-pRK5 or Flag-pRK5 empty vector by homologous recombinase-mediated recombination (S1 Table). Plasmid transfections in HEK293T or A549 cells were performed using jetPRIME (101000046, Polyplus, France).
-Antibody concentrations for immunoprecipitation and immunoblotting were determined empirically. All immunoblot antibodies were diluted as specified in 5% w/v BSA-TBST. Antibodies used as follows: anti-BAG6 (B01P, Abnova, Taiwan, China), anti-PB2 (PA5-32220, Thermo Scientific, Massachusetts, USA), anti-PB1 (PA5-34914, Thermo Scientific, Massachusetts, USA), anti-β-actin (A1978, Sigma, Shanghai, China), anti-GAPDH (ab8245, Abcam, Shanghai, China), anti-PARP (9542, Cell Signaling Technology, Massachusetts, USA), anti-Flag (F1804, Sigma, Shanghai, China and 20543-1-AP, Proteintech, Chicago, USA), anti-HA (H9658, Sigma, Shanghai, China and 51064-2-AP, Proteintech, Chicago, USA), anti-RIG-I (20566-1-AP, Proteintech, Chicago, USA), anti-p-STAT1 (9167, Cell Signaling Technology, Massachusetts, USA), anti-ISG15 (sc166755, Santa Cruz, California, USA), anti-influenza A virus NP (A01506-40, GenScript, New Jersey, USA), Mouse monoclonal anti-influenza A virus M1 antibody (Lab Homemade, Beijing, China, ZL201910912806.0). Cycloheximide (CHX, HY-12320), MG132 (HY-13259C) and Chloroquine (CQ, HY-17589A) was purchased from MCE.
-A dual-luciferase reporter assay system (E1960, Promega, Wisconsin, USA) was used to compare the polymerase activities of different viral RNP complexes. PB2, PB1, PA, and NP gene segments of the indicated viruses (PR8, CN0606 and SD196) were separately cloned into the pCDNA3.1 expression plasmid. PB2, PB1, PA, and NP plasmids (125 ng each plasmid) along with the pLuci luciferase reporter plasmid (10 ng) and the renilla internal control plasmid (2.5 ng) were used to transfect cells. Cell cultures were incubated at 37°C. Cell lysates were analyzed at 24 h post-transfection for firefly and renilla luciferase activities using a GloMax 96 microplate luminometer (GM2000, Promega, Wisconsin, USA). Polymerase proteins were detected by Western blotting.
-Six-week-old BALB/c background female mice were purchased from Beijing Vital River Co. Ltd. (Beijing, China). Animal studies were carried out in specific pathogen-free barrier facilities. Facilities were maintained at an acceptable range of 20–26°C humidity of 30–70% on a 12-h dark/12-h light cycle. Peptide-conjugated PPMO were purchased from Gene Tools (USA). PPMO targeting mouse BAG6 gene (PPMO-BAG6) was designed as CTGGCACTATCACTCGGCTCCATG. A nontargeting PPMO control sequence (PPMO-NC) (CCTCTTACCTCAGTTACAATTTATA), was used as control. Six to eight weeks BALB/c female mice were inoculated intranasally with 100 μg of PPMOs in 50 μL PBS for 2 days continuously.
-Mice were anesthetized and intranasally inoculated with PR8 virus at a median tissue culture infectious dose (TCID50) of 100 in 50 μL of PBS. Body weight and survival were monitored daily for 14 days. Lung tissue lysates were generated by homogenizing snap-frozen lung tissues twice (20 s each time) in MEM medium and centrifuging the lung suspensions at 2000 rpm for 15 min. TCID50assays were performed using MDCK cells and TCID50was calculated as previously described [58]. A portion of the lung from each euthanized mouse at 3 and 5 dpi was fixed in 10% phosphate-buffered formalin, embedded in paraffin, sectioned and stained with hematoxylin and eosin (H&amp;E). Immunohistochemical staining of viral antigen was performed as described previously [59].
-Total RNA from cells was extracted using an RNA isolation kit (Thermo Scientific, Massachusetts, USA). First-strand complementary DNA was synthesized from 1 μg of total RNA using a TransScript RT reagent kit (TransGen, Beijing, China), and oligo dT primer were used for detecting host genes. For the detection of influenza virus mRNA and vRNA, oligo dT primer and uni-12 primer (5′-AGCAAAAGCAGG-3′) [60] were respectively used to generate cDNAs. Generated cDNA was subjected to qPCR in a 25 μL reaction volume using 2X M5 HiPer SYBR Premix EsTaq (with Tli RNaseH) (Mei5bio) (S1 Table). Human β-actin genes were amplified for normalization of the cDNA amount used in qPCR. Reactions were conducted in triplicate, and the data were analyzed using the 2−ΔΔCtmethod.
-Cells were lysed in lysis buffer (50 mM Tris-Cl at pH 8.0, 150 mM NaCl, 1% Tri-ton X-100, 1 mM DTT, 1× complete protease inhibitor cocktail, and 10% glycerol) and pre-cleared with Protein A/G PLUS-Agarose beads (sc-2003, Santa Cruz Biotechnology, USA) for 2 h at 4°C. The lysates were then immunoprecipitated with indicated antibodies or isotype-matched control antibodies plus protein G Sepharose beads at 4°C for 2–4 h. The beads were then washed three times and boiled. Protein samples were analyzed by Western blotting. For Western blotting, protein samples were mixed with 6× loading buffer supplemented with 10% β-mercaptoethanol, heated at 100°C for 5 min and separated on a 10% SDS-PAGE under reducing conditions. After electrophoresis, protein samples were electroblotted onto polyvinylidene difluoride membranes (Bio-Rad, CA, USA) and blocked for 2 h in Tris-buffered saline (10 mM Tris-HCl, pH 8.0, containing 150 mM NaCl) containing 5% (w/v) non-fat dry milk and 0.5‰ (v/v) Tween-20. The blots were incubated with the primary antibodies overnight at 4°C. The next day, the blots were incubated with corresponding horseradish peroxidase (HRP)-conjugated secondary antibodies for 1 h at room temperature (RT). HRP antibody binding was detected using a standard enhanced chemiluminescence (ECL) kit (wbluf0500, Millipore, USA).
-HEK293T cell lines were cotransfected with PB2-Flag plasmid with empty vector or BAG6-HA plasmid. After 24 h post-transfection, CHX (50 μg/mL) was added to the medium and cells were harvested at different time points. Western blotting of cell lysates was performed to detect PB2-Flag, BAG6-HA and β-actin. To investigate the cellular pathway of BAG6-mediated PB2 degradation, at 24 h post-transfection, or infection with PR8 (H1N1), MG132 (20 μM) or CQ (150 μM) was added to the medium, and the cells were harvested 6 h after treatment. Three independent experiments were performed.
-HEK293T cells were transfected with HA-tagged ubiquitin (Ub-HA) plasmids, BAG6-HA or empty plasmids, and PB2-Flag or PB2-Flag with Lysine mutations. At 24 h post-transfection, the cells were treated with MG132 (20 μM) for 6 h and then lysed in 1% SDS lysis buffer. After being boiled for 10 min, the lysates were diluted 10 times with cold lysis buffer supplemented with 1× complete protease inhibitor cocktail, 10 mM DTT, and 10 mM NEM. PB2-Flag protein was then purified with anti-Flag antibody and subjected to western blotting analysis. Ubiquitinated PB2-Flag was detected by anti-HA antibody.
-We downloaded all available PB2 amino acid sequences of human and avian origin for influenza viruses of subtypes H1, H3, H5, H7, and H9 from the Global Initiative on Sharing Avian Influenza Data (GISAID,www.epicov.org) (date of access: Jan. 22, 2024), and multiple sequence alignment was performed using MAFFT v7.0 [61], and then the amino acid categories and percentages of the 189 amino acid residues were counted.
-Cells on coverslips were washed twice with prewarmed PBS and fixed with 4% paraformaldehyde for 15 min at room temperature. Cells were subsequently permeabilized with immunostaining permeabilization buffer containing Triton X-100 (P0096, Beyotime, Shanghai, China) for 10 min and blocked with QuickBlock blocking buffer (P0220, Beyotime, Shanghai, China) for 20 min at room temperature. Fixed cells were incubated with indicated antibodies diluted in immunostaining primary antibody dilution buffer at 4°C overnight. Coverslips were then washed three times with PBS and incubated with Alexa Fluor 488-conjugated secondary antibodies or Alexa Fluor 555-conjugated secondary antibodies for 1 h at 37°C. Coverslips were finally washed three times and mounted onto microscope slides with DAPI staining solution (C1006, Beyotime, Shanghai, China) for 8 min and examined by confocal microscopy. Immunoassayed cells were visualized using a Nikon super-resolution laser scanning confocal microscope under a 100-time oil objective and analyzed using the Imaris 9.2 platform.
-An online software, ColabFold, was used for the prediction of protein structures and complexes by combining the fast homology search of MMseqs2 with AlphaFold2 or RoseTTAFold. Sequence alignments/templates are generated through MMseqs2 and HHsearch [62]. The amino acid sequences of BAG6 protein N-terminal 1-255aa and PB2 protein N-terminal 1-247aa were used for the prediction of protein complex at the open-source website ColabFold v1.5.2 (https://colab.research.google.com/github/sokrypton/ColabFold/blob/main/AlphaFold2.ipynb#scrollTo=mbaIO9pWjaN0), and the predicted results were viewed and analyzed using PyMOL v2.5.0.
-WT A549 and BAG6-KO A549 cells or WT HeLa and BAG6-KO HeLa cells were plated in 96-well plates at a density of 2000 cells in 100 μL of medium per well. The cell viability was then assayed according to the CCK8 kit instructions (C0042, Beyotime, Shanghai, China).</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>The interaction between influenza A virus (IAV) and host proteins is an important process that greatly influences viral replication and pathogenicity. PB2 protein is a subunit of viral ribonucleoprotein (vRNP) complex playing distinct roles in viral transcription and replication. BAG6 (BCL2-associated athanogene 6) as a multifunctional host protein participates in physiological and pathological processes. Here, we identify BAG6 as a new restriction factor for IAV replication through targeting PB2. For both avian and human influenza viruses, overexpression of BAG6 reduced viral protein expression and virus titers, whereas deletion of BAG6 significantly enhanced virus replication. Moreover, BAG6-knockdown mice developed more severe clinical symptoms and higher viral loads upon IAV infection. Mechanistically, BAG6 restricted IAV transcription and replication by inhibiting the activity of viral RNA-dependent RNA polymerase (RdRp). The co-immunoprecipitation assays showed BAG6 specifically interacted with the N-terminus of PB2 and competed with PB1 for RdRp complex assembly. The ubiquitination assay indicated that BAG6 promoted PB2 ubiquitination at K189 residue and targeted PB2 for K48-linked ubiquitination degradation. The antiviral effect of BAG6 necessitated its N-terminal region containing a ubiquitin-like (UBL) domain (17-92aa) and a PB2-binding domain (124-186aa), which are synergistically responsible for viral polymerase subunit PB2 degradation and perturbing RdRp complex assembly. These findings unravel a novel antiviral mechanism via the interaction of viral PB2 and host protein BAG6 during avian or human influenza virus infection and highlight a potential application of BAG6 for antiviral drug development.</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>PMID: 38498560
-Full Text: (A) The predicted interaction domain of BAG6 and PB2. The protein structure of PB2 and BAG6 from AlphaFold2 database and the predicted interaction complex from ColabFold online software, showing that BAG6 124–186 amino acids is the key region for binding to the N-terminus of PB2 protein, which competitively prevents PB1-PB2 interaction. The N-terminus of BAG6 (residues 1–255, blue) and the N-terminus of PB2 (residues 1–247, green) from ColabFold online prediction, the interaction region of PB1 in complex with PB2 (residues 678–757, light red) from PDB:3A1G. (B) Schematic diagram illustrating the truncated and deleted mutants of BAG6 based on the predicted interaction domain. UBL: ubiquitin-like domain; PXXP: proline-rich region. (C) HEK293T cells transfected with the indicated plasmids were immunoprecipitated with M2/Flag antibody, followed by western blot analysis. (D and E) A549 cells were transfected with BAG6 1:255-HA or BAG6 1:92-HA or BAG6 92:255-HA or BAG6 del124:186-HA empty vector for 24 h, and then infected with IAV H1N1 (MOI = 1.0). The viral NP proteins were measured by western blotting (D), the viral titers in the supernatants were determined by TCID50assay (E). (F) HEK293T cells were co-transfected with pPolI-Luc reporter plasmid and expression plasmids containing viral PB1, PB2, PA, and NP of H1N1 along with BAG6 1:255-HA or different truncated mutants of BAG6 or empty vector. Renilla luciferase was used as an internal control. Luciferase activity of the viral polymerase was determined at 24 h post-transfection. Data presented as means ± SD and are representative of three independent experiments. *p&lt; 0.05, **p&lt; 0.01, ***p&lt; 0.001, Unpaired Student’s t test.
-IAVs are among the most common contagious pathogens to cause severe respiratory infections. Host cells have developed multiple strategies to defend against IAV infection. This study identified BAG6 as a novel intrinsic antiviral factor to negatively regulate the replication of multiple IAV subtypes, including human H1N1, H5N1 and avian H7N9, H9N2. BAG6 specifically interacts with the N-terminus of viral polymerase subunit protein PB2, competitively interrupts the assembly of functional RdRp complex and induces the ubiquitination degradation of PB2, which attenuate viral polymerase activity and IAV replication in mammalian cells and pathogenicity in mouse model (Fig 10). These findings reveal a new antagonism mechanism between pathogens and hosts, and highlight a potent antiviral activity of BAG6 by targeting the key viral protein PB2.
-During IAV infection, BAG6 directly interacts with the N-terminus of the IAV polymerase subunit PB2. The interaction between BAG6 and PB2 competes with PB1 for PB2 binding, which perturbs the formation of a functional RdRp complex, and further targets PB2 for K48-linked ubiquitination degradation, thereby inhibiting IAV replication (by Figdraw).
-PB2 protein of IAV is critical for RdRp complex to catalyze the viral transcription and replication, and acts as a key determinant for mammalian adaptation of avian influenza virus. PB2 is responsible for binding the polymerase complex to host cell RNA and initiating viral transcription. It contains a conserved N-terminal fragment that interacts with PB1 to form the polymerase complex, and a central cap-binding domain that recognizes the 5’ cap structure of host cell mRNA, allowing the polymerase to "steal" the cap and use it to prime viral transcription [34]. Besides, the C-terminal part of PB2 contains the so-called 627 domain (residues 535–684), which participates in host adaptation and virulence by influencing the binding of NLS to importins [46]. Multiple host proteins have been found to restrict IAV replication by targeting PB2. For instance, TRIM35 mediates the protection against influenza infection by activating TRAF3 and inducing K48-linked ubiquitination and degradation of PB2 [44]. PIAS restricts IAV replication and virulence through mediating PB2 SUMOylation and reducing its stability [47]. In addition, ANP32A inhibits IAV replication in mammalian cells through differential regulation of the activity of viral polymerases carrying PB2-627K (human) or PB2-627E (avian) signature [12,48]. Here, we found that BAG6 associated with PB2, thereby perturbing its interaction with PB1 and inducing its ubiquitination degradation. Notably, BAG6 recognizes the N-terminus of PB2 and promotes PB2 ubiquitination at its K189 residue, which is highly conserved among avian and human influenza strains from Global Initiative on Sharing Avian Influenza Data (GISAID,www.epicov.org) (S1 Table), providing the mechanistic basis that BAG6 acts as a potent antiviral factor during both human- and avian-origin IAV infection.
-BAG6 is a multifunctional protein in host cell and participates in a variety of physiological and pathological processes [19]. BAG6 functions as an essential factor in ubiquitin-mediated metabolism of neo-synthesized defective polypeptides and misfolded/mislocalized proteins [49–51]. It can capture these defective or mislocalized substrates by interacting with their unprocessed or non-inserted hydrophobic domains [45], and at the same time, recruit the E3 ligases, primarily RNF126, to its N-terminal UBL domain for efficient ubiquitination and degradation [40]. Besides, BAG6 is necessary for DNA damage-induced apoptosis by controlling the p53 signaling pathway [52]. It promotes p53 transactivation by stabilizing its interaction with the acetyltransferase p300 and enhancing p53 acetylation during apoptosis and autophagy [21,22,53]. A recent study reported that BAG6 was capable of regulating the activation of IFN-I by inhibiting RIG-I/VISA-mediated recognition of RNA ligand [29]. However, the role of BAG6 in virus infection remains opaque. In this study, we provide evidence that BAG6 can potently inhibit influenza virus replicationin vitroandin vivo. Further investigation found that the overexpression of BAG6 neither affected cell apoptosis during IAV infection (S4 Fig), nor relied on the IFN-I antiviral response to inhibit IAV replication (Fig 4), whereas BAG6 directly interacts with viral polymerase subunit PB2 and targets it for ubiquitination degradation. These findings reveal a novel mechanism by which BAG6 serves as an antiviral factor to specifically target viral protein through its protein quality control function.
-In the recent years, there has been increased interest in harnessing targeted protein degradation (TPD) technology in the development of antiviral therapies by inducing the degradation of either viral or host-related protein targets, but the off-target side effects and toxicity greatly limit its use [54–57]. In this study, we found the N-terminus of host protein BAG6 contains a ubiquitin-like domain (UBL, 17-92aa), which was previously reported to recruit E3 ligase RNF126 and ubiquitinates BAG6-associated clients [40], and a PB2-binding domain (124-186aa), which was proved to interact with viral polymerase subunit PB2 protein during IAV infection. Interestingly, although the BAG6:92-255aa mutant lacking the UBL domain weakened BAG6-meditated antiviral activity against IAV, it still significantly restricted viral polymerase activity and replication (Fig 9E and 9F). This mirrors the findings that BAG6 could suppress the viral polymerase activity by competing with PB1 for PB2 binding and interfering with RdRp assembly (Fig 6E and 6F), even in the situation with PB2 degradation resistance. These data indicate that both UBL and PB2-binding domains are essential for the efficient PB2 degradation and BAG6-mediated antiviral activity. This unique structure thus allows BAG6 naturally possessing a proteolysis-targeting function. By targeting viral PB2, BAG6 is more likely to become a potential candidate for antiviral drug development.
-The laboratory animal usage license number is SYXK-Beijing-2018-0038, certified by Beijing Association for Science and Technology. All animal research was performed in compliance with the Beijing Laboratory Animal Welfare and Ethics guidelines, as issued by the Beijing Administration Committee of Laboratory Animals, and the China Agricultural University (CAU) Institutional Animal Care and Use Committee guidelines (ID: SKLAB-B-2010-003) approved by the Animal Welfare Committee of CAU. All experiments with live viruses were performed in Biosafety Level II laboratory (BSL-2) in CAU. All animal research involved in this study was approved by the Animal Welfare Committee of CAU (No.AW03503202-2-2).
-Human lung adenocarcinoma epithelial cells (A549), HeLa cell, Madin-Darby canine kidney cells (MDCK), Vero cell and human embryonic kidney cells (HEK293T) were purchased from ATCC. IRF9-KO HeLa cells were generated as previous indicated [30,31]. BAG6 KO A549 cells and BAG6 KO HeLa cells were generated using CRISPR/Cas 9-based knockout of BAG6 gene. In brief, the BAG6 gene target sequences, #1 5’- CACCGCGGTACTGGTACTATCATT-3’ and #2 5’- CACCAGGCTCCTCCACAGCGGTAC-3’, were inserted into the guide RNA (gRNA) expression cassette of the pUC19 vector, which also contains an expression cassette of Cas9. The pUC19 plasmid containing the BAG6 target sequence was then transfected into A549 or HeLa cells. The transfected cells were trypsinized 24 h later into single cells, which were diluted and inoculated into a 96-well plate by infinite dilution. Each colony was individually propagated in a 96-well plate, and the knockout of BAG6 expression was confirmed by western blotting. Cells were cultured in DMEM supplemented with 10% v/v heat-inactivated fetal bovine serum (10099141C, Gibco, USA), 100 U mL−1penicillin and 100 μg mL−1streptomycin at 37°C in a 5% CO2atmosphere.
-Influenza A/Puerto Rico/8/1934 (PR8, H1N1, accession HA number:CY045764), A/chicken/China/0606-13/2017 (CN0606, H7N9, accession HA number:MK530478), and A/chicken/Shandong/196/2011 (SD196, H9N2, accession HA number:KR002651) and A/Anhui/1/2005 (AH1, H5N1, accession HA number:HM172104) viruses were maintained in the laboratory. All experiments using non-H5 live viruses were performed in the Biosafety Level II laboratory (BSL-2), and experiments using H5 viruses were performed in the Biosafety Level III Laboratory (BSL-3) in CAU.
-Protein expression plasmids BAG6-HA, BAG6 1:255-HA, BAG6 1:753-HA, BAG6 482:753-HA, BAG6 482:1126-HA, BAG6 642:1126-HA, PB2-Flag, N-terminal PB2-Flag, PB1-Flag, PA-Flag, NP-Flag, M1-Flag, PB2-K5R-Flag, PB2-K33R-Flag, PB2-K41R-Flag, PB2-K48R-Flag, PB2-K61R-Flag, PB2-K187R-Flag, PB2-K189R-Flag, PB2-K331R-Flag, PB2-K339R-Flag, PB2-K353R-Flag, PB2-K482R-Flag, PB2-K561R-Flag, PB2-K617R-Flag, PB2-K699R-Flag, PB2-K721R-Flag, PB2-K736R-Flag, PB2-K738R-Flag, PB2-K752R-Flag, Ub-HA, K48-Ub-HA and K63-Ub-HA were generated by subcloning the corresponding coding segment into the HA-pRK5 or Flag-pRK5 empty vector by homologous recombinase-mediated recombination (S1 Table). Plasmid transfections in HEK293T or A549 cells were performed using jetPRIME (101000046, Polyplus, France).
-Antibody concentrations for immunoprecipitation and immunoblotting were determined empirically. All immunoblot antibodies were diluted as specified in 5% w/v BSA-TBST. Antibodies used as follows: anti-BAG6 (B01P, Abnova, Taiwan, China), anti-PB2 (PA5-32220, Thermo Scientific, Massachusetts, USA), anti-PB1 (PA5-34914, Thermo Scientific, Massachusetts, USA), anti-β-actin (A1978, Sigma, Shanghai, China), anti-GAPDH (ab8245, Abcam, Shanghai, China), anti-PARP (9542, Cell Signaling Technology, Massachusetts, USA), anti-Flag (F1804, Sigma, Shanghai, China and 20543-1-AP, Proteintech, Chicago, USA), anti-HA (H9658, Sigma, Shanghai, China and 51064-2-AP, Proteintech, Chicago, USA), anti-RIG-I (20566-1-AP, Proteintech, Chicago, USA), anti-p-STAT1 (9167, Cell Signaling Technology, Massachusetts, USA), anti-ISG15 (sc166755, Santa Cruz, California, USA), anti-influenza A virus NP (A01506-40, GenScript, New Jersey, USA), Mouse monoclonal anti-influenza A virus M1 antibody (Lab Homemade, Beijing, China, ZL201910912806.0). Cycloheximide (CHX, HY-12320), MG132 (HY-13259C) and Chloroquine (CQ, HY-17589A) was purchased from MCE.
-A dual-luciferase reporter assay system (E1960, Promega, Wisconsin, USA) was used to compare the polymerase activities of different viral RNP complexes. PB2, PB1, PA, and NP gene segments of the indicated viruses (PR8, CN0606 and SD196) were separately cloned into the pCDNA3.1 expression plasmid. PB2, PB1, PA, and NP plasmids (125 ng each plasmid) along with the pLuci luciferase reporter plasmid (10 ng) and the renilla internal control plasmid (2.5 ng) were used to transfect cells. Cell cultures were incubated at 37°C. Cell lysates were analyzed at 24 h post-transfection for firefly and renilla luciferase activities using a GloMax 96 microplate luminometer (GM2000, Promega, Wisconsin, USA). Polymerase proteins were detected by Western blotting.
-Six-week-old BALB/c background female mice were purchased from Beijing Vital River Co. Ltd. (Beijing, China). Animal studies were carried out in specific pathogen-free barrier facilities. Facilities were maintained at an acceptable range of 20–26°C humidity of 30–70% on a 12-h dark/12-h light cycle. Peptide-conjugated PPMO were purchased from Gene Tools (USA). PPMO targeting mouse BAG6 gene (PPMO-BAG6) was designed as CTGGCACTATCACTCGGCTCCATG. A nontargeting PPMO control sequence (PPMO-NC) (CCTCTTACCTCAGTTACAATTTATA), was used as control. Six to eight weeks BALB/c female mice were inoculated intranasally with 100 μg of PPMOs in 50 μL PBS for 2 days continuously.
-Mice were anesthetized and intranasally inoculated with PR8 virus at a median tissue culture infectious dose (TCID50) of 100 in 50 μL of PBS. Body weight and survival were monitored daily for 14 days. Lung tissue lysates were generated by homogenizing snap-frozen lung tissues twice (20 s each time) in MEM medium and centrifuging the lung suspensions at 2000 rpm for 15 min. TCID50assays were performed using MDCK cells and TCID50was calculated as previously described [58]. A portion of the lung from each euthanized mouse at 3 and 5 dpi was fixed in 10% phosphate-buffered formalin, embedded in paraffin, sectioned and stained with hematoxylin and eosin (H&amp;E). Immunohistochemical staining of viral antigen was performed as described previously [59].
-Total RNA from cells was extracted using an RNA isolation kit (Thermo Scientific, Massachusetts, USA). First-strand complementary DNA was synthesized from 1 μg of total RNA using a TransScript RT reagent kit (TransGen, Beijing, China), and oligo dT primer were used for detecting host genes. For the detection of influenza virus mRNA and vRNA, oligo dT primer and uni-12 primer (5′-AGCAAAAGCAGG-3′) [60] were respectively used to generate cDNAs. Generated cDNA was subjected to qPCR in a 25 μL reaction volume using 2X M5 HiPer SYBR Premix EsTaq (with Tli RNaseH) (Mei5bio) (S1 Table). Human β-actin genes were amplified for normalization of the cDNA amount used in qPCR. Reactions were conducted in triplicate, and the data were analyzed using the 2−ΔΔCtmethod.
-Cells were lysed in lysis buffer (50 mM Tris-Cl at pH 8.0, 150 mM NaCl, 1% Tri-ton X-100, 1 mM DTT, 1× complete protease inhibitor cocktail, and 10% glycerol) and pre-cleared with Protein A/G PLUS-Agarose beads (sc-2003, Santa Cruz Biotechnology, USA) for 2 h at 4°C. The lysates were then immunoprecipitated with indicated antibodies or isotype-matched control antibodies plus protein G Sepharose beads at 4°C for 2–4 h. The beads were then washed three times and boiled. Protein samples were analyzed by Western blotting. For Western blotting, protein samples were mixed with 6× loading buffer supplemented with 10% β-mercaptoethanol, heated at 100°C for 5 min and separated on a 10% SDS-PAGE under reducing conditions. After electrophoresis, protein samples were electroblotted onto polyvinylidene difluoride membranes (Bio-Rad, CA, USA) and blocked for 2 h in Tris-buffered saline (10 mM Tris-HCl, pH 8.0, containing 150 mM NaCl) containing 5% (w/v) non-fat dry milk and 0.5‰ (v/v) Tween-20. The blots were incubated with the primary antibodies overnight at 4°C. The next day, the blots were incubated with corresponding horseradish peroxidase (HRP)-conjugated secondary antibodies for 1 h at room temperature (RT). HRP antibody binding was detected using a standard enhanced chemiluminescence (ECL) kit (wbluf0500, Millipore, USA).
-HEK293T cell lines were cotransfected with PB2-Flag plasmid with empty vector or BAG6-HA plasmid. After 24 h post-transfection, CHX (50 μg/mL) was added to the medium and cells were harvested at different time points. Western blotting of cell lysates was performed to detect PB2-Flag, BAG6-HA and β-actin. To investigate the cellular pathway of BAG6-mediated PB2 degradation, at 24 h post-transfection, or infection with PR8 (H1N1), MG132 (20 μM) or CQ (150 μM) was added to the medium, and the cells were harvested 6 h after treatment. Three independent experiments were performed.
-HEK293T cells were transfected with HA-tagged ubiquitin (Ub-HA) plasmids, BAG6-HA or empty plasmids, and PB2-Flag or PB2-Flag with Lysine mutations. At 24 h post-transfection, the cells were treated with MG132 (20 μM) for 6 h and then lysed in 1% SDS lysis buffer. After being boiled for 10 min, the lysates were diluted 10 times with cold lysis buffer supplemented with 1× complete protease inhibitor cocktail, 10 mM DTT, and 10 mM NEM. PB2-Flag protein was then purified with anti-Flag antibody and subjected to western blotting analysis. Ubiquitinated PB2-Flag was detected by anti-HA antibody.
-We downloaded all available PB2 amino acid sequences of human and avian origin for influenza viruses of subtypes H1, H3, H5, H7, and H9 from the Global Initiative on Sharing Avian Influenza Data (GISAID,www.epicov.org) (date of access: Jan. 22, 2024), and multiple sequence alignment was performed using MAFFT v7.0 [61], and then the amino acid categories and percentages of the 189 amino acid residues were counted.
-Cells on coverslips were washed twice with prewarmed PBS and fixed with 4% paraformaldehyde for 15 min at room temperature. Cells were subsequently permeabilized with immunostaining permeabilization buffer containing Triton X-100 (P0096, Beyotime, Shanghai, China) for 10 min and blocked with QuickBlock blocking buffer (P0220, Beyotime, Shanghai, China) for 20 min at room temperature. Fixed cells were incubated with indicated antibodies diluted in immunostaining primary antibody dilution buffer at 4°C overnight. Coverslips were then washed three times with PBS and incubated with Alexa Fluor 488-conjugated secondary antibodies or Alexa Fluor 555-conjugated secondary antibodies for 1 h at 37°C. Coverslips were finally washed three times and mounted onto microscope slides with DAPI staining solution (C1006, Beyotime, Shanghai, China) for 8 min and examined by confocal microscopy. Immunoassayed cells were visualized using a Nikon super-resolution laser scanning confocal microscope under a 100-time oil objective and analyzed using the Imaris 9.2 platform.
-An online software, ColabFold, was used for the prediction of protein structures and complexes by combining the fast homology search of MMseqs2 with AlphaFold2 or RoseTTAFold. Sequence alignments/templates are generated through MMseqs2 and HHsearch [62]. The amino acid sequences of BAG6 protein N-terminal 1-255aa and PB2 protein N-terminal 1-247aa were used for the prediction of protein complex at the open-source website ColabFold v1.5.2 (https://colab.research.google.com/github/sokrypton/ColabFold/blob/main/AlphaFold2.ipynb#scrollTo=mbaIO9pWjaN0), and the predicted results were viewed and analyzed using PyMOL v2.5.0.
-WT A549 and BAG6-KO A549 cells or WT HeLa and BAG6-KO HeLa cells were plated in 96-well plates at a density of 2000 cells in 100 μL of medium per well. The cell viability was then assayed according to the CCK8 kit instructions (C0042, Beyotime, Shanghai, China).</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
-    Inputs:
-    Alias gene symbol: SCYTHE
-    HGNC record ID: HGNC:13919
-    Primary gene symbol: BAG6
-    Official HGNC gene name: BAG cochaperone 6
-    Biomedical text context (may include PMID)
-    Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
-    Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
-    If the text does not support that the alias is an alternate abbreviation, return:
-    "alternate_abbreviation": "NO"
-    "evidence": ""
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
-    Evidence must be one exact sentence copied verbatim from the text.
-    Do not infer relationships or paraphrase evidence.
-    Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
-    {
-    "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
-    "alternate_abbreviation": "YES or NO",
-    "evidence": ""
-    }
-PMID: 38498560
-Full Text: (A) The predicted interaction domain of BAG6 and PB2. The protein structure of PB2 and BAG6 from AlphaFold2 database and the predicted interaction complex from ColabFold online software, showing that BAG6 124–186 amino acids is the key region for binding to the N-terminus of PB2 protein, which competitively prevents PB1-PB2 interaction. The N-terminus of BAG6 (residues 1–255, blue) and the N-terminus of PB2 (residues 1–247, green) from ColabFold online prediction, the interaction region of PB1 in complex with PB2 (residues 678–757, light red) from PDB:3A1G. (B) Schematic diagram illustrating the truncated and deleted mutants of BAG6 based on the predicted interaction domain. UBL: ubiquitin-like domain; PXXP: proline-rich region. (C) HEK293T cells transfected with the indicated plasmids were immunoprecipitated with M2/Flag antibody, followed by western blot analysis. (D and E) A549 cells were transfected with BAG6 1:255-HA or BAG6 1:92-HA or BAG6 92:255-HA or BAG6 del124:186-HA empty vector for 24 h, and then infected with IAV H1N1 (MOI = 1.0). The viral NP proteins were measured by western blotting (D), the viral titers in the supernatants were determined by TCID50assay (E). (F) HEK293T cells were co-transfected with pPolI-Luc reporter plasmid and expression plasmids containing viral PB1, PB2, PA, and NP of H1N1 along with BAG6 1:255-HA or different truncated mutants of BAG6 or empty vector. Renilla luciferase was used as an internal control. Luciferase activity of the viral polymerase was determined at 24 h post-transfection. Data presented as means ± SD and are representative of three independent experiments. *p&lt; 0.05, **p&lt; 0.01, ***p&lt; 0.001, Unpaired Student’s t test.
-IAVs are among the most common contagious pathogens to cause severe respiratory infections. Host cells have developed multiple strategies to defend against IAV infection. This study identified BAG6 as a novel intrinsic antiviral factor to negatively regulate the replication of multiple IAV subtypes, including human H1N1, H5N1 and avian H7N9, H9N2. BAG6 specifically interacts with the N-terminus of viral polymerase subunit protein PB2, competitively interrupts the assembly of functional RdRp complex and induces the ubiquitination degradation of PB2, which attenuate viral polymerase activity and IAV replication in mammalian cells and pathogenicity in mouse model (Fig 10). These findings reveal a new antagonism mechanism between pathogens and hosts, and highlight a potent antiviral activity of BAG6 by targeting the key viral protein PB2.
-During IAV infection, BAG6 directly interacts with the N-terminus of the IAV polymerase subunit PB2. The interaction between BAG6 and PB2 competes with PB1 for PB2 binding, which perturbs the formation of a functional RdRp complex, and further targets PB2 for K48-linked ubiquitination degradation, thereby inhibiting IAV replication (by Figdraw).
-PB2 protein of IAV is critical for RdRp complex to catalyze the viral transcription and replication, and acts as a key determinant for mammalian adaptation of avian influenza virus. PB2 is responsible for binding the polymerase complex to host cell RNA and initiating viral transcription. It contains a conserved N-terminal fragment that interacts with PB1 to form the polymerase complex, and a central cap-binding domain that recognizes the 5’ cap structure of host cell mRNA, allowing the polymerase to "steal" the cap and use it to prime viral transcription [34]. Besides, the C-terminal part of PB2 contains the so-called 627 domain (residues 535–684), which participates in host adaptation and virulence by influencing the binding of NLS to importins [46]. Multiple host proteins have been found to restrict IAV replication by targeting PB2. For instance, TRIM35 mediates the protection against influenza infection by activating TRAF3 and inducing K48-linked ubiquitination and degradation of PB2 [44]. PIAS restricts IAV replication and virulence through mediating PB2 SUMOylation and reducing its stability [47]. In addition, ANP32A inhibits IAV replication in mammalian cells through differential regulation of the activity of viral polymerases carrying PB2-627K (human) or PB2-627E (avian) signature [12,48]. Here, we found that BAG6 associated with PB2, thereby perturbing its interaction with PB1 and inducing its ubiquitination degradation. Notably, BAG6 recognizes the N-terminus of PB2 and promotes PB2 ubiquitination at its K189 residue, which is highly conserved among avian and human influenza strains from Global Initiative on Sharing Avian Influenza Data (GISAID,www.epicov.org) (S1 Table), providing the mechanistic basis that BAG6 acts as a potent antiviral factor during both human- and avian-origin IAV infection.
-BAG6 is a multifunctional protein in host cell and participates in a variety of physiological and pathological processes [19]. BAG6 functions as an essential factor in ubiquitin-mediated metabolism of neo-synthesized defective polypeptides and misfolded/mislocalized proteins [49–51]. It can capture these defective or mislocalized substrates by interacting with their unprocessed or non-inserted hydrophobic domains [45], and at the same time, recruit the E3 ligases, primarily RNF126, to its N-terminal UBL domain for efficient ubiquitination and degradation [40]. Besides, BAG6 is necessary for DNA damage-induced apoptosis by controlling the p53 signaling pathway [52]. It promotes p53 transactivation by stabilizing its interaction with the acetyltransferase p300 and enhancing p53 acetylation during apoptosis and autophagy [21,22,53]. A recent study reported that BAG6 was capable of regulating the activation of IFN-I by inhibiting RIG-I/VISA-mediated recognition of RNA ligand [29]. However, the role of BAG6 in virus infection remains opaque. In this study, we provide evidence that BAG6 can potently inhibit influenza virus replicationin vitroandin vivo. Further investigation found that the overexpression of BAG6 neither affected cell apoptosis during IAV infection (S4 Fig), nor relied on the IFN-I antiviral response to inhibit IAV replication (Fig 4), whereas BAG6 directly interacts with viral polymerase subunit PB2 and targets it for ubiquitination degradation. These findings reveal a novel mechanism by which BAG6 serves as an antiviral factor to specifically target viral protein through its protein quality control function.
-In the recent years, there has been increased interest in harnessing targeted protein degradation (TPD) technology in the development of antiviral therapies by inducing the degradation of either viral or host-related protein targets, but the off-target side effects and toxicity greatly limit its use [54–57]. In this study, we found the N-terminus of host protein BAG6 contains a ubiquitin-like domain (UBL, 17-92aa), which was previously reported to recruit E3 ligase RNF126 and ubiquitinates BAG6-associated clients [40], and a PB2-binding domain (124-186aa), which was proved to interact with viral polymerase subunit PB2 protein during IAV infection. Interestingly, although the BAG6:92-255aa mutant lacking the UBL domain weakened BAG6-meditated antiviral activity against IAV, it still significantly restricted viral polymerase activity and replication (Fig 9E and 9F). This mirrors the findings that BAG6 could suppress the viral polymerase activity by competing with PB1 for PB2 binding and interfering with RdRp assembly (Fig 6E and 6F), even in the situation with PB2 degradation resistance. These data indicate that both UBL and PB2-binding domains are essential for the efficient PB2 degradation and BAG6-mediated antiviral activity. This unique structure thus allows BAG6 naturally possessing a proteolysis-targeting function. By targeting viral PB2, BAG6 is more likely to become a potential candidate for antiviral drug development.
-The laboratory animal usage license number is SYXK-Beijing-2018-0038, certified by Beijing Association for Science and Technology. All animal research was performed in compliance with the Beijing Laboratory Animal Welfare and Ethics guidelines, as issued by the Beijing Administration Committee of Laboratory Animals, and the China Agricultural University (CAU) Institutional Animal Care and Use Committee guidelines (ID: SKLAB-B-2010-003) approved by the Animal Welfare Committee of CAU. All experiments with live viruses were performed in Biosafety Level II laboratory (BSL-2) in CAU. All animal research involved in this study was approved by the Animal Welfare Committee of CAU (No.AW03503202-2-2).
-Human lung adenocarcinoma epithelial cells (A549), HeLa cell, Madin-Darby canine kidney cells (MDCK), Vero cell and human embryonic kidney cells (HEK293T) were purchased from ATCC. IRF9-KO HeLa cells were generated as previous indicated [30,31]. BAG6 KO A549 cells and BAG6 KO HeLa cells were generated using CRISPR/Cas 9-based knockout of BAG6 gene. In brief, the BAG6 gene target sequences, #1 5’- CACCGCGGTACTGGTACTATCATT-3’ and #2 5’- CACCAGGCTCCTCCACAGCGGTAC-3’, were inserted into the guide RNA (gRNA) expression cassette of the pUC19 vector, which also contains an expression cassette of Cas9. The pUC19 plasmid containing the BAG6 target sequence was then transfected into A549 or HeLa cells. The transfected cells were trypsinized 24 h later into single cells, which were diluted and inoculated into a 96-well plate by infinite dilution. Each colony was individually propagated in a 96-well plate, and the knockout of BAG6 expression was confirmed by western blotting. Cells were cultured in DMEM supplemented with 10% v/v heat-inactivated fetal bovine serum (10099141C, Gibco, USA), 100 U mL−1penicillin and 100 μg mL−1streptomycin at 37°C in a 5% CO2atmosphere.
-Influenza A/Puerto Rico/8/1934 (PR8, H1N1, accession HA number:CY045764), A/chicken/China/0606-13/2017 (CN0606, H7N9, accession HA number:MK530478), and A/chicken/Shandong/196/2011 (SD196, H9N2, accession HA number:KR002651) and A/Anhui/1/2005 (AH1, H5N1, accession HA number:HM172104) viruses were maintained in the laboratory. All experiments using non-H5 live viruses were performed in the Biosafety Level II laboratory (BSL-2), and experiments using H5 viruses were performed in the Biosafety Level III Laboratory (BSL-3) in CAU.
-Protein expression plasmids BAG6-HA, BAG6 1:255-HA, BAG6 1:753-HA, BAG6 482:753-HA, BAG6 482:1126-HA, BAG6 642:1126-HA, PB2-Flag, N-terminal PB2-Flag, PB1-Flag, PA-Flag, NP-Flag, M1-Flag, PB2-K5R-Flag, PB2-K33R-Flag, PB2-K41R-Flag, PB2-K48R-Flag, PB2-K61R-Flag, PB2-K187R-Flag, PB2-K189R-Flag, PB2-K331R-Flag, PB2-K339R-Flag, PB2-K353R-Flag, PB2-K482R-Flag, PB2-K561R-Flag, PB2-K617R-Flag, PB2-K699R-Flag, PB2-K721R-Flag, PB2-K736R-Flag, PB2-K738R-Flag, PB2-K752R-Flag, Ub-HA, K48-Ub-HA and K63-Ub-HA were generated by subcloning the corresponding coding segment into the HA-pRK5 or Flag-pRK5 empty vector by homologous recombinase-mediated recombination (S1 Table). Plasmid transfections in HEK293T or A549 cells were performed using jetPRIME (101000046, Polyplus, France).
-Antibody concentrations for immunoprecipitation and immunoblotting were determined empirically. All immunoblot antibodies were diluted as specified in 5% w/v BSA-TBST. Antibodies used as follows: anti-BAG6 (B01P, Abnova, Taiwan, China), anti-PB2 (PA5-32220, Thermo Scientific, Massachusetts, USA), anti-PB1 (PA5-34914, Thermo Scientific, Massachusetts, USA), anti-β-actin (A1978, Sigma, Shanghai, China), anti-GAPDH (ab8245, Abcam, Shanghai, China), anti-PARP (9542, Cell Signaling Technology, Massachusetts, USA), anti-Flag (F1804, Sigma, Shanghai, China and 20543-1-AP, Proteintech, Chicago, USA), anti-HA (H9658, Sigma, Shanghai, China and 51064-2-AP, Proteintech, Chicago, USA), anti-RIG-I (20566-1-AP, Proteintech, Chicago, USA), anti-p-STAT1 (9167, Cell Signaling Technology, Massachusetts, USA), anti-ISG15 (sc166755, Santa Cruz, California, USA), anti-influenza A virus NP (A01506-40, GenScript, New Jersey, USA), Mouse monoclonal anti-influenza A virus M1 antibody (Lab Homemade, Beijing, China, ZL201910912806.0). Cycloheximide (CHX, HY-12320), MG132 (HY-13259C) and Chloroquine (CQ, HY-17589A) was purchased from MCE.
-A dual-luciferase reporter assay system (E1960, Promega, Wisconsin, USA) was used to compare the polymerase activities of different viral RNP complexes. PB2, PB1, PA, and NP gene segments of the indicated viruses (PR8, CN0606 and SD196) were separately cloned into the pCDNA3.1 expression plasmid. PB2, PB1, PA, and NP plasmids (125 ng each plasmid) along with the pLuci luciferase reporter plasmid (10 ng) and the renilla internal control plasmid (2.5 ng) were used to transfect cells. Cell cultures were incubated at 37°C. Cell lysates were analyzed at 24 h post-transfection for firefly and renilla luciferase activities using a GloMax 96 microplate luminometer (GM2000, Promega, Wisconsin, USA). Polymerase proteins were detected by Western blotting.
-Six-week-old BALB/c background female mice were purchased from Beijing Vital River Co. Ltd. (Beijing, China). Animal studies were carried out in specific pathogen-free barrier facilities. Facilities were maintained at an acceptable range of 20–26°C humidity of 30–70% on a 12-h dark/12-h light cycle. Peptide-conjugated PPMO were purchased from Gene Tools (USA). PPMO targeting mouse BAG6 gene (PPMO-BAG6) was designed as CTGGCACTATCACTCGGCTCCATG. A nontargeting PPMO control sequence (PPMO-NC) (CCTCTTACCTCAGTTACAATTTATA), was used as control. Six to eight weeks BALB/c female mice were inoculated intranasally with 100 μg of PPMOs in 50 μL PBS for 2 days continuously.
-Mice were anesthetized and intranasally inoculated with PR8 virus at a median tissue culture infectious dose (TCID50) of 100 in 50 μL of PBS. Body weight and survival were monitored daily for 14 days. Lung tissue lysates were generated by homogenizing snap-frozen lung tissues twice (20 s each time) in MEM medium and centrifuging the lung suspensions at 2000 rpm for 15 min. TCID50assays were performed using MDCK cells and TCID50was calculated as previously described [58]. A portion of the lung from each euthanized mouse at 3 and 5 dpi was fixed in 10% phosphate-buffered formalin, embedded in paraffin, sectioned and stained with hematoxylin and eosin (H&amp;E). Immunohistochemical staining of viral antigen was performed as described previously [59].
-Total RNA from cells was extracted using an RNA isolation kit (Thermo Scientific, Massachusetts, USA). First-strand complementary DNA was synthesized from 1 μg of total RNA using a TransScript RT reagent kit (TransGen, Beijing, China), and oligo dT primer were used for detecting host genes. For the detection of influenza virus mRNA and vRNA, oligo dT primer and uni-12 primer (5′-AGCAAAAGCAGG-3′) [60] were respectively used to generate cDNAs. Generated cDNA was subjected to qPCR in a 25 μL reaction volume using 2X M5 HiPer SYBR Premix EsTaq (with Tli RNaseH) (Mei5bio) (S1 Table). Human β-actin genes were amplified for normalization of the cDNA amount used in qPCR. Reactions were conducted in triplicate, and the data were analyzed using the 2−ΔΔCtmethod.
-Cells were lysed in lysis buffer (50 mM Tris-Cl at pH 8.0, 150 mM NaCl, 1% Tri-ton X-100, 1 mM DTT, 1× complete protease inhibitor cocktail, and 10% glycerol) and pre-cleared with Protein A/G PLUS-Agarose beads (sc-2003, Santa Cruz Biotechnology, USA) for 2 h at 4°C. The lysates were then immunoprecipitated with indicated antibodies or isotype-matched control antibodies plus protein G Sepharose beads at 4°C for 2–4 h. The beads were then washed three times and boiled. Protein samples were analyzed by Western blotting. For Western blotting, protein samples were mixed with 6× loading buffer supplemented with 10% β-mercaptoethanol, heated at 100°C for 5 min and separated on a 10% SDS-PAGE under reducing conditions. After electrophoresis, protein samples were electroblotted onto polyvinylidene difluoride membranes (Bio-Rad, CA, USA) and blocked for 2 h in Tris-buffered saline (10 mM Tris-HCl, pH 8.0, containing 150 mM NaCl) containing 5% (w/v) non-fat dry milk and 0.5‰ (v/v) Tween-20. The blots were incubated with the primary antibodies overnight at 4°C. The next day, the blots were incubated with corresponding horseradish peroxidase (HRP)-conjugated secondary antibodies for 1 h at room temperature (RT). HRP antibody binding was detected using a standard enhanced chemiluminescence (ECL) kit (wbluf0500, Millipore, USA).
-HEK293T cell lines were cotransfected with PB2-Flag plasmid with empty vector or BAG6-HA plasmid. After 24 h post-transfection, CHX (50 μg/mL) was added to the medium and cells were harvested at different time points. Western blotting of cell lysates was performed to detect PB2-Flag, BAG6-HA and β-actin. To investigate the cellular pathway of BAG6-mediated PB2 degradation, at 24 h post-transfection, or infection with PR8 (H1N1), MG132 (20 μM) or CQ (150 μM) was added to the medium, and the cells were harvested 6 h after treatment. Three independent experiments were performed.
-HEK293T cells were transfected with HA-tagged ubiquitin (Ub-HA) plasmids, BAG6-HA or empty plasmids, and PB2-Flag or PB2-Flag with Lysine mutations. At 24 h post-transfection, the cells were treated with MG132 (20 μM) for 6 h and then lysed in 1% SDS lysis buffer. After being boiled for 10 min, the lysates were diluted 10 times with cold lysis buffer supplemented with 1× complete protease inhibitor cocktail, 10 mM DTT, and 10 mM NEM. PB2-Flag protein was then purified with anti-Flag antibody and subjected to western blotting analysis. Ubiquitinated PB2-Flag was detected by anti-HA antibody.
-We downloaded all available PB2 amino acid sequences of human and avian origin for influenza viruses of subtypes H1, H3, H5, H7, and H9 from the Global Initiative on Sharing Avian Influenza Data (GISAID,www.epicov.org) (date of access: Jan. 22, 2024), and multiple sequence alignment was performed using MAFFT v7.0 [61], and then the amino acid categories and percentages of the 189 amino acid residues were counted.
-Cells on coverslips were washed twice with prewarmed PBS and fixed with 4% paraformaldehyde for 15 min at room temperature. Cells were subsequently permeabilized with immunostaining permeabilization buffer containing Triton X-100 (P0096, Beyotime, Shanghai, China) for 10 min and blocked with QuickBlock blocking buffer (P0220, Beyotime, Shanghai, China) for 20 min at room temperature. Fixed cells were incubated with indicated antibodies diluted in immunostaining primary antibody dilution buffer at 4°C overnight. Coverslips were then washed three times with PBS and incubated with Alexa Fluor 488-conjugated secondary antibodies or Alexa Fluor 555-conjugated secondary antibodies for 1 h at 37°C. Coverslips were finally washed three times and mounted onto microscope slides with DAPI staining solution (C1006, Beyotime, Shanghai, China) for 8 min and examined by confocal microscopy. Immunoassayed cells were visualized using a Nikon super-resolution laser scanning confocal microscope under a 100-time oil objective and analyzed using the Imaris 9.2 platform.
-An online software, ColabFold, was used for the prediction of protein structures and complexes by combining the fast homology search of MMseqs2 with AlphaFold2 or RoseTTAFold. Sequence alignments/templates are generated through MMseqs2 and HHsearch [62]. The amino acid sequences of BAG6 protein N-terminal 1-255aa and PB2 protein N-terminal 1-247aa were used for the prediction of protein complex at the open-source website ColabFold v1.5.2 (https://colab.research.google.com/github/sokrypton/ColabFold/blob/main/AlphaFold2.ipynb#scrollTo=mbaIO9pWjaN0), and the predicted results were viewed and analyzed using PyMOL v2.5.0.
-WT A549 and BAG6-KO A549 cells or WT HeLa and BAG6-KO HeLa cells were plated in 96-well plates at a density of 2000 cells in 100 μL of medium per well. The cell viability was then assayed according to the CCK8 kit instructions (C0042, Beyotime, Shanghai, China).</t>
-        </is>
-      </c>
       <c r="V21" t="inlineStr">
         <is>
           <t>Based on the provided text, here is my analysis:
@@ -5404,11 +5450,10 @@
 "alias_symbol": "SCYTHE",
 "primary_gene_symbol": "BAG6",
 "name": "BAG cochaperone 6",
-"alias_symbol_represents_primary_gene": "YES",
 "alternate_abbreviation": "NO",
-"evidence": "BAG6 is a multifunctional protein in host cell and participates in a variety of physiological and pathological processes [19]."
+"evidence": ""
 }
-The text clearly refers to BAG6 throughout and discusses its functions, indicating that SCYTHE does represent the same gene as BAG6. However, there is no evidence that SCYTHE is used as an alternate abbreviation or expanded to match the official gene name. The provided evidence sentence confirms that BAG6 is being discussed but does not mention the SCYTHE alias.</t>
+The text does not provide any evidence that SCYTHE is used as an alternate abbreviation for BAG6 or BAG cochaperone 6. The text consistently refers to the gene as BAG6 throughout and does not mention SCYTHE or link it to BAG6 in any way. Therefore, there is no support for SCYTHE being an alternate abbreviation in this context.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: Alternate Abbreviation Symbols LLM Experiment Trial 5 (#86)
* add more samples where the correct annotation would be "alternate abbreviation" (previously there was only one)

* remove negative examples and remove "alias" and "other" as annotation options

* run all samples

* remove first question from prompt

* something is wrong with the full text import

* add confusion matrix and precision and recall analysis

* discrepancy in accuracy rates due to grouping after assigning T/F values-corrected

* add confusion matrix and precision and recall analysis

* update alt abb nb
</commit_message>
<xml_diff>
--- a/output/test20_alt_abbrev_annotation_with_prompt_using_fulltext_and_abstract_df.xlsx
+++ b/output/test20_alt_abbrev_annotation_with_prompt_using_fulltext_and_abstract_df.xlsx
@@ -572,44 +572,42 @@
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>36612533</t>
-        </is>
+      <c r="H2" t="n">
+        <v>7479945</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>mouse phenotype biomarker</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>primer</t>
-        </is>
-      </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>methods</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>The primers were as follows: forward primer RD5 5_-ATC TGG TTG ATC CTG CCA GT-3_ and reverse primer BhRDr 5_-GAG CTT TTTA ACT GCA ACA ACG-3_</t>
+          <t>We report a mouse model of type I Usher syndrome, rd5, whose linkage on mouse chromosome 7 to Hbb and tub has homology to human Usher I reported on human chromosome 11p15. The electroretinogram in homozygous rd5/rd5 mouse is never normal with reduced amplitudes that extinguish by 6 months.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr"/>
@@ -618,7 +616,773 @@
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Usher syndrome is a group of diseases with autosomal recessive inheritance, congenital hearing loss, and the development of retinitis pigmentosa, a progressive retinal degeneration characterized by night blindness and visual field loss over several decades. The causes of Usher syndrome are unknown and no animal models have been available for study. Four human gene sites have been reported, suggesting at least four separate forms of Usher syndrome. We report a mouse model of type I Usher syndrome, rd5, whose linkage on mouse chromosome 7 to Hbb and tub has homology to human Usher I reported on human chromosome 11p15. The electroretinogram in homozygous rd5/rd5 mouse is never normal with reduced amplitudes that extinguish by 6 months. Auditory-evoked response testing demonstrates increased hearing thresholds more than control at 3 weeks of about 30 decibels (dB) that worsen to about 45 dB by 6 months.</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>PMID: 7479945
+Abstract: Usher syndrome is a group of diseases with autosomal recessive inheritance, congenital hearing loss, and the development of retinitis pigmentosa, a progressive retinal degeneration characterized by night blindness and visual field loss over several decades. The causes of Usher syndrome are unknown and no animal models have been available for study. Four human gene sites have been reported, suggesting at least four separate forms of Usher syndrome. We report a mouse model of type I Usher syndrome, rd5, whose linkage on mouse chromosome 7 to Hbb and tub has homology to human Usher I reported on human chromosome 11p15. The electroretinogram in homozygous rd5/rd5 mouse is never normal with reduced amplitudes that extinguish by 6 months. Auditory-evoked response testing demonstrates increased hearing thresholds more than control at 3 weeks of about 30 decibels (dB) that worsen to about 45 dB by 6 months.</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
+    Inputs:
+    Alias gene symbol: rd5
+    HGNC record ID: HGNC:12406
+    Primary gene symbol: TUB
+    Official HGNC gene name: TUB bipartite transcription factor
+    Biomedical text context
+    Task:
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
+    Rules:
+    If the text does not support that the alias is an alternate abbreviation, return:
+    "alternate_abbreviation": "NO"
+    "evidence": ""
+    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
+    Evidence must be one exact sentence copied verbatim from the text.
+    Do not infer relationships or paraphrase evidence.
+    Output (Strict):
+    Output only one JSON object. No markdown.
+    {
+    "pmid": "",
+    "alias_symbol": "",
+    "primary_gene_symbol": "",
+    "name": "",
+    "alternate_abbreviation": "YES or NO",
+    "evidence": ""
+    }
+PMID: 7479945
+Abstract: Usher syndrome is a group of diseases with autosomal recessive inheritance, congenital hearing loss, and the development of retinitis pigmentosa, a progressive retinal degeneration characterized by night blindness and visual field loss over several decades. The causes of Usher syndrome are unknown and no animal models have been available for study. Four human gene sites have been reported, suggesting at least four separate forms of Usher syndrome. We report a mouse model of type I Usher syndrome, rd5, whose linkage on mouse chromosome 7 to Hbb and tub has homology to human Usher I reported on human chromosome 11p15. The electroretinogram in homozygous rd5/rd5 mouse is never normal with reduced amplitudes that extinguish by 6 months. Auditory-evoked response testing demonstrates increased hearing thresholds more than control at 3 weeks of about 30 decibels (dB) that worsen to about 45 dB by 6 months.</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>{
+"pmid": "7479945",
+"alias_symbol": "rd5",
+"primary_gene_symbol": "TUB",
+"name": "TUB bipartite transcription factor",
+"alternate_abbreviation": "NO",
+"evidence": ""
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HGNC:12406</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ENSG00000166402</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GENE ID:7275</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>TUB</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>rd5</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>9390831</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>mouse phenotype biomarker</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Mice homozygous for a defect of the tub (rd5) gene exhibit cochlear and retinal degeneration combined with obesity, and resemble certain human autosomal recessive sensory deficit syndromes.</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>TUB bipartite transcription factor</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>These authors contributed equally to this work.
+These authors jointly coordinated this work.
+Inherited retinal degeneration (IRD) represents a clinically variable and genetically heterogeneous group of disorders characterized by photoreceptor dysfunction. These diseases typically present with progressive severe vision loss and variable onset, ranging from birth to adulthood. Genomic sequencing has allowed to identify novel IRD-related genes, most of which encode proteins contributing to photoreceptor-cilia biogenesis and/or function. Despite these insights, knowledge gaps hamper a molecular diagnosis in one-third of IRD cases. By exome sequencing in a cohort of molecularly unsolved individuals with IRD, we identified a homozygous splice site variant affecting the transcript processing of TUB, encoding the first member of the Tubby family of bipartite transcription factors, in a sporadic case with retinal dystrophy. A truncating homozygous variant in this gene had previously been reported in a single family with three subjects sharing retinal dystrophy and obesity. The clinical assessment of the present patient documented a slightly increased body mass index and no changes in metabolic markers of obesity, but confirmed the occurrence of retinal detachment. In vitro studies using patient-derived fibroblasts showed the accelerated degradation of the encoded protein and aberrant cilium morphology and biogenesis. These findings definitely link impaired TUB function to retinal dystrophy and provide new data on the clinical characterization of this ultra-rare retinal ciliopathy.
+Inherited retinal degeneration (IRD) occurs in a clinically variable and genetically heterogeneous group of conditions characterized by photoreceptor degeneration and/or dysfunction [1]. The prevalence of monogenic IRD is estimated as 1 in 2000 individuals, affecting more than 2 million people worldwide [2]. This group of disorders typically present with severe vision loss that can be progressive, having an onset ranging from birth to late adulthood. Severe visual impairment affects mobility and independence, posing relevant psychological and economic burdens [3]. In the last ten years, genomic sequencing has allowed the identification of several genes implicated in IRD (for an updated list see the RetNet database,https://sph.uth.edu/retnet/). These genes encode proteins that have different roles in visual function, contributing to key processes in the cells of the pigmented cell layer and neurosensory retina [4,5]. Notably, retinal degeneration is frequently observed in ciliopathies, and a portion of IRD-related genes codifies for proteins involved in biogenesis and the maintenance of photoreceptor primary cilium [6,7,8,9]. Among these genes,TUB[MIM #601197], which encodes the first member of the Tubby family of bipartite transcription factors, has recently reported to be associated with a novel condition characterized by retinal dystrophy and obesity [MIM #616188] [10]. A truncating homozygousTUBvariant [c.1194_1195delAG, p.Arg398Serfs*9] was identified in a single family with three affected members, suggesting loss of function (LoF) as the pathomechanism underlying the disorder. The TUB family of transcription factors counts four members in vertebrates (TUB, TULP1, TULP2 and TULP3), sharing a similar domain organization including a highly conserved C-terminal domain mediating DNA binding and a divergent N-terminal region encompassing the nuclear localization signal and the transcriptional activation domain implicated in protein–protein binding [11]. A conserved region at the N-terminus enables some members of the Tubby family, including TUB, to bind to the ciliary intraflagellar transport A protein (IFTAP) [12]. Similar to the other members of the TULP family, TUB is also implicated in the control of the initiation of phagocytosis, facilitating the removal of apoptotic cells or cellular debris by retinal pigmented epithelium (RPE) cells and macrophages [13]. Since the original report, no other subject carrying biallelicTUBvariants has been described.
+In this study, we report on an additional subject with retinal dystrophy carrying a homozygous LoF variant inTUB. In vitro analyses provide evidence of the disruptive functional impact of the variant onTUBtranscript processing. We also show that the loss of TUB is associated with a defective cilium morphology and biogenesis in the primary patient’s fibroblasts. Our findings confirm the involvement of defective TUB function in retinal dystrophy and define this disorder as a novel ciliopathy.
+The proband is a 35-year-old male, the first child of healthy non-consanguineous parents of European descent (Figure 1). Family history was negative for retinal diseases or other congenital defects. The proband was born at term after an uneventful pregnancy. Length and weight at birth were reported as within the normal range. Apgar score was 8–10. No hearing impairment and/or learning difficulties were documented during the first year of age.
+At 5 years, the subject required consulting ophthalmologists for referring color blindness. A “blonde” aspect of the fundus oculi was observed and reduced full-field flash photopic and scotopic electroretinogram (ERG) responses were recorded. Visual acuity was not investigated at that time. Ophthalmological assessment at 26 years was suggestive of cone-rod dystrophy. Visual acuity was 0.8 Snellen in his right eye (RE) with myopic and astigmatic refractive error (RE: -4.50 dioptre sphere and -1 dioptre cylinder at 20°), and 0.2 Snellen in his left eye (LE) with myopic refractive error (LE: -2.00 dioptre sphere). Goldmann visual field was generally constricted, with reduced sensitivity in the superior central field in the RE and presented peripheral constriction and relative central scotoma in the LE. Light and dark adaptation sensitivity curves showed abnormal thresholds for both cones and rods. No number at the Ishihara charts were recognized. Intraocular pressure was within normal limits. The slit lamp examination biomicroscopy of the anterior segment was normal for cornea, iris and lens appearance. Fundus examination revealed bilateral optic disc pallor, depigmented aspect of the choroidal and retinal structures, diffuse retinal dystrophy with absence of intraretinal pigment dispersion or vitreous abnormalities and arteriolar attenuation. Full-field scotopic and photopic electroretinograms showed reduced a-wave and b-wave amplitude responses and delayed implicit times. Multifocal ERG ring analysis documented reduced response amplitude densities in all examined areas from the foveal center up to 20° of foveal eccentricity in both eyes (LE &gt; RE). After reduced visual field in his LE, a large area of retinoschisis in the infero-temporal sector was observed by fundoscopy, which later progressed, resulting in full retinal detachment of the LE. The subject underwent to pars plana vitrectomy with silicon oil (30% polydimethylsiloxane, PDMS) tamponade. He underwent cataract surgery in his LE and to subsequent vitreo-retinal surgeries for relapsing retinal detachments in same eye (PDMS/perfluorocarbon liquid (PFCL)/PDMS tamponades exchange and intra-operatory laser treatment; PDMS/heavy silicon oil tamponades exchange and intra-operatory laser). One year later, he developed vitreo-retinal proliferation and retinal fibrosis in the LE, and visual acuity was hand motion; therefore, the subject underwent retinotomy and heavy silicon oil/PDMS tamponades exchange.
+At last evaluation (35 years), the subject presented with a good clinical condition. No cognitive deficit nor behavioral issues were observed, and no craniofacial dysmorphism and truncal obesity were noticed. An accurate endocrinological examination was uninformative. Anthropometric assessment displayed a height of 177.5 cm (+0.1 SD), weight of 95.70 kg (+1.6 SD), and OFC 60 cm (+0.2 SD) and BMI of 30.30 Kg/m2(+1.6 SD). Tanner stage was Ph5Pg5, with a testicular volume 20 mL bilaterally. The subject’s visual acuity was 0.8 Snellen in his RE and light perception in his LE. Fundus oculi showed the unmodified condition of RE and diffuse chorio-retinal atrophy in the LE, as for visible vitreo-retinal surgical outcomes. Ultrawide field fundus photography showed macular atrophy in absence of peripheral pigment and confirmed a “blonde” aspect of the retina (Figure 2A). Fundus autofluorescence (FAF) revealed an hypoautoflorescent area in the macula due to RPE atrophy and hyper/hypoautofluorescence mottling in the posterior pole and immediately outside the vascular arcades (Figure 2B). The SD-OCT showed a disruption of the outer retina, including ELM, ellipsoid zone and RPE with outer retinal debris at the level of the RPE in the parafoveal region (Figure 2C). Full-field flash scotopic (Figure 2D) and photopic ERG confirmed reduced a-wave and b-wave amplitude responses and delayed implicit times in the RE. Similarly, multifocal ERG ring analysis, recordable only in the RE, showed the worsening of the response amplitude densities in all examined areas (0–20°) (Figure 2E), as compared to the previous examinations. Similarly, Goldmann visual field in his RE showed progressive constriction of the peripheral isopters and a ring scotoma enclosed between 10–20° of the visual field (Figure 2F); it was not executable, however, in his LE. Color blindness was also confirmed. Neck and abdominal ultrasound assessment did not reveal any abnormality. Measurements of basal hormones by the anterior pituitary, glycaemia and insulin were within the normal range. Basal plasma leptin level was in the low normal range, showing no leptin resistance. During his follow-up, clinical and ophthalmological assessments of other family members (parents and younger brother) were unremarkable.
+Trio-based WES allowed to identify a homozygous splice siteTUBvariant (chr11:8122545G &gt; A, GRCh37.p13; c.1387 + 1G &gt; A,NM_177972.3) as the only clinically and functionally relevant event putatively linked to the disorder (Supplemental Table S1). The variant had previously been annotated in public databases (dbSNP, rs1040410003) with low frequency (gnomAD v3.1, MAF = 0.00001972) at the heterozygous state. It was classified as likely pathogenic (PVS1/PM2/PP5) according to the American College of Medical Genetics and Genomics-Association for Molecular Pathology (ACMG-AMP) criteria (ClinVar: VCV000865971.1) [14]. Sanger sequencing confirmed the homozygosity for the variant in the proband and the heterozygous status in the healthy parents and unaffected sib (Figure 1).
+Since the variant was predicted to affect the exon 11 donor splice site, the total RNA from patient-derived skin primary fibroblasts was used to characterize the impact of the nucleotide change on transcript processing. The cDNA fragment encompassing the relevant exons was amplified, confirming the presence of two aberrantly spliced products (Figure 3A). The two aberrant PCR amplicons were isolated from agarose gel, purified and sequenced via Sanger. The former (500 bp) was derived from skipping of the penultimate exon (exon 11, ENST00000299506.3), resulting in a premature termination codon (i.e., p.Glu406Argfs*4), while the latter (1172 bp) was the result of retention of intron 10, resulting in a TUB protein having a divergent 19-residue-long C-terminus and lacking the last 44 amino acids (p.Pro463Hisfs*19) (Figure 3B).
+In the patient’s skin fibroblasts, the predicted TUBGlu406Argfs*4protein was undetectable by Western blot [WB] analysis, while the TUBPro463Hisfs*19protein was poorly detectable likely due to accelerated degradation (Figure 3C, left panel). Consistently, the endogenous TUBPro463Hisfs*19level was partially rescued by blocking the proteasomal degradation pathway using MG132 (Figure 3C, right panel).
+To investigate the cellular localization of the mutated protein, cytoplasm and nuclear cell fractions were obtained and analyzed by WB. The results demonstrate that both the wild-type (wt) and mutant TUB proteins were almost exclusively localized in the nucleus (Figure 3D). This finding was also confirmed by confocal microscopy analysis that evidenced the nuclear localization of the TUB mutant (Figure 4A).
+Based on the documented role of TUB in early ciliogenesis [15], we assessed the localization of TUB at the cilium, but we failed to observe any consistent co-localization, possibly due to the low diffused levels of the protein in the cytoplasm To investigate the impact of defective TUB function on the morphogenesis of the primary cilium, a confocal analysis on primary fibroblasts was performed using antibodies against ARL13B, which localizes to primary cilia, and pericentrin, a component of the centrosome, which stains the basal body. As shown inFigure 4B, while almost all the control cells showed a primary cilium, 40% of the fibroblasts carrying the homozygous splice site variant inTUBdid not show a primary cilium. Moreover, while no significant difference was observed in ciliary axoneme length between the starved control and mutant cells, a large percentage of the latter showed an abnormal cilium morphology and a poorly defined and disorganized basal body (Figure 4C).
+The loss of TUB function was recently reported to underlie a novel IRD condition based on the identification of homozygosity for a 2 bp deletion (c.1194_1195delAG) causing the premature termination of the protein (p.Arg398Serfs*9) shared by three affected members of a single consanguineous family [10]. While the combination of retinal dystrophy and early onset obesity can be reminiscent of other disorders (e.g., Bardet–Biedl syndrome (MIM#PS209900) and Alstrom syndrome (MIM#203800)), the absence of other clinically relevant feature/sign was suggestive of a previously unreported ciliopathy [10]. In this paper, we report on a second disruptive variant (c.1387 + 1G &gt; A) affectingTUBin a subject with features that overlap with those previously described in the affected members of the original family.
+In the present and previously reported affected individuals, the ocular phenotype associated with defective TUB function is characterized by widespread retinal pigment epithelial (RPE) atrophy, deteriorating vision, the myopic and astigmatic refractive defect, the blonde fundus appearance, the ERG and OCT findings and progression of the disease (Figure 2). Notably, retinal detachment, without vitreous hemorrhage, was invariantly documented in the four individuals with biallelic inactivatingTUBvariants, suggesting that this feature likely represent a common finding in the disorder.
+Early onset obesity had previously been considered a major feature of the TUB-related condition [10], even though only two of three affected sibs were found obese (BMI &gt; 30), and the glycemic and lipid profiles in one of affected sibs were found within the normal range. The finding of obesity in the apparently healthy father (heterozygous carrier) suggests a possible co-occurring genetic event contributing to obesity in the family. In the present report, the clinical assessment of the affected individual documented increased weight (95.7 kg, +1.6 SD) and BMI (30.3, +1.6 SD), thus indicating overweight, in absence of other signs of obesity. Although evidence suggests that a defective TUB function may result in disturbances in insulin and leptin activity and obesity in mice [16,17,18,19], based on the collected findings, the relevance of TUB in human obesity requires further study. To assess whether TUB LoF could impact on hypothalamic pathways, food intake and adiposity, the metabolic profile of the affected individual was investigated. Accurate endocrinological examination did not reveal any abnormality, and the measurements of basal hormones by the anterior pituitary, glycaemia, insulin and leptin were within the normal range, thus ruling out insulin or leptin resistance. Consistently, instrumental investigations (X-ray and ultrasound analyses) documented no sign of glycogen accumulation in the internal organs. Consistently, the absence of significant changes in lipid storage was demonstrated by thin-layer chromatography (HPTLC) analysis in proband-derived fibroblast (Figure S1), allowing to confirm an apparently normal endocrine–metabolic profile in the affected individual. Of note, the Tubby protein has been involved in cochlear degeneration [20,21]. Based on this functional link, we evaluated the occurrence of hearing problems and cochlear degeneration, which were not observed.
+The homozygousTUBvariant was predicted to affect transcript processing, causing the skipping of exon 11 and intron retention, resulting in a frameshift with the premature termination of the TUB protein. mRNA analysis in proband-derived fibroblasts confirmed a disruptive impact of the splice site change documenting two aberrantly processed transcripts predicted to encode a 406-residue-long protein (p.Glu406Argfs*4) that probably is not able to proceed in protein synthesis, and a 481-residue-long protein (p.Pro463Hisfs*19) characterized by a divergent C-terminus characterized by accelerated degradation (Figure 3B). These findings confirm LoF as the pathomechanism underlying this disorder.
+Primary cilia are microtubule-based organelles that extend from the apical surface of the majority of mammalian cells. Cilia act as “cellular antennae”, receiving different inputs from the extracellular environment and transducing signals in response to stimuli [22]. A complex process required for proper cilia biogenesis function is the intraflagellar transport, which is required for assembling cilia and trafficking within primary cilia [23]. In this context, IFT-A has historically been believed to mediate retrograde intraflagellar transport inside the cilia and an IFT-A-binding domain at the TUB N-terminus has been demonstrated recently [24]. Moreover, co-localization between TUB and rootletin, the major structural component of the ciliary rootlet, has been observed in human retinal photoreceptors [10]. The use of a more informative in vitro model (e.g., induced pluripotent-stem-cell-derived retinal-pigment epithelium cells) and experimental strategies (e.g., siRNA-mediated TUB silencing) is required to appreciate more accurately the functional relevance of TUB in an appropriate cellular context.
+In summary, we confirm the link between TUB LoF and a new condition of human retinal ciliopathy and provide evidence of an altered cilium morphology/biogenesis in patient-derived fibroblasts. In fact, these cells displayed a reduced number of cilia when compared to the control cells, with a poorly defined and disorganized basal body structure, which are expected to prevent normal protein trafficking along the cilium. While these findings could explain the degeneration of photoreceptors characterizing this disorder, a relatively overall mild presentation has been associated with mutations in this gene. Multiple factors might contribute to this picture. First, the functional relevance of TUB in the context of ciliogenesis and cilium function might vary in different cell lineages. Second, functional compensation exerted by other related proteins might contribute to buffer the severity of the endophenotype. Third, specific cell lineages (e.g., rod and cone cells) might be particularly sensitive to TUB LoF. The collection of additional patients with biallelic variants in the gene will allow a more accurate characterization of the clinical spectrum associated with TUB LoF. Based on these considerations, TUB loss of function could be considered as responsible for a novel form of isolated retinal ciliopathy.</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Mice homozygous for a defect of the tub (rd5) gene exhibit cochlear and retinal degeneration combined with obesity, and resemble certain human autosomal recessive sensory deficit syndromes. To establish the progressive nature of sensory cell loss associated with the tub gene, and to differentiate tub-related losses from those associated with the C57 background on which tub arose, we evaluated cochleas and retinas from tub/tub, tub/+, and +/+ mice, aged 2 weeks to 1 year by light and electron microscopy. Cochleas from mice of all three genotypes show progressive inner (IHC) and outer hair cell (OHC) loss. Relative to tub/+ and +/+ animals, however, tub homozygotes show accelerated OHC loss, affecting the extreme cochlear base (hook region) by 1 month, and the apex by 6 months. IHC loss in tub/tub animals is accelerated in the basal half of the cochlea, affecting the hook region by 6 months. Spiral ganglion cell losses were observed only in tub/tub mice, and only in the cochlear base. Retinas of tub/tub mice are abnormal at maturity, exhibiting shortened photoreceptor outer segments by 2 weeks, and progressive photoreceptor loss thereafter. Because the tub mutation causes degeneration of sensory cells in the ear and eye but has no other neurological effects, tubby mice hold unique promise for the study of human syndromic sensory loss.</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>PMID: 9390831
+Full Text: These authors contributed equally to this work.
+These authors jointly coordinated this work.
+Inherited retinal degeneration (IRD) represents a clinically variable and genetically heterogeneous group of disorders characterized by photoreceptor dysfunction. These diseases typically present with progressive severe vision loss and variable onset, ranging from birth to adulthood. Genomic sequencing has allowed to identify novel IRD-related genes, most of which encode proteins contributing to photoreceptor-cilia biogenesis and/or function. Despite these insights, knowledge gaps hamper a molecular diagnosis in one-third of IRD cases. By exome sequencing in a cohort of molecularly unsolved individuals with IRD, we identified a homozygous splice site variant affecting the transcript processing of TUB, encoding the first member of the Tubby family of bipartite transcription factors, in a sporadic case with retinal dystrophy. A truncating homozygous variant in this gene had previously been reported in a single family with three subjects sharing retinal dystrophy and obesity. The clinical assessment of the present patient documented a slightly increased body mass index and no changes in metabolic markers of obesity, but confirmed the occurrence of retinal detachment. In vitro studies using patient-derived fibroblasts showed the accelerated degradation of the encoded protein and aberrant cilium morphology and biogenesis. These findings definitely link impaired TUB function to retinal dystrophy and provide new data on the clinical characterization of this ultra-rare retinal ciliopathy.
+Inherited retinal degeneration (IRD) occurs in a clinically variable and genetically heterogeneous group of conditions characterized by photoreceptor degeneration and/or dysfunction [1]. The prevalence of monogenic IRD is estimated as 1 in 2000 individuals, affecting more than 2 million people worldwide [2]. This group of disorders typically present with severe vision loss that can be progressive, having an onset ranging from birth to late adulthood. Severe visual impairment affects mobility and independence, posing relevant psychological and economic burdens [3]. In the last ten years, genomic sequencing has allowed the identification of several genes implicated in IRD (for an updated list see the RetNet database,https://sph.uth.edu/retnet/). These genes encode proteins that have different roles in visual function, contributing to key processes in the cells of the pigmented cell layer and neurosensory retina [4,5]. Notably, retinal degeneration is frequently observed in ciliopathies, and a portion of IRD-related genes codifies for proteins involved in biogenesis and the maintenance of photoreceptor primary cilium [6,7,8,9]. Among these genes,TUB[MIM #601197], which encodes the first member of the Tubby family of bipartite transcription factors, has recently reported to be associated with a novel condition characterized by retinal dystrophy and obesity [MIM #616188] [10]. A truncating homozygousTUBvariant [c.1194_1195delAG, p.Arg398Serfs*9] was identified in a single family with three affected members, suggesting loss of function (LoF) as the pathomechanism underlying the disorder. The TUB family of transcription factors counts four members in vertebrates (TUB, TULP1, TULP2 and TULP3), sharing a similar domain organization including a highly conserved C-terminal domain mediating DNA binding and a divergent N-terminal region encompassing the nuclear localization signal and the transcriptional activation domain implicated in protein–protein binding [11]. A conserved region at the N-terminus enables some members of the Tubby family, including TUB, to bind to the ciliary intraflagellar transport A protein (IFTAP) [12]. Similar to the other members of the TULP family, TUB is also implicated in the control of the initiation of phagocytosis, facilitating the removal of apoptotic cells or cellular debris by retinal pigmented epithelium (RPE) cells and macrophages [13]. Since the original report, no other subject carrying biallelicTUBvariants has been described.
+In this study, we report on an additional subject with retinal dystrophy carrying a homozygous LoF variant inTUB. In vitro analyses provide evidence of the disruptive functional impact of the variant onTUBtranscript processing. We also show that the loss of TUB is associated with a defective cilium morphology and biogenesis in the primary patient’s fibroblasts. Our findings confirm the involvement of defective TUB function in retinal dystrophy and define this disorder as a novel ciliopathy.
+The proband is a 35-year-old male, the first child of healthy non-consanguineous parents of European descent (Figure 1). Family history was negative for retinal diseases or other congenital defects. The proband was born at term after an uneventful pregnancy. Length and weight at birth were reported as within the normal range. Apgar score was 8–10. No hearing impairment and/or learning difficulties were documented during the first year of age.
+At 5 years, the subject required consulting ophthalmologists for referring color blindness. A “blonde” aspect of the fundus oculi was observed and reduced full-field flash photopic and scotopic electroretinogram (ERG) responses were recorded. Visual acuity was not investigated at that time. Ophthalmological assessment at 26 years was suggestive of cone-rod dystrophy. Visual acuity was 0.8 Snellen in his right eye (RE) with myopic and astigmatic refractive error (RE: -4.50 dioptre sphere and -1 dioptre cylinder at 20°), and 0.2 Snellen in his left eye (LE) with myopic refractive error (LE: -2.00 dioptre sphere). Goldmann visual field was generally constricted, with reduced sensitivity in the superior central field in the RE and presented peripheral constriction and relative central scotoma in the LE. Light and dark adaptation sensitivity curves showed abnormal thresholds for both cones and rods. No number at the Ishihara charts were recognized. Intraocular pressure was within normal limits. The slit lamp examination biomicroscopy of the anterior segment was normal for cornea, iris and lens appearance. Fundus examination revealed bilateral optic disc pallor, depigmented aspect of the choroidal and retinal structures, diffuse retinal dystrophy with absence of intraretinal pigment dispersion or vitreous abnormalities and arteriolar attenuation. Full-field scotopic and photopic electroretinograms showed reduced a-wave and b-wave amplitude responses and delayed implicit times. Multifocal ERG ring analysis documented reduced response amplitude densities in all examined areas from the foveal center up to 20° of foveal eccentricity in both eyes (LE &gt; RE). After reduced visual field in his LE, a large area of retinoschisis in the infero-temporal sector was observed by fundoscopy, which later progressed, resulting in full retinal detachment of the LE. The subject underwent to pars plana vitrectomy with silicon oil (30% polydimethylsiloxane, PDMS) tamponade. He underwent cataract surgery in his LE and to subsequent vitreo-retinal surgeries for relapsing retinal detachments in same eye (PDMS/perfluorocarbon liquid (PFCL)/PDMS tamponades exchange and intra-operatory laser treatment; PDMS/heavy silicon oil tamponades exchange and intra-operatory laser). One year later, he developed vitreo-retinal proliferation and retinal fibrosis in the LE, and visual acuity was hand motion; therefore, the subject underwent retinotomy and heavy silicon oil/PDMS tamponades exchange.
+At last evaluation (35 years), the subject presented with a good clinical condition. No cognitive deficit nor behavioral issues were observed, and no craniofacial dysmorphism and truncal obesity were noticed. An accurate endocrinological examination was uninformative. Anthropometric assessment displayed a height of 177.5 cm (+0.1 SD), weight of 95.70 kg (+1.6 SD), and OFC 60 cm (+0.2 SD) and BMI of 30.30 Kg/m2(+1.6 SD). Tanner stage was Ph5Pg5, with a testicular volume 20 mL bilaterally. The subject’s visual acuity was 0.8 Snellen in his RE and light perception in his LE. Fundus oculi showed the unmodified condition of RE and diffuse chorio-retinal atrophy in the LE, as for visible vitreo-retinal surgical outcomes. Ultrawide field fundus photography showed macular atrophy in absence of peripheral pigment and confirmed a “blonde” aspect of the retina (Figure 2A). Fundus autofluorescence (FAF) revealed an hypoautoflorescent area in the macula due to RPE atrophy and hyper/hypoautofluorescence mottling in the posterior pole and immediately outside the vascular arcades (Figure 2B). The SD-OCT showed a disruption of the outer retina, including ELM, ellipsoid zone and RPE with outer retinal debris at the level of the RPE in the parafoveal region (Figure 2C). Full-field flash scotopic (Figure 2D) and photopic ERG confirmed reduced a-wave and b-wave amplitude responses and delayed implicit times in the RE. Similarly, multifocal ERG ring analysis, recordable only in the RE, showed the worsening of the response amplitude densities in all examined areas (0–20°) (Figure 2E), as compared to the previous examinations. Similarly, Goldmann visual field in his RE showed progressive constriction of the peripheral isopters and a ring scotoma enclosed between 10–20° of the visual field (Figure 2F); it was not executable, however, in his LE. Color blindness was also confirmed. Neck and abdominal ultrasound assessment did not reveal any abnormality. Measurements of basal hormones by the anterior pituitary, glycaemia and insulin were within the normal range. Basal plasma leptin level was in the low normal range, showing no leptin resistance. During his follow-up, clinical and ophthalmological assessments of other family members (parents and younger brother) were unremarkable.
+Trio-based WES allowed to identify a homozygous splice siteTUBvariant (chr11:8122545G &gt; A, GRCh37.p13; c.1387 + 1G &gt; A,NM_177972.3) as the only clinically and functionally relevant event putatively linked to the disorder (Supplemental Table S1). The variant had previously been annotated in public databases (dbSNP, rs1040410003) with low frequency (gnomAD v3.1, MAF = 0.00001972) at the heterozygous state. It was classified as likely pathogenic (PVS1/PM2/PP5) according to the American College of Medical Genetics and Genomics-Association for Molecular Pathology (ACMG-AMP) criteria (ClinVar: VCV000865971.1) [14]. Sanger sequencing confirmed the homozygosity for the variant in the proband and the heterozygous status in the healthy parents and unaffected sib (Figure 1).
+Since the variant was predicted to affect the exon 11 donor splice site, the total RNA from patient-derived skin primary fibroblasts was used to characterize the impact of the nucleotide change on transcript processing. The cDNA fragment encompassing the relevant exons was amplified, confirming the presence of two aberrantly spliced products (Figure 3A). The two aberrant PCR amplicons were isolated from agarose gel, purified and sequenced via Sanger. The former (500 bp) was derived from skipping of the penultimate exon (exon 11, ENST00000299506.3), resulting in a premature termination codon (i.e., p.Glu406Argfs*4), while the latter (1172 bp) was the result of retention of intron 10, resulting in a TUB protein having a divergent 19-residue-long C-terminus and lacking the last 44 amino acids (p.Pro463Hisfs*19) (Figure 3B).
+In the patient’s skin fibroblasts, the predicted TUBGlu406Argfs*4protein was undetectable by Western blot [WB] analysis, while the TUBPro463Hisfs*19protein was poorly detectable likely due to accelerated degradation (Figure 3C, left panel). Consistently, the endogenous TUBPro463Hisfs*19level was partially rescued by blocking the proteasomal degradation pathway using MG132 (Figure 3C, right panel).
+To investigate the cellular localization of the mutated protein, cytoplasm and nuclear cell fractions were obtained and analyzed by WB. The results demonstrate that both the wild-type (wt) and mutant TUB proteins were almost exclusively localized in the nucleus (Figure 3D). This finding was also confirmed by confocal microscopy analysis that evidenced the nuclear localization of the TUB mutant (Figure 4A).
+Based on the documented role of TUB in early ciliogenesis [15], we assessed the localization of TUB at the cilium, but we failed to observe any consistent co-localization, possibly due to the low diffused levels of the protein in the cytoplasm To investigate the impact of defective TUB function on the morphogenesis of the primary cilium, a confocal analysis on primary fibroblasts was performed using antibodies against ARL13B, which localizes to primary cilia, and pericentrin, a component of the centrosome, which stains the basal body. As shown inFigure 4B, while almost all the control cells showed a primary cilium, 40% of the fibroblasts carrying the homozygous splice site variant inTUBdid not show a primary cilium. Moreover, while no significant difference was observed in ciliary axoneme length between the starved control and mutant cells, a large percentage of the latter showed an abnormal cilium morphology and a poorly defined and disorganized basal body (Figure 4C).
+The loss of TUB function was recently reported to underlie a novel IRD condition based on the identification of homozygosity for a 2 bp deletion (c.1194_1195delAG) causing the premature termination of the protein (p.Arg398Serfs*9) shared by three affected members of a single consanguineous family [10]. While the combination of retinal dystrophy and early onset obesity can be reminiscent of other disorders (e.g., Bardet–Biedl syndrome (MIM#PS209900) and Alstrom syndrome (MIM#203800)), the absence of other clinically relevant feature/sign was suggestive of a previously unreported ciliopathy [10]. In this paper, we report on a second disruptive variant (c.1387 + 1G &gt; A) affectingTUBin a subject with features that overlap with those previously described in the affected members of the original family.
+In the present and previously reported affected individuals, the ocular phenotype associated with defective TUB function is characterized by widespread retinal pigment epithelial (RPE) atrophy, deteriorating vision, the myopic and astigmatic refractive defect, the blonde fundus appearance, the ERG and OCT findings and progression of the disease (Figure 2). Notably, retinal detachment, without vitreous hemorrhage, was invariantly documented in the four individuals with biallelic inactivatingTUBvariants, suggesting that this feature likely represent a common finding in the disorder.
+Early onset obesity had previously been considered a major feature of the TUB-related condition [10], even though only two of three affected sibs were found obese (BMI &gt; 30), and the glycemic and lipid profiles in one of affected sibs were found within the normal range. The finding of obesity in the apparently healthy father (heterozygous carrier) suggests a possible co-occurring genetic event contributing to obesity in the family. In the present report, the clinical assessment of the affected individual documented increased weight (95.7 kg, +1.6 SD) and BMI (30.3, +1.6 SD), thus indicating overweight, in absence of other signs of obesity. Although evidence suggests that a defective TUB function may result in disturbances in insulin and leptin activity and obesity in mice [16,17,18,19], based on the collected findings, the relevance of TUB in human obesity requires further study. To assess whether TUB LoF could impact on hypothalamic pathways, food intake and adiposity, the metabolic profile of the affected individual was investigated. Accurate endocrinological examination did not reveal any abnormality, and the measurements of basal hormones by the anterior pituitary, glycaemia, insulin and leptin were within the normal range, thus ruling out insulin or leptin resistance. Consistently, instrumental investigations (X-ray and ultrasound analyses) documented no sign of glycogen accumulation in the internal organs. Consistently, the absence of significant changes in lipid storage was demonstrated by thin-layer chromatography (HPTLC) analysis in proband-derived fibroblast (Figure S1), allowing to confirm an apparently normal endocrine–metabolic profile in the affected individual. Of note, the Tubby protein has been involved in cochlear degeneration [20,21]. Based on this functional link, we evaluated the occurrence of hearing problems and cochlear degeneration, which were not observed.
+The homozygousTUBvariant was predicted to affect transcript processing, causing the skipping of exon 11 and intron retention, resulting in a frameshift with the premature termination of the TUB protein. mRNA analysis in proband-derived fibroblasts confirmed a disruptive impact of the splice site change documenting two aberrantly processed transcripts predicted to encode a 406-residue-long protein (p.Glu406Argfs*4) that probably is not able to proceed in protein synthesis, and a 481-residue-long protein (p.Pro463Hisfs*19) characterized by a divergent C-terminus characterized by accelerated degradation (Figure 3B). These findings confirm LoF as the pathomechanism underlying this disorder.
+Primary cilia are microtubule-based organelles that extend from the apical surface of the majority of mammalian cells. Cilia act as “cellular antennae”, receiving different inputs from the extracellular environment and transducing signals in response to stimuli [22]. A complex process required for proper cilia biogenesis function is the intraflagellar transport, which is required for assembling cilia and trafficking within primary cilia [23]. In this context, IFT-A has historically been believed to mediate retrograde intraflagellar transport inside the cilia and an IFT-A-binding domain at the TUB N-terminus has been demonstrated recently [24]. Moreover, co-localization between TUB and rootletin, the major structural component of the ciliary rootlet, has been observed in human retinal photoreceptors [10]. The use of a more informative in vitro model (e.g., induced pluripotent-stem-cell-derived retinal-pigment epithelium cells) and experimental strategies (e.g., siRNA-mediated TUB silencing) is required to appreciate more accurately the functional relevance of TUB in an appropriate cellular context.
+In summary, we confirm the link between TUB LoF and a new condition of human retinal ciliopathy and provide evidence of an altered cilium morphology/biogenesis in patient-derived fibroblasts. In fact, these cells displayed a reduced number of cilia when compared to the control cells, with a poorly defined and disorganized basal body structure, which are expected to prevent normal protein trafficking along the cilium. While these findings could explain the degeneration of photoreceptors characterizing this disorder, a relatively overall mild presentation has been associated with mutations in this gene. Multiple factors might contribute to this picture. First, the functional relevance of TUB in the context of ciliogenesis and cilium function might vary in different cell lineages. Second, functional compensation exerted by other related proteins might contribute to buffer the severity of the endophenotype. Third, specific cell lineages (e.g., rod and cone cells) might be particularly sensitive to TUB LoF. The collection of additional patients with biallelic variants in the gene will allow a more accurate characterization of the clinical spectrum associated with TUB LoF. Based on these considerations, TUB loss of function could be considered as responsible for a novel form of isolated retinal ciliopathy.</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
+    Inputs:
+    Alias gene symbol: rd5
+    HGNC record ID: HGNC:12406
+    Primary gene symbol: TUB
+    Official HGNC gene name: TUB bipartite transcription factor
+    Biomedical text context
+    Task:
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
+    Rules:
+    If the text does not support that the alias is an alternate abbreviation, return:
+    "alternate_abbreviation": "NO"
+    "evidence": ""
+    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
+    Evidence must be one exact sentence copied verbatim from the text.
+    Do not infer relationships or paraphrase evidence.
+    Output (Strict):
+    Output only one JSON object. No markdown.
+    {
+    "pmid": "",
+    "alias_symbol": "",
+    "primary_gene_symbol": "",
+    "name": "",
+    "alternate_abbreviation": "YES or NO",
+    "evidence": ""
+    }
+PMID: 9390831
+Full Text: These authors contributed equally to this work.
+These authors jointly coordinated this work.
+Inherited retinal degeneration (IRD) represents a clinically variable and genetically heterogeneous group of disorders characterized by photoreceptor dysfunction. These diseases typically present with progressive severe vision loss and variable onset, ranging from birth to adulthood. Genomic sequencing has allowed to identify novel IRD-related genes, most of which encode proteins contributing to photoreceptor-cilia biogenesis and/or function. Despite these insights, knowledge gaps hamper a molecular diagnosis in one-third of IRD cases. By exome sequencing in a cohort of molecularly unsolved individuals with IRD, we identified a homozygous splice site variant affecting the transcript processing of TUB, encoding the first member of the Tubby family of bipartite transcription factors, in a sporadic case with retinal dystrophy. A truncating homozygous variant in this gene had previously been reported in a single family with three subjects sharing retinal dystrophy and obesity. The clinical assessment of the present patient documented a slightly increased body mass index and no changes in metabolic markers of obesity, but confirmed the occurrence of retinal detachment. In vitro studies using patient-derived fibroblasts showed the accelerated degradation of the encoded protein and aberrant cilium morphology and biogenesis. These findings definitely link impaired TUB function to retinal dystrophy and provide new data on the clinical characterization of this ultra-rare retinal ciliopathy.
+Inherited retinal degeneration (IRD) occurs in a clinically variable and genetically heterogeneous group of conditions characterized by photoreceptor degeneration and/or dysfunction [1]. The prevalence of monogenic IRD is estimated as 1 in 2000 individuals, affecting more than 2 million people worldwide [2]. This group of disorders typically present with severe vision loss that can be progressive, having an onset ranging from birth to late adulthood. Severe visual impairment affects mobility and independence, posing relevant psychological and economic burdens [3]. In the last ten years, genomic sequencing has allowed the identification of several genes implicated in IRD (for an updated list see the RetNet database,https://sph.uth.edu/retnet/). These genes encode proteins that have different roles in visual function, contributing to key processes in the cells of the pigmented cell layer and neurosensory retina [4,5]. Notably, retinal degeneration is frequently observed in ciliopathies, and a portion of IRD-related genes codifies for proteins involved in biogenesis and the maintenance of photoreceptor primary cilium [6,7,8,9]. Among these genes,TUB[MIM #601197], which encodes the first member of the Tubby family of bipartite transcription factors, has recently reported to be associated with a novel condition characterized by retinal dystrophy and obesity [MIM #616188] [10]. A truncating homozygousTUBvariant [c.1194_1195delAG, p.Arg398Serfs*9] was identified in a single family with three affected members, suggesting loss of function (LoF) as the pathomechanism underlying the disorder. The TUB family of transcription factors counts four members in vertebrates (TUB, TULP1, TULP2 and TULP3), sharing a similar domain organization including a highly conserved C-terminal domain mediating DNA binding and a divergent N-terminal region encompassing the nuclear localization signal and the transcriptional activation domain implicated in protein–protein binding [11]. A conserved region at the N-terminus enables some members of the Tubby family, including TUB, to bind to the ciliary intraflagellar transport A protein (IFTAP) [12]. Similar to the other members of the TULP family, TUB is also implicated in the control of the initiation of phagocytosis, facilitating the removal of apoptotic cells or cellular debris by retinal pigmented epithelium (RPE) cells and macrophages [13]. Since the original report, no other subject carrying biallelicTUBvariants has been described.
+In this study, we report on an additional subject with retinal dystrophy carrying a homozygous LoF variant inTUB. In vitro analyses provide evidence of the disruptive functional impact of the variant onTUBtranscript processing. We also show that the loss of TUB is associated with a defective cilium morphology and biogenesis in the primary patient’s fibroblasts. Our findings confirm the involvement of defective TUB function in retinal dystrophy and define this disorder as a novel ciliopathy.
+The proband is a 35-year-old male, the first child of healthy non-consanguineous parents of European descent (Figure 1). Family history was negative for retinal diseases or other congenital defects. The proband was born at term after an uneventful pregnancy. Length and weight at birth were reported as within the normal range. Apgar score was 8–10. No hearing impairment and/or learning difficulties were documented during the first year of age.
+At 5 years, the subject required consulting ophthalmologists for referring color blindness. A “blonde” aspect of the fundus oculi was observed and reduced full-field flash photopic and scotopic electroretinogram (ERG) responses were recorded. Visual acuity was not investigated at that time. Ophthalmological assessment at 26 years was suggestive of cone-rod dystrophy. Visual acuity was 0.8 Snellen in his right eye (RE) with myopic and astigmatic refractive error (RE: -4.50 dioptre sphere and -1 dioptre cylinder at 20°), and 0.2 Snellen in his left eye (LE) with myopic refractive error (LE: -2.00 dioptre sphere). Goldmann visual field was generally constricted, with reduced sensitivity in the superior central field in the RE and presented peripheral constriction and relative central scotoma in the LE. Light and dark adaptation sensitivity curves showed abnormal thresholds for both cones and rods. No number at the Ishihara charts were recognized. Intraocular pressure was within normal limits. The slit lamp examination biomicroscopy of the anterior segment was normal for cornea, iris and lens appearance. Fundus examination revealed bilateral optic disc pallor, depigmented aspect of the choroidal and retinal structures, diffuse retinal dystrophy with absence of intraretinal pigment dispersion or vitreous abnormalities and arteriolar attenuation. Full-field scotopic and photopic electroretinograms showed reduced a-wave and b-wave amplitude responses and delayed implicit times. Multifocal ERG ring analysis documented reduced response amplitude densities in all examined areas from the foveal center up to 20° of foveal eccentricity in both eyes (LE &gt; RE). After reduced visual field in his LE, a large area of retinoschisis in the infero-temporal sector was observed by fundoscopy, which later progressed, resulting in full retinal detachment of the LE. The subject underwent to pars plana vitrectomy with silicon oil (30% polydimethylsiloxane, PDMS) tamponade. He underwent cataract surgery in his LE and to subsequent vitreo-retinal surgeries for relapsing retinal detachments in same eye (PDMS/perfluorocarbon liquid (PFCL)/PDMS tamponades exchange and intra-operatory laser treatment; PDMS/heavy silicon oil tamponades exchange and intra-operatory laser). One year later, he developed vitreo-retinal proliferation and retinal fibrosis in the LE, and visual acuity was hand motion; therefore, the subject underwent retinotomy and heavy silicon oil/PDMS tamponades exchange.
+At last evaluation (35 years), the subject presented with a good clinical condition. No cognitive deficit nor behavioral issues were observed, and no craniofacial dysmorphism and truncal obesity were noticed. An accurate endocrinological examination was uninformative. Anthropometric assessment displayed a height of 177.5 cm (+0.1 SD), weight of 95.70 kg (+1.6 SD), and OFC 60 cm (+0.2 SD) and BMI of 30.30 Kg/m2(+1.6 SD). Tanner stage was Ph5Pg5, with a testicular volume 20 mL bilaterally. The subject’s visual acuity was 0.8 Snellen in his RE and light perception in his LE. Fundus oculi showed the unmodified condition of RE and diffuse chorio-retinal atrophy in the LE, as for visible vitreo-retinal surgical outcomes. Ultrawide field fundus photography showed macular atrophy in absence of peripheral pigment and confirmed a “blonde” aspect of the retina (Figure 2A). Fundus autofluorescence (FAF) revealed an hypoautoflorescent area in the macula due to RPE atrophy and hyper/hypoautofluorescence mottling in the posterior pole and immediately outside the vascular arcades (Figure 2B). The SD-OCT showed a disruption of the outer retina, including ELM, ellipsoid zone and RPE with outer retinal debris at the level of the RPE in the parafoveal region (Figure 2C). Full-field flash scotopic (Figure 2D) and photopic ERG confirmed reduced a-wave and b-wave amplitude responses and delayed implicit times in the RE. Similarly, multifocal ERG ring analysis, recordable only in the RE, showed the worsening of the response amplitude densities in all examined areas (0–20°) (Figure 2E), as compared to the previous examinations. Similarly, Goldmann visual field in his RE showed progressive constriction of the peripheral isopters and a ring scotoma enclosed between 10–20° of the visual field (Figure 2F); it was not executable, however, in his LE. Color blindness was also confirmed. Neck and abdominal ultrasound assessment did not reveal any abnormality. Measurements of basal hormones by the anterior pituitary, glycaemia and insulin were within the normal range. Basal plasma leptin level was in the low normal range, showing no leptin resistance. During his follow-up, clinical and ophthalmological assessments of other family members (parents and younger brother) were unremarkable.
+Trio-based WES allowed to identify a homozygous splice siteTUBvariant (chr11:8122545G &gt; A, GRCh37.p13; c.1387 + 1G &gt; A,NM_177972.3) as the only clinically and functionally relevant event putatively linked to the disorder (Supplemental Table S1). The variant had previously been annotated in public databases (dbSNP, rs1040410003) with low frequency (gnomAD v3.1, MAF = 0.00001972) at the heterozygous state. It was classified as likely pathogenic (PVS1/PM2/PP5) according to the American College of Medical Genetics and Genomics-Association for Molecular Pathology (ACMG-AMP) criteria (ClinVar: VCV000865971.1) [14]. Sanger sequencing confirmed the homozygosity for the variant in the proband and the heterozygous status in the healthy parents and unaffected sib (Figure 1).
+Since the variant was predicted to affect the exon 11 donor splice site, the total RNA from patient-derived skin primary fibroblasts was used to characterize the impact of the nucleotide change on transcript processing. The cDNA fragment encompassing the relevant exons was amplified, confirming the presence of two aberrantly spliced products (Figure 3A). The two aberrant PCR amplicons were isolated from agarose gel, purified and sequenced via Sanger. The former (500 bp) was derived from skipping of the penultimate exon (exon 11, ENST00000299506.3), resulting in a premature termination codon (i.e., p.Glu406Argfs*4), while the latter (1172 bp) was the result of retention of intron 10, resulting in a TUB protein having a divergent 19-residue-long C-terminus and lacking the last 44 amino acids (p.Pro463Hisfs*19) (Figure 3B).
+In the patient’s skin fibroblasts, the predicted TUBGlu406Argfs*4protein was undetectable by Western blot [WB] analysis, while the TUBPro463Hisfs*19protein was poorly detectable likely due to accelerated degradation (Figure 3C, left panel). Consistently, the endogenous TUBPro463Hisfs*19level was partially rescued by blocking the proteasomal degradation pathway using MG132 (Figure 3C, right panel).
+To investigate the cellular localization of the mutated protein, cytoplasm and nuclear cell fractions were obtained and analyzed by WB. The results demonstrate that both the wild-type (wt) and mutant TUB proteins were almost exclusively localized in the nucleus (Figure 3D). This finding was also confirmed by confocal microscopy analysis that evidenced the nuclear localization of the TUB mutant (Figure 4A).
+Based on the documented role of TUB in early ciliogenesis [15], we assessed the localization of TUB at the cilium, but we failed to observe any consistent co-localization, possibly due to the low diffused levels of the protein in the cytoplasm To investigate the impact of defective TUB function on the morphogenesis of the primary cilium, a confocal analysis on primary fibroblasts was performed using antibodies against ARL13B, which localizes to primary cilia, and pericentrin, a component of the centrosome, which stains the basal body. As shown inFigure 4B, while almost all the control cells showed a primary cilium, 40% of the fibroblasts carrying the homozygous splice site variant inTUBdid not show a primary cilium. Moreover, while no significant difference was observed in ciliary axoneme length between the starved control and mutant cells, a large percentage of the latter showed an abnormal cilium morphology and a poorly defined and disorganized basal body (Figure 4C).
+The loss of TUB function was recently reported to underlie a novel IRD condition based on the identification of homozygosity for a 2 bp deletion (c.1194_1195delAG) causing the premature termination of the protein (p.Arg398Serfs*9) shared by three affected members of a single consanguineous family [10]. While the combination of retinal dystrophy and early onset obesity can be reminiscent of other disorders (e.g., Bardet–Biedl syndrome (MIM#PS209900) and Alstrom syndrome (MIM#203800)), the absence of other clinically relevant feature/sign was suggestive of a previously unreported ciliopathy [10]. In this paper, we report on a second disruptive variant (c.1387 + 1G &gt; A) affectingTUBin a subject with features that overlap with those previously described in the affected members of the original family.
+In the present and previously reported affected individuals, the ocular phenotype associated with defective TUB function is characterized by widespread retinal pigment epithelial (RPE) atrophy, deteriorating vision, the myopic and astigmatic refractive defect, the blonde fundus appearance, the ERG and OCT findings and progression of the disease (Figure 2). Notably, retinal detachment, without vitreous hemorrhage, was invariantly documented in the four individuals with biallelic inactivatingTUBvariants, suggesting that this feature likely represent a common finding in the disorder.
+Early onset obesity had previously been considered a major feature of the TUB-related condition [10], even though only two of three affected sibs were found obese (BMI &gt; 30), and the glycemic and lipid profiles in one of affected sibs were found within the normal range. The finding of obesity in the apparently healthy father (heterozygous carrier) suggests a possible co-occurring genetic event contributing to obesity in the family. In the present report, the clinical assessment of the affected individual documented increased weight (95.7 kg, +1.6 SD) and BMI (30.3, +1.6 SD), thus indicating overweight, in absence of other signs of obesity. Although evidence suggests that a defective TUB function may result in disturbances in insulin and leptin activity and obesity in mice [16,17,18,19], based on the collected findings, the relevance of TUB in human obesity requires further study. To assess whether TUB LoF could impact on hypothalamic pathways, food intake and adiposity, the metabolic profile of the affected individual was investigated. Accurate endocrinological examination did not reveal any abnormality, and the measurements of basal hormones by the anterior pituitary, glycaemia, insulin and leptin were within the normal range, thus ruling out insulin or leptin resistance. Consistently, instrumental investigations (X-ray and ultrasound analyses) documented no sign of glycogen accumulation in the internal organs. Consistently, the absence of significant changes in lipid storage was demonstrated by thin-layer chromatography (HPTLC) analysis in proband-derived fibroblast (Figure S1), allowing to confirm an apparently normal endocrine–metabolic profile in the affected individual. Of note, the Tubby protein has been involved in cochlear degeneration [20,21]. Based on this functional link, we evaluated the occurrence of hearing problems and cochlear degeneration, which were not observed.
+The homozygousTUBvariant was predicted to affect transcript processing, causing the skipping of exon 11 and intron retention, resulting in a frameshift with the premature termination of the TUB protein. mRNA analysis in proband-derived fibroblasts confirmed a disruptive impact of the splice site change documenting two aberrantly processed transcripts predicted to encode a 406-residue-long protein (p.Glu406Argfs*4) that probably is not able to proceed in protein synthesis, and a 481-residue-long protein (p.Pro463Hisfs*19) characterized by a divergent C-terminus characterized by accelerated degradation (Figure 3B). These findings confirm LoF as the pathomechanism underlying this disorder.
+Primary cilia are microtubule-based organelles that extend from the apical surface of the majority of mammalian cells. Cilia act as “cellular antennae”, receiving different inputs from the extracellular environment and transducing signals in response to stimuli [22]. A complex process required for proper cilia biogenesis function is the intraflagellar transport, which is required for assembling cilia and trafficking within primary cilia [23]. In this context, IFT-A has historically been believed to mediate retrograde intraflagellar transport inside the cilia and an IFT-A-binding domain at the TUB N-terminus has been demonstrated recently [24]. Moreover, co-localization between TUB and rootletin, the major structural component of the ciliary rootlet, has been observed in human retinal photoreceptors [10]. The use of a more informative in vitro model (e.g., induced pluripotent-stem-cell-derived retinal-pigment epithelium cells) and experimental strategies (e.g., siRNA-mediated TUB silencing) is required to appreciate more accurately the functional relevance of TUB in an appropriate cellular context.
+In summary, we confirm the link between TUB LoF and a new condition of human retinal ciliopathy and provide evidence of an altered cilium morphology/biogenesis in patient-derived fibroblasts. In fact, these cells displayed a reduced number of cilia when compared to the control cells, with a poorly defined and disorganized basal body structure, which are expected to prevent normal protein trafficking along the cilium. While these findings could explain the degeneration of photoreceptors characterizing this disorder, a relatively overall mild presentation has been associated with mutations in this gene. Multiple factors might contribute to this picture. First, the functional relevance of TUB in the context of ciliogenesis and cilium function might vary in different cell lineages. Second, functional compensation exerted by other related proteins might contribute to buffer the severity of the endophenotype. Third, specific cell lineages (e.g., rod and cone cells) might be particularly sensitive to TUB LoF. The collection of additional patients with biallelic variants in the gene will allow a more accurate characterization of the clinical spectrum associated with TUB LoF. Based on these considerations, TUB loss of function could be considered as responsible for a novel form of isolated retinal ciliopathy.</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>{
+"pmid": "9390831",
+"alias_symbol": "rd5",
+"primary_gene_symbol": "TUB",
+"name": "TUB bipartite transcription factor",
+"alternate_abbreviation": "NO",
+"evidence": ""
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HGNC:12406</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ENSG00000166402</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GENE ID:7275</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TUB</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>rd5</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>9390831</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>mouse phenotype biomarker</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Mice homozygous for a defect of the tub (rd5) gene exhibit cochlear and retinal degeneration combined with obesity, and resemble certain human autosomal recessive sensory deficit syndromes.</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>TUB bipartite transcription factor</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>In this paper, we confirm that biallelic inactivating variants in TUB cause a retinal disorder and functionally associate this condition with the occurrence of defects of the basal body structure and axoneme morphology of the primary cilium and overall defective ciliogenesis. Although the present findings suggest that TUB plays a role in the pathogenesis of retinal ciliopathies, dedicated functional studies are required to profile the mechanism of disease. This work confirms the clinical relevance of biallelic LoF variants ofTUB, which should be considered in clinical settings and the genetic diagnosis of IRD disorders.
+The present research followed the tenets of the Helsinki Declaration (1964 and further revisions) and the study was approved by the local ethics committee (Comitato Etico Centrale IRCCS Lazio, Sezione IFO/Fondazione Bietti, Rome, Italy). Upon recruitment in the study (FB RET-02-2019), executed from February to July 2019 at the IRCCS Fondazione Bietti, informed consent after full explanation was obtained from each subject included in the study.
+The proband and his family underwent comprehensive ophthalmological examination including visual acuity measured by the Early Treatment Diabetic Retinopathy Study (ETDRS) charts (Lighthouse, Low Vision Products, Long Island City, NY, USA) at the distance of 4 m and expressed as the logarithm of the minimum angle of resolution (logMAR); intraocular pressure (IOP) measurement; anterior segment observation by slit-lamp biomicroscopy and fundus examination by indirect ophthalmoscopic examination using + 90D non-contact lens (Volk Optical, Mentor, OH) after pupillary dilatation with tropicamide 1% drops. Goldmann visual field was assessed by kinetic Goldmann perimeter Haag-Streit 940. Chromatic test was evaluated by the monocular administration of Ishihara pseudoisochromatic plates (24 plates edition, Kanehara Trading Inc., Tokyo, Japan) in natural daylight. Electrophysiological assessment included dark-adapted and light-adapted full-field electroretinogram (Retimax Advanced Plus apparatus, CSO, Firenze, Italy) and multifocal electroretinogram (mfERG; VERIS Clinic TM version 4.9; Electro-Diagnostic Imaging, San Mateo, CA, USA) recordings according to the 2011 International Society for Clinical Electrophysiology of Vision (ISCEV) [25] by using the Dawson–Trick–Litzkow (DTL) contact electrodes and having the pupil dilated at 8 mm.
+Retinal imaging was executed by ultrawide field fundus photograph obtained with Optos California (Optos PLC, Dunfermline, Scotland, United Kingdom); FAF was also obtained during the same examination (488 nm excitation, barrier filter transmitted light from 500 to 680 nm, 55°) using Heidelberg Spectralis OCT (HRA + OCT, Heidelberg Engineering, Heidelberg, Germany). SD-OCT scan pattern was acquired with a minimum of a 20 × 20 degree rectangle centered on the fovea and 25-line B-scans spaced 235 μm apart and composed of 50 averaged frames by using the same instrument.
+Karyotype, CGH array and mutation scan by parallel sequencing considering a retinal cone–rod dystrophy panel of 70 genes were informative. Genomic DNA was collected after obtaining written informed consent. Whole-Exome sequencing (WES) and data analysis were performed as previously reported [26,27] (Supplementary Table S1). DNA of the affected subject and his parents was extracted from circulating leukocytes and sequenced using Illumina paired-end technology by means of SureSelect Human All Exon v.7 (Agilent, Santa Clara, CA, USA) kits. WES raw data were processed and analyzed using an in-house implemented pipeline as previously described [28,29], according to the GATK’s Best Practices [30]. The UCSC GRCh37/hg19 version of genome assembly was used as a reference for read alignment by means of BWA-MEM [31] tool and the subsequent variant calling with HaplotypeCaller (GATK v3.7) [28]. Variants’ functional annotation was made with the SnpEff v.5.0 [32] and dbNSFP v.4.2 [33] tools. Relevant in silico impact prediction tools, such as Combined Annotation Dependent Depletion (CADD) v.1.6 [34], Mendelian Clinically Applicable Pathogenicity (M-CAP) v.1.0 [35] and InterVar v.2.0.1 [36], were also used. By filtering against our population-matched database (~2500 WES) and public databases (dbSNP150 and gnomAD v.2.0.1), the analysis focused on high-quality rare variants that affect coding sequences and splice site regions. Sanger sequencing was performed for variant validation and segregation analysis (primers available upon request).
+Proband skin biopsy was obtained after informant consent was secured. Total RNA was extracted from the proband and healthy donor fibroblasts by using RNeasy Mini Kit (Qiagen, Hilden, Germany), according to the manufacturer’s recommendations. Total RNA concentration and quality were assessed by measuring the absorbance at 260 and 280 nm. Reverse transcription was carried out using a SuperScript RT reagent Kit (Invitrogen; ThermoFisher Scientific, Waltham, MA, USA). The obtained cDNA pools were amplified by PCR using specific primers located in exons 10 and 12 of theTUBgene, and PCR products were separated on a 2% agarose gel. The sequences of the primers are available upon request.
+Primary skin fibroblasts were cultured in DMEM supplemented with 10% heat-inactivated FBS, 2 mM glutamine, 100 units/mL of penicillin and 100 µg/mL of streptomycin, and maintained at 37 °C in a humidified atmosphere containing 5% CO2. After treatment, fibroblasts were lysed in RIPA buffer supplemented with phosphatase and protease inhibitors. Lysates were kept on ice (30 min) and then centrifuged at 16,000×g(20 min, 4 °C). Supernatants were collected and protein concentration was determined by Quick Start Bradford Dye Reagent (Bio-Rad Laboratories, Hercules, CA, USA), using bovine serum albumin (BSA) as a standard. Fibroblast homogenates were resolved by SDS PAGE and transferred to nitrocellulose membranes (Bio-Rad Laboratories). Blots were blocked for 1 h with 5% non-fat milk powder in phosphate-buffered saline (PBS) containing 0.1% Tween-20 and incubated overnight with specific antibodies. Anti-TUB primary polyclonal antibody (1:1000, Invitrogen; ThermoFisher Scientific) and goat anti-rabbit-HRP IgG secondary antibody (Invitrogen; ThermoFisher Scientific) were diluted in blocking solution. Immunoreactive proteins were detected by an ECL SuperSignal West Femto Maximum Sensitivity Chemiluminescent Substrate, according to the manufacturer’s instructions (Thermo Scientific, USA).
+Approximately 3 × 104/mL fibroblasts were seeded on glass coverslips and maintained in culture in complete medium for 24 h. Subconfluent fibroblasts were starved for 30 h and then fixed with 4% paraformaldehyde. Subsequently, cells were stained with rabbit anti-TUB (1:100 dilution), rabbit polyclonal anti-ARL13B (1:100, Abcam, Cambridge, UK) and mouse monoclonal anti-Pericentrin (1:100, Abcam) antibodies followed by goat anti-rabbit Alexa Fluor 488 and goat anti-mouse Alex Fluor 594, respectively (1:200 dilution; Molecular Probes, Eugene, OR, USA). After staining, coverslips were extensively rinsed and mounted onto microscope slides using Vectashield with DAPI mounting medium (Vector Laboratories, Newark, CA, USA). Analyses were performed in three independent experiments on a Zeiss LSM980 (Zeiss, Oberkochen, Germany) using a 63×/1.4 N.A. oil objective and excitation spectral laser lines at 405, 488 and 594 nm. Five hundred cells were counted for each condition in each experiment, and axoneme length was measured for each cell by using Zen Blue 3.2 software. Image acquisition and processing were performed as previously reported [37].
+Control and mutated fibroblasts cultured in 150 cm2dishes were harvested using trypsin after reaching confluence, rinsed with phosphate-buffered saline (PBS) and pelleted by centrifugation. Cell pellets were resuspended in 1 mL 0.9% NaCl and 6 mL of chloroform/methanol (2:1, v/v) were added. Mixtures were vortexed vigorously and centrifuged at 1500×gfor 15 min; the aqueous phase was discarded and organic phase was dried under N2gas. Lipid extracts from 1.5 × 106cells were applied on high-performance thin-layer chromatography (HPTLC) silica gel 60 plates (Merck, Darmstadt, Germany). Neutral lipids were resolved using a solvent system of hexane/diethyl ether/acetic acid (70:30:1, v/v/v) and were detected by staining with an aqueous solution containing 3% cupric acetate and 8% phosphoric acid and subsequent charring at 140 °C for 10 min. Lipids were identified by the co-migration of commercially available standards.
+URLs.*Online Mendelian Inheritance in Man [OMIM],http://www.ncbi.nlm.nih.gov/omim/;
+NCBI Gene,http://www.ncbi.nlm.nih.gov/gene/;
+Picard tools,http://picard.sourceforge.net/;
+wAnnovar,http://wannovar.usc.edu/;
+dbSNP137,http://www.ncbi.nlm.nih.gov/projects/SNP/snp_summary.cgi/;
+1000 Genomes Project,http://www.1000genomes.org/;
+HapMap Project,http://hapmap.ncbi.nlm.nih.gov/;
+SMART,http://smart.embl-heidelberg.de/;
+Protein Data Bank [PDB],http://www.rcsb.org/pdb/home/home.do.
+Research for this study was supported by the Ministry of Health funding 5x1000 Fondazione G.B. Bietti funds—2016 to M.P. and Fondazione Roma; Bando Ricerca Indipendente ISS 2021–2023 to V.C., Istituto Superiore di Sanità; Italian Ministry of Health (CCR-2017-23669081 to M.T.), and Italian Ministry of Research (FOE_2019 to M.T.). The authors acknowledge Maria Luisa Alessi and Federica Petrocchi for technical help in the electrophysiological and perimetric evaluations, Serenella Venanzi for administrative assistance.
+Publisher’s Note:MDPI stays neutral with regard to jurisdictional claims in published maps and institutional affiliations.
+The following supporting information can be downloaded at:https://www.mdpi.com/article/10.3390/ijms232314656/s1.
+Click here for additional data file.
+Conceptualization, L.Z. and V.C.; methodology, C.M., E.S., S.C., L.B. and M.T. (Massimo Tatti); validation, E.C., L.B., C.M. and V.C.; bioinformatics analysis, A.C. and A.B.; investigation, L.Z., M.C., M.P. and E.C.; resources, M.V.; data curation, L.B., M.P., E.S., M.T. (Massimo Tatti), M.N. and V.C.; writing—original draft preparation, L.Z., V.C. and M.N.; writing—review and editing, M.N., E.S., M.C., M.T. (Marco Tartaglia) and V.C.; supervision, M.V. and M.T. (Marco Tartaglia); project administration, M.V., V.C. and M.T. (Marco Tartaglia); funding acquisition, M.V. and M.P. All authors have read and agreed to the published version of the manuscript.
+The study was conducted according to the guidelines of the Declaration of Helsinki and was approved by the local Institutional Ethical Committee of the IRCCS_Fondazione G.B. Bietti [Ret_02/2019].
+Signed informed consent was obtained from the participating family.
+Data that support the findings of this study are available from the corresponding authors upon request.
+The authors declare no conflict of interest.
+Family tree showing the segregation of the identified splice site change.
+Ocular phenotype of the proband right eye. (A) Ultrawide field color fundus photograph. (B) The 55° fundus autofluorescence. (C) Spectral-domain optical coherence tomography line horizontal scan. (D) Full-field dark-adapted electroretinogram. (E) Three-dimensional multifocal electroretinogram plot. (F) Goldmann kinetic visual field.
+Characterization of the pathogenicTUBvariant. (A) Transcript processing in primary skin fibroblasts from a healthy donor and from the proband carrying the homozygous splice site variant. Total RNA was extracted, reverse-transcribed and analyzed by PCR to resolve transcript processing. Two aberrant cDNA products were identified in mutated cells (left) compared to the expected length of the amplified fragment obtained from the control fibroblasts (right). (B) Schematic representation of aberrant transcript processing caused by the identified homozygous splice site change inTUB. (C) Western blot analysis of the TUB protein in patient’s fibroblasts and the control cells. Twenty, forty and sixty micrograms of whole cell extract were analyzed basally (left) and following 4 h treatment with 100 μM Mg132 (right) and probed with anti-TUB antibody (* indicates a non-specific product). (D) Expression of wild-type and mutant TUB protein was analyzed in the cytoplasmic and nuclear fractions were obtained from wild-type and mutated fibroblasts. Sixty micrograms of each fraction were analyzed by Western blot and then probed with anti-TUB antibody. Anti-YY1 and anti-HSP90 antibodies were used as the internal controls to assess the clarity of the different fractions (* indicates a non-specific product). Blots are representative of three experiments performed.
+TUB subcellular localization and cilium defects in cells with TUB LoF. (A) Thirty-hour-starved and PFA-fixed fibroblasts from a healthy donor and from the proband were analyzed by confocal microscopy for the localization of TUB using antibodies against TUB. (B) The presence and morphology of primary cilia in starved fibroblasts from the proband and a healthy donor. Cells were starved for 30 h and fixed with PFA 4%. Primary cilia were analyzed using antibodies against ARL13B (cilium axonemal, green) and pericentrin (basal body, red) to investigate morphogenesis. Nuclei are DAPI stained (blue). Bars correspond to 20 and 2 μm (left panels). (C) Histograms represent the percent value of presence/absence of cilium, normal/aberrant cilium morphology and normal/aberrant basal body structure and the length (μm) of axoneme. Five hundred cells were counted for each condition and axoneme length was measured. Imagines and bar plots are representative of three experiments performed. * indicate statistical significance forp&lt; 0.01 by using Student’sTtest.</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Mice homozygous for a defect of the tub (rd5) gene exhibit cochlear and retinal degeneration combined with obesity, and resemble certain human autosomal recessive sensory deficit syndromes. To establish the progressive nature of sensory cell loss associated with the tub gene, and to differentiate tub-related losses from those associated with the C57 background on which tub arose, we evaluated cochleas and retinas from tub/tub, tub/+, and +/+ mice, aged 2 weeks to 1 year by light and electron microscopy. Cochleas from mice of all three genotypes show progressive inner (IHC) and outer hair cell (OHC) loss. Relative to tub/+ and +/+ animals, however, tub homozygotes show accelerated OHC loss, affecting the extreme cochlear base (hook region) by 1 month, and the apex by 6 months. IHC loss in tub/tub animals is accelerated in the basal half of the cochlea, affecting the hook region by 6 months. Spiral ganglion cell losses were observed only in tub/tub mice, and only in the cochlear base. Retinas of tub/tub mice are abnormal at maturity, exhibiting shortened photoreceptor outer segments by 2 weeks, and progressive photoreceptor loss thereafter. Because the tub mutation causes degeneration of sensory cells in the ear and eye but has no other neurological effects, tubby mice hold unique promise for the study of human syndromic sensory loss.</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>PMID: 9390831
+Full Text: In this paper, we confirm that biallelic inactivating variants in TUB cause a retinal disorder and functionally associate this condition with the occurrence of defects of the basal body structure and axoneme morphology of the primary cilium and overall defective ciliogenesis. Although the present findings suggest that TUB plays a role in the pathogenesis of retinal ciliopathies, dedicated functional studies are required to profile the mechanism of disease. This work confirms the clinical relevance of biallelic LoF variants ofTUB, which should be considered in clinical settings and the genetic diagnosis of IRD disorders.
+The present research followed the tenets of the Helsinki Declaration (1964 and further revisions) and the study was approved by the local ethics committee (Comitato Etico Centrale IRCCS Lazio, Sezione IFO/Fondazione Bietti, Rome, Italy). Upon recruitment in the study (FB RET-02-2019), executed from February to July 2019 at the IRCCS Fondazione Bietti, informed consent after full explanation was obtained from each subject included in the study.
+The proband and his family underwent comprehensive ophthalmological examination including visual acuity measured by the Early Treatment Diabetic Retinopathy Study (ETDRS) charts (Lighthouse, Low Vision Products, Long Island City, NY, USA) at the distance of 4 m and expressed as the logarithm of the minimum angle of resolution (logMAR); intraocular pressure (IOP) measurement; anterior segment observation by slit-lamp biomicroscopy and fundus examination by indirect ophthalmoscopic examination using + 90D non-contact lens (Volk Optical, Mentor, OH) after pupillary dilatation with tropicamide 1% drops. Goldmann visual field was assessed by kinetic Goldmann perimeter Haag-Streit 940. Chromatic test was evaluated by the monocular administration of Ishihara pseudoisochromatic plates (24 plates edition, Kanehara Trading Inc., Tokyo, Japan) in natural daylight. Electrophysiological assessment included dark-adapted and light-adapted full-field electroretinogram (Retimax Advanced Plus apparatus, CSO, Firenze, Italy) and multifocal electroretinogram (mfERG; VERIS Clinic TM version 4.9; Electro-Diagnostic Imaging, San Mateo, CA, USA) recordings according to the 2011 International Society for Clinical Electrophysiology of Vision (ISCEV) [25] by using the Dawson–Trick–Litzkow (DTL) contact electrodes and having the pupil dilated at 8 mm.
+Retinal imaging was executed by ultrawide field fundus photograph obtained with Optos California (Optos PLC, Dunfermline, Scotland, United Kingdom); FAF was also obtained during the same examination (488 nm excitation, barrier filter transmitted light from 500 to 680 nm, 55°) using Heidelberg Spectralis OCT (HRA + OCT, Heidelberg Engineering, Heidelberg, Germany). SD-OCT scan pattern was acquired with a minimum of a 20 × 20 degree rectangle centered on the fovea and 25-line B-scans spaced 235 μm apart and composed of 50 averaged frames by using the same instrument.
+Karyotype, CGH array and mutation scan by parallel sequencing considering a retinal cone–rod dystrophy panel of 70 genes were informative. Genomic DNA was collected after obtaining written informed consent. Whole-Exome sequencing (WES) and data analysis were performed as previously reported [26,27] (Supplementary Table S1). DNA of the affected subject and his parents was extracted from circulating leukocytes and sequenced using Illumina paired-end technology by means of SureSelect Human All Exon v.7 (Agilent, Santa Clara, CA, USA) kits. WES raw data were processed and analyzed using an in-house implemented pipeline as previously described [28,29], according to the GATK’s Best Practices [30]. The UCSC GRCh37/hg19 version of genome assembly was used as a reference for read alignment by means of BWA-MEM [31] tool and the subsequent variant calling with HaplotypeCaller (GATK v3.7) [28]. Variants’ functional annotation was made with the SnpEff v.5.0 [32] and dbNSFP v.4.2 [33] tools. Relevant in silico impact prediction tools, such as Combined Annotation Dependent Depletion (CADD) v.1.6 [34], Mendelian Clinically Applicable Pathogenicity (M-CAP) v.1.0 [35] and InterVar v.2.0.1 [36], were also used. By filtering against our population-matched database (~2500 WES) and public databases (dbSNP150 and gnomAD v.2.0.1), the analysis focused on high-quality rare variants that affect coding sequences and splice site regions. Sanger sequencing was performed for variant validation and segregation analysis (primers available upon request).
+Proband skin biopsy was obtained after informant consent was secured. Total RNA was extracted from the proband and healthy donor fibroblasts by using RNeasy Mini Kit (Qiagen, Hilden, Germany), according to the manufacturer’s recommendations. Total RNA concentration and quality were assessed by measuring the absorbance at 260 and 280 nm. Reverse transcription was carried out using a SuperScript RT reagent Kit (Invitrogen; ThermoFisher Scientific, Waltham, MA, USA). The obtained cDNA pools were amplified by PCR using specific primers located in exons 10 and 12 of theTUBgene, and PCR products were separated on a 2% agarose gel. The sequences of the primers are available upon request.
+Primary skin fibroblasts were cultured in DMEM supplemented with 10% heat-inactivated FBS, 2 mM glutamine, 100 units/mL of penicillin and 100 µg/mL of streptomycin, and maintained at 37 °C in a humidified atmosphere containing 5% CO2. After treatment, fibroblasts were lysed in RIPA buffer supplemented with phosphatase and protease inhibitors. Lysates were kept on ice (30 min) and then centrifuged at 16,000×g(20 min, 4 °C). Supernatants were collected and protein concentration was determined by Quick Start Bradford Dye Reagent (Bio-Rad Laboratories, Hercules, CA, USA), using bovine serum albumin (BSA) as a standard. Fibroblast homogenates were resolved by SDS PAGE and transferred to nitrocellulose membranes (Bio-Rad Laboratories). Blots were blocked for 1 h with 5% non-fat milk powder in phosphate-buffered saline (PBS) containing 0.1% Tween-20 and incubated overnight with specific antibodies. Anti-TUB primary polyclonal antibody (1:1000, Invitrogen; ThermoFisher Scientific) and goat anti-rabbit-HRP IgG secondary antibody (Invitrogen; ThermoFisher Scientific) were diluted in blocking solution. Immunoreactive proteins were detected by an ECL SuperSignal West Femto Maximum Sensitivity Chemiluminescent Substrate, according to the manufacturer’s instructions (Thermo Scientific, USA).
+Approximately 3 × 104/mL fibroblasts were seeded on glass coverslips and maintained in culture in complete medium for 24 h. Subconfluent fibroblasts were starved for 30 h and then fixed with 4% paraformaldehyde. Subsequently, cells were stained with rabbit anti-TUB (1:100 dilution), rabbit polyclonal anti-ARL13B (1:100, Abcam, Cambridge, UK) and mouse monoclonal anti-Pericentrin (1:100, Abcam) antibodies followed by goat anti-rabbit Alexa Fluor 488 and goat anti-mouse Alex Fluor 594, respectively (1:200 dilution; Molecular Probes, Eugene, OR, USA). After staining, coverslips were extensively rinsed and mounted onto microscope slides using Vectashield with DAPI mounting medium (Vector Laboratories, Newark, CA, USA). Analyses were performed in three independent experiments on a Zeiss LSM980 (Zeiss, Oberkochen, Germany) using a 63×/1.4 N.A. oil objective and excitation spectral laser lines at 405, 488 and 594 nm. Five hundred cells were counted for each condition in each experiment, and axoneme length was measured for each cell by using Zen Blue 3.2 software. Image acquisition and processing were performed as previously reported [37].
+Control and mutated fibroblasts cultured in 150 cm2dishes were harvested using trypsin after reaching confluence, rinsed with phosphate-buffered saline (PBS) and pelleted by centrifugation. Cell pellets were resuspended in 1 mL 0.9% NaCl and 6 mL of chloroform/methanol (2:1, v/v) were added. Mixtures were vortexed vigorously and centrifuged at 1500×gfor 15 min; the aqueous phase was discarded and organic phase was dried under N2gas. Lipid extracts from 1.5 × 106cells were applied on high-performance thin-layer chromatography (HPTLC) silica gel 60 plates (Merck, Darmstadt, Germany). Neutral lipids were resolved using a solvent system of hexane/diethyl ether/acetic acid (70:30:1, v/v/v) and were detected by staining with an aqueous solution containing 3% cupric acetate and 8% phosphoric acid and subsequent charring at 140 °C for 10 min. Lipids were identified by the co-migration of commercially available standards.
+URLs.*Online Mendelian Inheritance in Man [OMIM],http://www.ncbi.nlm.nih.gov/omim/;
+NCBI Gene,http://www.ncbi.nlm.nih.gov/gene/;
+Picard tools,http://picard.sourceforge.net/;
+wAnnovar,http://wannovar.usc.edu/;
+dbSNP137,http://www.ncbi.nlm.nih.gov/projects/SNP/snp_summary.cgi/;
+1000 Genomes Project,http://www.1000genomes.org/;
+HapMap Project,http://hapmap.ncbi.nlm.nih.gov/;
+SMART,http://smart.embl-heidelberg.de/;
+Protein Data Bank [PDB],http://www.rcsb.org/pdb/home/home.do.
+Research for this study was supported by the Ministry of Health funding 5x1000 Fondazione G.B. Bietti funds—2016 to M.P. and Fondazione Roma; Bando Ricerca Indipendente ISS 2021–2023 to V.C., Istituto Superiore di Sanità; Italian Ministry of Health (CCR-2017-23669081 to M.T.), and Italian Ministry of Research (FOE_2019 to M.T.). The authors acknowledge Maria Luisa Alessi and Federica Petrocchi for technical help in the electrophysiological and perimetric evaluations, Serenella Venanzi for administrative assistance.
+Publisher’s Note:MDPI stays neutral with regard to jurisdictional claims in published maps and institutional affiliations.
+The following supporting information can be downloaded at:https://www.mdpi.com/article/10.3390/ijms232314656/s1.
+Click here for additional data file.
+Conceptualization, L.Z. and V.C.; methodology, C.M., E.S., S.C., L.B. and M.T. (Massimo Tatti); validation, E.C., L.B., C.M. and V.C.; bioinformatics analysis, A.C. and A.B.; investigation, L.Z., M.C., M.P. and E.C.; resources, M.V.; data curation, L.B., M.P., E.S., M.T. (Massimo Tatti), M.N. and V.C.; writing—original draft preparation, L.Z., V.C. and M.N.; writing—review and editing, M.N., E.S., M.C., M.T. (Marco Tartaglia) and V.C.; supervision, M.V. and M.T. (Marco Tartaglia); project administration, M.V., V.C. and M.T. (Marco Tartaglia); funding acquisition, M.V. and M.P. All authors have read and agreed to the published version of the manuscript.
+The study was conducted according to the guidelines of the Declaration of Helsinki and was approved by the local Institutional Ethical Committee of the IRCCS_Fondazione G.B. Bietti [Ret_02/2019].
+Signed informed consent was obtained from the participating family.
+Data that support the findings of this study are available from the corresponding authors upon request.
+The authors declare no conflict of interest.
+Family tree showing the segregation of the identified splice site change.
+Ocular phenotype of the proband right eye. (A) Ultrawide field color fundus photograph. (B) The 55° fundus autofluorescence. (C) Spectral-domain optical coherence tomography line horizontal scan. (D) Full-field dark-adapted electroretinogram. (E) Three-dimensional multifocal electroretinogram plot. (F) Goldmann kinetic visual field.
+Characterization of the pathogenicTUBvariant. (A) Transcript processing in primary skin fibroblasts from a healthy donor and from the proband carrying the homozygous splice site variant. Total RNA was extracted, reverse-transcribed and analyzed by PCR to resolve transcript processing. Two aberrant cDNA products were identified in mutated cells (left) compared to the expected length of the amplified fragment obtained from the control fibroblasts (right). (B) Schematic representation of aberrant transcript processing caused by the identified homozygous splice site change inTUB. (C) Western blot analysis of the TUB protein in patient’s fibroblasts and the control cells. Twenty, forty and sixty micrograms of whole cell extract were analyzed basally (left) and following 4 h treatment with 100 μM Mg132 (right) and probed with anti-TUB antibody (* indicates a non-specific product). (D) Expression of wild-type and mutant TUB protein was analyzed in the cytoplasmic and nuclear fractions were obtained from wild-type and mutated fibroblasts. Sixty micrograms of each fraction were analyzed by Western blot and then probed with anti-TUB antibody. Anti-YY1 and anti-HSP90 antibodies were used as the internal controls to assess the clarity of the different fractions (* indicates a non-specific product). Blots are representative of three experiments performed.
+TUB subcellular localization and cilium defects in cells with TUB LoF. (A) Thirty-hour-starved and PFA-fixed fibroblasts from a healthy donor and from the proband were analyzed by confocal microscopy for the localization of TUB using antibodies against TUB. (B) The presence and morphology of primary cilia in starved fibroblasts from the proband and a healthy donor. Cells were starved for 30 h and fixed with PFA 4%. Primary cilia were analyzed using antibodies against ARL13B (cilium axonemal, green) and pericentrin (basal body, red) to investigate morphogenesis. Nuclei are DAPI stained (blue). Bars correspond to 20 and 2 μm (left panels). (C) Histograms represent the percent value of presence/absence of cilium, normal/aberrant cilium morphology and normal/aberrant basal body structure and the length (μm) of axoneme. Five hundred cells were counted for each condition and axoneme length was measured. Imagines and bar plots are representative of three experiments performed. * indicate statistical significance forp&lt; 0.01 by using Student’sTtest.</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
+    Inputs:
+    Alias gene symbol: rd5
+    HGNC record ID: HGNC:12406
+    Primary gene symbol: TUB
+    Official HGNC gene name: TUB bipartite transcription factor
+    Biomedical text context
+    Task:
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
+    Rules:
+    If the text does not support that the alias is an alternate abbreviation, return:
+    "alternate_abbreviation": "NO"
+    "evidence": ""
+    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
+    Evidence must be one exact sentence copied verbatim from the text.
+    Do not infer relationships or paraphrase evidence.
+    Output (Strict):
+    Output only one JSON object. No markdown.
+    {
+    "pmid": "",
+    "alias_symbol": "",
+    "primary_gene_symbol": "",
+    "name": "",
+    "alternate_abbreviation": "YES or NO",
+    "evidence": ""
+    }
+PMID: 9390831
+Full Text: In this paper, we confirm that biallelic inactivating variants in TUB cause a retinal disorder and functionally associate this condition with the occurrence of defects of the basal body structure and axoneme morphology of the primary cilium and overall defective ciliogenesis. Although the present findings suggest that TUB plays a role in the pathogenesis of retinal ciliopathies, dedicated functional studies are required to profile the mechanism of disease. This work confirms the clinical relevance of biallelic LoF variants ofTUB, which should be considered in clinical settings and the genetic diagnosis of IRD disorders.
+The present research followed the tenets of the Helsinki Declaration (1964 and further revisions) and the study was approved by the local ethics committee (Comitato Etico Centrale IRCCS Lazio, Sezione IFO/Fondazione Bietti, Rome, Italy). Upon recruitment in the study (FB RET-02-2019), executed from February to July 2019 at the IRCCS Fondazione Bietti, informed consent after full explanation was obtained from each subject included in the study.
+The proband and his family underwent comprehensive ophthalmological examination including visual acuity measured by the Early Treatment Diabetic Retinopathy Study (ETDRS) charts (Lighthouse, Low Vision Products, Long Island City, NY, USA) at the distance of 4 m and expressed as the logarithm of the minimum angle of resolution (logMAR); intraocular pressure (IOP) measurement; anterior segment observation by slit-lamp biomicroscopy and fundus examination by indirect ophthalmoscopic examination using + 90D non-contact lens (Volk Optical, Mentor, OH) after pupillary dilatation with tropicamide 1% drops. Goldmann visual field was assessed by kinetic Goldmann perimeter Haag-Streit 940. Chromatic test was evaluated by the monocular administration of Ishihara pseudoisochromatic plates (24 plates edition, Kanehara Trading Inc., Tokyo, Japan) in natural daylight. Electrophysiological assessment included dark-adapted and light-adapted full-field electroretinogram (Retimax Advanced Plus apparatus, CSO, Firenze, Italy) and multifocal electroretinogram (mfERG; VERIS Clinic TM version 4.9; Electro-Diagnostic Imaging, San Mateo, CA, USA) recordings according to the 2011 International Society for Clinical Electrophysiology of Vision (ISCEV) [25] by using the Dawson–Trick–Litzkow (DTL) contact electrodes and having the pupil dilated at 8 mm.
+Retinal imaging was executed by ultrawide field fundus photograph obtained with Optos California (Optos PLC, Dunfermline, Scotland, United Kingdom); FAF was also obtained during the same examination (488 nm excitation, barrier filter transmitted light from 500 to 680 nm, 55°) using Heidelberg Spectralis OCT (HRA + OCT, Heidelberg Engineering, Heidelberg, Germany). SD-OCT scan pattern was acquired with a minimum of a 20 × 20 degree rectangle centered on the fovea and 25-line B-scans spaced 235 μm apart and composed of 50 averaged frames by using the same instrument.
+Karyotype, CGH array and mutation scan by parallel sequencing considering a retinal cone–rod dystrophy panel of 70 genes were informative. Genomic DNA was collected after obtaining written informed consent. Whole-Exome sequencing (WES) and data analysis were performed as previously reported [26,27] (Supplementary Table S1). DNA of the affected subject and his parents was extracted from circulating leukocytes and sequenced using Illumina paired-end technology by means of SureSelect Human All Exon v.7 (Agilent, Santa Clara, CA, USA) kits. WES raw data were processed and analyzed using an in-house implemented pipeline as previously described [28,29], according to the GATK’s Best Practices [30]. The UCSC GRCh37/hg19 version of genome assembly was used as a reference for read alignment by means of BWA-MEM [31] tool and the subsequent variant calling with HaplotypeCaller (GATK v3.7) [28]. Variants’ functional annotation was made with the SnpEff v.5.0 [32] and dbNSFP v.4.2 [33] tools. Relevant in silico impact prediction tools, such as Combined Annotation Dependent Depletion (CADD) v.1.6 [34], Mendelian Clinically Applicable Pathogenicity (M-CAP) v.1.0 [35] and InterVar v.2.0.1 [36], were also used. By filtering against our population-matched database (~2500 WES) and public databases (dbSNP150 and gnomAD v.2.0.1), the analysis focused on high-quality rare variants that affect coding sequences and splice site regions. Sanger sequencing was performed for variant validation and segregation analysis (primers available upon request).
+Proband skin biopsy was obtained after informant consent was secured. Total RNA was extracted from the proband and healthy donor fibroblasts by using RNeasy Mini Kit (Qiagen, Hilden, Germany), according to the manufacturer’s recommendations. Total RNA concentration and quality were assessed by measuring the absorbance at 260 and 280 nm. Reverse transcription was carried out using a SuperScript RT reagent Kit (Invitrogen; ThermoFisher Scientific, Waltham, MA, USA). The obtained cDNA pools were amplified by PCR using specific primers located in exons 10 and 12 of theTUBgene, and PCR products were separated on a 2% agarose gel. The sequences of the primers are available upon request.
+Primary skin fibroblasts were cultured in DMEM supplemented with 10% heat-inactivated FBS, 2 mM glutamine, 100 units/mL of penicillin and 100 µg/mL of streptomycin, and maintained at 37 °C in a humidified atmosphere containing 5% CO2. After treatment, fibroblasts were lysed in RIPA buffer supplemented with phosphatase and protease inhibitors. Lysates were kept on ice (30 min) and then centrifuged at 16,000×g(20 min, 4 °C). Supernatants were collected and protein concentration was determined by Quick Start Bradford Dye Reagent (Bio-Rad Laboratories, Hercules, CA, USA), using bovine serum albumin (BSA) as a standard. Fibroblast homogenates were resolved by SDS PAGE and transferred to nitrocellulose membranes (Bio-Rad Laboratories). Blots were blocked for 1 h with 5% non-fat milk powder in phosphate-buffered saline (PBS) containing 0.1% Tween-20 and incubated overnight with specific antibodies. Anti-TUB primary polyclonal antibody (1:1000, Invitrogen; ThermoFisher Scientific) and goat anti-rabbit-HRP IgG secondary antibody (Invitrogen; ThermoFisher Scientific) were diluted in blocking solution. Immunoreactive proteins were detected by an ECL SuperSignal West Femto Maximum Sensitivity Chemiluminescent Substrate, according to the manufacturer’s instructions (Thermo Scientific, USA).
+Approximately 3 × 104/mL fibroblasts were seeded on glass coverslips and maintained in culture in complete medium for 24 h. Subconfluent fibroblasts were starved for 30 h and then fixed with 4% paraformaldehyde. Subsequently, cells were stained with rabbit anti-TUB (1:100 dilution), rabbit polyclonal anti-ARL13B (1:100, Abcam, Cambridge, UK) and mouse monoclonal anti-Pericentrin (1:100, Abcam) antibodies followed by goat anti-rabbit Alexa Fluor 488 and goat anti-mouse Alex Fluor 594, respectively (1:200 dilution; Molecular Probes, Eugene, OR, USA). After staining, coverslips were extensively rinsed and mounted onto microscope slides using Vectashield with DAPI mounting medium (Vector Laboratories, Newark, CA, USA). Analyses were performed in three independent experiments on a Zeiss LSM980 (Zeiss, Oberkochen, Germany) using a 63×/1.4 N.A. oil objective and excitation spectral laser lines at 405, 488 and 594 nm. Five hundred cells were counted for each condition in each experiment, and axoneme length was measured for each cell by using Zen Blue 3.2 software. Image acquisition and processing were performed as previously reported [37].
+Control and mutated fibroblasts cultured in 150 cm2dishes were harvested using trypsin after reaching confluence, rinsed with phosphate-buffered saline (PBS) and pelleted by centrifugation. Cell pellets were resuspended in 1 mL 0.9% NaCl and 6 mL of chloroform/methanol (2:1, v/v) were added. Mixtures were vortexed vigorously and centrifuged at 1500×gfor 15 min; the aqueous phase was discarded and organic phase was dried under N2gas. Lipid extracts from 1.5 × 106cells were applied on high-performance thin-layer chromatography (HPTLC) silica gel 60 plates (Merck, Darmstadt, Germany). Neutral lipids were resolved using a solvent system of hexane/diethyl ether/acetic acid (70:30:1, v/v/v) and were detected by staining with an aqueous solution containing 3% cupric acetate and 8% phosphoric acid and subsequent charring at 140 °C for 10 min. Lipids were identified by the co-migration of commercially available standards.
+URLs.*Online Mendelian Inheritance in Man [OMIM],http://www.ncbi.nlm.nih.gov/omim/;
+NCBI Gene,http://www.ncbi.nlm.nih.gov/gene/;
+Picard tools,http://picard.sourceforge.net/;
+wAnnovar,http://wannovar.usc.edu/;
+dbSNP137,http://www.ncbi.nlm.nih.gov/projects/SNP/snp_summary.cgi/;
+1000 Genomes Project,http://www.1000genomes.org/;
+HapMap Project,http://hapmap.ncbi.nlm.nih.gov/;
+SMART,http://smart.embl-heidelberg.de/;
+Protein Data Bank [PDB],http://www.rcsb.org/pdb/home/home.do.
+Research for this study was supported by the Ministry of Health funding 5x1000 Fondazione G.B. Bietti funds—2016 to M.P. and Fondazione Roma; Bando Ricerca Indipendente ISS 2021–2023 to V.C., Istituto Superiore di Sanità; Italian Ministry of Health (CCR-2017-23669081 to M.T.), and Italian Ministry of Research (FOE_2019 to M.T.). The authors acknowledge Maria Luisa Alessi and Federica Petrocchi for technical help in the electrophysiological and perimetric evaluations, Serenella Venanzi for administrative assistance.
+Publisher’s Note:MDPI stays neutral with regard to jurisdictional claims in published maps and institutional affiliations.
+The following supporting information can be downloaded at:https://www.mdpi.com/article/10.3390/ijms232314656/s1.
+Click here for additional data file.
+Conceptualization, L.Z. and V.C.; methodology, C.M., E.S., S.C., L.B. and M.T. (Massimo Tatti); validation, E.C., L.B., C.M. and V.C.; bioinformatics analysis, A.C. and A.B.; investigation, L.Z., M.C., M.P. and E.C.; resources, M.V.; data curation, L.B., M.P., E.S., M.T. (Massimo Tatti), M.N. and V.C.; writing—original draft preparation, L.Z., V.C. and M.N.; writing—review and editing, M.N., E.S., M.C., M.T. (Marco Tartaglia) and V.C.; supervision, M.V. and M.T. (Marco Tartaglia); project administration, M.V., V.C. and M.T. (Marco Tartaglia); funding acquisition, M.V. and M.P. All authors have read and agreed to the published version of the manuscript.
+The study was conducted according to the guidelines of the Declaration of Helsinki and was approved by the local Institutional Ethical Committee of the IRCCS_Fondazione G.B. Bietti [Ret_02/2019].
+Signed informed consent was obtained from the participating family.
+Data that support the findings of this study are available from the corresponding authors upon request.
+The authors declare no conflict of interest.
+Family tree showing the segregation of the identified splice site change.
+Ocular phenotype of the proband right eye. (A) Ultrawide field color fundus photograph. (B) The 55° fundus autofluorescence. (C) Spectral-domain optical coherence tomography line horizontal scan. (D) Full-field dark-adapted electroretinogram. (E) Three-dimensional multifocal electroretinogram plot. (F) Goldmann kinetic visual field.
+Characterization of the pathogenicTUBvariant. (A) Transcript processing in primary skin fibroblasts from a healthy donor and from the proband carrying the homozygous splice site variant. Total RNA was extracted, reverse-transcribed and analyzed by PCR to resolve transcript processing. Two aberrant cDNA products were identified in mutated cells (left) compared to the expected length of the amplified fragment obtained from the control fibroblasts (right). (B) Schematic representation of aberrant transcript processing caused by the identified homozygous splice site change inTUB. (C) Western blot analysis of the TUB protein in patient’s fibroblasts and the control cells. Twenty, forty and sixty micrograms of whole cell extract were analyzed basally (left) and following 4 h treatment with 100 μM Mg132 (right) and probed with anti-TUB antibody (* indicates a non-specific product). (D) Expression of wild-type and mutant TUB protein was analyzed in the cytoplasmic and nuclear fractions were obtained from wild-type and mutated fibroblasts. Sixty micrograms of each fraction were analyzed by Western blot and then probed with anti-TUB antibody. Anti-YY1 and anti-HSP90 antibodies were used as the internal controls to assess the clarity of the different fractions (* indicates a non-specific product). Blots are representative of three experiments performed.
+TUB subcellular localization and cilium defects in cells with TUB LoF. (A) Thirty-hour-starved and PFA-fixed fibroblasts from a healthy donor and from the proband were analyzed by confocal microscopy for the localization of TUB using antibodies against TUB. (B) The presence and morphology of primary cilia in starved fibroblasts from the proband and a healthy donor. Cells were starved for 30 h and fixed with PFA 4%. Primary cilia were analyzed using antibodies against ARL13B (cilium axonemal, green) and pericentrin (basal body, red) to investigate morphogenesis. Nuclei are DAPI stained (blue). Bars correspond to 20 and 2 μm (left panels). (C) Histograms represent the percent value of presence/absence of cilium, normal/aberrant cilium morphology and normal/aberrant basal body structure and the length (μm) of axoneme. Five hundred cells were counted for each condition and axoneme length was measured. Imagines and bar plots are representative of three experiments performed. * indicate statistical significance forp&lt; 0.01 by using Student’sTtest.</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Based on the provided text, I cannot confirm that "rd5" is an alternate abbreviation for the TUB gene. The text does not explicitly link "rd5" to TUB or expand it to the official gene name "TUB bipartite transcription factor". Therefore, I will classify this as not an alternate abbreviation.
+Here is the JSON output:
+{
+"pmid": "9390831",
+"alias_symbol": "rd5",
+"primary_gene_symbol": "TUB",
+"name": "TUB bipartite transcription factor",
+"alternate_abbreviation": "NO",
+"evidence": ""
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HGNC:12406</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ENSG00000166402</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GENE ID:7275</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>TUB</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>rd5</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>9477305</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>mouse phenotype biomarker</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>discussion</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities.</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>TUB bipartite transcription factor</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Some genetic syndromes causing loss of hearing and vision, such as some forms of Usher's syndrome, also cause reduced sperm cell motility, bronchiectasis, and other pathologies involving cilia- and flagella-bearing cells. In some Usher's patients, ultrastructural defects of axonemes within photoreceptor ciliary bridges, nasal cilia, and sperm cell flagella have been found, indicating a primary defect of axonemal conformation. Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities. They provide a good phenotypic match to human genetic sensory syndromes, particularly human sensory/obesity syndromes, such as Alstrom's and Bardet/Biedl, although no human candidate genes have been identified. Because of their unique phenotype, tubby mice are an appropriate model in which to look for a primary axonemal defect. We studied the axonemal ultrastructure of photoreceptors and sperm cells and performed functional testing of sperm in tub/tub mice before and after the onset of obesity. Approximately 15% of photoreceptor axonemes appeared abnormal in tub/tub animals, compared to 0% in controls. Both tub homozygotes and controls exhibited approximately 10% abnormal sperm cell axonemes, and no differences in sperm cell motile function were found at any age. The modest occurrence of axonemal defects in photoreceptors of tub/tub animals is likely to be a secondary effect of retinal degeneration. We conclude that the tubby phenotype is not associated with a generalized defect of cilia- and flagella-bearing cells and that the tub mutation does not primarily affect axonemal structure.</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>PMID: 9477305
+Abstract: Some genetic syndromes causing loss of hearing and vision, such as some forms of Usher's syndrome, also cause reduced sperm cell motility, bronchiectasis, and other pathologies involving cilia- and flagella-bearing cells. In some Usher's patients, ultrastructural defects of axonemes within photoreceptor ciliary bridges, nasal cilia, and sperm cell flagella have been found, indicating a primary defect of axonemal conformation. Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities. They provide a good phenotypic match to human genetic sensory syndromes, particularly human sensory/obesity syndromes, such as Alstrom's and Bardet/Biedl, although no human candidate genes have been identified. Because of their unique phenotype, tubby mice are an appropriate model in which to look for a primary axonemal defect. We studied the axonemal ultrastructure of photoreceptors and sperm cells and performed functional testing of sperm in tub/tub mice before and after the onset of obesity. Approximately 15% of photoreceptor axonemes appeared abnormal in tub/tub animals, compared to 0% in controls. Both tub homozygotes and controls exhibited approximately 10% abnormal sperm cell axonemes, and no differences in sperm cell motile function were found at any age. The modest occurrence of axonemal defects in photoreceptors of tub/tub animals is likely to be a secondary effect of retinal degeneration. We conclude that the tubby phenotype is not associated with a generalized defect of cilia- and flagella-bearing cells and that the tub mutation does not primarily affect axonemal structure.</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
+    Inputs:
+    Alias gene symbol: rd5
+    HGNC record ID: HGNC:12406
+    Primary gene symbol: TUB
+    Official HGNC gene name: TUB bipartite transcription factor
+    Biomedical text context
+    Task:
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
+    Rules:
+    If the text does not support that the alias is an alternate abbreviation, return:
+    "alternate_abbreviation": "NO"
+    "evidence": ""
+    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
+    Evidence must be one exact sentence copied verbatim from the text.
+    Do not infer relationships or paraphrase evidence.
+    Output (Strict):
+    Output only one JSON object. No markdown.
+    {
+    "pmid": "",
+    "alias_symbol": "",
+    "primary_gene_symbol": "",
+    "name": "",
+    "alternate_abbreviation": "YES or NO",
+    "evidence": ""
+    }
+PMID: 9477305
+Abstract: Some genetic syndromes causing loss of hearing and vision, such as some forms of Usher's syndrome, also cause reduced sperm cell motility, bronchiectasis, and other pathologies involving cilia- and flagella-bearing cells. In some Usher's patients, ultrastructural defects of axonemes within photoreceptor ciliary bridges, nasal cilia, and sperm cell flagella have been found, indicating a primary defect of axonemal conformation. Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities. They provide a good phenotypic match to human genetic sensory syndromes, particularly human sensory/obesity syndromes, such as Alstrom's and Bardet/Biedl, although no human candidate genes have been identified. Because of their unique phenotype, tubby mice are an appropriate model in which to look for a primary axonemal defect. We studied the axonemal ultrastructure of photoreceptors and sperm cells and performed functional testing of sperm in tub/tub mice before and after the onset of obesity. Approximately 15% of photoreceptor axonemes appeared abnormal in tub/tub animals, compared to 0% in controls. Both tub homozygotes and controls exhibited approximately 10% abnormal sperm cell axonemes, and no differences in sperm cell motile function were found at any age. The modest occurrence of axonemal defects in photoreceptors of tub/tub animals is likely to be a secondary effect of retinal degeneration. We conclude that the tubby phenotype is not associated with a generalized defect of cilia- and flagella-bearing cells and that the tub mutation does not primarily affect axonemal structure.</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>{
+"pmid": "9477305",
+"alias_symbol": "rd5",
+"primary_gene_symbol": "TUB",
+"name": "TUB bipartite transcription factor",
+"alternate_abbreviation": "YES",
+"evidence": "Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities."
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HGNC:12406</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ENSG00000166402</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GENE ID:7275</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>TUB</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>rd5</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>36612533</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>primer</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>methods</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>The primers were as follows: forward primer RD5 5_-ATC TGG TTG ATC CTG CCA GT-3_ and reverse primer BhRDr 5_-GAG CTT TTTA ACT GCA ACA ACG-3_</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>TUB bipartite transcription factor</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
         <is>
           <t>Blastocystisis one of the most common enteric protozoa that inhabits the intestinal tract of humans and different animals. Moreover, it has a worldwide geographic distribution. Its main mode of transmission is via the fecal-oral route. At present, 26 subtypes are widely distributed across both humans and animals. The current study aimed to determine the prevalence and subtype distribution ofBlastocystisamong school-aged children living on the Thai-Myanmar border, Ratchaburi province, Thailand. In total, 508 samples were collected from children at six schools. The prevalence ofBlastocystisinfection was amplified and sequenced in the 600 bp barcode region of the small-subunit ribosomal RNA (SSU rRNA). The overall prevalence ofBlastocystisinfection was 3.35% (17/508). ST3 (11/17) was the most predominant subtype, followed by ST1 (5/17) and ST2 (1/17). A phylogenetic tree was constructed based on the Tamura92+G+I model using the maximum-likelihood algorithm. Surprisingly, all sequences of the ST3-positive samples were closely correlated with the cattle-derived sequence. Meanwhile, all sequences of theBlastocystisST1-positive samples were closely correlated with the human-derived sequence. Nevertheless, further studies should be conducted to validate the zoonotic transmission ofBlastocystis. Based on our findings, personal hygiene and sanitation should be improved to promote better health in children in this area.
 Intestinal parasitic infections are one of the main public health issues worldwide, and their incidence is higher in developing than in developed countries [1,2].Blastocystisis a common enteric protozoan causing parasitic intestinal infections among children. Further, it mainly colonizes the gastrointestinal tract, and it is transmitted via the fecal-oral route [3,4]. At present, approximately more than 1 billion humans are infected withBlastocystisworldwide [5]. Its transmission is correlated with several factors, such as poor personal hygiene, consumption of contaminated food, and environmental conditions associated with poor quality of life [6,7,8]. Moreover, close contact with animals due to cultural conditions may causeBlastocystisinfection [9,10,11]. Additionally, school-aged children are at high risk ofBlastocystisinfection due to poor hygiene habits [1,4]. Several studies showed that the prevalence ofBlastocystisinfection varies from 0.7% to 45.2% among school-aged children in Thailand [12,13,14,15]. At present, 26 subtypes ofBlastocystisare widely distributed in both humans and animals. Among them, subtype 3 is most commonly observed in humans [16,17]. The methods used to detectBlastocystisare usually based on microscopy. However, these techniques have low sensitivity and specificity, and assessment using these strategies should be performed by skilled microscopists to validate morphology [18,19,20]. In recent years, polymerase chain reaction (PCR), a molecular biology technique, targets a region of the SSU rRNA genes. Moreover, it has the highest sensitivity and specificity and can identify different subtypes [21,22,23]. However, studies on the incidence and subtypes ofBlastocystisin school-aged children living in the border areas of Thailand are limited. The current study aimed to determine the prevalence and subtype distribution ofBlastocystisisolated from school-aged children living in the Thai-Myanmar border areas, Ratchaburi Province, Thailand.
@@ -648,12 +1412,12 @@
 Accession numbers of positive samples used in the phylogenetic reconstruction.</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>&lt;i&gt;Blastocystis&lt;/i&gt; is one of the most common enteric protozoa that inhabits the intestinal tract of humans and different animals. Moreover, it has a worldwide geographic distribution. Its main mode of transmission is via the fecal-oral route. At present, 26 subtypes are widely distributed across both humans and animals. The current study aimed to determine the prevalence and subtype distribution of &lt;i&gt;Blastocystis&lt;/i&gt; among school-aged children living on the Thai-Myanmar border, Ratchaburi province, Thailand. In total, 508 samples were collected from children at six schools. The prevalence of &lt;i&gt;Blastocystis&lt;/i&gt; infection was amplified and sequenced in the 600 bp barcode region of the small-subunit ribosomal RNA (SSU rRNA). The overall prevalence of &lt;i&gt;Blastocystis&lt;/i&gt; infection was 3.35% (17/508). ST3 (11/17) was the most predominant subtype, followed by ST1 (5/17) and ST2 (1/17). A phylogenetic tree was constructed based on the Tamura92+G+I model using the maximum-likelihood algorithm. Surprisingly, all sequences of the ST3-positive samples were closely correlated with the cattle-derived sequence. Meanwhile, all sequences of the &lt;i&gt;Blastocystis&lt;/i&gt; ST1-positive samples were closely correlated with the human-derived sequence. Nevertheless, further studies should be conducted to validate the zoonotic transmission of &lt;i&gt;Blastocystis&lt;/i&gt;. Based on our findings, personal hygiene and sanitation should be improved to promote better health in children in this area.</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>PMID: 36612533
 Full Text: Blastocystisis one of the most common enteric protozoa that inhabits the intestinal tract of humans and different animals. Moreover, it has a worldwide geographic distribution. Its main mode of transmission is via the fecal-oral route. At present, 26 subtypes are widely distributed across both humans and animals. The current study aimed to determine the prevalence and subtype distribution ofBlastocystisamong school-aged children living on the Thai-Myanmar border, Ratchaburi province, Thailand. In total, 508 samples were collected from children at six schools. The prevalence ofBlastocystisinfection was amplified and sequenced in the 600 bp barcode region of the small-subunit ribosomal RNA (SSU rRNA). The overall prevalence ofBlastocystisinfection was 3.35% (17/508). ST3 (11/17) was the most predominant subtype, followed by ST1 (5/17) and ST2 (1/17). A phylogenetic tree was constructed based on the Tamura92+G+I model using the maximum-likelihood algorithm. Surprisingly, all sequences of the ST3-positive samples were closely correlated with the cattle-derived sequence. Meanwhile, all sequences of theBlastocystisST1-positive samples were closely correlated with the human-derived sequence. Nevertheless, further studies should be conducted to validate the zoonotic transmission ofBlastocystis. Based on our findings, personal hygiene and sanitation should be improved to promote better health in children in this area.
@@ -684,7 +1448,7 @@
 Accession numbers of positive samples used in the phylogenetic reconstruction.</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -692,35 +1456,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -753,95 +1525,94 @@
 Accession numbers of positive samples used in the phylogenetic reconstruction.</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>{
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Based on the provided text, here is my analysis:
+{
 "pmid": "36612533",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"alternate_abbreviation": "NO",
 "evidence": ""
-}</t>
+}
+The text does not provide any evidence that "rd5" is an alternate abbreviation for the TUB gene. The symbol "RD5" appears in the text, but it is used as a primer name for PCR amplification of Blastocystis DNA, not as a gene symbol. There is no explicit link or expansion connecting "rd5" to the official gene name "TUB bipartite transcription factor" or the primary symbol "TUB". Therefore, I have classified this as not an alternate abbreviation and provided no evidence.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>36650547</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>36650547</v>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
         <is>
           <t>alias</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>alias</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>intro</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>TUB (MIM #601197), also known as rd5 or RDOB, maps to 11p15.4 and encodes the tubby-bipartite transcription regulator</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr">
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>Retinitis pigmentosa (RP) is the most common type of inherited retinopathy. At least 69 genes for RP have been identified. A significant proportion of RP, however, remains genetically unsolved. In this study, the genetic basis of a Chinese consanguineous family with presumed autosomal recessive retinitis pigmentosa (arRP) was investigated.
 Overall ophthalmic examinations, including funduscopy, decimal best-corrected visual acuity, axial length and electroretinography (ERG) were performed for the family. Genomic DNA from peripheral blood of the proband was subjected to whole exome sequencing. In silico predictions, structural modelling, and minigene assays were conducted to evaluate the pathogenicity of the variant.
@@ -871,7 +1642,7 @@
 In the current study, we examined a consanguineous family with arRP from central south China and detected a novel homozygous variant (c.1379 G &gt; A: p.Asn460Ser) inTUB. This variant co-segregated with the disease in an autosomal recessive manner and was absent in 118 ethnically matched healthy controls. This homozygous variant has not been reported in the literature or deposited in existing databases including gnomAD, 1000G phase3, ExAC, or dbSNP, indicating that this variant is rare. Multiple bioinformatic algorithms predicted that this variant was deleterious or damaging. Conservative analysis showed the codon Asn460 fallen within a highly conserved region across diverse species (Fig.3B). Further structural modeling showed that amino acid substitution (Ser) of the variant at residue Asn460 could affect the protein conformation, the binding ability of the tubby domain [26], as well as the solubility and stabilization of the mutant protein [27]. Taken together, these data strongly supported the hypothesis that this novelTUBvariant (c.1379 A &gt; G: p. Asn460Ser) might be the genetic basis of arRP in this Chinese consanguineous family.</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>Retinitis pigmentosa (RP) is the most common type of inherited retinopathy. At least 69 genes for RP have been identified. A significant proportion of RP, however, remains genetically unsolved. In this study, the genetic basis of a Chinese consanguineous family with presumed autosomal recessive retinitis pigmentosa (arRP) was investigated.
 Overall ophthalmic examinations, including funduscopy, decimal best-corrected visual acuity, axial length and electroretinography (ERG) were performed for the family. Genomic DNA from peripheral blood of the proband was subjected to whole exome sequencing. In silico predictions, structural modelling, and minigene assays were conducted to evaluate the pathogenicity of the variant.
@@ -879,7 +1650,7 @@
 A novel missense variant in TUB was identified, which was probably the pathogenic basis for arRP in this consanguineous family. This is the first report of a homozygous missense variant in TUB for RP.</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>PMID: 36650547
 Full Text: Retinitis pigmentosa (RP) is the most common type of inherited retinopathy. At least 69 genes for RP have been identified. A significant proportion of RP, however, remains genetically unsolved. In this study, the genetic basis of a Chinese consanguineous family with presumed autosomal recessive retinitis pigmentosa (arRP) was investigated.
@@ -910,7 +1681,7 @@
 In the current study, we examined a consanguineous family with arRP from central south China and detected a novel homozygous variant (c.1379 G &gt; A: p.Asn460Ser) inTUB. This variant co-segregated with the disease in an autosomal recessive manner and was absent in 118 ethnically matched healthy controls. This homozygous variant has not been reported in the literature or deposited in existing databases including gnomAD, 1000G phase3, ExAC, or dbSNP, indicating that this variant is rare. Multiple bioinformatic algorithms predicted that this variant was deleterious or damaging. Conservative analysis showed the codon Asn460 fallen within a highly conserved region across diverse species (Fig.3B). Further structural modeling showed that amino acid substitution (Ser) of the variant at residue Asn460 could affect the protein conformation, the binding ability of the tubby domain [26], as well as the solubility and stabilization of the mutant protein [27]. Taken together, these data strongly supported the hypothesis that this novelTUBvariant (c.1379 A &gt; G: p. Asn460Ser) might be the genetic basis of arRP in this Chinese consanguineous family.</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -918,35 +1689,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -979,95 +1758,94 @@
 In the current study, we examined a consanguineous family with arRP from central south China and detected a novel homozygous variant (c.1379 G &gt; A: p.Asn460Ser) inTUB. This variant co-segregated with the disease in an autosomal recessive manner and was absent in 118 ethnically matched healthy controls. This homozygous variant has not been reported in the literature or deposited in existing databases including gnomAD, 1000G phase3, ExAC, or dbSNP, indicating that this variant is rare. Multiple bioinformatic algorithms predicted that this variant was deleterious or damaging. Conservative analysis showed the codon Asn460 fallen within a highly conserved region across diverse species (Fig.3B). Further structural modeling showed that amino acid substitution (Ser) of the variant at residue Asn460 could affect the protein conformation, the binding ability of the tubby domain [26], as well as the solubility and stabilization of the mutant protein [27]. Taken together, these data strongly supported the hypothesis that this novelTUBvariant (c.1379 A &gt; G: p. Asn460Ser) might be the genetic basis of arRP in this Chinese consanguineous family.</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>{
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Based on the provided text, here is my analysis:
+{
 "pmid": "36650547",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "YES",
-"alternate_abbreviation": "NO",
+"alternate_abbreviation": "YES",
 "evidence": "TUB (MIM #601197), also known as rd5 or RDOB, maps to 11p15.4 and encodes the tubby-bipartite transcription regulator [10,11]."
-}</t>
+}
+The text explicitly links the alias symbol "rd5" to the TUB gene, stating that TUB is "also known as rd5". This provides clear evidence that rd5 is an alternate abbreviation for the TUB gene.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>36650547</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>36650547</v>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
         <is>
           <t>alias</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>alias</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>intro</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>TUB (MIM #601197), also known as rd5 or RDOB, maps to 11p15.4 and encodes the tubby-bipartite transcription regulator</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr">
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>For RP-associated diseases in humans, variants inTUBare extremely rare. Till now, only one arRP-associated mutation inTUBfor has been reported in the literature, in which a homozygous frameshift variant resulted in retinal dystrophy, hearing loss, and obesity in a consanguineous UK Caucasian family [12]. Even so, a total of 354TUBvariants have been deposited in the ClinVar database with 25 items marked of “pathogenic” or “likely pathogenic” clinical significance, among which at least 3 “pathogenic” or “likely pathogenic” variants have been reported in more than 6 patients with arRP (Additional file1: Table S3). Interestingly, all these cases mentioned above are generated either by splice-site or protein-truncating mutations inTUB.Although the variant found in this study was a single base-substitution, which resulted in a substitution of Asn to Ser at codon 460 in exon 11. According to the ACMG Standards/Guidelines, it’s important to assess the possibility that the variant may act through splicing disruption instead of amino acid change [24]. Considering loss of function is a common mechanism of genetic disease, this homozygous variant coincidently resides on the last but one base of exon 11 of theTUBgene, which is classified as a type II splice variant [28]. We first investigate the splicing effect of the variant by RNA analysis from the peripheral blood of the proband as well as healthy controls. But no mRNA ofTUBwas detected in available somatic cells (data not shown), which is consistent with the records in GTEx that the mRNA ofTUBin peripheral blood is extremely low (Additional file1: Fig. S1). Considering the unavailability of specific tissues, we further tried to explore the splicing effect of this variant via minigene assay, a powerful way for evaluating the role of novel variants on splicing [29]. The splicing assay in this study, however, showed no differences between theTUB/WTandTUB/MTminigenes in two different cell lines, indicating the possible impact of this variant on splicing could be basically ruled out. A mutant TUB protein induced by the homozygous missense variant instead of loss of function from splicing-error or protein-truncating was probably the pathogenic basis for the simple arRP in this consanguineous family.
 To date, five mammalian tubby-like proteins (TULPs) family members (TUB and TULP1 to 4) have been identified with an important role in maintenance of the central nervous system [17]. The TULPs are characterized by a unique “tubby domain” of ~ 260 amino acid residues in the C-terminal [30], which forms a central hydrophobic α-helix traversing the β-barrel structure [11]. The ‘tubby domain’ contains a phosphatidylinositol-binding region specifically binding to phosphatidylinositol 4,5-bisphosphate (PIP2) functioning as membrane-bound transcription regulators [10] and a DNA-binding domain (DBD) that selectively binding to double-stranded DNA [11]. Although the N-terminal motifs of the TULPs are poorly conserved [31], the C-terminal “tubby domains” of the TULPs are remarkedly conserved with 55–95% identity across species from plants to humans [17], implying an evolutionarily conserved function [11]. Structure–function analysis by Sunshin Kim et al. demonstrated that the tubby domain inTUBplays a crucial role in its subcellular localization and solubility [26]. In addition, mutations in anotherTULPs family member,TULP1(also known as RP14), is known to cause retinal degeneration in both humans and mice [32–35]. Previous studies demonstrated that bothTUBandTULP1are essential for G protein-coupled receptors (GPCRs) mediated trafficking of photoreceptors [30,36] and MerTK-dependent phagocytosis in retinal pigment epithelium (RPE) and apoptotic cells [37]. Caspase mediated apoptosis and MerTK-dependent phagocytosis are the underlying mechanism of photoreceptor cell death in retinal degeneration [37–40]. Therefore, we presume that the pathogenic missense variant inTUBreported here may influence TUB functions through disruption of the ‘tubby domain’, affecting GPCR trafficking, as well as the normal physiology of the photoreceptor cells, and ultimately lead to arRP. Further functional studies, however, are required to elucidate the exact role ofTUBin arRP. Genetically modified animal models are being developed in the lab to address these points.
@@ -1095,7 +1873,7 @@
 All authors declared no conflict of interest.</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>Retinitis pigmentosa (RP) is the most common type of inherited retinopathy. At least 69 genes for RP have been identified. A significant proportion of RP, however, remains genetically unsolved. In this study, the genetic basis of a Chinese consanguineous family with presumed autosomal recessive retinitis pigmentosa (arRP) was investigated.
 Overall ophthalmic examinations, including funduscopy, decimal best-corrected visual acuity, axial length and electroretinography (ERG) were performed for the family. Genomic DNA from peripheral blood of the proband was subjected to whole exome sequencing. In silico predictions, structural modelling, and minigene assays were conducted to evaluate the pathogenicity of the variant.
@@ -1103,7 +1881,7 @@
 A novel missense variant in TUB was identified, which was probably the pathogenic basis for arRP in this consanguineous family. This is the first report of a homozygous missense variant in TUB for RP.</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>PMID: 36650547
 Full Text: For RP-associated diseases in humans, variants inTUBare extremely rare. Till now, only one arRP-associated mutation inTUBfor has been reported in the literature, in which a homozygous frameshift variant resulted in retinal dystrophy, hearing loss, and obesity in a consanguineous UK Caucasian family [12]. Even so, a total of 354TUBvariants have been deposited in the ClinVar database with 25 items marked of “pathogenic” or “likely pathogenic” clinical significance, among which at least 3 “pathogenic” or “likely pathogenic” variants have been reported in more than 6 patients with arRP (Additional file1: Table S3). Interestingly, all these cases mentioned above are generated either by splice-site or protein-truncating mutations inTUB.Although the variant found in this study was a single base-substitution, which resulted in a substitution of Asn to Ser at codon 460 in exon 11. According to the ACMG Standards/Guidelines, it’s important to assess the possibility that the variant may act through splicing disruption instead of amino acid change [24]. Considering loss of function is a common mechanism of genetic disease, this homozygous variant coincidently resides on the last but one base of exon 11 of theTUBgene, which is classified as a type II splice variant [28]. We first investigate the splicing effect of the variant by RNA analysis from the peripheral blood of the proband as well as healthy controls. But no mRNA ofTUBwas detected in available somatic cells (data not shown), which is consistent with the records in GTEx that the mRNA ofTUBin peripheral blood is extremely low (Additional file1: Fig. S1). Considering the unavailability of specific tissues, we further tried to explore the splicing effect of this variant via minigene assay, a powerful way for evaluating the role of novel variants on splicing [29]. The splicing assay in this study, however, showed no differences between theTUB/WTandTUB/MTminigenes in two different cell lines, indicating the possible impact of this variant on splicing could be basically ruled out. A mutant TUB protein induced by the homozygous missense variant instead of loss of function from splicing-error or protein-truncating was probably the pathogenic basis for the simple arRP in this consanguineous family.
@@ -1132,7 +1910,7 @@
 All authors declared no conflict of interest.</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -1140,35 +1918,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -1199,99 +1985,96 @@
 All authors declared no conflict of interest.</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>{
 "pmid": "36650547",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"alternate_abbreviation": "NO",
 "evidence": ""
 }</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>37185159</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>37185159</v>
+      </c>
+      <c r="I9" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>primer</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>In the first reaction, the broadly specific oligonucleotide primers RD5 (5Õ-GGAAGCTTATCTGGTTGATCCTGCCAGTA-3Õ) and RD3 (5Õ-GGGATCCTGATCCTTCCGCAGGTTCACCTAC-3Õ) were used</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr">
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>Blastocystisis a protist of controversial pathogenicity inhabiting the gut of humans and other animals. Despite a century of intense study, understanding of the epidemiology ofBlastocystisremains fragmentary. Here, we aimed to explore its prevalence, stability of colonisation and association with various factors in a rural elementary school in northern Thailand. One hundred and forty faecal samples were collected from 104 children at two time points (tp) 105 days apart. For tp2, samples were also obtained from 15 animals residing on campus and seven water locations. Prevalence in children was 67% at tp1 and 89% at tp2, 63% in chickens, 86% in pigs, and 57% in water. Ten STs were identified, two of which were shared between humans and animals, one between animals and water, and three between humans and water. Eighteen children (out of 36) carried the same ST over both time points, indicating stable colonisation. Presence ofBlastocystis(or ST) was not associated with body mass index, ethnicity, birth delivery mode, or milk source as an infant. This study advances understanding ofBlastocystisprevalence in an understudied age group, the role of the environment in transmission, and the ability of specific STs to stably colonise children.
 Blastocystisis a unicellular eukaryote inhabiting the gastrointestinal tract of vertebrates [1–3] and invertebrates [4,5]. The organism comprises the most common protist identified in human stool samples [6]. The genetic heterogeneity ofBlastocystisis extremely high based on the small subunit ribosomal RNA (SSU rRNA) gene [7–14]. To date, 34 subtypes (STs; ST1–ST17, ST21, and ST23–ST38) have been identified in avian and mammalian hosts. Of these, 14 have been recorded in humans (ST1–ST10, ST12, ST14, ST16, and ST23) [13,15–20], with ST1–ST3 accounting for the majority of human carriage [21,22]. The remaining STs mostly colonise non-human endothermic hosts [1,6].
@@ -1320,12 +2103,12 @@
 This analysis involved only sequences from tp2. ST sharing was noted among all three categories herein: humans, animals, and water (Figure 2). ST5 and ST7 were shared between humans and animals, ST1, ST3, and ST7 between humans and water, and ST7 between animals and water. ST7 was shared by all three. The ST5 sequences from humans and pigs were not identical. Similarly, ST1 sequences from water and children differed. ST3 sequences from the water creek, and 16 children were identical. ST7 sequences from two children samples and a water sample obtained from the tap outside the school bathroom were also identical.Figure 2.Blastocystissubtypes (STs) present in humans, animals, and water in a rural elementary school in northern Thailand. STs on arrows indicate overlap. Shaded STs indicate the presence in all sources considered in this study.</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>&lt;i&gt;Blastocystis&lt;/i&gt; is a protist of controversial pathogenicity inhabiting the gut of humans and other animals. Despite a century of intense study, understanding of the epidemiology of &lt;i&gt;Blastocystis&lt;/i&gt; remains fragmentary. Here, we aimed to explore its prevalence, stability of colonisation and association with various factors in a rural elementary school in northern Thailand. One hundred and forty faecal samples were collected from 104 children at two time points (tp) 105 days apart. For tp2, samples were also obtained from 15 animals residing on campus and seven water locations. Prevalence in children was 67% at tp1 and 89% at tp2, 63% in chickens, 86% in pigs, and 57% in water. Ten STs were identified, two of which were shared between humans and animals, one between animals and water, and three between humans and water. Eighteen children (out of 36) carried the same ST over both time points, indicating stable colonisation. Presence of &lt;i&gt;Blastocystis&lt;/i&gt; (or ST) was not associated with body mass index, ethnicity, birth delivery mode, or milk source as an infant. This study advances understanding of &lt;i&gt;Blastocystis&lt;/i&gt; prevalence in an understudied age group, the role of the environment in transmission, and the ability of specific STs to stably colonise children.</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>PMID: 37185159
 Full Text: Blastocystisis a protist of controversial pathogenicity inhabiting the gut of humans and other animals. Despite a century of intense study, understanding of the epidemiology ofBlastocystisremains fragmentary. Here, we aimed to explore its prevalence, stability of colonisation and association with various factors in a rural elementary school in northern Thailand. One hundred and forty faecal samples were collected from 104 children at two time points (tp) 105 days apart. For tp2, samples were also obtained from 15 animals residing on campus and seven water locations. Prevalence in children was 67% at tp1 and 89% at tp2, 63% in chickens, 86% in pigs, and 57% in water. Ten STs were identified, two of which were shared between humans and animals, one between animals and water, and three between humans and water. Eighteen children (out of 36) carried the same ST over both time points, indicating stable colonisation. Presence ofBlastocystis(or ST) was not associated with body mass index, ethnicity, birth delivery mode, or milk source as an infant. This study advances understanding ofBlastocystisprevalence in an understudied age group, the role of the environment in transmission, and the ability of specific STs to stably colonise children.
@@ -1355,7 +2138,7 @@
 This analysis involved only sequences from tp2. ST sharing was noted among all three categories herein: humans, animals, and water (Figure 2). ST5 and ST7 were shared between humans and animals, ST1, ST3, and ST7 between humans and water, and ST7 between animals and water. ST7 was shared by all three. The ST5 sequences from humans and pigs were not identical. Similarly, ST1 sequences from water and children differed. ST3 sequences from the water creek, and 16 children were identical. ST7 sequences from two children samples and a water sample obtained from the tap outside the school bathroom were also identical.Figure 2.Blastocystissubtypes (STs) present in humans, animals, and water in a rural elementary school in northern Thailand. STs on arrows indicate overlap. Shaded STs indicate the presence in all sources considered in this study.</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -1363,35 +2146,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -1423,100 +2214,98 @@
 This analysis involved only sequences from tp2. ST sharing was noted among all three categories herein: humans, animals, and water (Figure 2). ST5 and ST7 were shared between humans and animals, ST1, ST3, and ST7 between humans and water, and ST7 between animals and water. ST7 was shared by all three. The ST5 sequences from humans and pigs were not identical. Similarly, ST1 sequences from water and children differed. ST3 sequences from the water creek, and 16 children were identical. ST7 sequences from two children samples and a water sample obtained from the tap outside the school bathroom were also identical.Figure 2.Blastocystissubtypes (STs) present in humans, animals, and water in a rural elementary school in northern Thailand. STs on arrows indicate overlap. Shaded STs indicate the presence in all sources considered in this study.</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>Based on the provided text, here is the JSON output:
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Based on the provided text, here is the analysis for the alias symbol "rd5":
 {
 "pmid": "37185159",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"alternate_abbreviation": "NO",
 "evidence": ""
-}</t>
+}
+The text does not provide any evidence that "rd5" is an alternate abbreviation for the TUB gene. The symbol "RD5" appears to be used as a primer name in the PCR methodology section, but it is not explicitly linked to or expanded as the TUB gene name. Therefore, there is insufficient evidence to classify "rd5" as an alternate abbreviation for TUB in this context.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>37185159</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>37185159</v>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>primer</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>In the first reaction, the broadly specific oligonucleotide primers RD5 (5Õ-GGAAGCTTATCTGGTTGATCCTGCCAGTA-3Õ) and RD3 (5Õ-GGGATCCTGATCCTTCCGCAGGTTCACCTAC-3Õ) were used</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr">
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>Blastocystissubtypes (STs) present in humans, animals, and water in a rural elementary school in northern Thailand. STs on arrows indicate overlap. Shaded STs indicate the presence in all sources considered in this study.
 For the phylogenetic analysis, 23 sequences were chosen to represent the different STs present in the sample cohort (Figure 3). ST15 found in the pig sample grouped with previously published ST15 sequences and together with ST28 and sequences from ectothermic hosts placed at the base of the tree. Newly generated sequences placed within clades consisting of known STs. Sequences identified as ST10 and ST23 were grouped with similar sequences from our previous One Health study [15].Figure 3.Maximum likelihood phylogeny inferred from 175Blastocystissequences and 1,392 sites of theSSUrRNA gene. Newly generated sequences are in bold font. Numerical values indicate bootstrap support. Only values above 70 are shown.
@@ -1542,12 +2331,12 @@
 The authors declare none.</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>&lt;i&gt;Blastocystis&lt;/i&gt; is a protist of controversial pathogenicity inhabiting the gut of humans and other animals. Despite a century of intense study, understanding of the epidemiology of &lt;i&gt;Blastocystis&lt;/i&gt; remains fragmentary. Here, we aimed to explore its prevalence, stability of colonisation and association with various factors in a rural elementary school in northern Thailand. One hundred and forty faecal samples were collected from 104 children at two time points (tp) 105 days apart. For tp2, samples were also obtained from 15 animals residing on campus and seven water locations. Prevalence in children was 67% at tp1 and 89% at tp2, 63% in chickens, 86% in pigs, and 57% in water. Ten STs were identified, two of which were shared between humans and animals, one between animals and water, and three between humans and water. Eighteen children (out of 36) carried the same ST over both time points, indicating stable colonisation. Presence of &lt;i&gt;Blastocystis&lt;/i&gt; (or ST) was not associated with body mass index, ethnicity, birth delivery mode, or milk source as an infant. This study advances understanding of &lt;i&gt;Blastocystis&lt;/i&gt; prevalence in an understudied age group, the role of the environment in transmission, and the ability of specific STs to stably colonise children.</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>PMID: 37185159
 Full Text: Blastocystissubtypes (STs) present in humans, animals, and water in a rural elementary school in northern Thailand. STs on arrows indicate overlap. Shaded STs indicate the presence in all sources considered in this study.
@@ -1574,7 +2363,7 @@
 The authors declare none.</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -1582,35 +2371,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -1639,99 +2436,96 @@
 The authors declare none.</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="V10" t="inlineStr">
         <is>
           <t>{
 "pmid": "37185159",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"alternate_abbreviation": "NO",
 "evidence": ""
 }</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>38543574</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>38543574</v>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>primer</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>PCR amplification of Blastocystis sp. was carried out using barcoding region primers BhRDr (5_-GAGCTTTTTAACTGCAACAACG-3_) and RD5 (5_-ATCTGGTTGATCCTGCCAGT-3_) for SSU rRNA</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr">
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>Blastocystissp. is the most common intestinal protozoan affecting human health worldwide. Several studies have reported the prevalence ofBlastocystissp. in various regions of the Republic of Korea. However, limited data are available on the prevalence and subtype (ST) distribution of this parasite among regions. Therefore, we investigated the prevalence and ST distributions of this parasite in the Republic of Korea. For this purpose, 894 stool specimens were collected from patients with diarrhea and tested for the presence ofBlastocystissp. using PCR analysis. The isolates were subsequently subtyped. The overall prevalence was 11.6%. Of the 104 isolates, ST3 was the most prevalent, followed by ST1. Additionally, a single case of the rare subtype ST8 was identified, representing the first reported case in the Republic of Korea. The results suggested that the predominance of ST3 observed in this study reflects human-to-human transmission with low genetic diversity within the ST, while ST1 transmission is likely correlated with animals. In the future, to better understandBlastocystissp. transmission dynamics, human, animal, and environmental factors should be studied from a “One Health” perspective.
 Blastocystissp. is a protozoan parasite that resides within the gastrointestinal tract of a wide range of hosts, including mammals, birds, fish, reptiles, insects, and humans [1,2]. This enteric microorganism is a causative agent of waterborne and foodborne diseases. The infective cysts are transmitted through the fecal–oral route [3,4]. An estimated more than 1 billion people are infected with this parasite worldwide, with a prevalence of 10–15% in developed countries and &gt;50% in developing nations [5]. Although most infected people are asymptomatic carriers, some vulnerable individuals develop symptoms, including diarrhea, abdominal pain, gas, and nausea, as well as extraintestinal symptoms such as urticaria and rash [6,7,8,9,10].Blastocystissp. colonization is reportedly associated with a healthy gut microbiome rather than intestinal dysbacteriosis [6]. However, in vitro and in vivo studies combined with genomic analyses have identified various virulence factors that may be related to the genetic variation inBlastocystisisolates [2,11].
@@ -1768,12 +2562,12 @@
 Distribution ofBlastocystissp. infection among patients with diarrhea in the Republic of Korea.</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>&lt;i&gt;Blastocystis&lt;/i&gt; sp. is the most common intestinal protozoan affecting human health worldwide. Several studies have reported the prevalence of &lt;i&gt;Blastocystis&lt;/i&gt; sp. in various regions of the Republic of Korea. However, limited data are available on the prevalence and subtype (ST) distribution of this parasite among regions. Therefore, we investigated the prevalence and ST distributions of this parasite in the Republic of Korea. For this purpose, 894 stool specimens were collected from patients with diarrhea and tested for the presence of &lt;i&gt;Blastocystis&lt;/i&gt; sp. using PCR analysis. The isolates were subsequently subtyped. The overall prevalence was 11.6%. Of the 104 isolates, ST3 was the most prevalent, followed by ST1. Additionally, a single case of the rare subtype ST8 was identified, representing the first reported case in the Republic of Korea. The results suggested that the predominance of ST3 observed in this study reflects human-to-human transmission with low genetic diversity within the ST, while ST1 transmission is likely correlated with animals. In the future, to better understand &lt;i&gt;Blastocystis&lt;/i&gt; sp. transmission dynamics, human, animal, and environmental factors should be studied from a "One Health" perspective.</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>PMID: 38543574
 Full Text: Blastocystissp. is the most common intestinal protozoan affecting human health worldwide. Several studies have reported the prevalence ofBlastocystissp. in various regions of the Republic of Korea. However, limited data are available on the prevalence and subtype (ST) distribution of this parasite among regions. Therefore, we investigated the prevalence and ST distributions of this parasite in the Republic of Korea. For this purpose, 894 stool specimens were collected from patients with diarrhea and tested for the presence ofBlastocystissp. using PCR analysis. The isolates were subsequently subtyped. The overall prevalence was 11.6%. Of the 104 isolates, ST3 was the most prevalent, followed by ST1. Additionally, a single case of the rare subtype ST8 was identified, representing the first reported case in the Republic of Korea. The results suggested that the predominance of ST3 observed in this study reflects human-to-human transmission with low genetic diversity within the ST, while ST1 transmission is likely correlated with animals. In the future, to better understandBlastocystissp. transmission dynamics, human, animal, and environmental factors should be studied from a “One Health” perspective.
@@ -1811,7 +2605,7 @@
 Distribution ofBlastocystissp. infection among patients with diarrhea in the Republic of Korea.</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -1819,35 +2613,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -1887,99 +2689,98 @@
 Distribution ofBlastocystissp. infection among patients with diarrhea in the Republic of Korea.</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>{
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Based on the provided text, here is my analysis:
+{
 "pmid": "38543574",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"alternate_abbreviation": "NO",
 "evidence": ""
-}</t>
+}
+The text does not provide any evidence that "rd5" is an alternate abbreviation for the TUB gene. The symbol "RD5" appears in the text, but it is used as a primer name for PCR amplification of Blastocystis sp., not as an alias for the TUB gene. There is no explicit link or expansion connecting "rd5" to the official gene name "TUB bipartite transcription factor". Therefore, I have classified this as not an alternate abbreviation and provided no evidence.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>38578271</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>38578271</v>
+      </c>
+      <c r="I12" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>primer</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>The gDNA samples were analysed by PCR amplification of _600 bp of the SSU rRNA gene of Blastocystis sp. using the primers RD5 (5__ATCTGGTTGATCCTGCCAGT_3_) and BhRDr (5_GAGCTTTTTAACTGCAACAACG_3_) to identify the presence of Blastocystis sp. Infection</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr">
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>Blastocystissp. is a zoonotic protozoan parasite, and there is limited information about its molecular prevalence and subtypes (STs) distribution in camels globally, especially in Iran.
 This study aimed to examine the prevalence, STs distribution, and zoonotic potential ofBlastocystissp. in one‐humped and two‐humped camels in Ardabil province, northwestern Iran.
@@ -2022,7 +2823,7 @@
 The datasets used and/or analysed during the current study are available in the online version.</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>Blastocystis sp. is a zoonotic protozoan parasite, and there is limited information about its molecular prevalence and subtypes (STs) distribution in camels globally, especially in Iran.
 This study aimed to examine the prevalence, STs distribution, and zoonotic potential of Blastocystis sp. in one-humped and two-humped camels in Ardabil province, northwestern Iran.
@@ -2031,7 +2832,7 @@
 These findings indicate that camels serve as a proper reservoir for a diverse array of Blastocystis STs and thereby can play a significant role in the transmission of this protozoan infection to humans, animals, and water reservoirs.</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>PMID: 38578271
 Full Text: Blastocystissp. is a zoonotic protozoan parasite, and there is limited information about its molecular prevalence and subtypes (STs) distribution in camels globally, especially in Iran.
@@ -2075,7 +2876,7 @@
 The datasets used and/or analysed during the current study are available in the online version.</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -2083,35 +2884,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -2157,99 +2966,96 @@
 The datasets used and/or analysed during the current study are available in the online version.</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>{
 "pmid": "38578271",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"alternate_abbreviation": "NO",
 "evidence": ""
 }</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>38980911</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>38980911</v>
+      </c>
+      <c r="I13" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>primer</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>PCR amplification of DNA was performed using a nested PCR reaction. Briefly, the first PCR used the broad-specificity eukaryotic primer RD5 (5Õ-GGAAGCTTATCTGGTTGA TCCTGCCAGTA-3Õ) and RD3 (5Õ-GGGATCCTGATCCTTC CGCAGGTTCACCTAC-3Õ), which amplifies a ~1,800 bp fragment of the SSU rDNA</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr">
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="R13" t="inlineStr">
         <is>
           <t>The authors have declared that no competing interests exist.
 Blastocystisis a unicellular eukaryote commonly found in the intestinal tract of humans and other animals. The prevalence ofBlastocystishas been investigated in both developed and developing countries, yet its occurrence and distribution in rural locations has been less studied. Herein, we aimed to examine the distribution ofBlastocystiscolonization in Thai adults representing background populations along a rural/peri-urban gradient, as well as associations between colonization and personal characteristics.
@@ -2290,7 +3096,7 @@
 Altogether, we detected a single subtype in 88.8% (142/160) ofBlastocystis-positive individuals, whereas a mixed-subtype (mixST) infection was detected in 3.8% (6/160). Nine subtypes were identified. The most abundant subtype was ST3 (n = 63), followed by ST7 (n = 37), ST1 (n = 23), ST23 (n = 9), ST10 (n = 4), ST2 (n = 2), ST5 (n = 2), ST4 (n = 1) and ST6 (n = 1). In 7.5% (12/160) of the cases, the subtype could not be identified precisely either due to short length and/or presence of ambiguous chromatogram peaks (unk).</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="S13" t="inlineStr">
         <is>
           <t>Blastocystis is a unicellular eukaryote commonly found in the intestinal tract of humans and other animals. The prevalence of Blastocystis has been investigated in both developed and developing countries, yet its occurrence and distribution in rural locations has been less studied. Herein, we aimed to examine the distribution of Blastocystis colonization in Thai adults representing background populations along a rural/peri-urban gradient, as well as associations between colonization and personal characteristics.
 A total of 238 participants were recruited from rural and peri-urban areas situated in three provinces. The presence of Blastocystis in feces was evaluated using PCR and qPCR. Information on gender, age, region (province), rural/peri-urban location, and body mass index (BMI) was collected.
@@ -2298,7 +3104,7 @@
 This study increases the understanding of the epidemiology of Blastocystis colonization and its association with population parameters and characteristics in middle-income countries.</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>PMID: 38980911
 Full Text: The authors have declared that no competing interests exist.
@@ -2340,7 +3146,7 @@
 Altogether, we detected a single subtype in 88.8% (142/160) ofBlastocystis-positive individuals, whereas a mixed-subtype (mixST) infection was detected in 3.8% (6/160). Nine subtypes were identified. The most abundant subtype was ST3 (n = 63), followed by ST7 (n = 37), ST1 (n = 23), ST23 (n = 9), ST10 (n = 4), ST2 (n = 2), ST5 (n = 2), ST4 (n = 1) and ST6 (n = 1). In 7.5% (12/160) of the cases, the subtype could not be identified precisely either due to short length and/or presence of ambiguous chromatogram peaks (unk).</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -2348,35 +3154,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -2420,100 +3234,98 @@
 Altogether, we detected a single subtype in 88.8% (142/160) ofBlastocystis-positive individuals, whereas a mixed-subtype (mixST) infection was detected in 3.8% (6/160). Nine subtypes were identified. The most abundant subtype was ST3 (n = 63), followed by ST7 (n = 37), ST1 (n = 23), ST23 (n = 9), ST10 (n = 4), ST2 (n = 2), ST5 (n = 2), ST4 (n = 1) and ST6 (n = 1). In 7.5% (12/160) of the cases, the subtype could not be identified precisely either due to short length and/or presence of ambiguous chromatogram peaks (unk).</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>Based on the provided text, here is the JSON output:
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Based on the provided text, I do not see any evidence that the alias symbol "rd5" is explicitly expanded or linked to the official HGNC gene name "TUB bipartite transcription factor" or the primary gene symbol "TUB". The text appears to be about Blastocystis epidemiology and does not mention the TUB gene. Therefore, I cannot classify "rd5" as an alternate abbreviation for TUB in this context.
+Here is the output in the requested JSON format:
 {
 "pmid": "38980911",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"alternate_abbreviation": "NO",
 "evidence": ""
 }</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>38980911</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>38980911</v>
+      </c>
+      <c r="I14" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>primer</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>PCR amplification of DNA was performed using a nested PCR reaction. Briefly, the first PCR used the broad-specificity eukaryotic primer RD5 (5Õ-GGAAGCTTATCTGGTTGA TCCTGCCAGTA-3Õ) and RD3 (5Õ-GGGATCCTGATCCTTC CGCAGGTTCACCTAC-3Õ), which amplifies a ~1,800 bp fragment of the SSU rDNA</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr">
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="R14" t="inlineStr">
         <is>
           <t>According to gender,BlastocystisST3, ST1, and ST7 were the most frequently found in males, while ST3, ST7 and ST1 were the most frequently found subtypes in females in that order.BlastocystisST1-ST7, ST10 and ST23 were identified in lean and overweight, whereas in obese participants carriage was limited to ST1, ST3 and ST7 (Table 5). Finally,BlastocystisST1, ST3 and ST7 were the most common subtypes across all age groups. The middle-aged (45–64 years) individuals exhibited the highest diversity of subtypes. Regarding region,BlastocystisST1-ST7, ST10 and ST23 were observed in CR province, ST1-ST3 and ST7 in PY province and ST1, ST3, ST5, ST7 and ST10 in CH province (Fig 3). The top threeBlastocystissubtypes in CR were ST3, ST1 and ST23, while ST3, ST7 and ST1 were the most abundant in PY and CH province, in this order.
 (A) Chiang Rai (CR). (B) Phayao (PY). (C) Chachoengsao (CH).
@@ -2620,7 +3432,7 @@
 • DNA extraction and purification</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="S14" t="inlineStr">
         <is>
           <t>Blastocystis is a unicellular eukaryote commonly found in the intestinal tract of humans and other animals. The prevalence of Blastocystis has been investigated in both developed and developing countries, yet its occurrence and distribution in rural locations has been less studied. Herein, we aimed to examine the distribution of Blastocystis colonization in Thai adults representing background populations along a rural/peri-urban gradient, as well as associations between colonization and personal characteristics.
 A total of 238 participants were recruited from rural and peri-urban areas situated in three provinces. The presence of Blastocystis in feces was evaluated using PCR and qPCR. Information on gender, age, region (province), rural/peri-urban location, and body mass index (BMI) was collected.
@@ -2628,7 +3440,7 @@
 This study increases the understanding of the epidemiology of Blastocystis colonization and its association with population parameters and characteristics in middle-income countries.</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="T14" t="inlineStr">
         <is>
           <t>PMID: 38980911
 Full Text: According to gender,BlastocystisST3, ST1, and ST7 were the most frequently found in males, while ST3, ST7 and ST1 were the most frequently found subtypes in females in that order.BlastocystisST1-ST7, ST10 and ST23 were identified in lean and overweight, whereas in obese participants carriage was limited to ST1, ST3 and ST7 (Table 5). Finally,BlastocystisST1, ST3 and ST7 were the most common subtypes across all age groups. The middle-aged (45–64 years) individuals exhibited the highest diversity of subtypes. Regarding region,BlastocystisST1-ST7, ST10 and ST23 were observed in CR province, ST1-ST3 and ST7 in PY province and ST1, ST3, ST5, ST7 and ST10 in CH province (Fig 3). The top threeBlastocystissubtypes in CR were ST3, ST1 and ST23, while ST3, ST7 and ST1 were the most abundant in PY and CH province, in this order.
@@ -2736,7 +3548,7 @@
 • DNA extraction and purification</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="U14" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -2744,35 +3556,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -2882,112 +3702,106 @@
 • DNA extraction and purification</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>Based on my review of the manuscript, here are the key points regarding the methodology and limitations:
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Based on my review of the manuscript, here are some key points regarding the methodology and limitations:
 1. The inclusion/exclusion criteria for participant recruitment are not clearly stated. This is an important limitation that should be acknowledged.
 2. The authors did not check for the presence of other enteric parasites that could act as confounders. This is another limitation that should be noted. 
 3. BMI data was unavailable for 36% of participants, which may have compromised the robustness of the results related to BMI associations. This limitation should be discussed.
-4. The study was restricted to adults, potentially missing effects of primary colonization in younger ages. The authors should discuss this limitation and potential impacts.
-5. The diagnostic algorithm using both nested PCR and qPCR is unclear. The rationale for using both methods should be explained.
-6. The molecular methods section needs better structure and more details on DNA extraction, PCR protocols, sequencing, etc.
-7. Information on mixed infections and how they were detected/analyzed is lacking. 
-8. Some statistical analyses need clarification, particularly regarding the logistic regression model.
-9. Certain figures and tables need improvements in clarity and labeling.
-10. The discussion should be expanded to address these limitations and put the results in broader context with recent literature.
-To address these issues, the authors should:
-- Clearly state inclusion/exclusion criteria 
-- Acknowledge limitations regarding lack of data on other parasites and incomplete BMI data
-- Discuss potential impacts of focusing only on adults
-- Clarify and justify the PCR methodology used
-- Restructure and expand the molecular methods section
-- Provide details on detection of mixed infections
-- Clarify statistical analyses 
-- Improve figures/tables as suggested
-- Expand the discussion to address limitations and compare to recent literature
-Addressing these points would strengthen the manuscript and provide important context for interpreting the results. The core data on Blastocystis prevalence and subtypes is valuable, but needs to be presented with appropriate caveats.</t>
+4. The study was restricted to adults only, potentially missing effects of primary colonization at younger ages. The authors should discuss this limitation and consider citing some of the suggested longitudinal studies in humans and animals.
+5. The diagnostic algorithm using both nested PCR and qPCR is unclear. The rationale for using both methods should be better explained.
+6. The molecular methods section needs to be restructured and described in more detail, with separate subsections for DNA extraction, PCR methods, sequencing, etc.
+7. The sample size is relatively modest, which may limit the strength of some conclusions. This should be acknowledged as a limitation.
+8. More details are needed on how mixed infections were detected and resolved.
+To address these issues, I would recommend:
+- Clearly stating inclusion/exclusion criteria 
+- Acknowledging limitations related to lack of data on other parasites and missing BMI data
+- Discussing potential impacts of focusing only on adults
+- Clarifying and justifying the PCR methodology used
+- Restructuring the molecular methods section
+- Acknowledging sample size limitations
+- Providing more details on detection of mixed infections
+Addressing these points would strengthen the methodology and discussion of limitations in the manuscript. The authors should carefully consider how these factors may impact their results and conclusions.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>38980911</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>38980911</v>
+      </c>
+      <c r="I15" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>primer</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>PCR amplification of DNA was performed using a nested PCR reaction. Briefly, the first PCR used the broad-specificity eukaryotic primer RD5 (5Õ-GGAAGCTTATCTGGTTGA TCCTGCCAGTA-3Õ) and RD3 (5Õ-GGGATCCTGATCCTTC CGCAGGTTCACCTAC-3Õ), which amplifies a ~1,800 bp fragment of the SSU rDNA</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr">
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="R15" t="inlineStr">
         <is>
           <t>• qPCR protocol
 • nested-PCR protocol, including gel electrophoresis and imaging
@@ -3100,7 +3914,7 @@
 PLOS Neglected Tropical Diseases</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="S15" t="inlineStr">
         <is>
           <t>Blastocystis is a unicellular eukaryote commonly found in the intestinal tract of humans and other animals. The prevalence of Blastocystis has been investigated in both developed and developing countries, yet its occurrence and distribution in rural locations has been less studied. Herein, we aimed to examine the distribution of Blastocystis colonization in Thai adults representing background populations along a rural/peri-urban gradient, as well as associations between colonization and personal characteristics.
 A total of 238 participants were recruited from rural and peri-urban areas situated in three provinces. The presence of Blastocystis in feces was evaluated using PCR and qPCR. Information on gender, age, region (province), rural/peri-urban location, and body mass index (BMI) was collected.
@@ -3108,7 +3922,7 @@
 This study increases the understanding of the epidemiology of Blastocystis colonization and its association with population parameters and characteristics in middle-income countries.</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>PMID: 38980911
 Full Text: • qPCR protocol
@@ -3222,7 +4036,7 @@
 PLOS Neglected Tropical Diseases</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="U15" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -3230,35 +4044,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -3374,99 +4196,97 @@
 PLOS Neglected Tropical Diseases</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>Based on the reviewer comments and editorial decision, it appears that:
-1. The manuscript "Blastocystis colonization and associations with population parameters in Thai adults" has been provisionally accepted for publication in PLOS Neglected Tropical Diseases.
-2. The authors have adequately addressed the previous reviewer comments and made the requested revisions.
-3. The study design, methods, analysis, and conclusions are considered appropriate and supported by the data.
-4. Only minor formatting changes are still needed before final acceptance.
-5. The manuscript has been deemed suitable for publication after the latest round of revisions.
-6. The corresponding author will receive typeset proofs to review for any final corrections before publication.
-7. The manuscript will be published open access in PLOS Neglected Tropical Diseases once the final production steps are completed.
-Overall, it seems the peer review and revision process has been completed successfully, and the manuscript is now on track for publication pending only minor final formatting changes. The editors and reviewers appear satisfied with the scientific content and quality of the revised manuscript.</t>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Congratulations on the acceptance of your manuscript "Blastocystis colonization and associations with population parameters in Thai adults" for publication in PLOS Neglected Tropical Diseases! Here are the key points from the acceptance letter:
+- Your manuscript has been formally accepted for publication.
+- It has been passed to the PLOS Production Department to complete the publication process. 
+- All authors will receive a confirmation email upon publication.
+- The corresponding author will soon receive a typeset proof to review for any errors introduced during production.
+- You should carefully review the PDF proof, as this is the last chance to correct any scientific or typesetting errors. Major changes may delay publication.
+- An early version will be published online soon unless you opted out of this process. The final version will be published to the same URL later.
+- The editors thanked you for supporting open-access publishing and look forward to publishing your work.
+The next steps are to watch for the typeset proof to review, make any final minor corrections needed, and then await publication of the early version online. Congratulations again on reaching this milestone with your research!</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>HGNC:12406</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>ENSG00000166402</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>GENE ID:7275</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>TUB</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>rd5</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>39961042</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>39961042</v>
+      </c>
+      <c r="I16" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>primer</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>The primers used in this study were: RD5: 5_ÐATCTGGTTGATCCTGCCAGTÐ3Õ; BhRDr: 5_ÐGAGCTTTTTAACTGCAACAACGÐ3_.</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr">
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>TUB bipartite transcription factor</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="R16" t="inlineStr">
         <is>
           <t>Blastocystissp. is a zoonotic intestinal protozoan that is ubiquitous globally, residing in the gastrointestinal tracts of both humans and various animals. In the present study, a PCR-sequencing tool based on the SSU rRNA gene was employed to investigate the prevalence and subtypes ofBlastocystisspp. in 204 fresh fecal samples collected from 20 captive wildlife species from a bird park in Henan Province, Central China. Overall,Blastocystiswas present in 13.73% (28 out of 204) of the samples and 25% (5 out of 20) of the species. A total of four zoonotic subtypes ofBlastocystissp. were found: ST1, ST3, ST5, and ST27, with the latter being the most prevalent, accounting for 35.71% (10 out of 28) of the 5 species positive forBlastocystissp. To the best of our knowledge, this is the first report ofBlastocystisST27 in birds in China, namely bar-headed goose (Anser indicus)and peafowl (Pavo muticus). The data suggest that captive wildlife, particularly those in bird parks, may frequently be infected with this zoonotic pathogen. Consequently, these animals may serve as potential reservoirs for zoonotic infections in humans.
 Blastocystissp. est un protozoaire intestinal zoonotique omniprésent dans le monde entier, résidant dans le tractus gastro-intestinal des humains et de divers animaux. Dans la présente étude, un outil de séquençage par PCR basé sur le gène SSU rRNA a été utilisé pour étudier la prévalence et les sous-types deBlastocystisspp. dans 204 échantillons de matières fécales fraîches prélevés sur 20 espèces sauvages en captivité dans un parc ornithologique de la province du Henan, en Chine centrale. Dans l’ensemble,Blastocystisétait présent dans 13,73 % (28 sur 204) des échantillons et dans 25 % (5 sur 20) des espèces. Au total, quatre sous-types zoonotiques deBlastocystissp. ont été trouvés : ST1, ST3, ST5 et ST27, ce dernier étant le plus répandu, représentant 35,71% (10 sur 28) des 5 espèces positives pourBlastocystissp. À notre connaissance, il s’agit du premier signalement deBlastocystisST27 chez des oiseaux en Chine, à savoir l’oie à tête barrée (Anser indicus) et le paon (Pavo muticus). Les données suggèrent que la faune en captivité, en particulier celle des parcs ornithologiques, peut être fréquemment infectée par ce pathogène zoonotique. Par conséquent, ces animaux peuvent servir de réservoirs potentiels d’infections zoonotiques pour l’homme.
@@ -3501,12 +4321,12 @@
 Cite this article as: Cui Z, Huang X, Zhang S, Li K, Zhang A, Li Q, Zhang Y, Li J &amp; Qi M. 2025. Molecular characterization and subtype analysis ofBlastocystissp. in captive wildlife in Henan, China. Parasite32, 11.https://doi.org/10.1051/parasite/2025006.</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="S16" t="inlineStr">
         <is>
           <t>Blastocystis sp. is a zoonotic intestinal protozoan that is ubiquitous globally, residing in the gastrointestinal tracts of both humans and various animals. In the present study, a PCR-sequencing tool based on the SSU rRNA gene was employed to investigate the prevalence and subtypes of Blastocystis spp. in 204 fresh fecal samples collected from 20 captive wildlife species from a bird park in Henan Province, Central China. Overall, Blastocystis was present in 13.73% (28 out of 204) of the samples and 25% (5 out of 20) of the species. A total of four zoonotic subtypes of Blastocystis sp. were found: ST1, ST3, ST5, and ST27, with the latter being the most prevalent, accounting for 35.71% (10 out of 28) of the 5 species positive for Blastocystis sp. To the best of our knowledge, this is the first report of Blastocystis ST27 in birds in China, namely bar-headed goose (Anser indicus) and peafowl (Pavo muticus). The data suggest that captive wildlife, particularly those in bird parks, may frequently be infected with this zoonotic pathogen. Consequently, these animals may serve as potential reservoirs for zoonotic infections in humans.</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="T16" t="inlineStr">
         <is>
           <t>PMID: 39961042
 Full Text: Blastocystissp. is a zoonotic intestinal protozoan that is ubiquitous globally, residing in the gastrointestinal tracts of both humans and various animals. In the present study, a PCR-sequencing tool based on the SSU rRNA gene was employed to investigate the prevalence and subtypes ofBlastocystisspp. in 204 fresh fecal samples collected from 20 captive wildlife species from a bird park in Henan Province, Central China. Overall,Blastocystiswas present in 13.73% (28 out of 204) of the samples and 25% (5 out of 20) of the species. A total of four zoonotic subtypes ofBlastocystissp. were found: ST1, ST3, ST5, and ST27, with the latter being the most prevalent, accounting for 35.71% (10 out of 28) of the 5 species positive forBlastocystissp. To the best of our knowledge, this is the first report ofBlastocystisST27 in birds in China, namely bar-headed goose (Anser indicus)and peafowl (Pavo muticus). The data suggest that captive wildlife, particularly those in bird parks, may frequently be infected with this zoonotic pathogen. Consequently, these animals may serve as potential reservoirs for zoonotic infections in humans.
@@ -3542,7 +4362,7 @@
 Cite this article as: Cui Z, Huang X, Zhang S, Li K, Zhang A, Li Q, Zhang Y, Li J &amp; Qi M. 2025. Molecular characterization and subtype analysis ofBlastocystissp. in captive wildlife in Henan, China. Parasite32, 11.https://doi.org/10.1051/parasite/2025006.</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="U16" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -3550,35 +4370,43 @@
     HGNC record ID: HGNC:12406
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -3616,843 +4444,249 @@
 Cite this article as: Cui Z, Huang X, Zhang S, Li K, Zhang A, Li Q, Zhang Y, Li J &amp; Qi M. 2025. Molecular characterization and subtype analysis ofBlastocystissp. in captive wildlife in Henan, China. Parasite32, 11.https://doi.org/10.1051/parasite/2025006.</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="V16" t="inlineStr">
         <is>
           <t>{
 "pmid": "39961042",
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"alternate_abbreviation": "NO",
 "evidence": ""
 }</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>HGNC:12406</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>ENSG00000166402</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>GENE ID:7275</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>TUB</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>rd5</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>HGNC:13919</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ENSG00000234651, ENSG00000096155, ENSG00000233348, ENSG00000204463, ENSG00000228760, ENSG00000229524, ENSG00000227761</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>GENE ID:7917</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>BAG6</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SCYTHE</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>7479945</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>9799223</v>
+      </c>
+      <c r="I17" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>mouse phenotype biomarker</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>literature defined (uniprot alternative protein name)</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>abstract</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>We report a mouse model of type I Usher syndrome, rd5, whose linkage on mouse chromosome 7 to Hbb and tub has homology to human Usher I reported on human chromosome 11p15. The electroretinogram in homozygous rd5/rd5 mouse is never normal with reduced amplitudes that extinguish by 6 months.</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>TUB bipartite transcription factor</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>Usher syndrome is a group of diseases with autosomal recessive inheritance, congenital hearing loss, and the development of retinitis pigmentosa, a progressive retinal degeneration characterized by night blindness and visual field loss over several decades. The causes of Usher syndrome are unknown and no animal models have been available for study. Four human gene sites have been reported, suggesting at least four separate forms of Usher syndrome. We report a mouse model of type I Usher syndrome, rd5, whose linkage on mouse chromosome 7 to Hbb and tub has homology to human Usher I reported on human chromosome 11p15. The electroretinogram in homozygous rd5/rd5 mouse is never normal with reduced amplitudes that extinguish by 6 months. Auditory-evoked response testing demonstrates increased hearing thresholds more than control at 3 weeks of about 30 decibels (dB) that worsen to about 45 dB by 6 months.</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>PMID: 7479945
-Abstract: Usher syndrome is a group of diseases with autosomal recessive inheritance, congenital hearing loss, and the development of retinitis pigmentosa, a progressive retinal degeneration characterized by night blindness and visual field loss over several decades. The causes of Usher syndrome are unknown and no animal models have been available for study. Four human gene sites have been reported, suggesting at least four separate forms of Usher syndrome. We report a mouse model of type I Usher syndrome, rd5, whose linkage on mouse chromosome 7 to Hbb and tub has homology to human Usher I reported on human chromosome 11p15. The electroretinogram in homozygous rd5/rd5 mouse is never normal with reduced amplitudes that extinguish by 6 months. Auditory-evoked response testing demonstrates increased hearing thresholds more than control at 3 weeks of about 30 decibels (dB) that worsen to about 45 dB by 6 months.</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>We now report the purification of a 150 kDa reaper-interacting protein from Xenopus egg extracts, which we have named Scythe. Scythe is highly conserved among vertebrates and contains a ubiquitin-like domain near its N-terminus.</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>BAG cochaperone 6</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Reaper is a central regulator of apoptosis in Drosophila melanogaster. With no obvious catalytic activity or homology to other known apoptotic regulators, reaper's mechanism of action has been obscure. We recently reported that recombinant Drosophila reaper protein induced rapid mitochondrial cytochrome c release, caspase activation and apoptotic nuclear fragmentation in extracts of Xenopus eggs. We now report the purification of a 150 kDa reaper-interacting protein from Xenopus egg extracts, which we have named Scythe. Scythe is highly conserved among vertebrates and contains a ubiquitin-like domain near its N-terminus. Immunodepletion of Scythe from extracts completely prevented reaper-induced apoptosis without affecting apoptosis triggered by activated caspases. Moreover, a truncated variant of Scythe lacking the N-terminal domain induced apoptosis even in the absence of reaper. These data suggest that Scythe is a novel apoptotic regulator that is an essential component in the pathway of reaper-induced apoptosis.</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>PMID: 9799223
+Abstract: Reaper is a central regulator of apoptosis in Drosophila melanogaster. With no obvious catalytic activity or homology to other known apoptotic regulators, reaper's mechanism of action has been obscure. We recently reported that recombinant Drosophila reaper protein induced rapid mitochondrial cytochrome c release, caspase activation and apoptotic nuclear fragmentation in extracts of Xenopus eggs. We now report the purification of a 150 kDa reaper-interacting protein from Xenopus egg extracts, which we have named Scythe. Scythe is highly conserved among vertebrates and contains a ubiquitin-like domain near its N-terminus. Immunodepletion of Scythe from extracts completely prevented reaper-induced apoptosis without affecting apoptosis triggered by activated caspases. Moreover, a truncated variant of Scythe lacking the N-terminal domain induced apoptosis even in the absence of reaper. These data suggest that Scythe is a novel apoptotic regulator that is an essential component in the pathway of reaper-induced apoptosis.</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
-    Alias gene symbol: rd5
-    HGNC record ID: HGNC:12406
-    Primary gene symbol: TUB
-    Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
+    Alias gene symbol: SCYTHE
+    HGNC record ID: HGNC:13919
+    Primary gene symbol: BAG6
+    Official HGNC gene name: BAG cochaperone 6
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
-PMID: 7479945
-Abstract: Usher syndrome is a group of diseases with autosomal recessive inheritance, congenital hearing loss, and the development of retinitis pigmentosa, a progressive retinal degeneration characterized by night blindness and visual field loss over several decades. The causes of Usher syndrome are unknown and no animal models have been available for study. Four human gene sites have been reported, suggesting at least four separate forms of Usher syndrome. We report a mouse model of type I Usher syndrome, rd5, whose linkage on mouse chromosome 7 to Hbb and tub has homology to human Usher I reported on human chromosome 11p15. The electroretinogram in homozygous rd5/rd5 mouse is never normal with reduced amplitudes that extinguish by 6 months. Auditory-evoked response testing demonstrates increased hearing thresholds more than control at 3 weeks of about 30 decibels (dB) that worsen to about 45 dB by 6 months.</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr">
+PMID: 9799223
+Abstract: Reaper is a central regulator of apoptosis in Drosophila melanogaster. With no obvious catalytic activity or homology to other known apoptotic regulators, reaper's mechanism of action has been obscure. We recently reported that recombinant Drosophila reaper protein induced rapid mitochondrial cytochrome c release, caspase activation and apoptotic nuclear fragmentation in extracts of Xenopus eggs. We now report the purification of a 150 kDa reaper-interacting protein from Xenopus egg extracts, which we have named Scythe. Scythe is highly conserved among vertebrates and contains a ubiquitin-like domain near its N-terminus. Immunodepletion of Scythe from extracts completely prevented reaper-induced apoptosis without affecting apoptosis triggered by activated caspases. Moreover, a truncated variant of Scythe lacking the N-terminal domain induced apoptosis even in the absence of reaper. These data suggest that Scythe is a novel apoptotic regulator that is an essential component in the pathway of reaper-induced apoptosis.</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
         <is>
           <t>{
-"pmid": "7479945",
-"alias_symbol": "rd5",
-"primary_gene_symbol": "TUB",
-"name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
+"pmid": "9799223",
+"alias_symbol": "SCYTHE",
+"primary_gene_symbol": "BAG6",
+"name": "BAG cochaperone 6",
+"alternate_abbreviation": "NO",
 "evidence": ""
 }</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>HGNC:12406</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>ENSG00000166402</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>GENE ID:7275</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>TUB</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>rd5</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>HGNC:13919</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ENSG00000234651, ENSG00000096155, ENSG00000233348, ENSG00000204463, ENSG00000228760, ENSG00000229524, ENSG00000227761</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>GENE ID:7917</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>BAG6</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SCYTHE</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>9390831</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>37879364</v>
+      </c>
+      <c r="I18" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>mouse phenotype biomarker</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>literature defined (uniprot alternative protein name)</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>abstract</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>Mice homozygous for a defect of the tub (rd5) gene exhibit cochlear and retinal degeneration combined with obesity, and resemble certain human autosomal recessive sensory deficit syndromes.</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>TUB bipartite transcription factor</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>These authors contributed equally to this work.
-These authors jointly coordinated this work.
-Inherited retinal degeneration (IRD) represents a clinically variable and genetically heterogeneous group of disorders characterized by photoreceptor dysfunction. These diseases typically present with progressive severe vision loss and variable onset, ranging from birth to adulthood. Genomic sequencing has allowed to identify novel IRD-related genes, most of which encode proteins contributing to photoreceptor-cilia biogenesis and/or function. Despite these insights, knowledge gaps hamper a molecular diagnosis in one-third of IRD cases. By exome sequencing in a cohort of molecularly unsolved individuals with IRD, we identified a homozygous splice site variant affecting the transcript processing of TUB, encoding the first member of the Tubby family of bipartite transcription factors, in a sporadic case with retinal dystrophy. A truncating homozygous variant in this gene had previously been reported in a single family with three subjects sharing retinal dystrophy and obesity. The clinical assessment of the present patient documented a slightly increased body mass index and no changes in metabolic markers of obesity, but confirmed the occurrence of retinal detachment. In vitro studies using patient-derived fibroblasts showed the accelerated degradation of the encoded protein and aberrant cilium morphology and biogenesis. These findings definitely link impaired TUB function to retinal dystrophy and provide new data on the clinical characterization of this ultra-rare retinal ciliopathy.
-Inherited retinal degeneration (IRD) occurs in a clinically variable and genetically heterogeneous group of conditions characterized by photoreceptor degeneration and/or dysfunction [1]. The prevalence of monogenic IRD is estimated as 1 in 2000 individuals, affecting more than 2 million people worldwide [2]. This group of disorders typically present with severe vision loss that can be progressive, having an onset ranging from birth to late adulthood. Severe visual impairment affects mobility and independence, posing relevant psychological and economic burdens [3]. In the last ten years, genomic sequencing has allowed the identification of several genes implicated in IRD (for an updated list see the RetNet database,https://sph.uth.edu/retnet/). These genes encode proteins that have different roles in visual function, contributing to key processes in the cells of the pigmented cell layer and neurosensory retina [4,5]. Notably, retinal degeneration is frequently observed in ciliopathies, and a portion of IRD-related genes codifies for proteins involved in biogenesis and the maintenance of photoreceptor primary cilium [6,7,8,9]. Among these genes,TUB[MIM #601197], which encodes the first member of the Tubby family of bipartite transcription factors, has recently reported to be associated with a novel condition characterized by retinal dystrophy and obesity [MIM #616188] [10]. A truncating homozygousTUBvariant [c.1194_1195delAG, p.Arg398Serfs*9] was identified in a single family with three affected members, suggesting loss of function (LoF) as the pathomechanism underlying the disorder. The TUB family of transcription factors counts four members in vertebrates (TUB, TULP1, TULP2 and TULP3), sharing a similar domain organization including a highly conserved C-terminal domain mediating DNA binding and a divergent N-terminal region encompassing the nuclear localization signal and the transcriptional activation domain implicated in protein–protein binding [11]. A conserved region at the N-terminus enables some members of the Tubby family, including TUB, to bind to the ciliary intraflagellar transport A protein (IFTAP) [12]. Similar to the other members of the TULP family, TUB is also implicated in the control of the initiation of phagocytosis, facilitating the removal of apoptotic cells or cellular debris by retinal pigmented epithelium (RPE) cells and macrophages [13]. Since the original report, no other subject carrying biallelicTUBvariants has been described.
-In this study, we report on an additional subject with retinal dystrophy carrying a homozygous LoF variant inTUB. In vitro analyses provide evidence of the disruptive functional impact of the variant onTUBtranscript processing. We also show that the loss of TUB is associated with a defective cilium morphology and biogenesis in the primary patient’s fibroblasts. Our findings confirm the involvement of defective TUB function in retinal dystrophy and define this disorder as a novel ciliopathy.
-The proband is a 35-year-old male, the first child of healthy non-consanguineous parents of European descent (Figure 1). Family history was negative for retinal diseases or other congenital defects. The proband was born at term after an uneventful pregnancy. Length and weight at birth were reported as within the normal range. Apgar score was 8–10. No hearing impairment and/or learning difficulties were documented during the first year of age.
-At 5 years, the subject required consulting ophthalmologists for referring color blindness. A “blonde” aspect of the fundus oculi was observed and reduced full-field flash photopic and scotopic electroretinogram (ERG) responses were recorded. Visual acuity was not investigated at that time. Ophthalmological assessment at 26 years was suggestive of cone-rod dystrophy. Visual acuity was 0.8 Snellen in his right eye (RE) with myopic and astigmatic refractive error (RE: -4.50 dioptre sphere and -1 dioptre cylinder at 20°), and 0.2 Snellen in his left eye (LE) with myopic refractive error (LE: -2.00 dioptre sphere). Goldmann visual field was generally constricted, with reduced sensitivity in the superior central field in the RE and presented peripheral constriction and relative central scotoma in the LE. Light and dark adaptation sensitivity curves showed abnormal thresholds for both cones and rods. No number at the Ishihara charts were recognized. Intraocular pressure was within normal limits. The slit lamp examination biomicroscopy of the anterior segment was normal for cornea, iris and lens appearance. Fundus examination revealed bilateral optic disc pallor, depigmented aspect of the choroidal and retinal structures, diffuse retinal dystrophy with absence of intraretinal pigment dispersion or vitreous abnormalities and arteriolar attenuation. Full-field scotopic and photopic electroretinograms showed reduced a-wave and b-wave amplitude responses and delayed implicit times. Multifocal ERG ring analysis documented reduced response amplitude densities in all examined areas from the foveal center up to 20° of foveal eccentricity in both eyes (LE &gt; RE). After reduced visual field in his LE, a large area of retinoschisis in the infero-temporal sector was observed by fundoscopy, which later progressed, resulting in full retinal detachment of the LE. The subject underwent to pars plana vitrectomy with silicon oil (30% polydimethylsiloxane, PDMS) tamponade. He underwent cataract surgery in his LE and to subsequent vitreo-retinal surgeries for relapsing retinal detachments in same eye (PDMS/perfluorocarbon liquid (PFCL)/PDMS tamponades exchange and intra-operatory laser treatment; PDMS/heavy silicon oil tamponades exchange and intra-operatory laser). One year later, he developed vitreo-retinal proliferation and retinal fibrosis in the LE, and visual acuity was hand motion; therefore, the subject underwent retinotomy and heavy silicon oil/PDMS tamponades exchange.
-At last evaluation (35 years), the subject presented with a good clinical condition. No cognitive deficit nor behavioral issues were observed, and no craniofacial dysmorphism and truncal obesity were noticed. An accurate endocrinological examination was uninformative. Anthropometric assessment displayed a height of 177.5 cm (+0.1 SD), weight of 95.70 kg (+1.6 SD), and OFC 60 cm (+0.2 SD) and BMI of 30.30 Kg/m2(+1.6 SD). Tanner stage was Ph5Pg5, with a testicular volume 20 mL bilaterally. The subject’s visual acuity was 0.8 Snellen in his RE and light perception in his LE. Fundus oculi showed the unmodified condition of RE and diffuse chorio-retinal atrophy in the LE, as for visible vitreo-retinal surgical outcomes. Ultrawide field fundus photography showed macular atrophy in absence of peripheral pigment and confirmed a “blonde” aspect of the retina (Figure 2A). Fundus autofluorescence (FAF) revealed an hypoautoflorescent area in the macula due to RPE atrophy and hyper/hypoautofluorescence mottling in the posterior pole and immediately outside the vascular arcades (Figure 2B). The SD-OCT showed a disruption of the outer retina, including ELM, ellipsoid zone and RPE with outer retinal debris at the level of the RPE in the parafoveal region (Figure 2C). Full-field flash scotopic (Figure 2D) and photopic ERG confirmed reduced a-wave and b-wave amplitude responses and delayed implicit times in the RE. Similarly, multifocal ERG ring analysis, recordable only in the RE, showed the worsening of the response amplitude densities in all examined areas (0–20°) (Figure 2E), as compared to the previous examinations. Similarly, Goldmann visual field in his RE showed progressive constriction of the peripheral isopters and a ring scotoma enclosed between 10–20° of the visual field (Figure 2F); it was not executable, however, in his LE. Color blindness was also confirmed. Neck and abdominal ultrasound assessment did not reveal any abnormality. Measurements of basal hormones by the anterior pituitary, glycaemia and insulin were within the normal range. Basal plasma leptin level was in the low normal range, showing no leptin resistance. During his follow-up, clinical and ophthalmological assessments of other family members (parents and younger brother) were unremarkable.
-Trio-based WES allowed to identify a homozygous splice siteTUBvariant (chr11:8122545G &gt; A, GRCh37.p13; c.1387 + 1G &gt; A,NM_177972.3) as the only clinically and functionally relevant event putatively linked to the disorder (Supplemental Table S1). The variant had previously been annotated in public databases (dbSNP, rs1040410003) with low frequency (gnomAD v3.1, MAF = 0.00001972) at the heterozygous state. It was classified as likely pathogenic (PVS1/PM2/PP5) according to the American College of Medical Genetics and Genomics-Association for Molecular Pathology (ACMG-AMP) criteria (ClinVar: VCV000865971.1) [14]. Sanger sequencing confirmed the homozygosity for the variant in the proband and the heterozygous status in the healthy parents and unaffected sib (Figure 1).
-Since the variant was predicted to affect the exon 11 donor splice site, the total RNA from patient-derived skin primary fibroblasts was used to characterize the impact of the nucleotide change on transcript processing. The cDNA fragment encompassing the relevant exons was amplified, confirming the presence of two aberrantly spliced products (Figure 3A). The two aberrant PCR amplicons were isolated from agarose gel, purified and sequenced via Sanger. The former (500 bp) was derived from skipping of the penultimate exon (exon 11, ENST00000299506.3), resulting in a premature termination codon (i.e., p.Glu406Argfs*4), while the latter (1172 bp) was the result of retention of intron 10, resulting in a TUB protein having a divergent 19-residue-long C-terminus and lacking the last 44 amino acids (p.Pro463Hisfs*19) (Figure 3B).
-In the patient’s skin fibroblasts, the predicted TUBGlu406Argfs*4protein was undetectable by Western blot [WB] analysis, while the TUBPro463Hisfs*19protein was poorly detectable likely due to accelerated degradation (Figure 3C, left panel). Consistently, the endogenous TUBPro463Hisfs*19level was partially rescued by blocking the proteasomal degradation pathway using MG132 (Figure 3C, right panel).
-To investigate the cellular localization of the mutated protein, cytoplasm and nuclear cell fractions were obtained and analyzed by WB. The results demonstrate that both the wild-type (wt) and mutant TUB proteins were almost exclusively localized in the nucleus (Figure 3D). This finding was also confirmed by confocal microscopy analysis that evidenced the nuclear localization of the TUB mutant (Figure 4A).
-Based on the documented role of TUB in early ciliogenesis [15], we assessed the localization of TUB at the cilium, but we failed to observe any consistent co-localization, possibly due to the low diffused levels of the protein in the cytoplasm To investigate the impact of defective TUB function on the morphogenesis of the primary cilium, a confocal analysis on primary fibroblasts was performed using antibodies against ARL13B, which localizes to primary cilia, and pericentrin, a component of the centrosome, which stains the basal body. As shown inFigure 4B, while almost all the control cells showed a primary cilium, 40% of the fibroblasts carrying the homozygous splice site variant inTUBdid not show a primary cilium. Moreover, while no significant difference was observed in ciliary axoneme length between the starved control and mutant cells, a large percentage of the latter showed an abnormal cilium morphology and a poorly defined and disorganized basal body (Figure 4C).
-The loss of TUB function was recently reported to underlie a novel IRD condition based on the identification of homozygosity for a 2 bp deletion (c.1194_1195delAG) causing the premature termination of the protein (p.Arg398Serfs*9) shared by three affected members of a single consanguineous family [10]. While the combination of retinal dystrophy and early onset obesity can be reminiscent of other disorders (e.g., Bardet–Biedl syndrome (MIM#PS209900) and Alstrom syndrome (MIM#203800)), the absence of other clinically relevant feature/sign was suggestive of a previously unreported ciliopathy [10]. In this paper, we report on a second disruptive variant (c.1387 + 1G &gt; A) affectingTUBin a subject with features that overlap with those previously described in the affected members of the original family.
-In the present and previously reported affected individuals, the ocular phenotype associated with defective TUB function is characterized by widespread retinal pigment epithelial (RPE) atrophy, deteriorating vision, the myopic and astigmatic refractive defect, the blonde fundus appearance, the ERG and OCT findings and progression of the disease (Figure 2). Notably, retinal detachment, without vitreous hemorrhage, was invariantly documented in the four individuals with biallelic inactivatingTUBvariants, suggesting that this feature likely represent a common finding in the disorder.
-Early onset obesity had previously been considered a major feature of the TUB-related condition [10], even though only two of three affected sibs were found obese (BMI &gt; 30), and the glycemic and lipid profiles in one of affected sibs were found within the normal range. The finding of obesity in the apparently healthy father (heterozygous carrier) suggests a possible co-occurring genetic event contributing to obesity in the family. In the present report, the clinical assessment of the affected individual documented increased weight (95.7 kg, +1.6 SD) and BMI (30.3, +1.6 SD), thus indicating overweight, in absence of other signs of obesity. Although evidence suggests that a defective TUB function may result in disturbances in insulin and leptin activity and obesity in mice [16,17,18,19], based on the collected findings, the relevance of TUB in human obesity requires further study. To assess whether TUB LoF could impact on hypothalamic pathways, food intake and adiposity, the metabolic profile of the affected individual was investigated. Accurate endocrinological examination did not reveal any abnormality, and the measurements of basal hormones by the anterior pituitary, glycaemia, insulin and leptin were within the normal range, thus ruling out insulin or leptin resistance. Consistently, instrumental investigations (X-ray and ultrasound analyses) documented no sign of glycogen accumulation in the internal organs. Consistently, the absence of significant changes in lipid storage was demonstrated by thin-layer chromatography (HPTLC) analysis in proband-derived fibroblast (Figure S1), allowing to confirm an apparently normal endocrine–metabolic profile in the affected individual. Of note, the Tubby protein has been involved in cochlear degeneration [20,21]. Based on this functional link, we evaluated the occurrence of hearing problems and cochlear degeneration, which were not observed.
-The homozygousTUBvariant was predicted to affect transcript processing, causing the skipping of exon 11 and intron retention, resulting in a frameshift with the premature termination of the TUB protein. mRNA analysis in proband-derived fibroblasts confirmed a disruptive impact of the splice site change documenting two aberrantly processed transcripts predicted to encode a 406-residue-long protein (p.Glu406Argfs*4) that probably is not able to proceed in protein synthesis, and a 481-residue-long protein (p.Pro463Hisfs*19) characterized by a divergent C-terminus characterized by accelerated degradation (Figure 3B). These findings confirm LoF as the pathomechanism underlying this disorder.
-Primary cilia are microtubule-based organelles that extend from the apical surface of the majority of mammalian cells. Cilia act as “cellular antennae”, receiving different inputs from the extracellular environment and transducing signals in response to stimuli [22]. A complex process required for proper cilia biogenesis function is the intraflagellar transport, which is required for assembling cilia and trafficking within primary cilia [23]. In this context, IFT-A has historically been believed to mediate retrograde intraflagellar transport inside the cilia and an IFT-A-binding domain at the TUB N-terminus has been demonstrated recently [24]. Moreover, co-localization between TUB and rootletin, the major structural component of the ciliary rootlet, has been observed in human retinal photoreceptors [10]. The use of a more informative in vitro model (e.g., induced pluripotent-stem-cell-derived retinal-pigment epithelium cells) and experimental strategies (e.g., siRNA-mediated TUB silencing) is required to appreciate more accurately the functional relevance of TUB in an appropriate cellular context.
-In summary, we confirm the link between TUB LoF and a new condition of human retinal ciliopathy and provide evidence of an altered cilium morphology/biogenesis in patient-derived fibroblasts. In fact, these cells displayed a reduced number of cilia when compared to the control cells, with a poorly defined and disorganized basal body structure, which are expected to prevent normal protein trafficking along the cilium. While these findings could explain the degeneration of photoreceptors characterizing this disorder, a relatively overall mild presentation has been associated with mutations in this gene. Multiple factors might contribute to this picture. First, the functional relevance of TUB in the context of ciliogenesis and cilium function might vary in different cell lineages. Second, functional compensation exerted by other related proteins might contribute to buffer the severity of the endophenotype. Third, specific cell lineages (e.g., rod and cone cells) might be particularly sensitive to TUB LoF. The collection of additional patients with biallelic variants in the gene will allow a more accurate characterization of the clinical spectrum associated with TUB LoF. Based on these considerations, TUB loss of function could be considered as responsible for a novel form of isolated retinal ciliopathy.</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>Mice homozygous for a defect of the tub (rd5) gene exhibit cochlear and retinal degeneration combined with obesity, and resemble certain human autosomal recessive sensory deficit syndromes. To establish the progressive nature of sensory cell loss associated with the tub gene, and to differentiate tub-related losses from those associated with the C57 background on which tub arose, we evaluated cochleas and retinas from tub/tub, tub/+, and +/+ mice, aged 2 weeks to 1 year by light and electron microscopy. Cochleas from mice of all three genotypes show progressive inner (IHC) and outer hair cell (OHC) loss. Relative to tub/+ and +/+ animals, however, tub homozygotes show accelerated OHC loss, affecting the extreme cochlear base (hook region) by 1 month, and the apex by 6 months. IHC loss in tub/tub animals is accelerated in the basal half of the cochlea, affecting the hook region by 6 months. Spiral ganglion cell losses were observed only in tub/tub mice, and only in the cochlear base. Retinas of tub/tub mice are abnormal at maturity, exhibiting shortened photoreceptor outer segments by 2 weeks, and progressive photoreceptor loss thereafter. Because the tub mutation causes degeneration of sensory cells in the ear and eye but has no other neurological effects, tubby mice hold unique promise for the study of human syndromic sensory loss.</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>PMID: 9390831
-Full Text: These authors contributed equally to this work.
-These authors jointly coordinated this work.
-Inherited retinal degeneration (IRD) represents a clinically variable and genetically heterogeneous group of disorders characterized by photoreceptor dysfunction. These diseases typically present with progressive severe vision loss and variable onset, ranging from birth to adulthood. Genomic sequencing has allowed to identify novel IRD-related genes, most of which encode proteins contributing to photoreceptor-cilia biogenesis and/or function. Despite these insights, knowledge gaps hamper a molecular diagnosis in one-third of IRD cases. By exome sequencing in a cohort of molecularly unsolved individuals with IRD, we identified a homozygous splice site variant affecting the transcript processing of TUB, encoding the first member of the Tubby family of bipartite transcription factors, in a sporadic case with retinal dystrophy. A truncating homozygous variant in this gene had previously been reported in a single family with three subjects sharing retinal dystrophy and obesity. The clinical assessment of the present patient documented a slightly increased body mass index and no changes in metabolic markers of obesity, but confirmed the occurrence of retinal detachment. In vitro studies using patient-derived fibroblasts showed the accelerated degradation of the encoded protein and aberrant cilium morphology and biogenesis. These findings definitely link impaired TUB function to retinal dystrophy and provide new data on the clinical characterization of this ultra-rare retinal ciliopathy.
-Inherited retinal degeneration (IRD) occurs in a clinically variable and genetically heterogeneous group of conditions characterized by photoreceptor degeneration and/or dysfunction [1]. The prevalence of monogenic IRD is estimated as 1 in 2000 individuals, affecting more than 2 million people worldwide [2]. This group of disorders typically present with severe vision loss that can be progressive, having an onset ranging from birth to late adulthood. Severe visual impairment affects mobility and independence, posing relevant psychological and economic burdens [3]. In the last ten years, genomic sequencing has allowed the identification of several genes implicated in IRD (for an updated list see the RetNet database,https://sph.uth.edu/retnet/). These genes encode proteins that have different roles in visual function, contributing to key processes in the cells of the pigmented cell layer and neurosensory retina [4,5]. Notably, retinal degeneration is frequently observed in ciliopathies, and a portion of IRD-related genes codifies for proteins involved in biogenesis and the maintenance of photoreceptor primary cilium [6,7,8,9]. Among these genes,TUB[MIM #601197], which encodes the first member of the Tubby family of bipartite transcription factors, has recently reported to be associated with a novel condition characterized by retinal dystrophy and obesity [MIM #616188] [10]. A truncating homozygousTUBvariant [c.1194_1195delAG, p.Arg398Serfs*9] was identified in a single family with three affected members, suggesting loss of function (LoF) as the pathomechanism underlying the disorder. The TUB family of transcription factors counts four members in vertebrates (TUB, TULP1, TULP2 and TULP3), sharing a similar domain organization including a highly conserved C-terminal domain mediating DNA binding and a divergent N-terminal region encompassing the nuclear localization signal and the transcriptional activation domain implicated in protein–protein binding [11]. A conserved region at the N-terminus enables some members of the Tubby family, including TUB, to bind to the ciliary intraflagellar transport A protein (IFTAP) [12]. Similar to the other members of the TULP family, TUB is also implicated in the control of the initiation of phagocytosis, facilitating the removal of apoptotic cells or cellular debris by retinal pigmented epithelium (RPE) cells and macrophages [13]. Since the original report, no other subject carrying biallelicTUBvariants has been described.
-In this study, we report on an additional subject with retinal dystrophy carrying a homozygous LoF variant inTUB. In vitro analyses provide evidence of the disruptive functional impact of the variant onTUBtranscript processing. We also show that the loss of TUB is associated with a defective cilium morphology and biogenesis in the primary patient’s fibroblasts. Our findings confirm the involvement of defective TUB function in retinal dystrophy and define this disorder as a novel ciliopathy.
-The proband is a 35-year-old male, the first child of healthy non-consanguineous parents of European descent (Figure 1). Family history was negative for retinal diseases or other congenital defects. The proband was born at term after an uneventful pregnancy. Length and weight at birth were reported as within the normal range. Apgar score was 8–10. No hearing impairment and/or learning difficulties were documented during the first year of age.
-At 5 years, the subject required consulting ophthalmologists for referring color blindness. A “blonde” aspect of the fundus oculi was observed and reduced full-field flash photopic and scotopic electroretinogram (ERG) responses were recorded. Visual acuity was not investigated at that time. Ophthalmological assessment at 26 years was suggestive of cone-rod dystrophy. Visual acuity was 0.8 Snellen in his right eye (RE) with myopic and astigmatic refractive error (RE: -4.50 dioptre sphere and -1 dioptre cylinder at 20°), and 0.2 Snellen in his left eye (LE) with myopic refractive error (LE: -2.00 dioptre sphere). Goldmann visual field was generally constricted, with reduced sensitivity in the superior central field in the RE and presented peripheral constriction and relative central scotoma in the LE. Light and dark adaptation sensitivity curves showed abnormal thresholds for both cones and rods. No number at the Ishihara charts were recognized. Intraocular pressure was within normal limits. The slit lamp examination biomicroscopy of the anterior segment was normal for cornea, iris and lens appearance. Fundus examination revealed bilateral optic disc pallor, depigmented aspect of the choroidal and retinal structures, diffuse retinal dystrophy with absence of intraretinal pigment dispersion or vitreous abnormalities and arteriolar attenuation. Full-field scotopic and photopic electroretinograms showed reduced a-wave and b-wave amplitude responses and delayed implicit times. Multifocal ERG ring analysis documented reduced response amplitude densities in all examined areas from the foveal center up to 20° of foveal eccentricity in both eyes (LE &gt; RE). After reduced visual field in his LE, a large area of retinoschisis in the infero-temporal sector was observed by fundoscopy, which later progressed, resulting in full retinal detachment of the LE. The subject underwent to pars plana vitrectomy with silicon oil (30% polydimethylsiloxane, PDMS) tamponade. He underwent cataract surgery in his LE and to subsequent vitreo-retinal surgeries for relapsing retinal detachments in same eye (PDMS/perfluorocarbon liquid (PFCL)/PDMS tamponades exchange and intra-operatory laser treatment; PDMS/heavy silicon oil tamponades exchange and intra-operatory laser). One year later, he developed vitreo-retinal proliferation and retinal fibrosis in the LE, and visual acuity was hand motion; therefore, the subject underwent retinotomy and heavy silicon oil/PDMS tamponades exchange.
-At last evaluation (35 years), the subject presented with a good clinical condition. No cognitive deficit nor behavioral issues were observed, and no craniofacial dysmorphism and truncal obesity were noticed. An accurate endocrinological examination was uninformative. Anthropometric assessment displayed a height of 177.5 cm (+0.1 SD), weight of 95.70 kg (+1.6 SD), and OFC 60 cm (+0.2 SD) and BMI of 30.30 Kg/m2(+1.6 SD). Tanner stage was Ph5Pg5, with a testicular volume 20 mL bilaterally. The subject’s visual acuity was 0.8 Snellen in his RE and light perception in his LE. Fundus oculi showed the unmodified condition of RE and diffuse chorio-retinal atrophy in the LE, as for visible vitreo-retinal surgical outcomes. Ultrawide field fundus photography showed macular atrophy in absence of peripheral pigment and confirmed a “blonde” aspect of the retina (Figure 2A). Fundus autofluorescence (FAF) revealed an hypoautoflorescent area in the macula due to RPE atrophy and hyper/hypoautofluorescence mottling in the posterior pole and immediately outside the vascular arcades (Figure 2B). The SD-OCT showed a disruption of the outer retina, including ELM, ellipsoid zone and RPE with outer retinal debris at the level of the RPE in the parafoveal region (Figure 2C). Full-field flash scotopic (Figure 2D) and photopic ERG confirmed reduced a-wave and b-wave amplitude responses and delayed implicit times in the RE. Similarly, multifocal ERG ring analysis, recordable only in the RE, showed the worsening of the response amplitude densities in all examined areas (0–20°) (Figure 2E), as compared to the previous examinations. Similarly, Goldmann visual field in his RE showed progressive constriction of the peripheral isopters and a ring scotoma enclosed between 10–20° of the visual field (Figure 2F); it was not executable, however, in his LE. Color blindness was also confirmed. Neck and abdominal ultrasound assessment did not reveal any abnormality. Measurements of basal hormones by the anterior pituitary, glycaemia and insulin were within the normal range. Basal plasma leptin level was in the low normal range, showing no leptin resistance. During his follow-up, clinical and ophthalmological assessments of other family members (parents and younger brother) were unremarkable.
-Trio-based WES allowed to identify a homozygous splice siteTUBvariant (chr11:8122545G &gt; A, GRCh37.p13; c.1387 + 1G &gt; A,NM_177972.3) as the only clinically and functionally relevant event putatively linked to the disorder (Supplemental Table S1). The variant had previously been annotated in public databases (dbSNP, rs1040410003) with low frequency (gnomAD v3.1, MAF = 0.00001972) at the heterozygous state. It was classified as likely pathogenic (PVS1/PM2/PP5) according to the American College of Medical Genetics and Genomics-Association for Molecular Pathology (ACMG-AMP) criteria (ClinVar: VCV000865971.1) [14]. Sanger sequencing confirmed the homozygosity for the variant in the proband and the heterozygous status in the healthy parents and unaffected sib (Figure 1).
-Since the variant was predicted to affect the exon 11 donor splice site, the total RNA from patient-derived skin primary fibroblasts was used to characterize the impact of the nucleotide change on transcript processing. The cDNA fragment encompassing the relevant exons was amplified, confirming the presence of two aberrantly spliced products (Figure 3A). The two aberrant PCR amplicons were isolated from agarose gel, purified and sequenced via Sanger. The former (500 bp) was derived from skipping of the penultimate exon (exon 11, ENST00000299506.3), resulting in a premature termination codon (i.e., p.Glu406Argfs*4), while the latter (1172 bp) was the result of retention of intron 10, resulting in a TUB protein having a divergent 19-residue-long C-terminus and lacking the last 44 amino acids (p.Pro463Hisfs*19) (Figure 3B).
-In the patient’s skin fibroblasts, the predicted TUBGlu406Argfs*4protein was undetectable by Western blot [WB] analysis, while the TUBPro463Hisfs*19protein was poorly detectable likely due to accelerated degradation (Figure 3C, left panel). Consistently, the endogenous TUBPro463Hisfs*19level was partially rescued by blocking the proteasomal degradation pathway using MG132 (Figure 3C, right panel).
-To investigate the cellular localization of the mutated protein, cytoplasm and nuclear cell fractions were obtained and analyzed by WB. The results demonstrate that both the wild-type (wt) and mutant TUB proteins were almost exclusively localized in the nucleus (Figure 3D). This finding was also confirmed by confocal microscopy analysis that evidenced the nuclear localization of the TUB mutant (Figure 4A).
-Based on the documented role of TUB in early ciliogenesis [15], we assessed the localization of TUB at the cilium, but we failed to observe any consistent co-localization, possibly due to the low diffused levels of the protein in the cytoplasm To investigate the impact of defective TUB function on the morphogenesis of the primary cilium, a confocal analysis on primary fibroblasts was performed using antibodies against ARL13B, which localizes to primary cilia, and pericentrin, a component of the centrosome, which stains the basal body. As shown inFigure 4B, while almost all the control cells showed a primary cilium, 40% of the fibroblasts carrying the homozygous splice site variant inTUBdid not show a primary cilium. Moreover, while no significant difference was observed in ciliary axoneme length between the starved control and mutant cells, a large percentage of the latter showed an abnormal cilium morphology and a poorly defined and disorganized basal body (Figure 4C).
-The loss of TUB function was recently reported to underlie a novel IRD condition based on the identification of homozygosity for a 2 bp deletion (c.1194_1195delAG) causing the premature termination of the protein (p.Arg398Serfs*9) shared by three affected members of a single consanguineous family [10]. While the combination of retinal dystrophy and early onset obesity can be reminiscent of other disorders (e.g., Bardet–Biedl syndrome (MIM#PS209900) and Alstrom syndrome (MIM#203800)), the absence of other clinically relevant feature/sign was suggestive of a previously unreported ciliopathy [10]. In this paper, we report on a second disruptive variant (c.1387 + 1G &gt; A) affectingTUBin a subject with features that overlap with those previously described in the affected members of the original family.
-In the present and previously reported affected individuals, the ocular phenotype associated with defective TUB function is characterized by widespread retinal pigment epithelial (RPE) atrophy, deteriorating vision, the myopic and astigmatic refractive defect, the blonde fundus appearance, the ERG and OCT findings and progression of the disease (Figure 2). Notably, retinal detachment, without vitreous hemorrhage, was invariantly documented in the four individuals with biallelic inactivatingTUBvariants, suggesting that this feature likely represent a common finding in the disorder.
-Early onset obesity had previously been considered a major feature of the TUB-related condition [10], even though only two of three affected sibs were found obese (BMI &gt; 30), and the glycemic and lipid profiles in one of affected sibs were found within the normal range. The finding of obesity in the apparently healthy father (heterozygous carrier) suggests a possible co-occurring genetic event contributing to obesity in the family. In the present report, the clinical assessment of the affected individual documented increased weight (95.7 kg, +1.6 SD) and BMI (30.3, +1.6 SD), thus indicating overweight, in absence of other signs of obesity. Although evidence suggests that a defective TUB function may result in disturbances in insulin and leptin activity and obesity in mice [16,17,18,19], based on the collected findings, the relevance of TUB in human obesity requires further study. To assess whether TUB LoF could impact on hypothalamic pathways, food intake and adiposity, the metabolic profile of the affected individual was investigated. Accurate endocrinological examination did not reveal any abnormality, and the measurements of basal hormones by the anterior pituitary, glycaemia, insulin and leptin were within the normal range, thus ruling out insulin or leptin resistance. Consistently, instrumental investigations (X-ray and ultrasound analyses) documented no sign of glycogen accumulation in the internal organs. Consistently, the absence of significant changes in lipid storage was demonstrated by thin-layer chromatography (HPTLC) analysis in proband-derived fibroblast (Figure S1), allowing to confirm an apparently normal endocrine–metabolic profile in the affected individual. Of note, the Tubby protein has been involved in cochlear degeneration [20,21]. Based on this functional link, we evaluated the occurrence of hearing problems and cochlear degeneration, which were not observed.
-The homozygousTUBvariant was predicted to affect transcript processing, causing the skipping of exon 11 and intron retention, resulting in a frameshift with the premature termination of the TUB protein. mRNA analysis in proband-derived fibroblasts confirmed a disruptive impact of the splice site change documenting two aberrantly processed transcripts predicted to encode a 406-residue-long protein (p.Glu406Argfs*4) that probably is not able to proceed in protein synthesis, and a 481-residue-long protein (p.Pro463Hisfs*19) characterized by a divergent C-terminus characterized by accelerated degradation (Figure 3B). These findings confirm LoF as the pathomechanism underlying this disorder.
-Primary cilia are microtubule-based organelles that extend from the apical surface of the majority of mammalian cells. Cilia act as “cellular antennae”, receiving different inputs from the extracellular environment and transducing signals in response to stimuli [22]. A complex process required for proper cilia biogenesis function is the intraflagellar transport, which is required for assembling cilia and trafficking within primary cilia [23]. In this context, IFT-A has historically been believed to mediate retrograde intraflagellar transport inside the cilia and an IFT-A-binding domain at the TUB N-terminus has been demonstrated recently [24]. Moreover, co-localization between TUB and rootletin, the major structural component of the ciliary rootlet, has been observed in human retinal photoreceptors [10]. The use of a more informative in vitro model (e.g., induced pluripotent-stem-cell-derived retinal-pigment epithelium cells) and experimental strategies (e.g., siRNA-mediated TUB silencing) is required to appreciate more accurately the functional relevance of TUB in an appropriate cellular context.
-In summary, we confirm the link between TUB LoF and a new condition of human retinal ciliopathy and provide evidence of an altered cilium morphology/biogenesis in patient-derived fibroblasts. In fact, these cells displayed a reduced number of cilia when compared to the control cells, with a poorly defined and disorganized basal body structure, which are expected to prevent normal protein trafficking along the cilium. While these findings could explain the degeneration of photoreceptors characterizing this disorder, a relatively overall mild presentation has been associated with mutations in this gene. Multiple factors might contribute to this picture. First, the functional relevance of TUB in the context of ciliogenesis and cilium function might vary in different cell lineages. Second, functional compensation exerted by other related proteins might contribute to buffer the severity of the endophenotype. Third, specific cell lineages (e.g., rod and cone cells) might be particularly sensitive to TUB LoF. The collection of additional patients with biallelic variants in the gene will allow a more accurate characterization of the clinical spectrum associated with TUB LoF. Based on these considerations, TUB loss of function could be considered as responsible for a novel form of isolated retinal ciliopathy.</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
-    Inputs:
-    Alias gene symbol: rd5
-    HGNC record ID: HGNC:12406
-    Primary gene symbol: TUB
-    Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
-    Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
-    Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
-    If the text does not support that the alias is an alternate abbreviation, return:
-    "alternate_abbreviation": "NO"
-    "evidence": ""
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
-    Evidence must be one exact sentence copied verbatim from the text.
-    Do not infer relationships or paraphrase evidence.
-    Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
-    {
-    "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
-    "alternate_abbreviation": "YES or NO",
-    "evidence": ""
-    }
-PMID: 9390831
-Full Text: These authors contributed equally to this work.
-These authors jointly coordinated this work.
-Inherited retinal degeneration (IRD) represents a clinically variable and genetically heterogeneous group of disorders characterized by photoreceptor dysfunction. These diseases typically present with progressive severe vision loss and variable onset, ranging from birth to adulthood. Genomic sequencing has allowed to identify novel IRD-related genes, most of which encode proteins contributing to photoreceptor-cilia biogenesis and/or function. Despite these insights, knowledge gaps hamper a molecular diagnosis in one-third of IRD cases. By exome sequencing in a cohort of molecularly unsolved individuals with IRD, we identified a homozygous splice site variant affecting the transcript processing of TUB, encoding the first member of the Tubby family of bipartite transcription factors, in a sporadic case with retinal dystrophy. A truncating homozygous variant in this gene had previously been reported in a single family with three subjects sharing retinal dystrophy and obesity. The clinical assessment of the present patient documented a slightly increased body mass index and no changes in metabolic markers of obesity, but confirmed the occurrence of retinal detachment. In vitro studies using patient-derived fibroblasts showed the accelerated degradation of the encoded protein and aberrant cilium morphology and biogenesis. These findings definitely link impaired TUB function to retinal dystrophy and provide new data on the clinical characterization of this ultra-rare retinal ciliopathy.
-Inherited retinal degeneration (IRD) occurs in a clinically variable and genetically heterogeneous group of conditions characterized by photoreceptor degeneration and/or dysfunction [1]. The prevalence of monogenic IRD is estimated as 1 in 2000 individuals, affecting more than 2 million people worldwide [2]. This group of disorders typically present with severe vision loss that can be progressive, having an onset ranging from birth to late adulthood. Severe visual impairment affects mobility and independence, posing relevant psychological and economic burdens [3]. In the last ten years, genomic sequencing has allowed the identification of several genes implicated in IRD (for an updated list see the RetNet database,https://sph.uth.edu/retnet/). These genes encode proteins that have different roles in visual function, contributing to key processes in the cells of the pigmented cell layer and neurosensory retina [4,5]. Notably, retinal degeneration is frequently observed in ciliopathies, and a portion of IRD-related genes codifies for proteins involved in biogenesis and the maintenance of photoreceptor primary cilium [6,7,8,9]. Among these genes,TUB[MIM #601197], which encodes the first member of the Tubby family of bipartite transcription factors, has recently reported to be associated with a novel condition characterized by retinal dystrophy and obesity [MIM #616188] [10]. A truncating homozygousTUBvariant [c.1194_1195delAG, p.Arg398Serfs*9] was identified in a single family with three affected members, suggesting loss of function (LoF) as the pathomechanism underlying the disorder. The TUB family of transcription factors counts four members in vertebrates (TUB, TULP1, TULP2 and TULP3), sharing a similar domain organization including a highly conserved C-terminal domain mediating DNA binding and a divergent N-terminal region encompassing the nuclear localization signal and the transcriptional activation domain implicated in protein–protein binding [11]. A conserved region at the N-terminus enables some members of the Tubby family, including TUB, to bind to the ciliary intraflagellar transport A protein (IFTAP) [12]. Similar to the other members of the TULP family, TUB is also implicated in the control of the initiation of phagocytosis, facilitating the removal of apoptotic cells or cellular debris by retinal pigmented epithelium (RPE) cells and macrophages [13]. Since the original report, no other subject carrying biallelicTUBvariants has been described.
-In this study, we report on an additional subject with retinal dystrophy carrying a homozygous LoF variant inTUB. In vitro analyses provide evidence of the disruptive functional impact of the variant onTUBtranscript processing. We also show that the loss of TUB is associated with a defective cilium morphology and biogenesis in the primary patient’s fibroblasts. Our findings confirm the involvement of defective TUB function in retinal dystrophy and define this disorder as a novel ciliopathy.
-The proband is a 35-year-old male, the first child of healthy non-consanguineous parents of European descent (Figure 1). Family history was negative for retinal diseases or other congenital defects. The proband was born at term after an uneventful pregnancy. Length and weight at birth were reported as within the normal range. Apgar score was 8–10. No hearing impairment and/or learning difficulties were documented during the first year of age.
-At 5 years, the subject required consulting ophthalmologists for referring color blindness. A “blonde” aspect of the fundus oculi was observed and reduced full-field flash photopic and scotopic electroretinogram (ERG) responses were recorded. Visual acuity was not investigated at that time. Ophthalmological assessment at 26 years was suggestive of cone-rod dystrophy. Visual acuity was 0.8 Snellen in his right eye (RE) with myopic and astigmatic refractive error (RE: -4.50 dioptre sphere and -1 dioptre cylinder at 20°), and 0.2 Snellen in his left eye (LE) with myopic refractive error (LE: -2.00 dioptre sphere). Goldmann visual field was generally constricted, with reduced sensitivity in the superior central field in the RE and presented peripheral constriction and relative central scotoma in the LE. Light and dark adaptation sensitivity curves showed abnormal thresholds for both cones and rods. No number at the Ishihara charts were recognized. Intraocular pressure was within normal limits. The slit lamp examination biomicroscopy of the anterior segment was normal for cornea, iris and lens appearance. Fundus examination revealed bilateral optic disc pallor, depigmented aspect of the choroidal and retinal structures, diffuse retinal dystrophy with absence of intraretinal pigment dispersion or vitreous abnormalities and arteriolar attenuation. Full-field scotopic and photopic electroretinograms showed reduced a-wave and b-wave amplitude responses and delayed implicit times. Multifocal ERG ring analysis documented reduced response amplitude densities in all examined areas from the foveal center up to 20° of foveal eccentricity in both eyes (LE &gt; RE). After reduced visual field in his LE, a large area of retinoschisis in the infero-temporal sector was observed by fundoscopy, which later progressed, resulting in full retinal detachment of the LE. The subject underwent to pars plana vitrectomy with silicon oil (30% polydimethylsiloxane, PDMS) tamponade. He underwent cataract surgery in his LE and to subsequent vitreo-retinal surgeries for relapsing retinal detachments in same eye (PDMS/perfluorocarbon liquid (PFCL)/PDMS tamponades exchange and intra-operatory laser treatment; PDMS/heavy silicon oil tamponades exchange and intra-operatory laser). One year later, he developed vitreo-retinal proliferation and retinal fibrosis in the LE, and visual acuity was hand motion; therefore, the subject underwent retinotomy and heavy silicon oil/PDMS tamponades exchange.
-At last evaluation (35 years), the subject presented with a good clinical condition. No cognitive deficit nor behavioral issues were observed, and no craniofacial dysmorphism and truncal obesity were noticed. An accurate endocrinological examination was uninformative. Anthropometric assessment displayed a height of 177.5 cm (+0.1 SD), weight of 95.70 kg (+1.6 SD), and OFC 60 cm (+0.2 SD) and BMI of 30.30 Kg/m2(+1.6 SD). Tanner stage was Ph5Pg5, with a testicular volume 20 mL bilaterally. The subject’s visual acuity was 0.8 Snellen in his RE and light perception in his LE. Fundus oculi showed the unmodified condition of RE and diffuse chorio-retinal atrophy in the LE, as for visible vitreo-retinal surgical outcomes. Ultrawide field fundus photography showed macular atrophy in absence of peripheral pigment and confirmed a “blonde” aspect of the retina (Figure 2A). Fundus autofluorescence (FAF) revealed an hypoautoflorescent area in the macula due to RPE atrophy and hyper/hypoautofluorescence mottling in the posterior pole and immediately outside the vascular arcades (Figure 2B). The SD-OCT showed a disruption of the outer retina, including ELM, ellipsoid zone and RPE with outer retinal debris at the level of the RPE in the parafoveal region (Figure 2C). Full-field flash scotopic (Figure 2D) and photopic ERG confirmed reduced a-wave and b-wave amplitude responses and delayed implicit times in the RE. Similarly, multifocal ERG ring analysis, recordable only in the RE, showed the worsening of the response amplitude densities in all examined areas (0–20°) (Figure 2E), as compared to the previous examinations. Similarly, Goldmann visual field in his RE showed progressive constriction of the peripheral isopters and a ring scotoma enclosed between 10–20° of the visual field (Figure 2F); it was not executable, however, in his LE. Color blindness was also confirmed. Neck and abdominal ultrasound assessment did not reveal any abnormality. Measurements of basal hormones by the anterior pituitary, glycaemia and insulin were within the normal range. Basal plasma leptin level was in the low normal range, showing no leptin resistance. During his follow-up, clinical and ophthalmological assessments of other family members (parents and younger brother) were unremarkable.
-Trio-based WES allowed to identify a homozygous splice siteTUBvariant (chr11:8122545G &gt; A, GRCh37.p13; c.1387 + 1G &gt; A,NM_177972.3) as the only clinically and functionally relevant event putatively linked to the disorder (Supplemental Table S1). The variant had previously been annotated in public databases (dbSNP, rs1040410003) with low frequency (gnomAD v3.1, MAF = 0.00001972) at the heterozygous state. It was classified as likely pathogenic (PVS1/PM2/PP5) according to the American College of Medical Genetics and Genomics-Association for Molecular Pathology (ACMG-AMP) criteria (ClinVar: VCV000865971.1) [14]. Sanger sequencing confirmed the homozygosity for the variant in the proband and the heterozygous status in the healthy parents and unaffected sib (Figure 1).
-Since the variant was predicted to affect the exon 11 donor splice site, the total RNA from patient-derived skin primary fibroblasts was used to characterize the impact of the nucleotide change on transcript processing. The cDNA fragment encompassing the relevant exons was amplified, confirming the presence of two aberrantly spliced products (Figure 3A). The two aberrant PCR amplicons were isolated from agarose gel, purified and sequenced via Sanger. The former (500 bp) was derived from skipping of the penultimate exon (exon 11, ENST00000299506.3), resulting in a premature termination codon (i.e., p.Glu406Argfs*4), while the latter (1172 bp) was the result of retention of intron 10, resulting in a TUB protein having a divergent 19-residue-long C-terminus and lacking the last 44 amino acids (p.Pro463Hisfs*19) (Figure 3B).
-In the patient’s skin fibroblasts, the predicted TUBGlu406Argfs*4protein was undetectable by Western blot [WB] analysis, while the TUBPro463Hisfs*19protein was poorly detectable likely due to accelerated degradation (Figure 3C, left panel). Consistently, the endogenous TUBPro463Hisfs*19level was partially rescued by blocking the proteasomal degradation pathway using MG132 (Figure 3C, right panel).
-To investigate the cellular localization of the mutated protein, cytoplasm and nuclear cell fractions were obtained and analyzed by WB. The results demonstrate that both the wild-type (wt) and mutant TUB proteins were almost exclusively localized in the nucleus (Figure 3D). This finding was also confirmed by confocal microscopy analysis that evidenced the nuclear localization of the TUB mutant (Figure 4A).
-Based on the documented role of TUB in early ciliogenesis [15], we assessed the localization of TUB at the cilium, but we failed to observe any consistent co-localization, possibly due to the low diffused levels of the protein in the cytoplasm To investigate the impact of defective TUB function on the morphogenesis of the primary cilium, a confocal analysis on primary fibroblasts was performed using antibodies against ARL13B, which localizes to primary cilia, and pericentrin, a component of the centrosome, which stains the basal body. As shown inFigure 4B, while almost all the control cells showed a primary cilium, 40% of the fibroblasts carrying the homozygous splice site variant inTUBdid not show a primary cilium. Moreover, while no significant difference was observed in ciliary axoneme length between the starved control and mutant cells, a large percentage of the latter showed an abnormal cilium morphology and a poorly defined and disorganized basal body (Figure 4C).
-The loss of TUB function was recently reported to underlie a novel IRD condition based on the identification of homozygosity for a 2 bp deletion (c.1194_1195delAG) causing the premature termination of the protein (p.Arg398Serfs*9) shared by three affected members of a single consanguineous family [10]. While the combination of retinal dystrophy and early onset obesity can be reminiscent of other disorders (e.g., Bardet–Biedl syndrome (MIM#PS209900) and Alstrom syndrome (MIM#203800)), the absence of other clinically relevant feature/sign was suggestive of a previously unreported ciliopathy [10]. In this paper, we report on a second disruptive variant (c.1387 + 1G &gt; A) affectingTUBin a subject with features that overlap with those previously described in the affected members of the original family.
-In the present and previously reported affected individuals, the ocular phenotype associated with defective TUB function is characterized by widespread retinal pigment epithelial (RPE) atrophy, deteriorating vision, the myopic and astigmatic refractive defect, the blonde fundus appearance, the ERG and OCT findings and progression of the disease (Figure 2). Notably, retinal detachment, without vitreous hemorrhage, was invariantly documented in the four individuals with biallelic inactivatingTUBvariants, suggesting that this feature likely represent a common finding in the disorder.
-Early onset obesity had previously been considered a major feature of the TUB-related condition [10], even though only two of three affected sibs were found obese (BMI &gt; 30), and the glycemic and lipid profiles in one of affected sibs were found within the normal range. The finding of obesity in the apparently healthy father (heterozygous carrier) suggests a possible co-occurring genetic event contributing to obesity in the family. In the present report, the clinical assessment of the affected individual documented increased weight (95.7 kg, +1.6 SD) and BMI (30.3, +1.6 SD), thus indicating overweight, in absence of other signs of obesity. Although evidence suggests that a defective TUB function may result in disturbances in insulin and leptin activity and obesity in mice [16,17,18,19], based on the collected findings, the relevance of TUB in human obesity requires further study. To assess whether TUB LoF could impact on hypothalamic pathways, food intake and adiposity, the metabolic profile of the affected individual was investigated. Accurate endocrinological examination did not reveal any abnormality, and the measurements of basal hormones by the anterior pituitary, glycaemia, insulin and leptin were within the normal range, thus ruling out insulin or leptin resistance. Consistently, instrumental investigations (X-ray and ultrasound analyses) documented no sign of glycogen accumulation in the internal organs. Consistently, the absence of significant changes in lipid storage was demonstrated by thin-layer chromatography (HPTLC) analysis in proband-derived fibroblast (Figure S1), allowing to confirm an apparently normal endocrine–metabolic profile in the affected individual. Of note, the Tubby protein has been involved in cochlear degeneration [20,21]. Based on this functional link, we evaluated the occurrence of hearing problems and cochlear degeneration, which were not observed.
-The homozygousTUBvariant was predicted to affect transcript processing, causing the skipping of exon 11 and intron retention, resulting in a frameshift with the premature termination of the TUB protein. mRNA analysis in proband-derived fibroblasts confirmed a disruptive impact of the splice site change documenting two aberrantly processed transcripts predicted to encode a 406-residue-long protein (p.Glu406Argfs*4) that probably is not able to proceed in protein synthesis, and a 481-residue-long protein (p.Pro463Hisfs*19) characterized by a divergent C-terminus characterized by accelerated degradation (Figure 3B). These findings confirm LoF as the pathomechanism underlying this disorder.
-Primary cilia are microtubule-based organelles that extend from the apical surface of the majority of mammalian cells. Cilia act as “cellular antennae”, receiving different inputs from the extracellular environment and transducing signals in response to stimuli [22]. A complex process required for proper cilia biogenesis function is the intraflagellar transport, which is required for assembling cilia and trafficking within primary cilia [23]. In this context, IFT-A has historically been believed to mediate retrograde intraflagellar transport inside the cilia and an IFT-A-binding domain at the TUB N-terminus has been demonstrated recently [24]. Moreover, co-localization between TUB and rootletin, the major structural component of the ciliary rootlet, has been observed in human retinal photoreceptors [10]. The use of a more informative in vitro model (e.g., induced pluripotent-stem-cell-derived retinal-pigment epithelium cells) and experimental strategies (e.g., siRNA-mediated TUB silencing) is required to appreciate more accurately the functional relevance of TUB in an appropriate cellular context.
-In summary, we confirm the link between TUB LoF and a new condition of human retinal ciliopathy and provide evidence of an altered cilium morphology/biogenesis in patient-derived fibroblasts. In fact, these cells displayed a reduced number of cilia when compared to the control cells, with a poorly defined and disorganized basal body structure, which are expected to prevent normal protein trafficking along the cilium. While these findings could explain the degeneration of photoreceptors characterizing this disorder, a relatively overall mild presentation has been associated with mutations in this gene. Multiple factors might contribute to this picture. First, the functional relevance of TUB in the context of ciliogenesis and cilium function might vary in different cell lineages. Second, functional compensation exerted by other related proteins might contribute to buffer the severity of the endophenotype. Third, specific cell lineages (e.g., rod and cone cells) might be particularly sensitive to TUB LoF. The collection of additional patients with biallelic variants in the gene will allow a more accurate characterization of the clinical spectrum associated with TUB LoF. Based on these considerations, TUB loss of function could be considered as responsible for a novel form of isolated retinal ciliopathy.</t>
-        </is>
-      </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>{
-"pmid": "9390831",
-"alias_symbol": "rd5",
-"primary_gene_symbol": "TUB",
-"name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
-"evidence": ""
-}</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>HGNC:12406</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>ENSG00000166402</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>GENE ID:7275</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>TUB</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>rd5</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>9390831</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>mouse phenotype biomarker</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>abstract</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>Mice homozygous for a defect of the tub (rd5) gene exhibit cochlear and retinal degeneration combined with obesity, and resemble certain human autosomal recessive sensory deficit syndromes.</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>TUB bipartite transcription factor</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>In this paper, we confirm that biallelic inactivating variants in TUB cause a retinal disorder and functionally associate this condition with the occurrence of defects of the basal body structure and axoneme morphology of the primary cilium and overall defective ciliogenesis. Although the present findings suggest that TUB plays a role in the pathogenesis of retinal ciliopathies, dedicated functional studies are required to profile the mechanism of disease. This work confirms the clinical relevance of biallelic LoF variants ofTUB, which should be considered in clinical settings and the genetic diagnosis of IRD disorders.
-The present research followed the tenets of the Helsinki Declaration (1964 and further revisions) and the study was approved by the local ethics committee (Comitato Etico Centrale IRCCS Lazio, Sezione IFO/Fondazione Bietti, Rome, Italy). Upon recruitment in the study (FB RET-02-2019), executed from February to July 2019 at the IRCCS Fondazione Bietti, informed consent after full explanation was obtained from each subject included in the study.
-The proband and his family underwent comprehensive ophthalmological examination including visual acuity measured by the Early Treatment Diabetic Retinopathy Study (ETDRS) charts (Lighthouse, Low Vision Products, Long Island City, NY, USA) at the distance of 4 m and expressed as the logarithm of the minimum angle of resolution (logMAR); intraocular pressure (IOP) measurement; anterior segment observation by slit-lamp biomicroscopy and fundus examination by indirect ophthalmoscopic examination using + 90D non-contact lens (Volk Optical, Mentor, OH) after pupillary dilatation with tropicamide 1% drops. Goldmann visual field was assessed by kinetic Goldmann perimeter Haag-Streit 940. Chromatic test was evaluated by the monocular administration of Ishihara pseudoisochromatic plates (24 plates edition, Kanehara Trading Inc., Tokyo, Japan) in natural daylight. Electrophysiological assessment included dark-adapted and light-adapted full-field electroretinogram (Retimax Advanced Plus apparatus, CSO, Firenze, Italy) and multifocal electroretinogram (mfERG; VERIS Clinic TM version 4.9; Electro-Diagnostic Imaging, San Mateo, CA, USA) recordings according to the 2011 International Society for Clinical Electrophysiology of Vision (ISCEV) [25] by using the Dawson–Trick–Litzkow (DTL) contact electrodes and having the pupil dilated at 8 mm.
-Retinal imaging was executed by ultrawide field fundus photograph obtained with Optos California (Optos PLC, Dunfermline, Scotland, United Kingdom); FAF was also obtained during the same examination (488 nm excitation, barrier filter transmitted light from 500 to 680 nm, 55°) using Heidelberg Spectralis OCT (HRA + OCT, Heidelberg Engineering, Heidelberg, Germany). SD-OCT scan pattern was acquired with a minimum of a 20 × 20 degree rectangle centered on the fovea and 25-line B-scans spaced 235 μm apart and composed of 50 averaged frames by using the same instrument.
-Karyotype, CGH array and mutation scan by parallel sequencing considering a retinal cone–rod dystrophy panel of 70 genes were informative. Genomic DNA was collected after obtaining written informed consent. Whole-Exome sequencing (WES) and data analysis were performed as previously reported [26,27] (Supplementary Table S1). DNA of the affected subject and his parents was extracted from circulating leukocytes and sequenced using Illumina paired-end technology by means of SureSelect Human All Exon v.7 (Agilent, Santa Clara, CA, USA) kits. WES raw data were processed and analyzed using an in-house implemented pipeline as previously described [28,29], according to the GATK’s Best Practices [30]. The UCSC GRCh37/hg19 version of genome assembly was used as a reference for read alignment by means of BWA-MEM [31] tool and the subsequent variant calling with HaplotypeCaller (GATK v3.7) [28]. Variants’ functional annotation was made with the SnpEff v.5.0 [32] and dbNSFP v.4.2 [33] tools. Relevant in silico impact prediction tools, such as Combined Annotation Dependent Depletion (CADD) v.1.6 [34], Mendelian Clinically Applicable Pathogenicity (M-CAP) v.1.0 [35] and InterVar v.2.0.1 [36], were also used. By filtering against our population-matched database (~2500 WES) and public databases (dbSNP150 and gnomAD v.2.0.1), the analysis focused on high-quality rare variants that affect coding sequences and splice site regions. Sanger sequencing was performed for variant validation and segregation analysis (primers available upon request).
-Proband skin biopsy was obtained after informant consent was secured. Total RNA was extracted from the proband and healthy donor fibroblasts by using RNeasy Mini Kit (Qiagen, Hilden, Germany), according to the manufacturer’s recommendations. Total RNA concentration and quality were assessed by measuring the absorbance at 260 and 280 nm. Reverse transcription was carried out using a SuperScript RT reagent Kit (Invitrogen; ThermoFisher Scientific, Waltham, MA, USA). The obtained cDNA pools were amplified by PCR using specific primers located in exons 10 and 12 of theTUBgene, and PCR products were separated on a 2% agarose gel. The sequences of the primers are available upon request.
-Primary skin fibroblasts were cultured in DMEM supplemented with 10% heat-inactivated FBS, 2 mM glutamine, 100 units/mL of penicillin and 100 µg/mL of streptomycin, and maintained at 37 °C in a humidified atmosphere containing 5% CO2. After treatment, fibroblasts were lysed in RIPA buffer supplemented with phosphatase and protease inhibitors. Lysates were kept on ice (30 min) and then centrifuged at 16,000×g(20 min, 4 °C). Supernatants were collected and protein concentration was determined by Quick Start Bradford Dye Reagent (Bio-Rad Laboratories, Hercules, CA, USA), using bovine serum albumin (BSA) as a standard. Fibroblast homogenates were resolved by SDS PAGE and transferred to nitrocellulose membranes (Bio-Rad Laboratories). Blots were blocked for 1 h with 5% non-fat milk powder in phosphate-buffered saline (PBS) containing 0.1% Tween-20 and incubated overnight with specific antibodies. Anti-TUB primary polyclonal antibody (1:1000, Invitrogen; ThermoFisher Scientific) and goat anti-rabbit-HRP IgG secondary antibody (Invitrogen; ThermoFisher Scientific) were diluted in blocking solution. Immunoreactive proteins were detected by an ECL SuperSignal West Femto Maximum Sensitivity Chemiluminescent Substrate, according to the manufacturer’s instructions (Thermo Scientific, USA).
-Approximately 3 × 104/mL fibroblasts were seeded on glass coverslips and maintained in culture in complete medium for 24 h. Subconfluent fibroblasts were starved for 30 h and then fixed with 4% paraformaldehyde. Subsequently, cells were stained with rabbit anti-TUB (1:100 dilution), rabbit polyclonal anti-ARL13B (1:100, Abcam, Cambridge, UK) and mouse monoclonal anti-Pericentrin (1:100, Abcam) antibodies followed by goat anti-rabbit Alexa Fluor 488 and goat anti-mouse Alex Fluor 594, respectively (1:200 dilution; Molecular Probes, Eugene, OR, USA). After staining, coverslips were extensively rinsed and mounted onto microscope slides using Vectashield with DAPI mounting medium (Vector Laboratories, Newark, CA, USA). Analyses were performed in three independent experiments on a Zeiss LSM980 (Zeiss, Oberkochen, Germany) using a 63×/1.4 N.A. oil objective and excitation spectral laser lines at 405, 488 and 594 nm. Five hundred cells were counted for each condition in each experiment, and axoneme length was measured for each cell by using Zen Blue 3.2 software. Image acquisition and processing were performed as previously reported [37].
-Control and mutated fibroblasts cultured in 150 cm2dishes were harvested using trypsin after reaching confluence, rinsed with phosphate-buffered saline (PBS) and pelleted by centrifugation. Cell pellets were resuspended in 1 mL 0.9% NaCl and 6 mL of chloroform/methanol (2:1, v/v) were added. Mixtures were vortexed vigorously and centrifuged at 1500×gfor 15 min; the aqueous phase was discarded and organic phase was dried under N2gas. Lipid extracts from 1.5 × 106cells were applied on high-performance thin-layer chromatography (HPTLC) silica gel 60 plates (Merck, Darmstadt, Germany). Neutral lipids were resolved using a solvent system of hexane/diethyl ether/acetic acid (70:30:1, v/v/v) and were detected by staining with an aqueous solution containing 3% cupric acetate and 8% phosphoric acid and subsequent charring at 140 °C for 10 min. Lipids were identified by the co-migration of commercially available standards.
-URLs.*Online Mendelian Inheritance in Man [OMIM],http://www.ncbi.nlm.nih.gov/omim/;
-NCBI Gene,http://www.ncbi.nlm.nih.gov/gene/;
-Picard tools,http://picard.sourceforge.net/;
-wAnnovar,http://wannovar.usc.edu/;
-dbSNP137,http://www.ncbi.nlm.nih.gov/projects/SNP/snp_summary.cgi/;
-1000 Genomes Project,http://www.1000genomes.org/;
-HapMap Project,http://hapmap.ncbi.nlm.nih.gov/;
-SMART,http://smart.embl-heidelberg.de/;
-Protein Data Bank [PDB],http://www.rcsb.org/pdb/home/home.do.
-Research for this study was supported by the Ministry of Health funding 5x1000 Fondazione G.B. Bietti funds—2016 to M.P. and Fondazione Roma; Bando Ricerca Indipendente ISS 2021–2023 to V.C., Istituto Superiore di Sanità; Italian Ministry of Health (CCR-2017-23669081 to M.T.), and Italian Ministry of Research (FOE_2019 to M.T.). The authors acknowledge Maria Luisa Alessi and Federica Petrocchi for technical help in the electrophysiological and perimetric evaluations, Serenella Venanzi for administrative assistance.
-Publisher’s Note:MDPI stays neutral with regard to jurisdictional claims in published maps and institutional affiliations.
-The following supporting information can be downloaded at:https://www.mdpi.com/article/10.3390/ijms232314656/s1.
-Click here for additional data file.
-Conceptualization, L.Z. and V.C.; methodology, C.M., E.S., S.C., L.B. and M.T. (Massimo Tatti); validation, E.C., L.B., C.M. and V.C.; bioinformatics analysis, A.C. and A.B.; investigation, L.Z., M.C., M.P. and E.C.; resources, M.V.; data curation, L.B., M.P., E.S., M.T. (Massimo Tatti), M.N. and V.C.; writing—original draft preparation, L.Z., V.C. and M.N.; writing—review and editing, M.N., E.S., M.C., M.T. (Marco Tartaglia) and V.C.; supervision, M.V. and M.T. (Marco Tartaglia); project administration, M.V., V.C. and M.T. (Marco Tartaglia); funding acquisition, M.V. and M.P. All authors have read and agreed to the published version of the manuscript.
-The study was conducted according to the guidelines of the Declaration of Helsinki and was approved by the local Institutional Ethical Committee of the IRCCS_Fondazione G.B. Bietti [Ret_02/2019].
-Signed informed consent was obtained from the participating family.
-Data that support the findings of this study are available from the corresponding authors upon request.
-The authors declare no conflict of interest.
-Family tree showing the segregation of the identified splice site change.
-Ocular phenotype of the proband right eye. (A) Ultrawide field color fundus photograph. (B) The 55° fundus autofluorescence. (C) Spectral-domain optical coherence tomography line horizontal scan. (D) Full-field dark-adapted electroretinogram. (E) Three-dimensional multifocal electroretinogram plot. (F) Goldmann kinetic visual field.
-Characterization of the pathogenicTUBvariant. (A) Transcript processing in primary skin fibroblasts from a healthy donor and from the proband carrying the homozygous splice site variant. Total RNA was extracted, reverse-transcribed and analyzed by PCR to resolve transcript processing. Two aberrant cDNA products were identified in mutated cells (left) compared to the expected length of the amplified fragment obtained from the control fibroblasts (right). (B) Schematic representation of aberrant transcript processing caused by the identified homozygous splice site change inTUB. (C) Western blot analysis of the TUB protein in patient’s fibroblasts and the control cells. Twenty, forty and sixty micrograms of whole cell extract were analyzed basally (left) and following 4 h treatment with 100 μM Mg132 (right) and probed with anti-TUB antibody (* indicates a non-specific product). (D) Expression of wild-type and mutant TUB protein was analyzed in the cytoplasmic and nuclear fractions were obtained from wild-type and mutated fibroblasts. Sixty micrograms of each fraction were analyzed by Western blot and then probed with anti-TUB antibody. Anti-YY1 and anti-HSP90 antibodies were used as the internal controls to assess the clarity of the different fractions (* indicates a non-specific product). Blots are representative of three experiments performed.
-TUB subcellular localization and cilium defects in cells with TUB LoF. (A) Thirty-hour-starved and PFA-fixed fibroblasts from a healthy donor and from the proband were analyzed by confocal microscopy for the localization of TUB using antibodies against TUB. (B) The presence and morphology of primary cilia in starved fibroblasts from the proband and a healthy donor. Cells were starved for 30 h and fixed with PFA 4%. Primary cilia were analyzed using antibodies against ARL13B (cilium axonemal, green) and pericentrin (basal body, red) to investigate morphogenesis. Nuclei are DAPI stained (blue). Bars correspond to 20 and 2 μm (left panels). (C) Histograms represent the percent value of presence/absence of cilium, normal/aberrant cilium morphology and normal/aberrant basal body structure and the length (μm) of axoneme. Five hundred cells were counted for each condition and axoneme length was measured. Imagines and bar plots are representative of three experiments performed. * indicate statistical significance forp&lt; 0.01 by using Student’sTtest.</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>Mice homozygous for a defect of the tub (rd5) gene exhibit cochlear and retinal degeneration combined with obesity, and resemble certain human autosomal recessive sensory deficit syndromes. To establish the progressive nature of sensory cell loss associated with the tub gene, and to differentiate tub-related losses from those associated with the C57 background on which tub arose, we evaluated cochleas and retinas from tub/tub, tub/+, and +/+ mice, aged 2 weeks to 1 year by light and electron microscopy. Cochleas from mice of all three genotypes show progressive inner (IHC) and outer hair cell (OHC) loss. Relative to tub/+ and +/+ animals, however, tub homozygotes show accelerated OHC loss, affecting the extreme cochlear base (hook region) by 1 month, and the apex by 6 months. IHC loss in tub/tub animals is accelerated in the basal half of the cochlea, affecting the hook region by 6 months. Spiral ganglion cell losses were observed only in tub/tub mice, and only in the cochlear base. Retinas of tub/tub mice are abnormal at maturity, exhibiting shortened photoreceptor outer segments by 2 weeks, and progressive photoreceptor loss thereafter. Because the tub mutation causes degeneration of sensory cells in the ear and eye but has no other neurological effects, tubby mice hold unique promise for the study of human syndromic sensory loss.</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>PMID: 9390831
-Full Text: In this paper, we confirm that biallelic inactivating variants in TUB cause a retinal disorder and functionally associate this condition with the occurrence of defects of the basal body structure and axoneme morphology of the primary cilium and overall defective ciliogenesis. Although the present findings suggest that TUB plays a role in the pathogenesis of retinal ciliopathies, dedicated functional studies are required to profile the mechanism of disease. This work confirms the clinical relevance of biallelic LoF variants ofTUB, which should be considered in clinical settings and the genetic diagnosis of IRD disorders.
-The present research followed the tenets of the Helsinki Declaration (1964 and further revisions) and the study was approved by the local ethics committee (Comitato Etico Centrale IRCCS Lazio, Sezione IFO/Fondazione Bietti, Rome, Italy). Upon recruitment in the study (FB RET-02-2019), executed from February to July 2019 at the IRCCS Fondazione Bietti, informed consent after full explanation was obtained from each subject included in the study.
-The proband and his family underwent comprehensive ophthalmological examination including visual acuity measured by the Early Treatment Diabetic Retinopathy Study (ETDRS) charts (Lighthouse, Low Vision Products, Long Island City, NY, USA) at the distance of 4 m and expressed as the logarithm of the minimum angle of resolution (logMAR); intraocular pressure (IOP) measurement; anterior segment observation by slit-lamp biomicroscopy and fundus examination by indirect ophthalmoscopic examination using + 90D non-contact lens (Volk Optical, Mentor, OH) after pupillary dilatation with tropicamide 1% drops. Goldmann visual field was assessed by kinetic Goldmann perimeter Haag-Streit 940. Chromatic test was evaluated by the monocular administration of Ishihara pseudoisochromatic plates (24 plates edition, Kanehara Trading Inc., Tokyo, Japan) in natural daylight. Electrophysiological assessment included dark-adapted and light-adapted full-field electroretinogram (Retimax Advanced Plus apparatus, CSO, Firenze, Italy) and multifocal electroretinogram (mfERG; VERIS Clinic TM version 4.9; Electro-Diagnostic Imaging, San Mateo, CA, USA) recordings according to the 2011 International Society for Clinical Electrophysiology of Vision (ISCEV) [25] by using the Dawson–Trick–Litzkow (DTL) contact electrodes and having the pupil dilated at 8 mm.
-Retinal imaging was executed by ultrawide field fundus photograph obtained with Optos California (Optos PLC, Dunfermline, Scotland, United Kingdom); FAF was also obtained during the same examination (488 nm excitation, barrier filter transmitted light from 500 to 680 nm, 55°) using Heidelberg Spectralis OCT (HRA + OCT, Heidelberg Engineering, Heidelberg, Germany). SD-OCT scan pattern was acquired with a minimum of a 20 × 20 degree rectangle centered on the fovea and 25-line B-scans spaced 235 μm apart and composed of 50 averaged frames by using the same instrument.
-Karyotype, CGH array and mutation scan by parallel sequencing considering a retinal cone–rod dystrophy panel of 70 genes were informative. Genomic DNA was collected after obtaining written informed consent. Whole-Exome sequencing (WES) and data analysis were performed as previously reported [26,27] (Supplementary Table S1). DNA of the affected subject and his parents was extracted from circulating leukocytes and sequenced using Illumina paired-end technology by means of SureSelect Human All Exon v.7 (Agilent, Santa Clara, CA, USA) kits. WES raw data were processed and analyzed using an in-house implemented pipeline as previously described [28,29], according to the GATK’s Best Practices [30]. The UCSC GRCh37/hg19 version of genome assembly was used as a reference for read alignment by means of BWA-MEM [31] tool and the subsequent variant calling with HaplotypeCaller (GATK v3.7) [28]. Variants’ functional annotation was made with the SnpEff v.5.0 [32] and dbNSFP v.4.2 [33] tools. Relevant in silico impact prediction tools, such as Combined Annotation Dependent Depletion (CADD) v.1.6 [34], Mendelian Clinically Applicable Pathogenicity (M-CAP) v.1.0 [35] and InterVar v.2.0.1 [36], were also used. By filtering against our population-matched database (~2500 WES) and public databases (dbSNP150 and gnomAD v.2.0.1), the analysis focused on high-quality rare variants that affect coding sequences and splice site regions. Sanger sequencing was performed for variant validation and segregation analysis (primers available upon request).
-Proband skin biopsy was obtained after informant consent was secured. Total RNA was extracted from the proband and healthy donor fibroblasts by using RNeasy Mini Kit (Qiagen, Hilden, Germany), according to the manufacturer’s recommendations. Total RNA concentration and quality were assessed by measuring the absorbance at 260 and 280 nm. Reverse transcription was carried out using a SuperScript RT reagent Kit (Invitrogen; ThermoFisher Scientific, Waltham, MA, USA). The obtained cDNA pools were amplified by PCR using specific primers located in exons 10 and 12 of theTUBgene, and PCR products were separated on a 2% agarose gel. The sequences of the primers are available upon request.
-Primary skin fibroblasts were cultured in DMEM supplemented with 10% heat-inactivated FBS, 2 mM glutamine, 100 units/mL of penicillin and 100 µg/mL of streptomycin, and maintained at 37 °C in a humidified atmosphere containing 5% CO2. After treatment, fibroblasts were lysed in RIPA buffer supplemented with phosphatase and protease inhibitors. Lysates were kept on ice (30 min) and then centrifuged at 16,000×g(20 min, 4 °C). Supernatants were collected and protein concentration was determined by Quick Start Bradford Dye Reagent (Bio-Rad Laboratories, Hercules, CA, USA), using bovine serum albumin (BSA) as a standard. Fibroblast homogenates were resolved by SDS PAGE and transferred to nitrocellulose membranes (Bio-Rad Laboratories). Blots were blocked for 1 h with 5% non-fat milk powder in phosphate-buffered saline (PBS) containing 0.1% Tween-20 and incubated overnight with specific antibodies. Anti-TUB primary polyclonal antibody (1:1000, Invitrogen; ThermoFisher Scientific) and goat anti-rabbit-HRP IgG secondary antibody (Invitrogen; ThermoFisher Scientific) were diluted in blocking solution. Immunoreactive proteins were detected by an ECL SuperSignal West Femto Maximum Sensitivity Chemiluminescent Substrate, according to the manufacturer’s instructions (Thermo Scientific, USA).
-Approximately 3 × 104/mL fibroblasts were seeded on glass coverslips and maintained in culture in complete medium for 24 h. Subconfluent fibroblasts were starved for 30 h and then fixed with 4% paraformaldehyde. Subsequently, cells were stained with rabbit anti-TUB (1:100 dilution), rabbit polyclonal anti-ARL13B (1:100, Abcam, Cambridge, UK) and mouse monoclonal anti-Pericentrin (1:100, Abcam) antibodies followed by goat anti-rabbit Alexa Fluor 488 and goat anti-mouse Alex Fluor 594, respectively (1:200 dilution; Molecular Probes, Eugene, OR, USA). After staining, coverslips were extensively rinsed and mounted onto microscope slides using Vectashield with DAPI mounting medium (Vector Laboratories, Newark, CA, USA). Analyses were performed in three independent experiments on a Zeiss LSM980 (Zeiss, Oberkochen, Germany) using a 63×/1.4 N.A. oil objective and excitation spectral laser lines at 405, 488 and 594 nm. Five hundred cells were counted for each condition in each experiment, and axoneme length was measured for each cell by using Zen Blue 3.2 software. Image acquisition and processing were performed as previously reported [37].
-Control and mutated fibroblasts cultured in 150 cm2dishes were harvested using trypsin after reaching confluence, rinsed with phosphate-buffered saline (PBS) and pelleted by centrifugation. Cell pellets were resuspended in 1 mL 0.9% NaCl and 6 mL of chloroform/methanol (2:1, v/v) were added. Mixtures were vortexed vigorously and centrifuged at 1500×gfor 15 min; the aqueous phase was discarded and organic phase was dried under N2gas. Lipid extracts from 1.5 × 106cells were applied on high-performance thin-layer chromatography (HPTLC) silica gel 60 plates (Merck, Darmstadt, Germany). Neutral lipids were resolved using a solvent system of hexane/diethyl ether/acetic acid (70:30:1, v/v/v) and were detected by staining with an aqueous solution containing 3% cupric acetate and 8% phosphoric acid and subsequent charring at 140 °C for 10 min. Lipids were identified by the co-migration of commercially available standards.
-URLs.*Online Mendelian Inheritance in Man [OMIM],http://www.ncbi.nlm.nih.gov/omim/;
-NCBI Gene,http://www.ncbi.nlm.nih.gov/gene/;
-Picard tools,http://picard.sourceforge.net/;
-wAnnovar,http://wannovar.usc.edu/;
-dbSNP137,http://www.ncbi.nlm.nih.gov/projects/SNP/snp_summary.cgi/;
-1000 Genomes Project,http://www.1000genomes.org/;
-HapMap Project,http://hapmap.ncbi.nlm.nih.gov/;
-SMART,http://smart.embl-heidelberg.de/;
-Protein Data Bank [PDB],http://www.rcsb.org/pdb/home/home.do.
-Research for this study was supported by the Ministry of Health funding 5x1000 Fondazione G.B. Bietti funds—2016 to M.P. and Fondazione Roma; Bando Ricerca Indipendente ISS 2021–2023 to V.C., Istituto Superiore di Sanità; Italian Ministry of Health (CCR-2017-23669081 to M.T.), and Italian Ministry of Research (FOE_2019 to M.T.). The authors acknowledge Maria Luisa Alessi and Federica Petrocchi for technical help in the electrophysiological and perimetric evaluations, Serenella Venanzi for administrative assistance.
-Publisher’s Note:MDPI stays neutral with regard to jurisdictional claims in published maps and institutional affiliations.
-The following supporting information can be downloaded at:https://www.mdpi.com/article/10.3390/ijms232314656/s1.
-Click here for additional data file.
-Conceptualization, L.Z. and V.C.; methodology, C.M., E.S., S.C., L.B. and M.T. (Massimo Tatti); validation, E.C., L.B., C.M. and V.C.; bioinformatics analysis, A.C. and A.B.; investigation, L.Z., M.C., M.P. and E.C.; resources, M.V.; data curation, L.B., M.P., E.S., M.T. (Massimo Tatti), M.N. and V.C.; writing—original draft preparation, L.Z., V.C. and M.N.; writing—review and editing, M.N., E.S., M.C., M.T. (Marco Tartaglia) and V.C.; supervision, M.V. and M.T. (Marco Tartaglia); project administration, M.V., V.C. and M.T. (Marco Tartaglia); funding acquisition, M.V. and M.P. All authors have read and agreed to the published version of the manuscript.
-The study was conducted according to the guidelines of the Declaration of Helsinki and was approved by the local Institutional Ethical Committee of the IRCCS_Fondazione G.B. Bietti [Ret_02/2019].
-Signed informed consent was obtained from the participating family.
-Data that support the findings of this study are available from the corresponding authors upon request.
-The authors declare no conflict of interest.
-Family tree showing the segregation of the identified splice site change.
-Ocular phenotype of the proband right eye. (A) Ultrawide field color fundus photograph. (B) The 55° fundus autofluorescence. (C) Spectral-domain optical coherence tomography line horizontal scan. (D) Full-field dark-adapted electroretinogram. (E) Three-dimensional multifocal electroretinogram plot. (F) Goldmann kinetic visual field.
-Characterization of the pathogenicTUBvariant. (A) Transcript processing in primary skin fibroblasts from a healthy donor and from the proband carrying the homozygous splice site variant. Total RNA was extracted, reverse-transcribed and analyzed by PCR to resolve transcript processing. Two aberrant cDNA products were identified in mutated cells (left) compared to the expected length of the amplified fragment obtained from the control fibroblasts (right). (B) Schematic representation of aberrant transcript processing caused by the identified homozygous splice site change inTUB. (C) Western blot analysis of the TUB protein in patient’s fibroblasts and the control cells. Twenty, forty and sixty micrograms of whole cell extract were analyzed basally (left) and following 4 h treatment with 100 μM Mg132 (right) and probed with anti-TUB antibody (* indicates a non-specific product). (D) Expression of wild-type and mutant TUB protein was analyzed in the cytoplasmic and nuclear fractions were obtained from wild-type and mutated fibroblasts. Sixty micrograms of each fraction were analyzed by Western blot and then probed with anti-TUB antibody. Anti-YY1 and anti-HSP90 antibodies were used as the internal controls to assess the clarity of the different fractions (* indicates a non-specific product). Blots are representative of three experiments performed.
-TUB subcellular localization and cilium defects in cells with TUB LoF. (A) Thirty-hour-starved and PFA-fixed fibroblasts from a healthy donor and from the proband were analyzed by confocal microscopy for the localization of TUB using antibodies against TUB. (B) The presence and morphology of primary cilia in starved fibroblasts from the proband and a healthy donor. Cells were starved for 30 h and fixed with PFA 4%. Primary cilia were analyzed using antibodies against ARL13B (cilium axonemal, green) and pericentrin (basal body, red) to investigate morphogenesis. Nuclei are DAPI stained (blue). Bars correspond to 20 and 2 μm (left panels). (C) Histograms represent the percent value of presence/absence of cilium, normal/aberrant cilium morphology and normal/aberrant basal body structure and the length (μm) of axoneme. Five hundred cells were counted for each condition and axoneme length was measured. Imagines and bar plots are representative of three experiments performed. * indicate statistical significance forp&lt; 0.01 by using Student’sTtest.</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
-    Inputs:
-    Alias gene symbol: rd5
-    HGNC record ID: HGNC:12406
-    Primary gene symbol: TUB
-    Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
-    Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
-    Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
-    If the text does not support that the alias is an alternate abbreviation, return:
-    "alternate_abbreviation": "NO"
-    "evidence": ""
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
-    Evidence must be one exact sentence copied verbatim from the text.
-    Do not infer relationships or paraphrase evidence.
-    Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
-    {
-    "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
-    "alternate_abbreviation": "YES or NO",
-    "evidence": ""
-    }
-PMID: 9390831
-Full Text: In this paper, we confirm that biallelic inactivating variants in TUB cause a retinal disorder and functionally associate this condition with the occurrence of defects of the basal body structure and axoneme morphology of the primary cilium and overall defective ciliogenesis. Although the present findings suggest that TUB plays a role in the pathogenesis of retinal ciliopathies, dedicated functional studies are required to profile the mechanism of disease. This work confirms the clinical relevance of biallelic LoF variants ofTUB, which should be considered in clinical settings and the genetic diagnosis of IRD disorders.
-The present research followed the tenets of the Helsinki Declaration (1964 and further revisions) and the study was approved by the local ethics committee (Comitato Etico Centrale IRCCS Lazio, Sezione IFO/Fondazione Bietti, Rome, Italy). Upon recruitment in the study (FB RET-02-2019), executed from February to July 2019 at the IRCCS Fondazione Bietti, informed consent after full explanation was obtained from each subject included in the study.
-The proband and his family underwent comprehensive ophthalmological examination including visual acuity measured by the Early Treatment Diabetic Retinopathy Study (ETDRS) charts (Lighthouse, Low Vision Products, Long Island City, NY, USA) at the distance of 4 m and expressed as the logarithm of the minimum angle of resolution (logMAR); intraocular pressure (IOP) measurement; anterior segment observation by slit-lamp biomicroscopy and fundus examination by indirect ophthalmoscopic examination using + 90D non-contact lens (Volk Optical, Mentor, OH) after pupillary dilatation with tropicamide 1% drops. Goldmann visual field was assessed by kinetic Goldmann perimeter Haag-Streit 940. Chromatic test was evaluated by the monocular administration of Ishihara pseudoisochromatic plates (24 plates edition, Kanehara Trading Inc., Tokyo, Japan) in natural daylight. Electrophysiological assessment included dark-adapted and light-adapted full-field electroretinogram (Retimax Advanced Plus apparatus, CSO, Firenze, Italy) and multifocal electroretinogram (mfERG; VERIS Clinic TM version 4.9; Electro-Diagnostic Imaging, San Mateo, CA, USA) recordings according to the 2011 International Society for Clinical Electrophysiology of Vision (ISCEV) [25] by using the Dawson–Trick–Litzkow (DTL) contact electrodes and having the pupil dilated at 8 mm.
-Retinal imaging was executed by ultrawide field fundus photograph obtained with Optos California (Optos PLC, Dunfermline, Scotland, United Kingdom); FAF was also obtained during the same examination (488 nm excitation, barrier filter transmitted light from 500 to 680 nm, 55°) using Heidelberg Spectralis OCT (HRA + OCT, Heidelberg Engineering, Heidelberg, Germany). SD-OCT scan pattern was acquired with a minimum of a 20 × 20 degree rectangle centered on the fovea and 25-line B-scans spaced 235 μm apart and composed of 50 averaged frames by using the same instrument.
-Karyotype, CGH array and mutation scan by parallel sequencing considering a retinal cone–rod dystrophy panel of 70 genes were informative. Genomic DNA was collected after obtaining written informed consent. Whole-Exome sequencing (WES) and data analysis were performed as previously reported [26,27] (Supplementary Table S1). DNA of the affected subject and his parents was extracted from circulating leukocytes and sequenced using Illumina paired-end technology by means of SureSelect Human All Exon v.7 (Agilent, Santa Clara, CA, USA) kits. WES raw data were processed and analyzed using an in-house implemented pipeline as previously described [28,29], according to the GATK’s Best Practices [30]. The UCSC GRCh37/hg19 version of genome assembly was used as a reference for read alignment by means of BWA-MEM [31] tool and the subsequent variant calling with HaplotypeCaller (GATK v3.7) [28]. Variants’ functional annotation was made with the SnpEff v.5.0 [32] and dbNSFP v.4.2 [33] tools. Relevant in silico impact prediction tools, such as Combined Annotation Dependent Depletion (CADD) v.1.6 [34], Mendelian Clinically Applicable Pathogenicity (M-CAP) v.1.0 [35] and InterVar v.2.0.1 [36], were also used. By filtering against our population-matched database (~2500 WES) and public databases (dbSNP150 and gnomAD v.2.0.1), the analysis focused on high-quality rare variants that affect coding sequences and splice site regions. Sanger sequencing was performed for variant validation and segregation analysis (primers available upon request).
-Proband skin biopsy was obtained after informant consent was secured. Total RNA was extracted from the proband and healthy donor fibroblasts by using RNeasy Mini Kit (Qiagen, Hilden, Germany), according to the manufacturer’s recommendations. Total RNA concentration and quality were assessed by measuring the absorbance at 260 and 280 nm. Reverse transcription was carried out using a SuperScript RT reagent Kit (Invitrogen; ThermoFisher Scientific, Waltham, MA, USA). The obtained cDNA pools were amplified by PCR using specific primers located in exons 10 and 12 of theTUBgene, and PCR products were separated on a 2% agarose gel. The sequences of the primers are available upon request.
-Primary skin fibroblasts were cultured in DMEM supplemented with 10% heat-inactivated FBS, 2 mM glutamine, 100 units/mL of penicillin and 100 µg/mL of streptomycin, and maintained at 37 °C in a humidified atmosphere containing 5% CO2. After treatment, fibroblasts were lysed in RIPA buffer supplemented with phosphatase and protease inhibitors. Lysates were kept on ice (30 min) and then centrifuged at 16,000×g(20 min, 4 °C). Supernatants were collected and protein concentration was determined by Quick Start Bradford Dye Reagent (Bio-Rad Laboratories, Hercules, CA, USA), using bovine serum albumin (BSA) as a standard. Fibroblast homogenates were resolved by SDS PAGE and transferred to nitrocellulose membranes (Bio-Rad Laboratories). Blots were blocked for 1 h with 5% non-fat milk powder in phosphate-buffered saline (PBS) containing 0.1% Tween-20 and incubated overnight with specific antibodies. Anti-TUB primary polyclonal antibody (1:1000, Invitrogen; ThermoFisher Scientific) and goat anti-rabbit-HRP IgG secondary antibody (Invitrogen; ThermoFisher Scientific) were diluted in blocking solution. Immunoreactive proteins were detected by an ECL SuperSignal West Femto Maximum Sensitivity Chemiluminescent Substrate, according to the manufacturer’s instructions (Thermo Scientific, USA).
-Approximately 3 × 104/mL fibroblasts were seeded on glass coverslips and maintained in culture in complete medium for 24 h. Subconfluent fibroblasts were starved for 30 h and then fixed with 4% paraformaldehyde. Subsequently, cells were stained with rabbit anti-TUB (1:100 dilution), rabbit polyclonal anti-ARL13B (1:100, Abcam, Cambridge, UK) and mouse monoclonal anti-Pericentrin (1:100, Abcam) antibodies followed by goat anti-rabbit Alexa Fluor 488 and goat anti-mouse Alex Fluor 594, respectively (1:200 dilution; Molecular Probes, Eugene, OR, USA). After staining, coverslips were extensively rinsed and mounted onto microscope slides using Vectashield with DAPI mounting medium (Vector Laboratories, Newark, CA, USA). Analyses were performed in three independent experiments on a Zeiss LSM980 (Zeiss, Oberkochen, Germany) using a 63×/1.4 N.A. oil objective and excitation spectral laser lines at 405, 488 and 594 nm. Five hundred cells were counted for each condition in each experiment, and axoneme length was measured for each cell by using Zen Blue 3.2 software. Image acquisition and processing were performed as previously reported [37].
-Control and mutated fibroblasts cultured in 150 cm2dishes were harvested using trypsin after reaching confluence, rinsed with phosphate-buffered saline (PBS) and pelleted by centrifugation. Cell pellets were resuspended in 1 mL 0.9% NaCl and 6 mL of chloroform/methanol (2:1, v/v) were added. Mixtures were vortexed vigorously and centrifuged at 1500×gfor 15 min; the aqueous phase was discarded and organic phase was dried under N2gas. Lipid extracts from 1.5 × 106cells were applied on high-performance thin-layer chromatography (HPTLC) silica gel 60 plates (Merck, Darmstadt, Germany). Neutral lipids were resolved using a solvent system of hexane/diethyl ether/acetic acid (70:30:1, v/v/v) and were detected by staining with an aqueous solution containing 3% cupric acetate and 8% phosphoric acid and subsequent charring at 140 °C for 10 min. Lipids were identified by the co-migration of commercially available standards.
-URLs.*Online Mendelian Inheritance in Man [OMIM],http://www.ncbi.nlm.nih.gov/omim/;
-NCBI Gene,http://www.ncbi.nlm.nih.gov/gene/;
-Picard tools,http://picard.sourceforge.net/;
-wAnnovar,http://wannovar.usc.edu/;
-dbSNP137,http://www.ncbi.nlm.nih.gov/projects/SNP/snp_summary.cgi/;
-1000 Genomes Project,http://www.1000genomes.org/;
-HapMap Project,http://hapmap.ncbi.nlm.nih.gov/;
-SMART,http://smart.embl-heidelberg.de/;
-Protein Data Bank [PDB],http://www.rcsb.org/pdb/home/home.do.
-Research for this study was supported by the Ministry of Health funding 5x1000 Fondazione G.B. Bietti funds—2016 to M.P. and Fondazione Roma; Bando Ricerca Indipendente ISS 2021–2023 to V.C., Istituto Superiore di Sanità; Italian Ministry of Health (CCR-2017-23669081 to M.T.), and Italian Ministry of Research (FOE_2019 to M.T.). The authors acknowledge Maria Luisa Alessi and Federica Petrocchi for technical help in the electrophysiological and perimetric evaluations, Serenella Venanzi for administrative assistance.
-Publisher’s Note:MDPI stays neutral with regard to jurisdictional claims in published maps and institutional affiliations.
-The following supporting information can be downloaded at:https://www.mdpi.com/article/10.3390/ijms232314656/s1.
-Click here for additional data file.
-Conceptualization, L.Z. and V.C.; methodology, C.M., E.S., S.C., L.B. and M.T. (Massimo Tatti); validation, E.C., L.B., C.M. and V.C.; bioinformatics analysis, A.C. and A.B.; investigation, L.Z., M.C., M.P. and E.C.; resources, M.V.; data curation, L.B., M.P., E.S., M.T. (Massimo Tatti), M.N. and V.C.; writing—original draft preparation, L.Z., V.C. and M.N.; writing—review and editing, M.N., E.S., M.C., M.T. (Marco Tartaglia) and V.C.; supervision, M.V. and M.T. (Marco Tartaglia); project administration, M.V., V.C. and M.T. (Marco Tartaglia); funding acquisition, M.V. and M.P. All authors have read and agreed to the published version of the manuscript.
-The study was conducted according to the guidelines of the Declaration of Helsinki and was approved by the local Institutional Ethical Committee of the IRCCS_Fondazione G.B. Bietti [Ret_02/2019].
-Signed informed consent was obtained from the participating family.
-Data that support the findings of this study are available from the corresponding authors upon request.
-The authors declare no conflict of interest.
-Family tree showing the segregation of the identified splice site change.
-Ocular phenotype of the proband right eye. (A) Ultrawide field color fundus photograph. (B) The 55° fundus autofluorescence. (C) Spectral-domain optical coherence tomography line horizontal scan. (D) Full-field dark-adapted electroretinogram. (E) Three-dimensional multifocal electroretinogram plot. (F) Goldmann kinetic visual field.
-Characterization of the pathogenicTUBvariant. (A) Transcript processing in primary skin fibroblasts from a healthy donor and from the proband carrying the homozygous splice site variant. Total RNA was extracted, reverse-transcribed and analyzed by PCR to resolve transcript processing. Two aberrant cDNA products were identified in mutated cells (left) compared to the expected length of the amplified fragment obtained from the control fibroblasts (right). (B) Schematic representation of aberrant transcript processing caused by the identified homozygous splice site change inTUB. (C) Western blot analysis of the TUB protein in patient’s fibroblasts and the control cells. Twenty, forty and sixty micrograms of whole cell extract were analyzed basally (left) and following 4 h treatment with 100 μM Mg132 (right) and probed with anti-TUB antibody (* indicates a non-specific product). (D) Expression of wild-type and mutant TUB protein was analyzed in the cytoplasmic and nuclear fractions were obtained from wild-type and mutated fibroblasts. Sixty micrograms of each fraction were analyzed by Western blot and then probed with anti-TUB antibody. Anti-YY1 and anti-HSP90 antibodies were used as the internal controls to assess the clarity of the different fractions (* indicates a non-specific product). Blots are representative of three experiments performed.
-TUB subcellular localization and cilium defects in cells with TUB LoF. (A) Thirty-hour-starved and PFA-fixed fibroblasts from a healthy donor and from the proband were analyzed by confocal microscopy for the localization of TUB using antibodies against TUB. (B) The presence and morphology of primary cilia in starved fibroblasts from the proband and a healthy donor. Cells were starved for 30 h and fixed with PFA 4%. Primary cilia were analyzed using antibodies against ARL13B (cilium axonemal, green) and pericentrin (basal body, red) to investigate morphogenesis. Nuclei are DAPI stained (blue). Bars correspond to 20 and 2 μm (left panels). (C) Histograms represent the percent value of presence/absence of cilium, normal/aberrant cilium morphology and normal/aberrant basal body structure and the length (μm) of axoneme. Five hundred cells were counted for each condition and axoneme length was measured. Imagines and bar plots are representative of three experiments performed. * indicate statistical significance forp&lt; 0.01 by using Student’sTtest.</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>{
-"pmid": "9390831",
-"alias_symbol": "rd5",
-"primary_gene_symbol": "TUB",
-"name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "",
-"evidence": ""
-}</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>HGNC:12406</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>ENSG00000166402</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>GENE ID:7275</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>TUB</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>rd5</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>9477305</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>mouse phenotype biomarker</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>discussion</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities.</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>TUB bipartite transcription factor</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>Some genetic syndromes causing loss of hearing and vision, such as some forms of Usher's syndrome, also cause reduced sperm cell motility, bronchiectasis, and other pathologies involving cilia- and flagella-bearing cells. In some Usher's patients, ultrastructural defects of axonemes within photoreceptor ciliary bridges, nasal cilia, and sperm cell flagella have been found, indicating a primary defect of axonemal conformation. Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities. They provide a good phenotypic match to human genetic sensory syndromes, particularly human sensory/obesity syndromes, such as Alstrom's and Bardet/Biedl, although no human candidate genes have been identified. Because of their unique phenotype, tubby mice are an appropriate model in which to look for a primary axonemal defect. We studied the axonemal ultrastructure of photoreceptors and sperm cells and performed functional testing of sperm in tub/tub mice before and after the onset of obesity. Approximately 15% of photoreceptor axonemes appeared abnormal in tub/tub animals, compared to 0% in controls. Both tub homozygotes and controls exhibited approximately 10% abnormal sperm cell axonemes, and no differences in sperm cell motile function were found at any age. The modest occurrence of axonemal defects in photoreceptors of tub/tub animals is likely to be a secondary effect of retinal degeneration. We conclude that the tubby phenotype is not associated with a generalized defect of cilia- and flagella-bearing cells and that the tub mutation does not primarily affect axonemal structure.</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>PMID: 9477305
-Abstract: Some genetic syndromes causing loss of hearing and vision, such as some forms of Usher's syndrome, also cause reduced sperm cell motility, bronchiectasis, and other pathologies involving cilia- and flagella-bearing cells. In some Usher's patients, ultrastructural defects of axonemes within photoreceptor ciliary bridges, nasal cilia, and sperm cell flagella have been found, indicating a primary defect of axonemal conformation. Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities. They provide a good phenotypic match to human genetic sensory syndromes, particularly human sensory/obesity syndromes, such as Alstrom's and Bardet/Biedl, although no human candidate genes have been identified. Because of their unique phenotype, tubby mice are an appropriate model in which to look for a primary axonemal defect. We studied the axonemal ultrastructure of photoreceptors and sperm cells and performed functional testing of sperm in tub/tub mice before and after the onset of obesity. Approximately 15% of photoreceptor axonemes appeared abnormal in tub/tub animals, compared to 0% in controls. Both tub homozygotes and controls exhibited approximately 10% abnormal sperm cell axonemes, and no differences in sperm cell motile function were found at any age. The modest occurrence of axonemal defects in photoreceptors of tub/tub animals is likely to be a secondary effect of retinal degeneration. We conclude that the tubby phenotype is not associated with a generalized defect of cilia- and flagella-bearing cells and that the tub mutation does not primarily affect axonemal structure.</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
-    Inputs:
-    Alias gene symbol: rd5
-    HGNC record ID: HGNC:12406
-    Primary gene symbol: TUB
-    Official HGNC gene name: TUB bipartite transcription factor
-    Biomedical text context (may include PMID)
-    Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
-    Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
-    If the text does not support that the alias is an alternate abbreviation, return:
-    "alternate_abbreviation": "NO"
-    "evidence": ""
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
-    Evidence must be one exact sentence copied verbatim from the text.
-    Do not infer relationships or paraphrase evidence.
-    Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
-    {
-    "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
-    "alternate_abbreviation": "YES or NO",
-    "evidence": ""
-    }
-PMID: 9477305
-Abstract: Some genetic syndromes causing loss of hearing and vision, such as some forms of Usher's syndrome, also cause reduced sperm cell motility, bronchiectasis, and other pathologies involving cilia- and flagella-bearing cells. In some Usher's patients, ultrastructural defects of axonemes within photoreceptor ciliary bridges, nasal cilia, and sperm cell flagella have been found, indicating a primary defect of axonemal conformation. Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities. They provide a good phenotypic match to human genetic sensory syndromes, particularly human sensory/obesity syndromes, such as Alstrom's and Bardet/Biedl, although no human candidate genes have been identified. Because of their unique phenotype, tubby mice are an appropriate model in which to look for a primary axonemal defect. We studied the axonemal ultrastructure of photoreceptors and sperm cells and performed functional testing of sperm in tub/tub mice before and after the onset of obesity. Approximately 15% of photoreceptor axonemes appeared abnormal in tub/tub animals, compared to 0% in controls. Both tub homozygotes and controls exhibited approximately 10% abnormal sperm cell axonemes, and no differences in sperm cell motile function were found at any age. The modest occurrence of axonemal defects in photoreceptors of tub/tub animals is likely to be a secondary effect of retinal degeneration. We conclude that the tubby phenotype is not associated with a generalized defect of cilia- and flagella-bearing cells and that the tub mutation does not primarily affect axonemal structure.</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>{
-"pmid": "9477305",
-"alias_symbol": "rd5",
-"primary_gene_symbol": "TUB",
-"name": "TUB bipartite transcription factor",
-"alias_symbol_represents_primary_gene": "YES",
-"alternate_abbreviation": "NO",
-"evidence": "Mice homozygous for the tub (rd5) mutation exhibit progressive retinal degeneration, sensorineural hearing loss, reduced fertility, and obesity, and presently represent the only animal model with neuroepithelial degeneration of both cochlea and retina without other neurological abnormalities."
-}</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>HGNC:13919</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>ENSG00000234651, ENSG00000096155, ENSG00000233348, ENSG00000204463, ENSG00000228760, ENSG00000229524, ENSG00000227761</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>GENE ID:7917</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>BAG6</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>SCYTHE</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>37879364</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>literature defined (uniprot alternative protein name)</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>discussion</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>PBF also interacts with 14_3_3_ and Scythe/BAT3 proteins, two important cellular proteins involved in the regulation of cell apoptosis.</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr">
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr">
         <is>
           <t>BAG cochaperone 6</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="R18" t="inlineStr">
         <is>
           <t>We previously identified papillomavirus binding factor (PBF) as an osteosarcoma antigen recognized by an autologous cytotoxic T lymphocyte clone. Vaccination with PBF‐derived peptide presented by HLA‐A24 (PBF peptide) elicited strong immune responses. In the present study, we generated T cell receptor‐engineered T cells (TCR‐T cells) directed against the PBF peptide (PBF TCR‐T cells). PBF TCR was successfully transduced into T cells and detected using HLA‐A*24:02/PBF peptide tetramer. PBF TCR‐T cells generated from a healthy donor were highly expanded and recognized T2‐A24 cells pulsed with PBF peptide, HLA‐A24+293T cells transfected with PBF cDNA, and sarcoma cell lines. To establish an adoptive cell therapy model, we modified the PBF TCR by replacing both α and β constant regions with those of mice (hybrid PBF TCR). Hybrid PBF TCR‐T cells also showed reactivity against T2‐A24 cells pulsed with PBF peptide and to HLA‐A24+293T cells transfected with various lengths of PBF cDNA including the PBF peptide sequence. Subsequently, we generated target cell lines highly expressing PBF (MFH03‐PBF [short] epitope [+]) containing PBF peptide with in vivo tumorigenicity. Hybrid PBF TCR‐T cells exhibited antitumor effects compared with mock T cells in NSG mice xenografted with MFH03‐PBF (short) epitope (+) cells. CD45+T cells significantly infiltrated xenografted tumors only in the hybrid PBF TCR T cell group and most of these cells were CD8‐positive. CD8+T cells also showed Ki‐67 expression and surrounded the CD8‐negative tumor cells expressing Ki‐67. These findings suggest that PBF TCR‐T cell therapy might be a candidate immunotherapy for sarcoma highly expressing PBF.
 We developed TCR‐T cells targeting sarcoma‐associated antigen PBF (PBF TCR‐T cells). PBF TCR‐T cells showed anti‐tumor effects against sarcoma cell lines in vitro and in vivo. PBF TCR‐T cell therapy might be a candidate immunotherapy for sarcoma highly expressing PBF.
@@ -4486,12 +4720,12 @@
 To assess the in vivo antitumor effects of hybrid PBF TCR‐T cells, we decided to generate target tumor cells with strong tumorigenesis in NSG mice and high expression of PBF. Therefore, we selected MFH03 cells, which exhibit strong tumorigenesis in mice, and stably transfected them with PBF cDNA containing the PBF epitope peptide; the cells were named MFH03‐PBF (short) epitope (+) cells (Figure4A). In parallel with the generation of hybrid PBF TCR‐T cells, mock T cells that were transduced with retroviral empty vector were also generated (Figure4B). Hybrid PBF TCR‐T cells showed cytotoxicity against MFH03‐PBF (short) epitope (+) cells (FigureS2). Adoptive cell transfer experiments were conducted with these effector cells and target cells. Hybrid PBF TCR‐T cells and mock T cells were administered on day 15 after the target cell inoculation. The results showed that tumor growth was suppressed in the hybrid PBF TCR‐T group compared with the mock T group, with significant differences in tumor volume observed on day 39 (p&lt; 0.0079, Figure4C,D, FigureS3).</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>We previously identified papillomavirus binding factor (PBF) as an osteosarcoma antigen recognized by an autologous cytotoxic T lymphocyte clone. Vaccination with PBF-derived peptide presented by HLA-A24 (PBF peptide) elicited strong immune responses. In the present study, we generated T cell receptor-engineered T cells (TCR-T cells) directed against the PBF peptide (PBF TCR-T cells). PBF TCR was successfully transduced into T cells and detected using HLA-A*24:02/PBF peptide tetramer. PBF TCR-T cells generated from a healthy donor were highly expanded and recognized T2-A24 cells pulsed with PBF peptide, HLA-A24&lt;sup&gt;+&lt;/sup&gt; 293T cells transfected with PBF cDNA, and sarcoma cell lines. To establish an adoptive cell therapy model, we modified the PBF TCR by replacing both α and β constant regions with those of mice (hybrid PBF TCR). Hybrid PBF TCR-T cells also showed reactivity against T2-A24 cells pulsed with PBF peptide and to HLA-A24&lt;sup&gt;+&lt;/sup&gt; 293T cells transfected with various lengths of PBF cDNA including the PBF peptide sequence. Subsequently, we generated target cell lines highly expressing PBF (MFH03-PBF [short] epitope [+]) containing PBF peptide with in vivo tumorigenicity. Hybrid PBF TCR-T cells exhibited antitumor effects compared with mock T cells in NSG mice xenografted with MFH03-PBF (short) epitope (+) cells. CD45&lt;sup&gt;+&lt;/sup&gt; T cells significantly infiltrated xenografted tumors only in the hybrid PBF TCR T cell group and most of these cells were CD8-positive. CD8&lt;sup&gt;+&lt;/sup&gt; T cells also showed Ki-67 expression and surrounded the CD8-negative tumor cells expressing Ki-67. These findings suggest that PBF TCR-T cell therapy might be a candidate immunotherapy for sarcoma highly expressing PBF.</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>PMID: 37879364
 Full Text: We previously identified papillomavirus binding factor (PBF) as an osteosarcoma antigen recognized by an autologous cytotoxic T lymphocyte clone. Vaccination with PBF‐derived peptide presented by HLA‐A24 (PBF peptide) elicited strong immune responses. In the present study, we generated T cell receptor‐engineered T cells (TCR‐T cells) directed against the PBF peptide (PBF TCR‐T cells). PBF TCR was successfully transduced into T cells and detected using HLA‐A*24:02/PBF peptide tetramer. PBF TCR‐T cells generated from a healthy donor were highly expanded and recognized T2‐A24 cells pulsed with PBF peptide, HLA‐A24+293T cells transfected with PBF cDNA, and sarcoma cell lines. To establish an adoptive cell therapy model, we modified the PBF TCR by replacing both α and β constant regions with those of mice (hybrid PBF TCR). Hybrid PBF TCR‐T cells also showed reactivity against T2‐A24 cells pulsed with PBF peptide and to HLA‐A24+293T cells transfected with various lengths of PBF cDNA including the PBF peptide sequence. Subsequently, we generated target cell lines highly expressing PBF (MFH03‐PBF [short] epitope [+]) containing PBF peptide with in vivo tumorigenicity. Hybrid PBF TCR‐T cells exhibited antitumor effects compared with mock T cells in NSG mice xenografted with MFH03‐PBF (short) epitope (+) cells. CD45+T cells significantly infiltrated xenografted tumors only in the hybrid PBF TCR T cell group and most of these cells were CD8‐positive. CD8+T cells also showed Ki‐67 expression and surrounded the CD8‐negative tumor cells expressing Ki‐67. These findings suggest that PBF TCR‐T cell therapy might be a candidate immunotherapy for sarcoma highly expressing PBF.
@@ -4526,7 +4760,7 @@
 To assess the in vivo antitumor effects of hybrid PBF TCR‐T cells, we decided to generate target tumor cells with strong tumorigenesis in NSG mice and high expression of PBF. Therefore, we selected MFH03 cells, which exhibit strong tumorigenesis in mice, and stably transfected them with PBF cDNA containing the PBF epitope peptide; the cells were named MFH03‐PBF (short) epitope (+) cells (Figure4A). In parallel with the generation of hybrid PBF TCR‐T cells, mock T cells that were transduced with retroviral empty vector were also generated (Figure4B). Hybrid PBF TCR‐T cells showed cytotoxicity against MFH03‐PBF (short) epitope (+) cells (FigureS2). Adoptive cell transfer experiments were conducted with these effector cells and target cells. Hybrid PBF TCR‐T cells and mock T cells were administered on day 15 after the target cell inoculation. The results showed that tumor growth was suppressed in the hybrid PBF TCR‐T group compared with the mock T group, with significant differences in tumor volume observed on day 39 (p&lt; 0.0079, Figure4C,D, FigureS3).</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -4534,35 +4768,43 @@
     HGNC record ID: HGNC:13919
     Primary gene symbol: BAG6
     Official HGNC gene name: BAG cochaperone 6
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -4599,99 +4841,98 @@
 To assess the in vivo antitumor effects of hybrid PBF TCR‐T cells, we decided to generate target tumor cells with strong tumorigenesis in NSG mice and high expression of PBF. Therefore, we selected MFH03 cells, which exhibit strong tumorigenesis in mice, and stably transfected them with PBF cDNA containing the PBF epitope peptide; the cells were named MFH03‐PBF (short) epitope (+) cells (Figure4A). In parallel with the generation of hybrid PBF TCR‐T cells, mock T cells that were transduced with retroviral empty vector were also generated (Figure4B). Hybrid PBF TCR‐T cells showed cytotoxicity against MFH03‐PBF (short) epitope (+) cells (FigureS2). Adoptive cell transfer experiments were conducted with these effector cells and target cells. Hybrid PBF TCR‐T cells and mock T cells were administered on day 15 after the target cell inoculation. The results showed that tumor growth was suppressed in the hybrid PBF TCR‐T group compared with the mock T group, with significant differences in tumor volume observed on day 39 (p&lt; 0.0079, Figure4C,D, FigureS3).</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>{
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>Based on the provided text, here is my analysis:
+{
 "pmid": "37879364",
-"alias_symbol": "SCYTHE",
+"alias_symbol": "PBF",
 "primary_gene_symbol": "BAG6",
 "name": "BAG cochaperone 6",
-"alias_symbol_represents_primary_gene": "NO",
 "alternate_abbreviation": "NO",
 "evidence": ""
-}</t>
+}
+The text does not provide evidence that PBF (papillomavirus binding factor) is an alternate abbreviation for BAG6 (BAG cochaperone 6). The text discusses PBF as a separate gene/protein that was identified as an osteosarcoma antigen. It does not link PBF to BAG6 or expand PBF to the official gene name "BAG cochaperone 6". Therefore, there is no evidence to classify PBF as an alternate abbreviation for BAG6 in this context.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>HGNC:13919</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>ENSG00000234651, ENSG00000096155, ENSG00000233348, ENSG00000204463, ENSG00000228760, ENSG00000229524, ENSG00000227761</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>GENE ID:7917</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>BAG6</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>SCYTHE</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>37879364</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>37879364</v>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>literature defined (uniprot alternative protein name)</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>discussion</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>PBF also interacts with 14_3_3_ and Scythe/BAT3 proteins, two important cellular proteins involved in the regulation of cell apoptosis.</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr">
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr">
         <is>
           <t>BAG cochaperone 6</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="R19" t="inlineStr">
         <is>
           <t>Papillomavirus binding factor (PBF) T cell receptor‐engineered T cells (TCR‐T cells) exert antitumor effects in a xenografted mouse model. (A) The PBF (short) epitope (+) gene was transduced into MFH03 cells for an in vivo assay. (B) Tetramer assay of PBF TCR‐T cells before adoptive cell transfer. (C) Tumor volume over time. The day on which tumor cells were transplanted into the mouse was set as day 0, and PBF TCR‐T cells or mock T cells were administered on day 14. (D) Tumor volume and weight at the endpoint. (E–H) Immunohistochemical findings of tumors excised from mice that were transferred with PBF TCR‐T cells. They were stained with monoclonal antibodies against CD45 (E and F), CD4, and CD8 (G) and both CD8 and Ki‐67 monoclonal antibodies (H). Black arrows indicate double‐stained cells (H). (I–N) Tetramer positivity rate (I and J) and the expression levels of PD‐1 (K and L) and Lag‐3 (M and N) in the removed mouse splenocytes were analyzed by flow cytometry (n= 5).
 Next, the infiltration of the transferred T cells into excised tumor tissues was analyzed by immunohistochemistry. The infiltration of CD45‐positive lymphocytes into the tumor was significantly higher in the TCR‐T group than in the mock group (p= 0.0021, Figure4E,F). The infiltrating lymphocytes were almost entirely CD8‐positive, in contrast to a few CD4‐positive lymphocytes (Figure4G). Moreover, hybrid PBF TCR‐T cells showed enhanced Ki‐67 expression, which suggested that these cells possessed a proliferative tendency in specific response to the antigen (Figure4H). In mouse spleens, PBF tetramer‐positive cells were detected in the hybrid PBF TCR‐T group (Figure4I,J). However, the expression levels of PD‐1 (Figure4K,L) and Lag‐3 (Figure4M,N) in the splenocytes were no different between hybrid PBF TCR‐T and mock T cells. The exhaustion status was not specific for the PBF TCR and might be a natural course of transferred T cells in the in vivo mouse model.
@@ -4711,12 +4952,12 @@
 The authors thank Ms. Asuka Akamatsu and Ms. Serina Tokita for technical assistance.</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="S19" t="inlineStr">
         <is>
           <t>We previously identified papillomavirus binding factor (PBF) as an osteosarcoma antigen recognized by an autologous cytotoxic T lymphocyte clone. Vaccination with PBF-derived peptide presented by HLA-A24 (PBF peptide) elicited strong immune responses. In the present study, we generated T cell receptor-engineered T cells (TCR-T cells) directed against the PBF peptide (PBF TCR-T cells). PBF TCR was successfully transduced into T cells and detected using HLA-A*24:02/PBF peptide tetramer. PBF TCR-T cells generated from a healthy donor were highly expanded and recognized T2-A24 cells pulsed with PBF peptide, HLA-A24&lt;sup&gt;+&lt;/sup&gt; 293T cells transfected with PBF cDNA, and sarcoma cell lines. To establish an adoptive cell therapy model, we modified the PBF TCR by replacing both α and β constant regions with those of mice (hybrid PBF TCR). Hybrid PBF TCR-T cells also showed reactivity against T2-A24 cells pulsed with PBF peptide and to HLA-A24&lt;sup&gt;+&lt;/sup&gt; 293T cells transfected with various lengths of PBF cDNA including the PBF peptide sequence. Subsequently, we generated target cell lines highly expressing PBF (MFH03-PBF [short] epitope [+]) containing PBF peptide with in vivo tumorigenicity. Hybrid PBF TCR-T cells exhibited antitumor effects compared with mock T cells in NSG mice xenografted with MFH03-PBF (short) epitope (+) cells. CD45&lt;sup&gt;+&lt;/sup&gt; T cells significantly infiltrated xenografted tumors only in the hybrid PBF TCR T cell group and most of these cells were CD8-positive. CD8&lt;sup&gt;+&lt;/sup&gt; T cells also showed Ki-67 expression and surrounded the CD8-negative tumor cells expressing Ki-67. These findings suggest that PBF TCR-T cell therapy might be a candidate immunotherapy for sarcoma highly expressing PBF.</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr">
+      <c r="T19" t="inlineStr">
         <is>
           <t>PMID: 37879364
 Full Text: Papillomavirus binding factor (PBF) T cell receptor‐engineered T cells (TCR‐T cells) exert antitumor effects in a xenografted mouse model. (A) The PBF (short) epitope (+) gene was transduced into MFH03 cells for an in vivo assay. (B) Tetramer assay of PBF TCR‐T cells before adoptive cell transfer. (C) Tumor volume over time. The day on which tumor cells were transplanted into the mouse was set as day 0, and PBF TCR‐T cells or mock T cells were administered on day 14. (D) Tumor volume and weight at the endpoint. (E–H) Immunohistochemical findings of tumors excised from mice that were transferred with PBF TCR‐T cells. They were stained with monoclonal antibodies against CD45 (E and F), CD4, and CD8 (G) and both CD8 and Ki‐67 monoclonal antibodies (H). Black arrows indicate double‐stained cells (H). (I–N) Tetramer positivity rate (I and J) and the expression levels of PD‐1 (K and L) and Lag‐3 (M and N) in the removed mouse splenocytes were analyzed by flow cytometry (n= 5).
@@ -4737,7 +4978,7 @@
 The authors thank Ms. Asuka Akamatsu and Ms. Serina Tokita for technical assistance.</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="U19" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -4745,35 +4986,43 @@
     HGNC record ID: HGNC:13919
     Primary gene symbol: BAG6
     Official HGNC gene name: BAG cochaperone 6
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -4796,99 +5045,96 @@
 The authors thank Ms. Asuka Akamatsu and Ms. Serina Tokita for technical assistance.</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr">
+      <c r="V19" t="inlineStr">
         <is>
           <t>{
 "pmid": "37879364",
 "alias_symbol": "SCYTHE",
 "primary_gene_symbol": "BAG6",
 "name": "BAG cochaperone 6",
-"alias_symbol_represents_primary_gene": "YES",
-"alternate_abbreviation": "NO",
-"evidence": "PBF also interacts with 14‐3‐3β and Scythe/BAT3 proteins, two important cellular proteins involved in the regulation of cell apoptosis.16,17"
+"alternate_abbreviation": "YES",
+"evidence": "PBF also interacts with 14‐3‐3β and Scythe/BAT3 proteins, two important cellular proteins involved in the regulation of cell apoptosis."
 }</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>HGNC:13919</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>ENSG00000234651, ENSG00000096155, ENSG00000233348, ENSG00000204463, ENSG00000228760, ENSG00000229524, ENSG00000227761</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>GENE ID:7917</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>BAG6</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>SCYTHE</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>38498560</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>38498560</v>
+      </c>
+      <c r="I20" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>alias</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>alias</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>intro</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>BAG6 (BCL2-associated athanogene 6, also known as BAT3 or Scythe) is a member of the BAG family due to a sequence homologous to the BAG domain at its C terminus and the collaboration with Heat Shock Protein 70 (Hsp70) family molecular chaperones</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr">
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr">
         <is>
           <t>BAG cochaperone 6</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="R20" t="inlineStr">
         <is>
           <t>The authors have declared that no competing interests exist.
 The interaction between influenza A virus (IAV) and host proteins is an important process that greatly influences viral replication and pathogenicity. PB2 protein is a subunit of viral ribonucleoprotein (vRNP) complex playing distinct roles in viral transcription and replication. BAG6 (BCL2-associated athanogene 6) as a multifunctional host protein participates in physiological and pathological processes. Here, we identify BAG6 as a new restriction factor for IAV replication through targeting PB2. For both avian and human influenza viruses, overexpression of BAG6 reduced viral protein expression and virus titers, whereas deletion of BAG6 significantly enhanced virus replication. Moreover, BAG6-knockdown mice developed more severe clinical symptoms and higher viral loads upon IAV infection. Mechanistically, BAG6 restricted IAV transcription and replication by inhibiting the activity of viral RNA-dependent RNA polymerase (RdRp). The co-immunoprecipitation assays showed BAG6 specifically interacted with the N-terminus of PB2 and competed with PB1 for RdRp complex assembly. The ubiquitination assay indicated that BAG6 promoted PB2 ubiquitination at K189 residue and targeted PB2 for K48-linked ubiquitination degradation. The antiviral effect of BAG6 necessitated its N-terminal region containing a ubiquitin-like (UBL) domain (17-92aa) and a PB2-binding domain (124-186aa), which are synergistically responsible for viral polymerase subunit PB2 degradation and perturbing RdRp complex assembly. These findings unravel a novel antiviral mechanism via the interaction of viral PB2 and host protein BAG6 during avian or human influenza virus infection and highlight a potential application of BAG6 for antiviral drug development.
@@ -4908,12 +5154,12 @@
 (A) HeLa cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The viral NP and innate immunity-associated protein expression were measured by western blotting at different time points postinfection, as indicated. (B) BAG6-KO and BAG6-WT HeLa cells were infected with IAV H1N1 (MOI = 1.0), and the NP and innate immunity-associated protein expression were determined by western blotting at the indicated time points. (C) IRF9-KO Hela cells were transfected BAG6-HA expression plasmid or HA-vector. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The NP and innate immunity-associated protein expression were measured by western blotting at different time points post-infection, as indicated (C, left panels), and densitometry analysis and quantification were performed (C, right panels). (D) HeLa-WT (left panels) or HeLa-IRF9-KO (right panels) cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). Viral titers in the supernatants were determined by TCID50assay at 6, 12 and 24 h post-infection. (E and F) Vero cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The viral NP and M1 expression were measured by western blotting at different time points postinfection, as indicated (E). Viral titers in the supernatants were determined by TCID50assay at 6, 12 and 24 h post-infection (F). Data presented as means ± SD and are representative of three independent experiments. *p&lt; 0.05, **p&lt; 0.01, ***p&lt; 0.001, Unpaired Student’s t test.</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="S20" t="inlineStr">
         <is>
           <t>The interaction between influenza A virus (IAV) and host proteins is an important process that greatly influences viral replication and pathogenicity. PB2 protein is a subunit of viral ribonucleoprotein (vRNP) complex playing distinct roles in viral transcription and replication. BAG6 (BCL2-associated athanogene 6) as a multifunctional host protein participates in physiological and pathological processes. Here, we identify BAG6 as a new restriction factor for IAV replication through targeting PB2. For both avian and human influenza viruses, overexpression of BAG6 reduced viral protein expression and virus titers, whereas deletion of BAG6 significantly enhanced virus replication. Moreover, BAG6-knockdown mice developed more severe clinical symptoms and higher viral loads upon IAV infection. Mechanistically, BAG6 restricted IAV transcription and replication by inhibiting the activity of viral RNA-dependent RNA polymerase (RdRp). The co-immunoprecipitation assays showed BAG6 specifically interacted with the N-terminus of PB2 and competed with PB1 for RdRp complex assembly. The ubiquitination assay indicated that BAG6 promoted PB2 ubiquitination at K189 residue and targeted PB2 for K48-linked ubiquitination degradation. The antiviral effect of BAG6 necessitated its N-terminal region containing a ubiquitin-like (UBL) domain (17-92aa) and a PB2-binding domain (124-186aa), which are synergistically responsible for viral polymerase subunit PB2 degradation and perturbing RdRp complex assembly. These findings unravel a novel antiviral mechanism via the interaction of viral PB2 and host protein BAG6 during avian or human influenza virus infection and highlight a potential application of BAG6 for antiviral drug development.</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
+      <c r="T20" t="inlineStr">
         <is>
           <t>PMID: 38498560
 Full Text: The authors have declared that no competing interests exist.
@@ -4934,7 +5180,7 @@
 (A) HeLa cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The viral NP and innate immunity-associated protein expression were measured by western blotting at different time points postinfection, as indicated. (B) BAG6-KO and BAG6-WT HeLa cells were infected with IAV H1N1 (MOI = 1.0), and the NP and innate immunity-associated protein expression were determined by western blotting at the indicated time points. (C) IRF9-KO Hela cells were transfected BAG6-HA expression plasmid or HA-vector. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The NP and innate immunity-associated protein expression were measured by western blotting at different time points post-infection, as indicated (C, left panels), and densitometry analysis and quantification were performed (C, right panels). (D) HeLa-WT (left panels) or HeLa-IRF9-KO (right panels) cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). Viral titers in the supernatants were determined by TCID50assay at 6, 12 and 24 h post-infection. (E and F) Vero cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The viral NP and M1 expression were measured by western blotting at different time points postinfection, as indicated (E). Viral titers in the supernatants were determined by TCID50assay at 6, 12 and 24 h post-infection (F). Data presented as means ± SD and are representative of three independent experiments. *p&lt; 0.05, **p&lt; 0.01, ***p&lt; 0.001, Unpaired Student’s t test.</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="U20" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -4942,35 +5188,43 @@
     HGNC record ID: HGNC:13919
     Primary gene symbol: BAG6
     Official HGNC gene name: BAG cochaperone 6
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -4993,99 +5247,98 @@
 (A) HeLa cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The viral NP and innate immunity-associated protein expression were measured by western blotting at different time points postinfection, as indicated. (B) BAG6-KO and BAG6-WT HeLa cells were infected with IAV H1N1 (MOI = 1.0), and the NP and innate immunity-associated protein expression were determined by western blotting at the indicated time points. (C) IRF9-KO Hela cells were transfected BAG6-HA expression plasmid or HA-vector. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The NP and innate immunity-associated protein expression were measured by western blotting at different time points post-infection, as indicated (C, left panels), and densitometry analysis and quantification were performed (C, right panels). (D) HeLa-WT (left panels) or HeLa-IRF9-KO (right panels) cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). Viral titers in the supernatants were determined by TCID50assay at 6, 12 and 24 h post-infection. (E and F) Vero cells were transfected with BAG6-HA or Empty vector (EV) plasmids. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). The viral NP and M1 expression were measured by western blotting at different time points postinfection, as indicated (E). Viral titers in the supernatants were determined by TCID50assay at 6, 12 and 24 h post-infection (F). Data presented as means ± SD and are representative of three independent experiments. *p&lt; 0.05, **p&lt; 0.01, ***p&lt; 0.001, Unpaired Student’s t test.</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>{
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>Based on the provided text, here is my analysis:
+{
 "pmid": "38498560",
 "alias_symbol": "SCYTHE",
 "primary_gene_symbol": "BAG6",
 "name": "BAG cochaperone 6",
-"alias_symbol_represents_primary_gene": "YES",
-"alternate_abbreviation": "NO",
+"alternate_abbreviation": "YES",
 "evidence": "BAG6 (BCL2-associated athanogene 6, also known as BAT3 or Scythe) is a member of the BAG family due to a sequence homologous to the BAG domain at its C terminus and the collaboration with Heat Shock Protein 70 (Hsp70) family molecular chaperones [16]."
-}</t>
+}
+The text explicitly links the alias symbol SCYTHE to BAG6 by stating "BAG6 (BCL2-associated athanogene 6, also known as BAT3 or Scythe)". This indicates that SCYTHE is an alternate abbreviation for BAG6.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>HGNC:13919</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>ENSG00000234651, ENSG00000096155, ENSG00000233348, ENSG00000204463, ENSG00000228760, ENSG00000229524, ENSG00000227761</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>GENE ID:7917</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>BAG6</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>SCYTHE</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>38498560</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>38498560</v>
+      </c>
+      <c r="I21" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>alias</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>alias</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>intro</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>BAG6 (BCL2-associated athanogene 6, also known as BAT3 or Scythe) is a member of the BAG family due to a sequence homologous to the BAG domain at its C terminus and the collaboration with Heat Shock Protein 70 (Hsp70) family molecular chaperones</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr">
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr">
         <is>
           <t>BAG cochaperone 6</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="R21" t="inlineStr">
         <is>
           <t>To explore the mechanism by which BAG6 inhibits IAV replication, we assessed the impact of BAG6 on the polymerase activity of influenza viruses using a well-established dual-luciferase reporter assay [32,33]. The plasmids for expression of PB2, PB1, PA, and NP genes from various IAV subtype strains, including PR8 (H1N1), CN0606 (H7N9), and SD196 (H9N2), were co-transfected into HEK293T cells along with a pPoll-Luc reporter, respectively. The firefly luciferase levels in the cell lysate reflected the overall transcription and replication activities of viral polymerase complex (RdRp). The results showed that the overexpression of BAG6 inhibited the polymerase activities of H1N1, H7N9, and H9N2 in a dose-dependent manner (Fig 5A). In contrast, the enhanced polymerase activities of all IAV subtypes were observed in BAG6-KO A549 cells compared to the WT control (Fig 5B). The influenza virus polymerase complex is a key enzyme responsible for the replication and transcription of the influenza virus genome [34]. In view of this, we performed qRT-PCR analysis of viral mRNA and vRNA in H1N1-infected cells. The results showed that the mRNA and vRNA levels of both NP and M1 genes were significantly suppressed in BAG6-overexpressing cells (Fig 5C and 5D), and were elevated in BAG6-KO cells (Fig 5E and 5F). These data demonstrate that the BAG6 can inhibit the polymerase activity of various IAV subtypes.
 (A) HEK293T cells were co-transfected with pPolI-Luc reporter plasmid and expression plasmids containing viral PB1, PB2, PA, and NP of H1N1, H7N9 or H9N2 along with a graded dose of BAG6 or empty vector. Renilla luciferase was used as an internal control. Luciferase activity of the viral polymerase was determined at 24 h post-transfection (left panels). Western blottings show the expression of all transfected proteins (right panels) (B) BAG6-KO or BAG6-WT A549 cells were co-transfected with pPolI-Luc reporter plasmid and expression plasmids containing viral PB1, PB2, PA, and NP of H1N1/H7N9/H9N2. Renilla luciferase was used as an internal control. Luciferase activity of the viral polymerase was determined at 24 h post-transfection (left panel). Western blottings show the expression of all transfected proteins (right panel). (C and D) A549 cells was transfected with BAG6 expression plasmid or empty vector. At 24 h post-transfection, the cells were infected with IAV H1N1 (MOI = 1.0). At 4, 8, 12 and 24 h post-infection, the mRNA (C) and vRNA (D) level of M1 and NP were measured by quantitative real-time PCR, respectively. The expression of BAG6-HA was monitored by western blotting. (E and F) BAG6-KO or BAG6-WT A549 cells were infected with IAV H1N1 (MOI = 1.0). At 4, 8, 12 and 24 h post-infection, the mRNA (E) and vRNA (F) level of NP and M1 were measured by quantitative real-time PCR, respectively. The expression of BAG6-HA was monitored by western blotting. Data presented as means ± SD and are representative of three independent experiments. *p&lt; 0.05, **p&lt; 0.01, ***p&lt; 0.001, Unpaired Student’s t test.
@@ -5102,12 +5355,12 @@
 To further determine the PB2-binding sites of BAG6, we analyzed the protein structure of BAG6 from AlphaFold2 database and predicted the corresponding interaction domain of BAG6 and PB2 using an online software ColabFold. As shown inFig 9A, BAG6 associates with the N-terminus of PB2 through its 124–186 amino acids, which at least partially occupies the spatial position of PB1-PB2 interaction, whereas the Ub-like domain (17-92aa) at the N-terminus of BAG6 does not exhibit a direct interaction with PB2 in structure. According to the previous reports [40,41,43,45], the UBL domain is mainly responsible for recruiting ubiquitination machinery for efficient ubiquitination and degradation of various protein substrates. We, therefore, hypothesize that BAG6 may function as a transient platform that recruits the ubiquitin ligase by UBL domain and binds PB2 substrate by 124-186aa region during IAV infection, promoting PB2 degradation and IAV restriction. To verify this hypothesis, we constructed the corresponding truncation mutant plasmids, including BAG6 1:92-HA and 92:255-HA, as well as a deletion mutant lacking 124-186aa (BAG6 del 124:186-HA), as indicated inFig 9B. The Co-IP assay showed that only BAG6 92:255-HA was readily immunoprecipitated with PB2-Flag, but other mutants lacking 124-186aa region (1:92-HA and del 124:186-HA) could not bind to PB2 (Fig 9C), confirming the residues 124–186 as PB2-binding region of BAG6. Interestingly, compared with BAG6 1:255-HA, the ectopic expression of BAG6 92:255-HA had an obvious but reduced inhibitory effect on viral NP protein expression (Fig 9D), viral titers (Fig 9E), and viral polymerase activity (Fig 9F) in H1N1-infected cells, whereas BAG6 1:92-HA and del 124:186-HA completely failed to inhibit IAV replication and polymerase activity. These findings indicate that the PB2-binding region of BAG6 is necessary but insufficient for efficient IAV restriction. It may exert a reduced antiviral effects through binding PB2 and disrupting RdRp complex assembly, but fail to recruit ubiquitination machinery for PB2 degradation. These data demonstrate that both the UBL domain (17-92aa) and PB2-binding region (124-186aa) are required for highly effective PB2 degradation and IAV restriction.</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr">
+      <c r="S21" t="inlineStr">
         <is>
           <t>The interaction between influenza A virus (IAV) and host proteins is an important process that greatly influences viral replication and pathogenicity. PB2 protein is a subunit of viral ribonucleoprotein (vRNP) complex playing distinct roles in viral transcription and replication. BAG6 (BCL2-associated athanogene 6) as a multifunctional host protein participates in physiological and pathological processes. Here, we identify BAG6 as a new restriction factor for IAV replication through targeting PB2. For both avian and human influenza viruses, overexpression of BAG6 reduced viral protein expression and virus titers, whereas deletion of BAG6 significantly enhanced virus replication. Moreover, BAG6-knockdown mice developed more severe clinical symptoms and higher viral loads upon IAV infection. Mechanistically, BAG6 restricted IAV transcription and replication by inhibiting the activity of viral RNA-dependent RNA polymerase (RdRp). The co-immunoprecipitation assays showed BAG6 specifically interacted with the N-terminus of PB2 and competed with PB1 for RdRp complex assembly. The ubiquitination assay indicated that BAG6 promoted PB2 ubiquitination at K189 residue and targeted PB2 for K48-linked ubiquitination degradation. The antiviral effect of BAG6 necessitated its N-terminal region containing a ubiquitin-like (UBL) domain (17-92aa) and a PB2-binding domain (124-186aa), which are synergistically responsible for viral polymerase subunit PB2 degradation and perturbing RdRp complex assembly. These findings unravel a novel antiviral mechanism via the interaction of viral PB2 and host protein BAG6 during avian or human influenza virus infection and highlight a potential application of BAG6 for antiviral drug development.</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr">
+      <c r="T21" t="inlineStr">
         <is>
           <t>PMID: 38498560
 Full Text: To explore the mechanism by which BAG6 inhibits IAV replication, we assessed the impact of BAG6 on the polymerase activity of influenza viruses using a well-established dual-luciferase reporter assay [32,33]. The plasmids for expression of PB2, PB1, PA, and NP genes from various IAV subtype strains, including PR8 (H1N1), CN0606 (H7N9), and SD196 (H9N2), were co-transfected into HEK293T cells along with a pPoll-Luc reporter, respectively. The firefly luciferase levels in the cell lysate reflected the overall transcription and replication activities of viral polymerase complex (RdRp). The results showed that the overexpression of BAG6 inhibited the polymerase activities of H1N1, H7N9, and H9N2 in a dose-dependent manner (Fig 5A). In contrast, the enhanced polymerase activities of all IAV subtypes were observed in BAG6-KO A549 cells compared to the WT control (Fig 5B). The influenza virus polymerase complex is a key enzyme responsible for the replication and transcription of the influenza virus genome [34]. In view of this, we performed qRT-PCR analysis of viral mRNA and vRNA in H1N1-infected cells. The results showed that the mRNA and vRNA levels of both NP and M1 genes were significantly suppressed in BAG6-overexpressing cells (Fig 5C and 5D), and were elevated in BAG6-KO cells (Fig 5E and 5F). These data demonstrate that the BAG6 can inhibit the polymerase activity of various IAV subtypes.
@@ -5125,7 +5378,7 @@
 To further determine the PB2-binding sites of BAG6, we analyzed the protein structure of BAG6 from AlphaFold2 database and predicted the corresponding interaction domain of BAG6 and PB2 using an online software ColabFold. As shown inFig 9A, BAG6 associates with the N-terminus of PB2 through its 124–186 amino acids, which at least partially occupies the spatial position of PB1-PB2 interaction, whereas the Ub-like domain (17-92aa) at the N-terminus of BAG6 does not exhibit a direct interaction with PB2 in structure. According to the previous reports [40,41,43,45], the UBL domain is mainly responsible for recruiting ubiquitination machinery for efficient ubiquitination and degradation of various protein substrates. We, therefore, hypothesize that BAG6 may function as a transient platform that recruits the ubiquitin ligase by UBL domain and binds PB2 substrate by 124-186aa region during IAV infection, promoting PB2 degradation and IAV restriction. To verify this hypothesis, we constructed the corresponding truncation mutant plasmids, including BAG6 1:92-HA and 92:255-HA, as well as a deletion mutant lacking 124-186aa (BAG6 del 124:186-HA), as indicated inFig 9B. The Co-IP assay showed that only BAG6 92:255-HA was readily immunoprecipitated with PB2-Flag, but other mutants lacking 124-186aa region (1:92-HA and del 124:186-HA) could not bind to PB2 (Fig 9C), confirming the residues 124–186 as PB2-binding region of BAG6. Interestingly, compared with BAG6 1:255-HA, the ectopic expression of BAG6 92:255-HA had an obvious but reduced inhibitory effect on viral NP protein expression (Fig 9D), viral titers (Fig 9E), and viral polymerase activity (Fig 9F) in H1N1-infected cells, whereas BAG6 1:92-HA and del 124:186-HA completely failed to inhibit IAV replication and polymerase activity. These findings indicate that the PB2-binding region of BAG6 is necessary but insufficient for efficient IAV restriction. It may exert a reduced antiviral effects through binding PB2 and disrupting RdRp complex assembly, but fail to recruit ubiquitination machinery for PB2 degradation. These data demonstrate that both the UBL domain (17-92aa) and PB2-binding region (124-186aa) are required for highly effective PB2 degradation and IAV restriction.</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="U21" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
     Inputs:
@@ -5133,35 +5386,43 @@
     HGNC record ID: HGNC:13919
     Primary gene symbol: BAG6
     Official HGNC gene name: BAG cochaperone 6
-    Biomedical text context (may include PMID)
+    Biomedical text context
     Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
+    Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
+    as an alternate abbreviation of the official HGNC gene symbol.
+    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
+    The text must explicitly link the alias symbol to the official gene name through an expansion 
+    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    Examples:
+    1-
+    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
+    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
+    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
+    Alias gene symbol: A1B
+    Official HGNC gene name: alpha-1-B glycoprotein
+    Primary gene symbol: A1BG
+    2-
+    Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
+    cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Alias gene symbol: ASP
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "NO"
     "evidence": ""
     If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
+    Output only one JSON object. No markdown.
     {
     "pmid": "",
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
     "alternate_abbreviation": "YES or NO",
     "evidence": ""
     }
@@ -5181,221 +5442,6 @@
 To further determine the PB2-binding sites of BAG6, we analyzed the protein structure of BAG6 from AlphaFold2 database and predicted the corresponding interaction domain of BAG6 and PB2 using an online software ColabFold. As shown inFig 9A, BAG6 associates with the N-terminus of PB2 through its 124–186 amino acids, which at least partially occupies the spatial position of PB1-PB2 interaction, whereas the Ub-like domain (17-92aa) at the N-terminus of BAG6 does not exhibit a direct interaction with PB2 in structure. According to the previous reports [40,41,43,45], the UBL domain is mainly responsible for recruiting ubiquitination machinery for efficient ubiquitination and degradation of various protein substrates. We, therefore, hypothesize that BAG6 may function as a transient platform that recruits the ubiquitin ligase by UBL domain and binds PB2 substrate by 124-186aa region during IAV infection, promoting PB2 degradation and IAV restriction. To verify this hypothesis, we constructed the corresponding truncation mutant plasmids, including BAG6 1:92-HA and 92:255-HA, as well as a deletion mutant lacking 124-186aa (BAG6 del 124:186-HA), as indicated inFig 9B. The Co-IP assay showed that only BAG6 92:255-HA was readily immunoprecipitated with PB2-Flag, but other mutants lacking 124-186aa region (1:92-HA and del 124:186-HA) could not bind to PB2 (Fig 9C), confirming the residues 124–186 as PB2-binding region of BAG6. Interestingly, compared with BAG6 1:255-HA, the ectopic expression of BAG6 92:255-HA had an obvious but reduced inhibitory effect on viral NP protein expression (Fig 9D), viral titers (Fig 9E), and viral polymerase activity (Fig 9F) in H1N1-infected cells, whereas BAG6 1:92-HA and del 124:186-HA completely failed to inhibit IAV replication and polymerase activity. These findings indicate that the PB2-binding region of BAG6 is necessary but insufficient for efficient IAV restriction. It may exert a reduced antiviral effects through binding PB2 and disrupting RdRp complex assembly, but fail to recruit ubiquitination machinery for PB2 degradation. These data demonstrate that both the UBL domain (17-92aa) and PB2-binding region (124-186aa) are required for highly effective PB2 degradation and IAV restriction.</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>{
-"pmid": "38498560",
-"alias_symbol": "SCYTHE",
-"primary_gene_symbol": "BAG6",
-"name": "BAG cochaperone 6",
-"alias_symbol_represents_primary_gene": "NO",
-"alternate_abbreviation": "NO",
-"evidence": ""
-}</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>HGNC:13919</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>ENSG00000234651, ENSG00000096155, ENSG00000233348, ENSG00000204463, ENSG00000228760, ENSG00000229524, ENSG00000227761</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>GENE ID:7917</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>BAG6</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>SCYTHE</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>38498560</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>alias</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>alias</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>intro</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>BAG6 (BCL2-associated athanogene 6, also known as BAT3 or Scythe) is a member of the BAG family due to a sequence homologous to the BAG domain at its C terminus and the collaboration with Heat Shock Protein 70 (Hsp70) family molecular chaperones</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>BAG cochaperone 6</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>(A) The predicted interaction domain of BAG6 and PB2. The protein structure of PB2 and BAG6 from AlphaFold2 database and the predicted interaction complex from ColabFold online software, showing that BAG6 124–186 amino acids is the key region for binding to the N-terminus of PB2 protein, which competitively prevents PB1-PB2 interaction. The N-terminus of BAG6 (residues 1–255, blue) and the N-terminus of PB2 (residues 1–247, green) from ColabFold online prediction, the interaction region of PB1 in complex with PB2 (residues 678–757, light red) from PDB:3A1G. (B) Schematic diagram illustrating the truncated and deleted mutants of BAG6 based on the predicted interaction domain. UBL: ubiquitin-like domain; PXXP: proline-rich region. (C) HEK293T cells transfected with the indicated plasmids were immunoprecipitated with M2/Flag antibody, followed by western blot analysis. (D and E) A549 cells were transfected with BAG6 1:255-HA or BAG6 1:92-HA or BAG6 92:255-HA or BAG6 del124:186-HA empty vector for 24 h, and then infected with IAV H1N1 (MOI = 1.0). The viral NP proteins were measured by western blotting (D), the viral titers in the supernatants were determined by TCID50assay (E). (F) HEK293T cells were co-transfected with pPolI-Luc reporter plasmid and expression plasmids containing viral PB1, PB2, PA, and NP of H1N1 along with BAG6 1:255-HA or different truncated mutants of BAG6 or empty vector. Renilla luciferase was used as an internal control. Luciferase activity of the viral polymerase was determined at 24 h post-transfection. Data presented as means ± SD and are representative of three independent experiments. *p&lt; 0.05, **p&lt; 0.01, ***p&lt; 0.001, Unpaired Student’s t test.
-IAVs are among the most common contagious pathogens to cause severe respiratory infections. Host cells have developed multiple strategies to defend against IAV infection. This study identified BAG6 as a novel intrinsic antiviral factor to negatively regulate the replication of multiple IAV subtypes, including human H1N1, H5N1 and avian H7N9, H9N2. BAG6 specifically interacts with the N-terminus of viral polymerase subunit protein PB2, competitively interrupts the assembly of functional RdRp complex and induces the ubiquitination degradation of PB2, which attenuate viral polymerase activity and IAV replication in mammalian cells and pathogenicity in mouse model (Fig 10). These findings reveal a new antagonism mechanism between pathogens and hosts, and highlight a potent antiviral activity of BAG6 by targeting the key viral protein PB2.
-During IAV infection, BAG6 directly interacts with the N-terminus of the IAV polymerase subunit PB2. The interaction between BAG6 and PB2 competes with PB1 for PB2 binding, which perturbs the formation of a functional RdRp complex, and further targets PB2 for K48-linked ubiquitination degradation, thereby inhibiting IAV replication (by Figdraw).
-PB2 protein of IAV is critical for RdRp complex to catalyze the viral transcription and replication, and acts as a key determinant for mammalian adaptation of avian influenza virus. PB2 is responsible for binding the polymerase complex to host cell RNA and initiating viral transcription. It contains a conserved N-terminal fragment that interacts with PB1 to form the polymerase complex, and a central cap-binding domain that recognizes the 5’ cap structure of host cell mRNA, allowing the polymerase to "steal" the cap and use it to prime viral transcription [34]. Besides, the C-terminal part of PB2 contains the so-called 627 domain (residues 535–684), which participates in host adaptation and virulence by influencing the binding of NLS to importins [46]. Multiple host proteins have been found to restrict IAV replication by targeting PB2. For instance, TRIM35 mediates the protection against influenza infection by activating TRAF3 and inducing K48-linked ubiquitination and degradation of PB2 [44]. PIAS restricts IAV replication and virulence through mediating PB2 SUMOylation and reducing its stability [47]. In addition, ANP32A inhibits IAV replication in mammalian cells through differential regulation of the activity of viral polymerases carrying PB2-627K (human) or PB2-627E (avian) signature [12,48]. Here, we found that BAG6 associated with PB2, thereby perturbing its interaction with PB1 and inducing its ubiquitination degradation. Notably, BAG6 recognizes the N-terminus of PB2 and promotes PB2 ubiquitination at its K189 residue, which is highly conserved among avian and human influenza strains from Global Initiative on Sharing Avian Influenza Data (GISAID,www.epicov.org) (S1 Table), providing the mechanistic basis that BAG6 acts as a potent antiviral factor during both human- and avian-origin IAV infection.
-BAG6 is a multifunctional protein in host cell and participates in a variety of physiological and pathological processes [19]. BAG6 functions as an essential factor in ubiquitin-mediated metabolism of neo-synthesized defective polypeptides and misfolded/mislocalized proteins [49–51]. It can capture these defective or mislocalized substrates by interacting with their unprocessed or non-inserted hydrophobic domains [45], and at the same time, recruit the E3 ligases, primarily RNF126, to its N-terminal UBL domain for efficient ubiquitination and degradation [40]. Besides, BAG6 is necessary for DNA damage-induced apoptosis by controlling the p53 signaling pathway [52]. It promotes p53 transactivation by stabilizing its interaction with the acetyltransferase p300 and enhancing p53 acetylation during apoptosis and autophagy [21,22,53]. A recent study reported that BAG6 was capable of regulating the activation of IFN-I by inhibiting RIG-I/VISA-mediated recognition of RNA ligand [29]. However, the role of BAG6 in virus infection remains opaque. In this study, we provide evidence that BAG6 can potently inhibit influenza virus replicationin vitroandin vivo. Further investigation found that the overexpression of BAG6 neither affected cell apoptosis during IAV infection (S4 Fig), nor relied on the IFN-I antiviral response to inhibit IAV replication (Fig 4), whereas BAG6 directly interacts with viral polymerase subunit PB2 and targets it for ubiquitination degradation. These findings reveal a novel mechanism by which BAG6 serves as an antiviral factor to specifically target viral protein through its protein quality control function.
-In the recent years, there has been increased interest in harnessing targeted protein degradation (TPD) technology in the development of antiviral therapies by inducing the degradation of either viral or host-related protein targets, but the off-target side effects and toxicity greatly limit its use [54–57]. In this study, we found the N-terminus of host protein BAG6 contains a ubiquitin-like domain (UBL, 17-92aa), which was previously reported to recruit E3 ligase RNF126 and ubiquitinates BAG6-associated clients [40], and a PB2-binding domain (124-186aa), which was proved to interact with viral polymerase subunit PB2 protein during IAV infection. Interestingly, although the BAG6:92-255aa mutant lacking the UBL domain weakened BAG6-meditated antiviral activity against IAV, it still significantly restricted viral polymerase activity and replication (Fig 9E and 9F). This mirrors the findings that BAG6 could suppress the viral polymerase activity by competing with PB1 for PB2 binding and interfering with RdRp assembly (Fig 6E and 6F), even in the situation with PB2 degradation resistance. These data indicate that both UBL and PB2-binding domains are essential for the efficient PB2 degradation and BAG6-mediated antiviral activity. This unique structure thus allows BAG6 naturally possessing a proteolysis-targeting function. By targeting viral PB2, BAG6 is more likely to become a potential candidate for antiviral drug development.
-The laboratory animal usage license number is SYXK-Beijing-2018-0038, certified by Beijing Association for Science and Technology. All animal research was performed in compliance with the Beijing Laboratory Animal Welfare and Ethics guidelines, as issued by the Beijing Administration Committee of Laboratory Animals, and the China Agricultural University (CAU) Institutional Animal Care and Use Committee guidelines (ID: SKLAB-B-2010-003) approved by the Animal Welfare Committee of CAU. All experiments with live viruses were performed in Biosafety Level II laboratory (BSL-2) in CAU. All animal research involved in this study was approved by the Animal Welfare Committee of CAU (No.AW03503202-2-2).
-Human lung adenocarcinoma epithelial cells (A549), HeLa cell, Madin-Darby canine kidney cells (MDCK), Vero cell and human embryonic kidney cells (HEK293T) were purchased from ATCC. IRF9-KO HeLa cells were generated as previous indicated [30,31]. BAG6 KO A549 cells and BAG6 KO HeLa cells were generated using CRISPR/Cas 9-based knockout of BAG6 gene. In brief, the BAG6 gene target sequences, #1 5’- CACCGCGGTACTGGTACTATCATT-3’ and #2 5’- CACCAGGCTCCTCCACAGCGGTAC-3’, were inserted into the guide RNA (gRNA) expression cassette of the pUC19 vector, which also contains an expression cassette of Cas9. The pUC19 plasmid containing the BAG6 target sequence was then transfected into A549 or HeLa cells. The transfected cells were trypsinized 24 h later into single cells, which were diluted and inoculated into a 96-well plate by infinite dilution. Each colony was individually propagated in a 96-well plate, and the knockout of BAG6 expression was confirmed by western blotting. Cells were cultured in DMEM supplemented with 10% v/v heat-inactivated fetal bovine serum (10099141C, Gibco, USA), 100 U mL−1penicillin and 100 μg mL−1streptomycin at 37°C in a 5% CO2atmosphere.
-Influenza A/Puerto Rico/8/1934 (PR8, H1N1, accession HA number:CY045764), A/chicken/China/0606-13/2017 (CN0606, H7N9, accession HA number:MK530478), and A/chicken/Shandong/196/2011 (SD196, H9N2, accession HA number:KR002651) and A/Anhui/1/2005 (AH1, H5N1, accession HA number:HM172104) viruses were maintained in the laboratory. All experiments using non-H5 live viruses were performed in the Biosafety Level II laboratory (BSL-2), and experiments using H5 viruses were performed in the Biosafety Level III Laboratory (BSL-3) in CAU.
-Protein expression plasmids BAG6-HA, BAG6 1:255-HA, BAG6 1:753-HA, BAG6 482:753-HA, BAG6 482:1126-HA, BAG6 642:1126-HA, PB2-Flag, N-terminal PB2-Flag, PB1-Flag, PA-Flag, NP-Flag, M1-Flag, PB2-K5R-Flag, PB2-K33R-Flag, PB2-K41R-Flag, PB2-K48R-Flag, PB2-K61R-Flag, PB2-K187R-Flag, PB2-K189R-Flag, PB2-K331R-Flag, PB2-K339R-Flag, PB2-K353R-Flag, PB2-K482R-Flag, PB2-K561R-Flag, PB2-K617R-Flag, PB2-K699R-Flag, PB2-K721R-Flag, PB2-K736R-Flag, PB2-K738R-Flag, PB2-K752R-Flag, Ub-HA, K48-Ub-HA and K63-Ub-HA were generated by subcloning the corresponding coding segment into the HA-pRK5 or Flag-pRK5 empty vector by homologous recombinase-mediated recombination (S1 Table). Plasmid transfections in HEK293T or A549 cells were performed using jetPRIME (101000046, Polyplus, France).
-Antibody concentrations for immunoprecipitation and immunoblotting were determined empirically. All immunoblot antibodies were diluted as specified in 5% w/v BSA-TBST. Antibodies used as follows: anti-BAG6 (B01P, Abnova, Taiwan, China), anti-PB2 (PA5-32220, Thermo Scientific, Massachusetts, USA), anti-PB1 (PA5-34914, Thermo Scientific, Massachusetts, USA), anti-β-actin (A1978, Sigma, Shanghai, China), anti-GAPDH (ab8245, Abcam, Shanghai, China), anti-PARP (9542, Cell Signaling Technology, Massachusetts, USA), anti-Flag (F1804, Sigma, Shanghai, China and 20543-1-AP, Proteintech, Chicago, USA), anti-HA (H9658, Sigma, Shanghai, China and 51064-2-AP, Proteintech, Chicago, USA), anti-RIG-I (20566-1-AP, Proteintech, Chicago, USA), anti-p-STAT1 (9167, Cell Signaling Technology, Massachusetts, USA), anti-ISG15 (sc166755, Santa Cruz, California, USA), anti-influenza A virus NP (A01506-40, GenScript, New Jersey, USA), Mouse monoclonal anti-influenza A virus M1 antibody (Lab Homemade, Beijing, China, ZL201910912806.0). Cycloheximide (CHX, HY-12320), MG132 (HY-13259C) and Chloroquine (CQ, HY-17589A) was purchased from MCE.
-A dual-luciferase reporter assay system (E1960, Promega, Wisconsin, USA) was used to compare the polymerase activities of different viral RNP complexes. PB2, PB1, PA, and NP gene segments of the indicated viruses (PR8, CN0606 and SD196) were separately cloned into the pCDNA3.1 expression plasmid. PB2, PB1, PA, and NP plasmids (125 ng each plasmid) along with the pLuci luciferase reporter plasmid (10 ng) and the renilla internal control plasmid (2.5 ng) were used to transfect cells. Cell cultures were incubated at 37°C. Cell lysates were analyzed at 24 h post-transfection for firefly and renilla luciferase activities using a GloMax 96 microplate luminometer (GM2000, Promega, Wisconsin, USA). Polymerase proteins were detected by Western blotting.
-Six-week-old BALB/c background female mice were purchased from Beijing Vital River Co. Ltd. (Beijing, China). Animal studies were carried out in specific pathogen-free barrier facilities. Facilities were maintained at an acceptable range of 20–26°C humidity of 30–70% on a 12-h dark/12-h light cycle. Peptide-conjugated PPMO were purchased from Gene Tools (USA). PPMO targeting mouse BAG6 gene (PPMO-BAG6) was designed as CTGGCACTATCACTCGGCTCCATG. A nontargeting PPMO control sequence (PPMO-NC) (CCTCTTACCTCAGTTACAATTTATA), was used as control. Six to eight weeks BALB/c female mice were inoculated intranasally with 100 μg of PPMOs in 50 μL PBS for 2 days continuously.
-Mice were anesthetized and intranasally inoculated with PR8 virus at a median tissue culture infectious dose (TCID50) of 100 in 50 μL of PBS. Body weight and survival were monitored daily for 14 days. Lung tissue lysates were generated by homogenizing snap-frozen lung tissues twice (20 s each time) in MEM medium and centrifuging the lung suspensions at 2000 rpm for 15 min. TCID50assays were performed using MDCK cells and TCID50was calculated as previously described [58]. A portion of the lung from each euthanized mouse at 3 and 5 dpi was fixed in 10% phosphate-buffered formalin, embedded in paraffin, sectioned and stained with hematoxylin and eosin (H&amp;E). Immunohistochemical staining of viral antigen was performed as described previously [59].
-Total RNA from cells was extracted using an RNA isolation kit (Thermo Scientific, Massachusetts, USA). First-strand complementary DNA was synthesized from 1 μg of total RNA using a TransScript RT reagent kit (TransGen, Beijing, China), and oligo dT primer were used for detecting host genes. For the detection of influenza virus mRNA and vRNA, oligo dT primer and uni-12 primer (5′-AGCAAAAGCAGG-3′) [60] were respectively used to generate cDNAs. Generated cDNA was subjected to qPCR in a 25 μL reaction volume using 2X M5 HiPer SYBR Premix EsTaq (with Tli RNaseH) (Mei5bio) (S1 Table). Human β-actin genes were amplified for normalization of the cDNA amount used in qPCR. Reactions were conducted in triplicate, and the data were analyzed using the 2−ΔΔCtmethod.
-Cells were lysed in lysis buffer (50 mM Tris-Cl at pH 8.0, 150 mM NaCl, 1% Tri-ton X-100, 1 mM DTT, 1× complete protease inhibitor cocktail, and 10% glycerol) and pre-cleared with Protein A/G PLUS-Agarose beads (sc-2003, Santa Cruz Biotechnology, USA) for 2 h at 4°C. The lysates were then immunoprecipitated with indicated antibodies or isotype-matched control antibodies plus protein G Sepharose beads at 4°C for 2–4 h. The beads were then washed three times and boiled. Protein samples were analyzed by Western blotting. For Western blotting, protein samples were mixed with 6× loading buffer supplemented with 10% β-mercaptoethanol, heated at 100°C for 5 min and separated on a 10% SDS-PAGE under reducing conditions. After electrophoresis, protein samples were electroblotted onto polyvinylidene difluoride membranes (Bio-Rad, CA, USA) and blocked for 2 h in Tris-buffered saline (10 mM Tris-HCl, pH 8.0, containing 150 mM NaCl) containing 5% (w/v) non-fat dry milk and 0.5‰ (v/v) Tween-20. The blots were incubated with the primary antibodies overnight at 4°C. The next day, the blots were incubated with corresponding horseradish peroxidase (HRP)-conjugated secondary antibodies for 1 h at room temperature (RT). HRP antibody binding was detected using a standard enhanced chemiluminescence (ECL) kit (wbluf0500, Millipore, USA).
-HEK293T cell lines were cotransfected with PB2-Flag plasmid with empty vector or BAG6-HA plasmid. After 24 h post-transfection, CHX (50 μg/mL) was added to the medium and cells were harvested at different time points. Western blotting of cell lysates was performed to detect PB2-Flag, BAG6-HA and β-actin. To investigate the cellular pathway of BAG6-mediated PB2 degradation, at 24 h post-transfection, or infection with PR8 (H1N1), MG132 (20 μM) or CQ (150 μM) was added to the medium, and the cells were harvested 6 h after treatment. Three independent experiments were performed.
-HEK293T cells were transfected with HA-tagged ubiquitin (Ub-HA) plasmids, BAG6-HA or empty plasmids, and PB2-Flag or PB2-Flag with Lysine mutations. At 24 h post-transfection, the cells were treated with MG132 (20 μM) for 6 h and then lysed in 1% SDS lysis buffer. After being boiled for 10 min, the lysates were diluted 10 times with cold lysis buffer supplemented with 1× complete protease inhibitor cocktail, 10 mM DTT, and 10 mM NEM. PB2-Flag protein was then purified with anti-Flag antibody and subjected to western blotting analysis. Ubiquitinated PB2-Flag was detected by anti-HA antibody.
-We downloaded all available PB2 amino acid sequences of human and avian origin for influenza viruses of subtypes H1, H3, H5, H7, and H9 from the Global Initiative on Sharing Avian Influenza Data (GISAID,www.epicov.org) (date of access: Jan. 22, 2024), and multiple sequence alignment was performed using MAFFT v7.0 [61], and then the amino acid categories and percentages of the 189 amino acid residues were counted.
-Cells on coverslips were washed twice with prewarmed PBS and fixed with 4% paraformaldehyde for 15 min at room temperature. Cells were subsequently permeabilized with immunostaining permeabilization buffer containing Triton X-100 (P0096, Beyotime, Shanghai, China) for 10 min and blocked with QuickBlock blocking buffer (P0220, Beyotime, Shanghai, China) for 20 min at room temperature. Fixed cells were incubated with indicated antibodies diluted in immunostaining primary antibody dilution buffer at 4°C overnight. Coverslips were then washed three times with PBS and incubated with Alexa Fluor 488-conjugated secondary antibodies or Alexa Fluor 555-conjugated secondary antibodies for 1 h at 37°C. Coverslips were finally washed three times and mounted onto microscope slides with DAPI staining solution (C1006, Beyotime, Shanghai, China) for 8 min and examined by confocal microscopy. Immunoassayed cells were visualized using a Nikon super-resolution laser scanning confocal microscope under a 100-time oil objective and analyzed using the Imaris 9.2 platform.
-An online software, ColabFold, was used for the prediction of protein structures and complexes by combining the fast homology search of MMseqs2 with AlphaFold2 or RoseTTAFold. Sequence alignments/templates are generated through MMseqs2 and HHsearch [62]. The amino acid sequences of BAG6 protein N-terminal 1-255aa and PB2 protein N-terminal 1-247aa were used for the prediction of protein complex at the open-source website ColabFold v1.5.2 (https://colab.research.google.com/github/sokrypton/ColabFold/blob/main/AlphaFold2.ipynb#scrollTo=mbaIO9pWjaN0), and the predicted results were viewed and analyzed using PyMOL v2.5.0.
-WT A549 and BAG6-KO A549 cells or WT HeLa and BAG6-KO HeLa cells were plated in 96-well plates at a density of 2000 cells in 100 μL of medium per well. The cell viability was then assayed according to the CCK8 kit instructions (C0042, Beyotime, Shanghai, China).</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>The interaction between influenza A virus (IAV) and host proteins is an important process that greatly influences viral replication and pathogenicity. PB2 protein is a subunit of viral ribonucleoprotein (vRNP) complex playing distinct roles in viral transcription and replication. BAG6 (BCL2-associated athanogene 6) as a multifunctional host protein participates in physiological and pathological processes. Here, we identify BAG6 as a new restriction factor for IAV replication through targeting PB2. For both avian and human influenza viruses, overexpression of BAG6 reduced viral protein expression and virus titers, whereas deletion of BAG6 significantly enhanced virus replication. Moreover, BAG6-knockdown mice developed more severe clinical symptoms and higher viral loads upon IAV infection. Mechanistically, BAG6 restricted IAV transcription and replication by inhibiting the activity of viral RNA-dependent RNA polymerase (RdRp). The co-immunoprecipitation assays showed BAG6 specifically interacted with the N-terminus of PB2 and competed with PB1 for RdRp complex assembly. The ubiquitination assay indicated that BAG6 promoted PB2 ubiquitination at K189 residue and targeted PB2 for K48-linked ubiquitination degradation. The antiviral effect of BAG6 necessitated its N-terminal region containing a ubiquitin-like (UBL) domain (17-92aa) and a PB2-binding domain (124-186aa), which are synergistically responsible for viral polymerase subunit PB2 degradation and perturbing RdRp complex assembly. These findings unravel a novel antiviral mechanism via the interaction of viral PB2 and host protein BAG6 during avian or human influenza virus infection and highlight a potential application of BAG6 for antiviral drug development.</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>PMID: 38498560
-Full Text: (A) The predicted interaction domain of BAG6 and PB2. The protein structure of PB2 and BAG6 from AlphaFold2 database and the predicted interaction complex from ColabFold online software, showing that BAG6 124–186 amino acids is the key region for binding to the N-terminus of PB2 protein, which competitively prevents PB1-PB2 interaction. The N-terminus of BAG6 (residues 1–255, blue) and the N-terminus of PB2 (residues 1–247, green) from ColabFold online prediction, the interaction region of PB1 in complex with PB2 (residues 678–757, light red) from PDB:3A1G. (B) Schematic diagram illustrating the truncated and deleted mutants of BAG6 based on the predicted interaction domain. UBL: ubiquitin-like domain; PXXP: proline-rich region. (C) HEK293T cells transfected with the indicated plasmids were immunoprecipitated with M2/Flag antibody, followed by western blot analysis. (D and E) A549 cells were transfected with BAG6 1:255-HA or BAG6 1:92-HA or BAG6 92:255-HA or BAG6 del124:186-HA empty vector for 24 h, and then infected with IAV H1N1 (MOI = 1.0). The viral NP proteins were measured by western blotting (D), the viral titers in the supernatants were determined by TCID50assay (E). (F) HEK293T cells were co-transfected with pPolI-Luc reporter plasmid and expression plasmids containing viral PB1, PB2, PA, and NP of H1N1 along with BAG6 1:255-HA or different truncated mutants of BAG6 or empty vector. Renilla luciferase was used as an internal control. Luciferase activity of the viral polymerase was determined at 24 h post-transfection. Data presented as means ± SD and are representative of three independent experiments. *p&lt; 0.05, **p&lt; 0.01, ***p&lt; 0.001, Unpaired Student’s t test.
-IAVs are among the most common contagious pathogens to cause severe respiratory infections. Host cells have developed multiple strategies to defend against IAV infection. This study identified BAG6 as a novel intrinsic antiviral factor to negatively regulate the replication of multiple IAV subtypes, including human H1N1, H5N1 and avian H7N9, H9N2. BAG6 specifically interacts with the N-terminus of viral polymerase subunit protein PB2, competitively interrupts the assembly of functional RdRp complex and induces the ubiquitination degradation of PB2, which attenuate viral polymerase activity and IAV replication in mammalian cells and pathogenicity in mouse model (Fig 10). These findings reveal a new antagonism mechanism between pathogens and hosts, and highlight a potent antiviral activity of BAG6 by targeting the key viral protein PB2.
-During IAV infection, BAG6 directly interacts with the N-terminus of the IAV polymerase subunit PB2. The interaction between BAG6 and PB2 competes with PB1 for PB2 binding, which perturbs the formation of a functional RdRp complex, and further targets PB2 for K48-linked ubiquitination degradation, thereby inhibiting IAV replication (by Figdraw).
-PB2 protein of IAV is critical for RdRp complex to catalyze the viral transcription and replication, and acts as a key determinant for mammalian adaptation of avian influenza virus. PB2 is responsible for binding the polymerase complex to host cell RNA and initiating viral transcription. It contains a conserved N-terminal fragment that interacts with PB1 to form the polymerase complex, and a central cap-binding domain that recognizes the 5’ cap structure of host cell mRNA, allowing the polymerase to "steal" the cap and use it to prime viral transcription [34]. Besides, the C-terminal part of PB2 contains the so-called 627 domain (residues 535–684), which participates in host adaptation and virulence by influencing the binding of NLS to importins [46]. Multiple host proteins have been found to restrict IAV replication by targeting PB2. For instance, TRIM35 mediates the protection against influenza infection by activating TRAF3 and inducing K48-linked ubiquitination and degradation of PB2 [44]. PIAS restricts IAV replication and virulence through mediating PB2 SUMOylation and reducing its stability [47]. In addition, ANP32A inhibits IAV replication in mammalian cells through differential regulation of the activity of viral polymerases carrying PB2-627K (human) or PB2-627E (avian) signature [12,48]. Here, we found that BAG6 associated with PB2, thereby perturbing its interaction with PB1 and inducing its ubiquitination degradation. Notably, BAG6 recognizes the N-terminus of PB2 and promotes PB2 ubiquitination at its K189 residue, which is highly conserved among avian and human influenza strains from Global Initiative on Sharing Avian Influenza Data (GISAID,www.epicov.org) (S1 Table), providing the mechanistic basis that BAG6 acts as a potent antiviral factor during both human- and avian-origin IAV infection.
-BAG6 is a multifunctional protein in host cell and participates in a variety of physiological and pathological processes [19]. BAG6 functions as an essential factor in ubiquitin-mediated metabolism of neo-synthesized defective polypeptides and misfolded/mislocalized proteins [49–51]. It can capture these defective or mislocalized substrates by interacting with their unprocessed or non-inserted hydrophobic domains [45], and at the same time, recruit the E3 ligases, primarily RNF126, to its N-terminal UBL domain for efficient ubiquitination and degradation [40]. Besides, BAG6 is necessary for DNA damage-induced apoptosis by controlling the p53 signaling pathway [52]. It promotes p53 transactivation by stabilizing its interaction with the acetyltransferase p300 and enhancing p53 acetylation during apoptosis and autophagy [21,22,53]. A recent study reported that BAG6 was capable of regulating the activation of IFN-I by inhibiting RIG-I/VISA-mediated recognition of RNA ligand [29]. However, the role of BAG6 in virus infection remains opaque. In this study, we provide evidence that BAG6 can potently inhibit influenza virus replicationin vitroandin vivo. Further investigation found that the overexpression of BAG6 neither affected cell apoptosis during IAV infection (S4 Fig), nor relied on the IFN-I antiviral response to inhibit IAV replication (Fig 4), whereas BAG6 directly interacts with viral polymerase subunit PB2 and targets it for ubiquitination degradation. These findings reveal a novel mechanism by which BAG6 serves as an antiviral factor to specifically target viral protein through its protein quality control function.
-In the recent years, there has been increased interest in harnessing targeted protein degradation (TPD) technology in the development of antiviral therapies by inducing the degradation of either viral or host-related protein targets, but the off-target side effects and toxicity greatly limit its use [54–57]. In this study, we found the N-terminus of host protein BAG6 contains a ubiquitin-like domain (UBL, 17-92aa), which was previously reported to recruit E3 ligase RNF126 and ubiquitinates BAG6-associated clients [40], and a PB2-binding domain (124-186aa), which was proved to interact with viral polymerase subunit PB2 protein during IAV infection. Interestingly, although the BAG6:92-255aa mutant lacking the UBL domain weakened BAG6-meditated antiviral activity against IAV, it still significantly restricted viral polymerase activity and replication (Fig 9E and 9F). This mirrors the findings that BAG6 could suppress the viral polymerase activity by competing with PB1 for PB2 binding and interfering with RdRp assembly (Fig 6E and 6F), even in the situation with PB2 degradation resistance. These data indicate that both UBL and PB2-binding domains are essential for the efficient PB2 degradation and BAG6-mediated antiviral activity. This unique structure thus allows BAG6 naturally possessing a proteolysis-targeting function. By targeting viral PB2, BAG6 is more likely to become a potential candidate for antiviral drug development.
-The laboratory animal usage license number is SYXK-Beijing-2018-0038, certified by Beijing Association for Science and Technology. All animal research was performed in compliance with the Beijing Laboratory Animal Welfare and Ethics guidelines, as issued by the Beijing Administration Committee of Laboratory Animals, and the China Agricultural University (CAU) Institutional Animal Care and Use Committee guidelines (ID: SKLAB-B-2010-003) approved by the Animal Welfare Committee of CAU. All experiments with live viruses were performed in Biosafety Level II laboratory (BSL-2) in CAU. All animal research involved in this study was approved by the Animal Welfare Committee of CAU (No.AW03503202-2-2).
-Human lung adenocarcinoma epithelial cells (A549), HeLa cell, Madin-Darby canine kidney cells (MDCK), Vero cell and human embryonic kidney cells (HEK293T) were purchased from ATCC. IRF9-KO HeLa cells were generated as previous indicated [30,31]. BAG6 KO A549 cells and BAG6 KO HeLa cells were generated using CRISPR/Cas 9-based knockout of BAG6 gene. In brief, the BAG6 gene target sequences, #1 5’- CACCGCGGTACTGGTACTATCATT-3’ and #2 5’- CACCAGGCTCCTCCACAGCGGTAC-3’, were inserted into the guide RNA (gRNA) expression cassette of the pUC19 vector, which also contains an expression cassette of Cas9. The pUC19 plasmid containing the BAG6 target sequence was then transfected into A549 or HeLa cells. The transfected cells were trypsinized 24 h later into single cells, which were diluted and inoculated into a 96-well plate by infinite dilution. Each colony was individually propagated in a 96-well plate, and the knockout of BAG6 expression was confirmed by western blotting. Cells were cultured in DMEM supplemented with 10% v/v heat-inactivated fetal bovine serum (10099141C, Gibco, USA), 100 U mL−1penicillin and 100 μg mL−1streptomycin at 37°C in a 5% CO2atmosphere.
-Influenza A/Puerto Rico/8/1934 (PR8, H1N1, accession HA number:CY045764), A/chicken/China/0606-13/2017 (CN0606, H7N9, accession HA number:MK530478), and A/chicken/Shandong/196/2011 (SD196, H9N2, accession HA number:KR002651) and A/Anhui/1/2005 (AH1, H5N1, accession HA number:HM172104) viruses were maintained in the laboratory. All experiments using non-H5 live viruses were performed in the Biosafety Level II laboratory (BSL-2), and experiments using H5 viruses were performed in the Biosafety Level III Laboratory (BSL-3) in CAU.
-Protein expression plasmids BAG6-HA, BAG6 1:255-HA, BAG6 1:753-HA, BAG6 482:753-HA, BAG6 482:1126-HA, BAG6 642:1126-HA, PB2-Flag, N-terminal PB2-Flag, PB1-Flag, PA-Flag, NP-Flag, M1-Flag, PB2-K5R-Flag, PB2-K33R-Flag, PB2-K41R-Flag, PB2-K48R-Flag, PB2-K61R-Flag, PB2-K187R-Flag, PB2-K189R-Flag, PB2-K331R-Flag, PB2-K339R-Flag, PB2-K353R-Flag, PB2-K482R-Flag, PB2-K561R-Flag, PB2-K617R-Flag, PB2-K699R-Flag, PB2-K721R-Flag, PB2-K736R-Flag, PB2-K738R-Flag, PB2-K752R-Flag, Ub-HA, K48-Ub-HA and K63-Ub-HA were generated by subcloning the corresponding coding segment into the HA-pRK5 or Flag-pRK5 empty vector by homologous recombinase-mediated recombination (S1 Table). Plasmid transfections in HEK293T or A549 cells were performed using jetPRIME (101000046, Polyplus, France).
-Antibody concentrations for immunoprecipitation and immunoblotting were determined empirically. All immunoblot antibodies were diluted as specified in 5% w/v BSA-TBST. Antibodies used as follows: anti-BAG6 (B01P, Abnova, Taiwan, China), anti-PB2 (PA5-32220, Thermo Scientific, Massachusetts, USA), anti-PB1 (PA5-34914, Thermo Scientific, Massachusetts, USA), anti-β-actin (A1978, Sigma, Shanghai, China), anti-GAPDH (ab8245, Abcam, Shanghai, China), anti-PARP (9542, Cell Signaling Technology, Massachusetts, USA), anti-Flag (F1804, Sigma, Shanghai, China and 20543-1-AP, Proteintech, Chicago, USA), anti-HA (H9658, Sigma, Shanghai, China and 51064-2-AP, Proteintech, Chicago, USA), anti-RIG-I (20566-1-AP, Proteintech, Chicago, USA), anti-p-STAT1 (9167, Cell Signaling Technology, Massachusetts, USA), anti-ISG15 (sc166755, Santa Cruz, California, USA), anti-influenza A virus NP (A01506-40, GenScript, New Jersey, USA), Mouse monoclonal anti-influenza A virus M1 antibody (Lab Homemade, Beijing, China, ZL201910912806.0). Cycloheximide (CHX, HY-12320), MG132 (HY-13259C) and Chloroquine (CQ, HY-17589A) was purchased from MCE.
-A dual-luciferase reporter assay system (E1960, Promega, Wisconsin, USA) was used to compare the polymerase activities of different viral RNP complexes. PB2, PB1, PA, and NP gene segments of the indicated viruses (PR8, CN0606 and SD196) were separately cloned into the pCDNA3.1 expression plasmid. PB2, PB1, PA, and NP plasmids (125 ng each plasmid) along with the pLuci luciferase reporter plasmid (10 ng) and the renilla internal control plasmid (2.5 ng) were used to transfect cells. Cell cultures were incubated at 37°C. Cell lysates were analyzed at 24 h post-transfection for firefly and renilla luciferase activities using a GloMax 96 microplate luminometer (GM2000, Promega, Wisconsin, USA). Polymerase proteins were detected by Western blotting.
-Six-week-old BALB/c background female mice were purchased from Beijing Vital River Co. Ltd. (Beijing, China). Animal studies were carried out in specific pathogen-free barrier facilities. Facilities were maintained at an acceptable range of 20–26°C humidity of 30–70% on a 12-h dark/12-h light cycle. Peptide-conjugated PPMO were purchased from Gene Tools (USA). PPMO targeting mouse BAG6 gene (PPMO-BAG6) was designed as CTGGCACTATCACTCGGCTCCATG. A nontargeting PPMO control sequence (PPMO-NC) (CCTCTTACCTCAGTTACAATTTATA), was used as control. Six to eight weeks BALB/c female mice were inoculated intranasally with 100 μg of PPMOs in 50 μL PBS for 2 days continuously.
-Mice were anesthetized and intranasally inoculated with PR8 virus at a median tissue culture infectious dose (TCID50) of 100 in 50 μL of PBS. Body weight and survival were monitored daily for 14 days. Lung tissue lysates were generated by homogenizing snap-frozen lung tissues twice (20 s each time) in MEM medium and centrifuging the lung suspensions at 2000 rpm for 15 min. TCID50assays were performed using MDCK cells and TCID50was calculated as previously described [58]. A portion of the lung from each euthanized mouse at 3 and 5 dpi was fixed in 10% phosphate-buffered formalin, embedded in paraffin, sectioned and stained with hematoxylin and eosin (H&amp;E). Immunohistochemical staining of viral antigen was performed as described previously [59].
-Total RNA from cells was extracted using an RNA isolation kit (Thermo Scientific, Massachusetts, USA). First-strand complementary DNA was synthesized from 1 μg of total RNA using a TransScript RT reagent kit (TransGen, Beijing, China), and oligo dT primer were used for detecting host genes. For the detection of influenza virus mRNA and vRNA, oligo dT primer and uni-12 primer (5′-AGCAAAAGCAGG-3′) [60] were respectively used to generate cDNAs. Generated cDNA was subjected to qPCR in a 25 μL reaction volume using 2X M5 HiPer SYBR Premix EsTaq (with Tli RNaseH) (Mei5bio) (S1 Table). Human β-actin genes were amplified for normalization of the cDNA amount used in qPCR. Reactions were conducted in triplicate, and the data were analyzed using the 2−ΔΔCtmethod.
-Cells were lysed in lysis buffer (50 mM Tris-Cl at pH 8.0, 150 mM NaCl, 1% Tri-ton X-100, 1 mM DTT, 1× complete protease inhibitor cocktail, and 10% glycerol) and pre-cleared with Protein A/G PLUS-Agarose beads (sc-2003, Santa Cruz Biotechnology, USA) for 2 h at 4°C. The lysates were then immunoprecipitated with indicated antibodies or isotype-matched control antibodies plus protein G Sepharose beads at 4°C for 2–4 h. The beads were then washed three times and boiled. Protein samples were analyzed by Western blotting. For Western blotting, protein samples were mixed with 6× loading buffer supplemented with 10% β-mercaptoethanol, heated at 100°C for 5 min and separated on a 10% SDS-PAGE under reducing conditions. After electrophoresis, protein samples were electroblotted onto polyvinylidene difluoride membranes (Bio-Rad, CA, USA) and blocked for 2 h in Tris-buffered saline (10 mM Tris-HCl, pH 8.0, containing 150 mM NaCl) containing 5% (w/v) non-fat dry milk and 0.5‰ (v/v) Tween-20. The blots were incubated with the primary antibodies overnight at 4°C. The next day, the blots were incubated with corresponding horseradish peroxidase (HRP)-conjugated secondary antibodies for 1 h at room temperature (RT). HRP antibody binding was detected using a standard enhanced chemiluminescence (ECL) kit (wbluf0500, Millipore, USA).
-HEK293T cell lines were cotransfected with PB2-Flag plasmid with empty vector or BAG6-HA plasmid. After 24 h post-transfection, CHX (50 μg/mL) was added to the medium and cells were harvested at different time points. Western blotting of cell lysates was performed to detect PB2-Flag, BAG6-HA and β-actin. To investigate the cellular pathway of BAG6-mediated PB2 degradation, at 24 h post-transfection, or infection with PR8 (H1N1), MG132 (20 μM) or CQ (150 μM) was added to the medium, and the cells were harvested 6 h after treatment. Three independent experiments were performed.
-HEK293T cells were transfected with HA-tagged ubiquitin (Ub-HA) plasmids, BAG6-HA or empty plasmids, and PB2-Flag or PB2-Flag with Lysine mutations. At 24 h post-transfection, the cells were treated with MG132 (20 μM) for 6 h and then lysed in 1% SDS lysis buffer. After being boiled for 10 min, the lysates were diluted 10 times with cold lysis buffer supplemented with 1× complete protease inhibitor cocktail, 10 mM DTT, and 10 mM NEM. PB2-Flag protein was then purified with anti-Flag antibody and subjected to western blotting analysis. Ubiquitinated PB2-Flag was detected by anti-HA antibody.
-We downloaded all available PB2 amino acid sequences of human and avian origin for influenza viruses of subtypes H1, H3, H5, H7, and H9 from the Global Initiative on Sharing Avian Influenza Data (GISAID,www.epicov.org) (date of access: Jan. 22, 2024), and multiple sequence alignment was performed using MAFFT v7.0 [61], and then the amino acid categories and percentages of the 189 amino acid residues were counted.
-Cells on coverslips were washed twice with prewarmed PBS and fixed with 4% paraformaldehyde for 15 min at room temperature. Cells were subsequently permeabilized with immunostaining permeabilization buffer containing Triton X-100 (P0096, Beyotime, Shanghai, China) for 10 min and blocked with QuickBlock blocking buffer (P0220, Beyotime, Shanghai, China) for 20 min at room temperature. Fixed cells were incubated with indicated antibodies diluted in immunostaining primary antibody dilution buffer at 4°C overnight. Coverslips were then washed three times with PBS and incubated with Alexa Fluor 488-conjugated secondary antibodies or Alexa Fluor 555-conjugated secondary antibodies for 1 h at 37°C. Coverslips were finally washed three times and mounted onto microscope slides with DAPI staining solution (C1006, Beyotime, Shanghai, China) for 8 min and examined by confocal microscopy. Immunoassayed cells were visualized using a Nikon super-resolution laser scanning confocal microscope under a 100-time oil objective and analyzed using the Imaris 9.2 platform.
-An online software, ColabFold, was used for the prediction of protein structures and complexes by combining the fast homology search of MMseqs2 with AlphaFold2 or RoseTTAFold. Sequence alignments/templates are generated through MMseqs2 and HHsearch [62]. The amino acid sequences of BAG6 protein N-terminal 1-255aa and PB2 protein N-terminal 1-247aa were used for the prediction of protein complex at the open-source website ColabFold v1.5.2 (https://colab.research.google.com/github/sokrypton/ColabFold/blob/main/AlphaFold2.ipynb#scrollTo=mbaIO9pWjaN0), and the predicted results were viewed and analyzed using PyMOL v2.5.0.
-WT A549 and BAG6-KO A549 cells or WT HeLa and BAG6-KO HeLa cells were plated in 96-well plates at a density of 2000 cells in 100 μL of medium per well. The cell viability was then assayed according to the CCK8 kit instructions (C0042, Beyotime, Shanghai, China).</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias resolution.
-    Inputs:
-    Alias gene symbol: SCYTHE
-    HGNC record ID: HGNC:13919
-    Primary gene symbol: BAG6
-    Official HGNC gene name: BAG cochaperone 6
-    Biomedical text context (may include PMID)
-    Task:
-    Determine whether the alias symbol in the given text refers to the gene represented by the provided HGNC record ID.
-    Rules:
-    If the text does not support that the alias refers to the provided gene, return:
-    "alias_symbol_represents_primary_gene": "NO"
-    "alternate_abbreviation": ""
-    "evidence": ""
-    If the text does support the gene identity, set "alias_symbol_represents_primary_gene": "YES" and 
-    determine whether the alias symbol in the given text is an alternate abbreviation for the primary gene symbol.
-    If the text does not support that the alias is an alternate abbreviation, return:
-    "alternate_abbreviation": "NO"
-    "evidence": ""
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
-    ALTERNATE ABBREVIATION → alias is expanded to a phrase identically matching the official HGNC gene name
-    ALTERNATE ABBREVIATION — POSITIVE EXAMPLE
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Primary gene symbol: A1BG
-    Evidence must be one exact sentence copied verbatim from the text.
-    Do not infer relationships or paraphrase evidence.
-    Output (Strict):
-    Output only one JSON object. No explanations. No markdown.
-    {
-    "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
-    "alias_symbol_represents_primary_gene": "YES or NO",
-    "alternate_abbreviation": "YES or NO",
-    "evidence": ""
-    }
-PMID: 38498560
-Full Text: (A) The predicted interaction domain of BAG6 and PB2. The protein structure of PB2 and BAG6 from AlphaFold2 database and the predicted interaction complex from ColabFold online software, showing that BAG6 124–186 amino acids is the key region for binding to the N-terminus of PB2 protein, which competitively prevents PB1-PB2 interaction. The N-terminus of BAG6 (residues 1–255, blue) and the N-terminus of PB2 (residues 1–247, green) from ColabFold online prediction, the interaction region of PB1 in complex with PB2 (residues 678–757, light red) from PDB:3A1G. (B) Schematic diagram illustrating the truncated and deleted mutants of BAG6 based on the predicted interaction domain. UBL: ubiquitin-like domain; PXXP: proline-rich region. (C) HEK293T cells transfected with the indicated plasmids were immunoprecipitated with M2/Flag antibody, followed by western blot analysis. (D and E) A549 cells were transfected with BAG6 1:255-HA or BAG6 1:92-HA or BAG6 92:255-HA or BAG6 del124:186-HA empty vector for 24 h, and then infected with IAV H1N1 (MOI = 1.0). The viral NP proteins were measured by western blotting (D), the viral titers in the supernatants were determined by TCID50assay (E). (F) HEK293T cells were co-transfected with pPolI-Luc reporter plasmid and expression plasmids containing viral PB1, PB2, PA, and NP of H1N1 along with BAG6 1:255-HA or different truncated mutants of BAG6 or empty vector. Renilla luciferase was used as an internal control. Luciferase activity of the viral polymerase was determined at 24 h post-transfection. Data presented as means ± SD and are representative of three independent experiments. *p&lt; 0.05, **p&lt; 0.01, ***p&lt; 0.001, Unpaired Student’s t test.
-IAVs are among the most common contagious pathogens to cause severe respiratory infections. Host cells have developed multiple strategies to defend against IAV infection. This study identified BAG6 as a novel intrinsic antiviral factor to negatively regulate the replication of multiple IAV subtypes, including human H1N1, H5N1 and avian H7N9, H9N2. BAG6 specifically interacts with the N-terminus of viral polymerase subunit protein PB2, competitively interrupts the assembly of functional RdRp complex and induces the ubiquitination degradation of PB2, which attenuate viral polymerase activity and IAV replication in mammalian cells and pathogenicity in mouse model (Fig 10). These findings reveal a new antagonism mechanism between pathogens and hosts, and highlight a potent antiviral activity of BAG6 by targeting the key viral protein PB2.
-During IAV infection, BAG6 directly interacts with the N-terminus of the IAV polymerase subunit PB2. The interaction between BAG6 and PB2 competes with PB1 for PB2 binding, which perturbs the formation of a functional RdRp complex, and further targets PB2 for K48-linked ubiquitination degradation, thereby inhibiting IAV replication (by Figdraw).
-PB2 protein of IAV is critical for RdRp complex to catalyze the viral transcription and replication, and acts as a key determinant for mammalian adaptation of avian influenza virus. PB2 is responsible for binding the polymerase complex to host cell RNA and initiating viral transcription. It contains a conserved N-terminal fragment that interacts with PB1 to form the polymerase complex, and a central cap-binding domain that recognizes the 5’ cap structure of host cell mRNA, allowing the polymerase to "steal" the cap and use it to prime viral transcription [34]. Besides, the C-terminal part of PB2 contains the so-called 627 domain (residues 535–684), which participates in host adaptation and virulence by influencing the binding of NLS to importins [46]. Multiple host proteins have been found to restrict IAV replication by targeting PB2. For instance, TRIM35 mediates the protection against influenza infection by activating TRAF3 and inducing K48-linked ubiquitination and degradation of PB2 [44]. PIAS restricts IAV replication and virulence through mediating PB2 SUMOylation and reducing its stability [47]. In addition, ANP32A inhibits IAV replication in mammalian cells through differential regulation of the activity of viral polymerases carrying PB2-627K (human) or PB2-627E (avian) signature [12,48]. Here, we found that BAG6 associated with PB2, thereby perturbing its interaction with PB1 and inducing its ubiquitination degradation. Notably, BAG6 recognizes the N-terminus of PB2 and promotes PB2 ubiquitination at its K189 residue, which is highly conserved among avian and human influenza strains from Global Initiative on Sharing Avian Influenza Data (GISAID,www.epicov.org) (S1 Table), providing the mechanistic basis that BAG6 acts as a potent antiviral factor during both human- and avian-origin IAV infection.
-BAG6 is a multifunctional protein in host cell and participates in a variety of physiological and pathological processes [19]. BAG6 functions as an essential factor in ubiquitin-mediated metabolism of neo-synthesized defective polypeptides and misfolded/mislocalized proteins [49–51]. It can capture these defective or mislocalized substrates by interacting with their unprocessed or non-inserted hydrophobic domains [45], and at the same time, recruit the E3 ligases, primarily RNF126, to its N-terminal UBL domain for efficient ubiquitination and degradation [40]. Besides, BAG6 is necessary for DNA damage-induced apoptosis by controlling the p53 signaling pathway [52]. It promotes p53 transactivation by stabilizing its interaction with the acetyltransferase p300 and enhancing p53 acetylation during apoptosis and autophagy [21,22,53]. A recent study reported that BAG6 was capable of regulating the activation of IFN-I by inhibiting RIG-I/VISA-mediated recognition of RNA ligand [29]. However, the role of BAG6 in virus infection remains opaque. In this study, we provide evidence that BAG6 can potently inhibit influenza virus replicationin vitroandin vivo. Further investigation found that the overexpression of BAG6 neither affected cell apoptosis during IAV infection (S4 Fig), nor relied on the IFN-I antiviral response to inhibit IAV replication (Fig 4), whereas BAG6 directly interacts with viral polymerase subunit PB2 and targets it for ubiquitination degradation. These findings reveal a novel mechanism by which BAG6 serves as an antiviral factor to specifically target viral protein through its protein quality control function.
-In the recent years, there has been increased interest in harnessing targeted protein degradation (TPD) technology in the development of antiviral therapies by inducing the degradation of either viral or host-related protein targets, but the off-target side effects and toxicity greatly limit its use [54–57]. In this study, we found the N-terminus of host protein BAG6 contains a ubiquitin-like domain (UBL, 17-92aa), which was previously reported to recruit E3 ligase RNF126 and ubiquitinates BAG6-associated clients [40], and a PB2-binding domain (124-186aa), which was proved to interact with viral polymerase subunit PB2 protein during IAV infection. Interestingly, although the BAG6:92-255aa mutant lacking the UBL domain weakened BAG6-meditated antiviral activity against IAV, it still significantly restricted viral polymerase activity and replication (Fig 9E and 9F). This mirrors the findings that BAG6 could suppress the viral polymerase activity by competing with PB1 for PB2 binding and interfering with RdRp assembly (Fig 6E and 6F), even in the situation with PB2 degradation resistance. These data indicate that both UBL and PB2-binding domains are essential for the efficient PB2 degradation and BAG6-mediated antiviral activity. This unique structure thus allows BAG6 naturally possessing a proteolysis-targeting function. By targeting viral PB2, BAG6 is more likely to become a potential candidate for antiviral drug development.
-The laboratory animal usage license number is SYXK-Beijing-2018-0038, certified by Beijing Association for Science and Technology. All animal research was performed in compliance with the Beijing Laboratory Animal Welfare and Ethics guidelines, as issued by the Beijing Administration Committee of Laboratory Animals, and the China Agricultural University (CAU) Institutional Animal Care and Use Committee guidelines (ID: SKLAB-B-2010-003) approved by the Animal Welfare Committee of CAU. All experiments with live viruses were performed in Biosafety Level II laboratory (BSL-2) in CAU. All animal research involved in this study was approved by the Animal Welfare Committee of CAU (No.AW03503202-2-2).
-Human lung adenocarcinoma epithelial cells (A549), HeLa cell, Madin-Darby canine kidney cells (MDCK), Vero cell and human embryonic kidney cells (HEK293T) were purchased from ATCC. IRF9-KO HeLa cells were generated as previous indicated [30,31]. BAG6 KO A549 cells and BAG6 KO HeLa cells were generated using CRISPR/Cas 9-based knockout of BAG6 gene. In brief, the BAG6 gene target sequences, #1 5’- CACCGCGGTACTGGTACTATCATT-3’ and #2 5’- CACCAGGCTCCTCCACAGCGGTAC-3’, were inserted into the guide RNA (gRNA) expression cassette of the pUC19 vector, which also contains an expression cassette of Cas9. The pUC19 plasmid containing the BAG6 target sequence was then transfected into A549 or HeLa cells. The transfected cells were trypsinized 24 h later into single cells, which were diluted and inoculated into a 96-well plate by infinite dilution. Each colony was individually propagated in a 96-well plate, and the knockout of BAG6 expression was confirmed by western blotting. Cells were cultured in DMEM supplemented with 10% v/v heat-inactivated fetal bovine serum (10099141C, Gibco, USA), 100 U mL−1penicillin and 100 μg mL−1streptomycin at 37°C in a 5% CO2atmosphere.
-Influenza A/Puerto Rico/8/1934 (PR8, H1N1, accession HA number:CY045764), A/chicken/China/0606-13/2017 (CN0606, H7N9, accession HA number:MK530478), and A/chicken/Shandong/196/2011 (SD196, H9N2, accession HA number:KR002651) and A/Anhui/1/2005 (AH1, H5N1, accession HA number:HM172104) viruses were maintained in the laboratory. All experiments using non-H5 live viruses were performed in the Biosafety Level II laboratory (BSL-2), and experiments using H5 viruses were performed in the Biosafety Level III Laboratory (BSL-3) in CAU.
-Protein expression plasmids BAG6-HA, BAG6 1:255-HA, BAG6 1:753-HA, BAG6 482:753-HA, BAG6 482:1126-HA, BAG6 642:1126-HA, PB2-Flag, N-terminal PB2-Flag, PB1-Flag, PA-Flag, NP-Flag, M1-Flag, PB2-K5R-Flag, PB2-K33R-Flag, PB2-K41R-Flag, PB2-K48R-Flag, PB2-K61R-Flag, PB2-K187R-Flag, PB2-K189R-Flag, PB2-K331R-Flag, PB2-K339R-Flag, PB2-K353R-Flag, PB2-K482R-Flag, PB2-K561R-Flag, PB2-K617R-Flag, PB2-K699R-Flag, PB2-K721R-Flag, PB2-K736R-Flag, PB2-K738R-Flag, PB2-K752R-Flag, Ub-HA, K48-Ub-HA and K63-Ub-HA were generated by subcloning the corresponding coding segment into the HA-pRK5 or Flag-pRK5 empty vector by homologous recombinase-mediated recombination (S1 Table). Plasmid transfections in HEK293T or A549 cells were performed using jetPRIME (101000046, Polyplus, France).
-Antibody concentrations for immunoprecipitation and immunoblotting were determined empirically. All immunoblot antibodies were diluted as specified in 5% w/v BSA-TBST. Antibodies used as follows: anti-BAG6 (B01P, Abnova, Taiwan, China), anti-PB2 (PA5-32220, Thermo Scientific, Massachusetts, USA), anti-PB1 (PA5-34914, Thermo Scientific, Massachusetts, USA), anti-β-actin (A1978, Sigma, Shanghai, China), anti-GAPDH (ab8245, Abcam, Shanghai, China), anti-PARP (9542, Cell Signaling Technology, Massachusetts, USA), anti-Flag (F1804, Sigma, Shanghai, China and 20543-1-AP, Proteintech, Chicago, USA), anti-HA (H9658, Sigma, Shanghai, China and 51064-2-AP, Proteintech, Chicago, USA), anti-RIG-I (20566-1-AP, Proteintech, Chicago, USA), anti-p-STAT1 (9167, Cell Signaling Technology, Massachusetts, USA), anti-ISG15 (sc166755, Santa Cruz, California, USA), anti-influenza A virus NP (A01506-40, GenScript, New Jersey, USA), Mouse monoclonal anti-influenza A virus M1 antibody (Lab Homemade, Beijing, China, ZL201910912806.0). Cycloheximide (CHX, HY-12320), MG132 (HY-13259C) and Chloroquine (CQ, HY-17589A) was purchased from MCE.
-A dual-luciferase reporter assay system (E1960, Promega, Wisconsin, USA) was used to compare the polymerase activities of different viral RNP complexes. PB2, PB1, PA, and NP gene segments of the indicated viruses (PR8, CN0606 and SD196) were separately cloned into the pCDNA3.1 expression plasmid. PB2, PB1, PA, and NP plasmids (125 ng each plasmid) along with the pLuci luciferase reporter plasmid (10 ng) and the renilla internal control plasmid (2.5 ng) were used to transfect cells. Cell cultures were incubated at 37°C. Cell lysates were analyzed at 24 h post-transfection for firefly and renilla luciferase activities using a GloMax 96 microplate luminometer (GM2000, Promega, Wisconsin, USA). Polymerase proteins were detected by Western blotting.
-Six-week-old BALB/c background female mice were purchased from Beijing Vital River Co. Ltd. (Beijing, China). Animal studies were carried out in specific pathogen-free barrier facilities. Facilities were maintained at an acceptable range of 20–26°C humidity of 30–70% on a 12-h dark/12-h light cycle. Peptide-conjugated PPMO were purchased from Gene Tools (USA). PPMO targeting mouse BAG6 gene (PPMO-BAG6) was designed as CTGGCACTATCACTCGGCTCCATG. A nontargeting PPMO control sequence (PPMO-NC) (CCTCTTACCTCAGTTACAATTTATA), was used as control. Six to eight weeks BALB/c female mice were inoculated intranasally with 100 μg of PPMOs in 50 μL PBS for 2 days continuously.
-Mice were anesthetized and intranasally inoculated with PR8 virus at a median tissue culture infectious dose (TCID50) of 100 in 50 μL of PBS. Body weight and survival were monitored daily for 14 days. Lung tissue lysates were generated by homogenizing snap-frozen lung tissues twice (20 s each time) in MEM medium and centrifuging the lung suspensions at 2000 rpm for 15 min. TCID50assays were performed using MDCK cells and TCID50was calculated as previously described [58]. A portion of the lung from each euthanized mouse at 3 and 5 dpi was fixed in 10% phosphate-buffered formalin, embedded in paraffin, sectioned and stained with hematoxylin and eosin (H&amp;E). Immunohistochemical staining of viral antigen was performed as described previously [59].
-Total RNA from cells was extracted using an RNA isolation kit (Thermo Scientific, Massachusetts, USA). First-strand complementary DNA was synthesized from 1 μg of total RNA using a TransScript RT reagent kit (TransGen, Beijing, China), and oligo dT primer were used for detecting host genes. For the detection of influenza virus mRNA and vRNA, oligo dT primer and uni-12 primer (5′-AGCAAAAGCAGG-3′) [60] were respectively used to generate cDNAs. Generated cDNA was subjected to qPCR in a 25 μL reaction volume using 2X M5 HiPer SYBR Premix EsTaq (with Tli RNaseH) (Mei5bio) (S1 Table). Human β-actin genes were amplified for normalization of the cDNA amount used in qPCR. Reactions were conducted in triplicate, and the data were analyzed using the 2−ΔΔCtmethod.
-Cells were lysed in lysis buffer (50 mM Tris-Cl at pH 8.0, 150 mM NaCl, 1% Tri-ton X-100, 1 mM DTT, 1× complete protease inhibitor cocktail, and 10% glycerol) and pre-cleared with Protein A/G PLUS-Agarose beads (sc-2003, Santa Cruz Biotechnology, USA) for 2 h at 4°C. The lysates were then immunoprecipitated with indicated antibodies or isotype-matched control antibodies plus protein G Sepharose beads at 4°C for 2–4 h. The beads were then washed three times and boiled. Protein samples were analyzed by Western blotting. For Western blotting, protein samples were mixed with 6× loading buffer supplemented with 10% β-mercaptoethanol, heated at 100°C for 5 min and separated on a 10% SDS-PAGE under reducing conditions. After electrophoresis, protein samples were electroblotted onto polyvinylidene difluoride membranes (Bio-Rad, CA, USA) and blocked for 2 h in Tris-buffered saline (10 mM Tris-HCl, pH 8.0, containing 150 mM NaCl) containing 5% (w/v) non-fat dry milk and 0.5‰ (v/v) Tween-20. The blots were incubated with the primary antibodies overnight at 4°C. The next day, the blots were incubated with corresponding horseradish peroxidase (HRP)-conjugated secondary antibodies for 1 h at room temperature (RT). HRP antibody binding was detected using a standard enhanced chemiluminescence (ECL) kit (wbluf0500, Millipore, USA).
-HEK293T cell lines were cotransfected with PB2-Flag plasmid with empty vector or BAG6-HA plasmid. After 24 h post-transfection, CHX (50 μg/mL) was added to the medium and cells were harvested at different time points. Western blotting of cell lysates was performed to detect PB2-Flag, BAG6-HA and β-actin. To investigate the cellular pathway of BAG6-mediated PB2 degradation, at 24 h post-transfection, or infection with PR8 (H1N1), MG132 (20 μM) or CQ (150 μM) was added to the medium, and the cells were harvested 6 h after treatment. Three independent experiments were performed.
-HEK293T cells were transfected with HA-tagged ubiquitin (Ub-HA) plasmids, BAG6-HA or empty plasmids, and PB2-Flag or PB2-Flag with Lysine mutations. At 24 h post-transfection, the cells were treated with MG132 (20 μM) for 6 h and then lysed in 1% SDS lysis buffer. After being boiled for 10 min, the lysates were diluted 10 times with cold lysis buffer supplemented with 1× complete protease inhibitor cocktail, 10 mM DTT, and 10 mM NEM. PB2-Flag protein was then purified with anti-Flag antibody and subjected to western blotting analysis. Ubiquitinated PB2-Flag was detected by anti-HA antibody.
-We downloaded all available PB2 amino acid sequences of human and avian origin for influenza viruses of subtypes H1, H3, H5, H7, and H9 from the Global Initiative on Sharing Avian Influenza Data (GISAID,www.epicov.org) (date of access: Jan. 22, 2024), and multiple sequence alignment was performed using MAFFT v7.0 [61], and then the amino acid categories and percentages of the 189 amino acid residues were counted.
-Cells on coverslips were washed twice with prewarmed PBS and fixed with 4% paraformaldehyde for 15 min at room temperature. Cells were subsequently permeabilized with immunostaining permeabilization buffer containing Triton X-100 (P0096, Beyotime, Shanghai, China) for 10 min and blocked with QuickBlock blocking buffer (P0220, Beyotime, Shanghai, China) for 20 min at room temperature. Fixed cells were incubated with indicated antibodies diluted in immunostaining primary antibody dilution buffer at 4°C overnight. Coverslips were then washed three times with PBS and incubated with Alexa Fluor 488-conjugated secondary antibodies or Alexa Fluor 555-conjugated secondary antibodies for 1 h at 37°C. Coverslips were finally washed three times and mounted onto microscope slides with DAPI staining solution (C1006, Beyotime, Shanghai, China) for 8 min and examined by confocal microscopy. Immunoassayed cells were visualized using a Nikon super-resolution laser scanning confocal microscope under a 100-time oil objective and analyzed using the Imaris 9.2 platform.
-An online software, ColabFold, was used for the prediction of protein structures and complexes by combining the fast homology search of MMseqs2 with AlphaFold2 or RoseTTAFold. Sequence alignments/templates are generated through MMseqs2 and HHsearch [62]. The amino acid sequences of BAG6 protein N-terminal 1-255aa and PB2 protein N-terminal 1-247aa were used for the prediction of protein complex at the open-source website ColabFold v1.5.2 (https://colab.research.google.com/github/sokrypton/ColabFold/blob/main/AlphaFold2.ipynb#scrollTo=mbaIO9pWjaN0), and the predicted results were viewed and analyzed using PyMOL v2.5.0.
-WT A549 and BAG6-KO A549 cells or WT HeLa and BAG6-KO HeLa cells were plated in 96-well plates at a density of 2000 cells in 100 μL of medium per well. The cell viability was then assayed according to the CCK8 kit instructions (C0042, Beyotime, Shanghai, China).</t>
-        </is>
-      </c>
       <c r="V21" t="inlineStr">
         <is>
           <t>Based on the provided text, here is my analysis:
@@ -5404,11 +5450,10 @@
 "alias_symbol": "SCYTHE",
 "primary_gene_symbol": "BAG6",
 "name": "BAG cochaperone 6",
-"alias_symbol_represents_primary_gene": "YES",
 "alternate_abbreviation": "NO",
-"evidence": "BAG6 is a multifunctional protein in host cell and participates in a variety of physiological and pathological processes [19]."
+"evidence": ""
 }
-The text clearly refers to BAG6 throughout and discusses its functions, indicating that SCYTHE does represent the same gene as BAG6. However, there is no evidence that SCYTHE is used as an alternate abbreviation or expanded to match the official gene name. The provided evidence sentence confirms that BAG6 is being discussed but does not mention the SCYTHE alias.</t>
+The text does not provide any evidence that SCYTHE is used as an alternate abbreviation for BAG6 or BAG cochaperone 6. The text consistently refers to the gene as BAG6 throughout and does not mention SCYTHE or link it to BAG6 in any way. Therefore, there is no support for SCYTHE being an alternate abbreviation in this context.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add a method to extract abbreviations, added a new positive example to the prompt lending for some flexibility
</commit_message>
<xml_diff>
--- a/output/test20_alt_abbrev_annotation_with_prompt_using_fulltext_and_abstract_df.xlsx
+++ b/output/test20_alt_abbrev_annotation_with_prompt_using_fulltext_and_abstract_df.xlsx
@@ -610,7 +610,18 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Gastric cancer is the second leading cause of cancer deaths worldwide, and more understanding of its molecular basis is urgently needed. Gastric gland mucin secreted from pyloric gland cells, mucous neck cells, and cardiac gland cells of the gastric mucosa harbors uniqueO‐glycans carrying terminal α1,4‐linkedN‐acetylglucosamine (αGlcNAc) residues. We previously reported that αGlcNAc loss correlated positively with poor outcomes for patients with differentiated‐type gastric cancer. However, the molecular mechanisms underlying these outcomes remained poorly understood. Here, we examined the effects of upregulated αGlcNAc expression on malignant phenotypes of the differentiated‐type gastric cancer cell lines, AGS and MKN7. Upregulation of αGlcNAc following ectopic expression of its biosynthetic enzyme attenuated cell proliferation, motility, and invasiveness of AGS and MKN7 cells in vitro. Moreover, AGS cell tumorigenicity was significantly suppressed by αGlcNAc overexpression in a xenograft model. To define the molecular mechanisms underlying these phenotypes, we investigated αGlcNAc binding proteins in AGS cells and identified Mucin‐1 (MUC1) and podocalyxin. Both proteins were colocalized with αGlcNAc on human gastric cancer cells. We also found that αGlcNAc was bound to MUC1 in murine normal gastric mucosa. When we assessed the effects of αGlcNAc binding to MUC1, we found that αGlcNAc blocked galectin‐3 binding to MUC1, phosphorylation of the MUC1 C‐terminus, and recruitment of Src and β‐catenin to that C‐terminus. These results suggest that αGlcNAc regulates cancer cell phenotypes by dampening MUC1 signal transduction.
+          <t>ABBREVIATIONS:
+αGlcNAc = α1,4‐linked N ‐acetylglucosamine
+α4GnT = α1,4‐ N ‐acetylglucosaminyltransferase
+Dox = doxycycline
+GSL II = Griffonia (Bandieraea) simplicifilia lectin II
+IP = immunoprecipitation
+MUC1 = Mucin‐1
+MUC1‐C = MUC1‐C terminus
+MUC1‐N = MUC1‐N terminus
+PODXL = podocalyxin
+WB = Western blotting
+Gastric cancer is the second leading cause of cancer deaths worldwide, and more understanding of its molecular basis is urgently needed. Gastric gland mucin secreted from pyloric gland cells, mucous neck cells, and cardiac gland cells of the gastric mucosa harbors uniqueO‐glycans carrying terminal α1,4‐linkedN‐acetylglucosamine (αGlcNAc) residues. We previously reported that αGlcNAc loss correlated positively with poor outcomes for patients with differentiated‐type gastric cancer. However, the molecular mechanisms underlying these outcomes remained poorly understood. Here, we examined the effects of upregulated αGlcNAc expression on malignant phenotypes of the differentiated‐type gastric cancer cell lines, AGS and MKN7. Upregulation of αGlcNAc following ectopic expression of its biosynthetic enzyme attenuated cell proliferation, motility, and invasiveness of AGS and MKN7 cells in vitro. Moreover, AGS cell tumorigenicity was significantly suppressed by αGlcNAc overexpression in a xenograft model. To define the molecular mechanisms underlying these phenotypes, we investigated αGlcNAc binding proteins in AGS cells and identified Mucin‐1 (MUC1) and podocalyxin. Both proteins were colocalized with αGlcNAc on human gastric cancer cells. We also found that αGlcNAc was bound to MUC1 in murine normal gastric mucosa. When we assessed the effects of αGlcNAc binding to MUC1, we found that αGlcNAc blocked galectin‐3 binding to MUC1, phosphorylation of the MUC1 C‐terminus, and recruitment of Src and β‐catenin to that C‐terminus. These results suggest that αGlcNAc regulates cancer cell phenotypes by dampening MUC1 signal transduction.
 We previously reported thatA4gnt, which encodes α4GnT, deficient mice completely lost αGlcNAc, and spontaneously developed differentiated‐type adenocarcinoma. Furthermore, loss of αGlcNAc correlated with poor outcome of differentiated‐type gastric cancer patients. However, the molecular mechanisms why loss of αGlcNAc leads to gastric cancer development are poorly understood. In this study, we demonstrate that malignant phenotypes are attenuated by forced expression of αGlcNAc in 2 differentiated‐type gastric cancer cell lines. We also show that αGlcNAc acts as a tumor suppressor by binding to MUC1, decreasing MUC1 signaling.
 FujiiC,HarumiyaS,SatoY,KawakuboM,MatobaH,NakayamaJ.α1,4‐LinkedN‐acetylglucosamine suppresses gastric cancer development by inhibiting Mucin‐1‐mediated signaling.Cancer Sci.2022;113:3852‐3863. doi:10.1111/cas.15530PMC963329435959971
 α1,4‐linkedN‐acetylglucosamine
@@ -651,7 +662,18 @@
       <c r="T2" t="inlineStr">
         <is>
           <t>PMID: 35959971
-Full Text: Gastric cancer is the second leading cause of cancer deaths worldwide, and more understanding of its molecular basis is urgently needed. Gastric gland mucin secreted from pyloric gland cells, mucous neck cells, and cardiac gland cells of the gastric mucosa harbors uniqueO‐glycans carrying terminal α1,4‐linkedN‐acetylglucosamine (αGlcNAc) residues. We previously reported that αGlcNAc loss correlated positively with poor outcomes for patients with differentiated‐type gastric cancer. However, the molecular mechanisms underlying these outcomes remained poorly understood. Here, we examined the effects of upregulated αGlcNAc expression on malignant phenotypes of the differentiated‐type gastric cancer cell lines, AGS and MKN7. Upregulation of αGlcNAc following ectopic expression of its biosynthetic enzyme attenuated cell proliferation, motility, and invasiveness of AGS and MKN7 cells in vitro. Moreover, AGS cell tumorigenicity was significantly suppressed by αGlcNAc overexpression in a xenograft model. To define the molecular mechanisms underlying these phenotypes, we investigated αGlcNAc binding proteins in AGS cells and identified Mucin‐1 (MUC1) and podocalyxin. Both proteins were colocalized with αGlcNAc on human gastric cancer cells. We also found that αGlcNAc was bound to MUC1 in murine normal gastric mucosa. When we assessed the effects of αGlcNAc binding to MUC1, we found that αGlcNAc blocked galectin‐3 binding to MUC1, phosphorylation of the MUC1 C‐terminus, and recruitment of Src and β‐catenin to that C‐terminus. These results suggest that αGlcNAc regulates cancer cell phenotypes by dampening MUC1 signal transduction.
+Full Text: ABBREVIATIONS:
+αGlcNAc = α1,4‐linked N ‐acetylglucosamine
+α4GnT = α1,4‐ N ‐acetylglucosaminyltransferase
+Dox = doxycycline
+GSL II = Griffonia (Bandieraea) simplicifilia lectin II
+IP = immunoprecipitation
+MUC1 = Mucin‐1
+MUC1‐C = MUC1‐C terminus
+MUC1‐N = MUC1‐N terminus
+PODXL = podocalyxin
+WB = Western blotting
+Gastric cancer is the second leading cause of cancer deaths worldwide, and more understanding of its molecular basis is urgently needed. Gastric gland mucin secreted from pyloric gland cells, mucous neck cells, and cardiac gland cells of the gastric mucosa harbors uniqueO‐glycans carrying terminal α1,4‐linkedN‐acetylglucosamine (αGlcNAc) residues. We previously reported that αGlcNAc loss correlated positively with poor outcomes for patients with differentiated‐type gastric cancer. However, the molecular mechanisms underlying these outcomes remained poorly understood. Here, we examined the effects of upregulated αGlcNAc expression on malignant phenotypes of the differentiated‐type gastric cancer cell lines, AGS and MKN7. Upregulation of αGlcNAc following ectopic expression of its biosynthetic enzyme attenuated cell proliferation, motility, and invasiveness of AGS and MKN7 cells in vitro. Moreover, AGS cell tumorigenicity was significantly suppressed by αGlcNAc overexpression in a xenograft model. To define the molecular mechanisms underlying these phenotypes, we investigated αGlcNAc binding proteins in AGS cells and identified Mucin‐1 (MUC1) and podocalyxin. Both proteins were colocalized with αGlcNAc on human gastric cancer cells. We also found that αGlcNAc was bound to MUC1 in murine normal gastric mucosa. When we assessed the effects of αGlcNAc binding to MUC1, we found that αGlcNAc blocked galectin‐3 binding to MUC1, phosphorylation of the MUC1 C‐terminus, and recruitment of Src and β‐catenin to that C‐terminus. These results suggest that αGlcNAc regulates cancer cell phenotypes by dampening MUC1 signal transduction.
 We previously reported thatA4gnt, which encodes α4GnT, deficient mice completely lost αGlcNAc, and spontaneously developed differentiated‐type adenocarcinoma. Furthermore, loss of αGlcNAc correlated with poor outcome of differentiated‐type gastric cancer patients. However, the molecular mechanisms why loss of αGlcNAc leads to gastric cancer development are poorly understood. In this study, we demonstrate that malignant phenotypes are attenuated by forced expression of αGlcNAc in 2 differentiated‐type gastric cancer cell lines. We also show that αGlcNAc acts as a tumor suppressor by binding to MUC1, decreasing MUC1 signaling.
 FujiiC,HarumiyaS,SatoY,KawakuboM,MatobaH,NakayamaJ.α1,4‐LinkedN‐acetylglucosamine suppresses gastric cancer development by inhibiting Mucin‐1‐mediated signaling.Cancer Sci.2022;113:3852‐3863. doi:10.1111/cas.15530PMC963329435959971
 α1,4‐linkedN‐acetylglucosamine
@@ -696,25 +718,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -733,7 +762,18 @@
     "evidence": ""
     }
 PMID: 35959971
-Full Text: Gastric cancer is the second leading cause of cancer deaths worldwide, and more understanding of its molecular basis is urgently needed. Gastric gland mucin secreted from pyloric gland cells, mucous neck cells, and cardiac gland cells of the gastric mucosa harbors uniqueO‐glycans carrying terminal α1,4‐linkedN‐acetylglucosamine (αGlcNAc) residues. We previously reported that αGlcNAc loss correlated positively with poor outcomes for patients with differentiated‐type gastric cancer. However, the molecular mechanisms underlying these outcomes remained poorly understood. Here, we examined the effects of upregulated αGlcNAc expression on malignant phenotypes of the differentiated‐type gastric cancer cell lines, AGS and MKN7. Upregulation of αGlcNAc following ectopic expression of its biosynthetic enzyme attenuated cell proliferation, motility, and invasiveness of AGS and MKN7 cells in vitro. Moreover, AGS cell tumorigenicity was significantly suppressed by αGlcNAc overexpression in a xenograft model. To define the molecular mechanisms underlying these phenotypes, we investigated αGlcNAc binding proteins in AGS cells and identified Mucin‐1 (MUC1) and podocalyxin. Both proteins were colocalized with αGlcNAc on human gastric cancer cells. We also found that αGlcNAc was bound to MUC1 in murine normal gastric mucosa. When we assessed the effects of αGlcNAc binding to MUC1, we found that αGlcNAc blocked galectin‐3 binding to MUC1, phosphorylation of the MUC1 C‐terminus, and recruitment of Src and β‐catenin to that C‐terminus. These results suggest that αGlcNAc regulates cancer cell phenotypes by dampening MUC1 signal transduction.
+Full Text: ABBREVIATIONS:
+αGlcNAc = α1,4‐linked N ‐acetylglucosamine
+α4GnT = α1,4‐ N ‐acetylglucosaminyltransferase
+Dox = doxycycline
+GSL II = Griffonia (Bandieraea) simplicifilia lectin II
+IP = immunoprecipitation
+MUC1 = Mucin‐1
+MUC1‐C = MUC1‐C terminus
+MUC1‐N = MUC1‐N terminus
+PODXL = podocalyxin
+WB = Western blotting
+Gastric cancer is the second leading cause of cancer deaths worldwide, and more understanding of its molecular basis is urgently needed. Gastric gland mucin secreted from pyloric gland cells, mucous neck cells, and cardiac gland cells of the gastric mucosa harbors uniqueO‐glycans carrying terminal α1,4‐linkedN‐acetylglucosamine (αGlcNAc) residues. We previously reported that αGlcNAc loss correlated positively with poor outcomes for patients with differentiated‐type gastric cancer. However, the molecular mechanisms underlying these outcomes remained poorly understood. Here, we examined the effects of upregulated αGlcNAc expression on malignant phenotypes of the differentiated‐type gastric cancer cell lines, AGS and MKN7. Upregulation of αGlcNAc following ectopic expression of its biosynthetic enzyme attenuated cell proliferation, motility, and invasiveness of AGS and MKN7 cells in vitro. Moreover, AGS cell tumorigenicity was significantly suppressed by αGlcNAc overexpression in a xenograft model. To define the molecular mechanisms underlying these phenotypes, we investigated αGlcNAc binding proteins in AGS cells and identified Mucin‐1 (MUC1) and podocalyxin. Both proteins were colocalized with αGlcNAc on human gastric cancer cells. We also found that αGlcNAc was bound to MUC1 in murine normal gastric mucosa. When we assessed the effects of αGlcNAc binding to MUC1, we found that αGlcNAc blocked galectin‐3 binding to MUC1, phosphorylation of the MUC1 C‐terminus, and recruitment of Src and β‐catenin to that C‐terminus. These results suggest that αGlcNAc regulates cancer cell phenotypes by dampening MUC1 signal transduction.
 We previously reported thatA4gnt, which encodes α4GnT, deficient mice completely lost αGlcNAc, and spontaneously developed differentiated‐type adenocarcinoma. Furthermore, loss of αGlcNAc correlated with poor outcome of differentiated‐type gastric cancer patients. However, the molecular mechanisms why loss of αGlcNAc leads to gastric cancer development are poorly understood. In this study, we demonstrate that malignant phenotypes are attenuated by forced expression of αGlcNAc in 2 differentiated‐type gastric cancer cell lines. We also show that αGlcNAc acts as a tumor suppressor by binding to MUC1, decreasing MUC1 signaling.
 FujiiC,HarumiyaS,SatoY,KawakuboM,MatobaH,NakayamaJ.α1,4‐LinkedN‐acetylglucosamine suppresses gastric cancer development by inhibiting Mucin‐1‐mediated signaling.Cancer Sci.2022;113:3852‐3863. doi:10.1111/cas.15530PMC963329435959971
 α1,4‐linkedN‐acetylglucosamine
@@ -768,16 +808,17 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Based on the provided text, I cannot confirm that ALPHA4GNT is explicitly used as an alternate abbreviation for the official gene name "alpha-1,4-N-acetylglucosaminyltransferase" associated with HGNC:17968. The text uses A4GNT and α4GnT as abbreviations, but does not explicitly link ALPHA4GNT to the full gene name. Therefore, I cannot classify ALPHA4GNT as an alternate abbreviation in this context.
-Here is the JSON output:
+          <t>Based on the provided text, here is my analysis:
 {
 "pmid": "35959971",
 "alias_symbol": "ALPHA4GNT",
-"primary_gene_symbol": "A4GNT",
+"primary_gene_symbol": "A4GNT", 
 "name": "alpha-1,4-N-acetylglucosaminyltransferase",
-"alternate_abbreviation": "FALSE",
-"evidence": ""
-}</t>
+"alternate_abbreviation": "TRUE",
+"evidence": "ABBREVIATIONS: α4GnT = α1,4‐ N ‐acetylglucosaminyltransferase"
+}
+Reasoning:
+The text provides direct evidence that ALPHA4GNT is an alternate abbreviation for A4GNT. In the abbreviations section, α4GnT is defined as "α1,4‐ N ‐acetylglucosaminyltransferase", which matches the official HGNC gene name. The only difference is that the Greek letter α is used instead of spelling out "alpha", but this is equivalent. Therefore, ALPHA4GNT can be considered an alternate abbreviation of the official gene symbol A4GNT.</t>
         </is>
       </c>
     </row>
@@ -967,25 +1008,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -1054,7 +1102,8 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Based on the provided text, here is the analysis for the gene alias GB3S:
+          <t>Based on the provided text, I do not see evidence that the alias symbol "GB3S" is an alternate abbreviation for the official gene name "alpha 1,4-galactosyltransferase (P1PK blood group)" or the primary gene symbol "A4GALT". The text discusses Gb3 (globotriaosylceramide) as a glycosphingolipid and potential cancer biomarker, but does not mention the gene responsible for its synthesis or any alternate gene symbols. Therefore, I cannot conclude that GB3S is an alternate abbreviation for A4GALT in this context.
+Here is the output in the requested JSON format:
 {
 "pmid": "21255370",
 "alias_symbol": "GB3S",
@@ -1062,8 +1111,7 @@
 "name": "alpha 1,4-galactosyltransferase (P1PK blood group)",
 "alternate_abbreviation": "FALSE",
 "evidence": ""
-}
-The text does not contain any explicit expansion or definition of GB3S as an abbreviation for the official gene name "alpha 1,4-galactosyltransferase (P1PK blood group)" or anything closely resembling it. The text discusses Gb3 (globotriaosylceramide) extensively, but does not link this to the A4GALT gene or the provided alias GB3S. Therefore, there is no evidence that GB3S is used as an alternate abbreviation for A4GALT in this context.</t>
+}</t>
         </is>
       </c>
     </row>
@@ -1237,25 +1285,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -1316,7 +1371,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Based on the provided text, I did not find any explicit evidence that the alias symbol "SCYTHE" is used as an alternate abbreviation for the official gene name "BAG cochaperone 6" or the primary gene symbol "BAG6". The text discusses BAG6 but does not mention or expand the alias "SCYTHE". Therefore, I cannot confirm that SCYTHE is used as an alternate abbreviation in this context.
+          <t>Based on the provided text, I did not find any evidence that the alias symbol "SCYTHE" is explicitly linked to or expanded as the official HGNC gene name "BAG cochaperone 6" or the primary gene symbol "BAG6". The text mentions BAG6 several times but does not connect it to the alias SCYTHE. Therefore, I cannot confirm that SCYTHE is used as an alternate abbreviation for BAG6 in this context.
 Here is the output in the requested JSON format:
 {
 "pmid": "39812643",
@@ -1451,25 +1506,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -1502,14 +1564,13 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Based on the provided text, I cannot confirm that NLRA is an alternate abbreviation for CIITA in this context. The text does not explicitly expand NLRA to "class II major histocompatibility complex transactivator" or provide a clear link between NLRA and CIITA. Therefore, I will classify this as not an alternate abbreviation.
-{
+          <t>{
 "pmid": "40643515",
 "alias_symbol": "NLRA",
 "primary_gene_symbol": "CIITA",
 "name": "class II major histocompatibility complex transactivator",
-"alternate_abbreviation": "FALSE",
-"evidence": ""
+"alternate_abbreviation": "TRUE",
+"evidence": "Moreover, to date, five subfamilies have been identified and constitute the NLR family, including NLRA (CIITA and Ciita), NLRB (NAIP and Naip1,2,4,5,6,7), NLRC (NOD1, NOD2, NLRC3, NLRC4, and NLRC5), NLRP (NLRP1-NLRP14) and NLRX (NLRX1 and NLRx1)."
 }</t>
         </is>
       </c>
@@ -1618,25 +1679,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -2671,25 +2739,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -3165,8 +3240,8 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Based on the provided text, I do not see any evidence that the alias symbol "GAB" is explicitly defined or expanded as an alternate abbreviation for the gene "alpha-1-B glycoprotein" (A1BG). The text appears to be about image processing techniques and does not mention the A1BG gene or expand GAB to its full name. Therefore, I cannot confirm that GAB is being used as an alternate abbreviation for A1BG in this context.
-Here is the JSON output:
+          <t>Based on the provided text, I do not see any evidence that the alias symbol "GAB" is being used as an alternate abbreviation for the gene A1BG (alpha-1-B glycoprotein). The text appears to be about image processing techniques and does not mention genes or proteins. Therefore, I cannot confirm that GAB is an alternate abbreviation for A1BG in this context.
+Here is the output in the requested JSON format:
 {
 "pmid": "40567688",
 "alias_symbol": "GAB",
@@ -3346,25 +3421,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -3591,25 +3673,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -3674,7 +3763,8 @@
 "alternate_abbreviation": "FALSE",
 "evidence": ""
 }
-The text does not provide any evidence that "rd5" is an alternate abbreviation for the TUB gene. The symbol "RD5" appears in the text, but it is used as a primer name for PCR amplification of Blastocystis sp., not as an alias for the TUB gene. There is no explicit link or expansion connecting "rd5" to the official gene name "TUB bipartite transcription factor". Therefore, I have classified it as not being an alternate abbreviation and provided no evidence.</t>
+Reasoning:
+The text does not contain any evidence that the alias symbol "rd5" is an alternate abbreviation for the TUB gene. The only mention of "RD5" in the text is as a primer name "RD5 (5′-ATCTGGTTGATCCTGCCAGT-3′)" used for PCR amplification of Blastocystis sp. This usage is unrelated to the TUB gene. There is no expansion or linking of "rd5" to the official gene name "TUB bipartite transcription factor" or anything similar. Therefore, this text does not support "rd5" being an alternate abbreviation for the TUB gene.</t>
         </is>
       </c>
     </row>
@@ -3830,25 +3920,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -3898,8 +3995,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Based on the provided text, I do not see evidence that SUR-2 is explicitly expanded to or linked with the official gene name "mediator complex subunit 23" or the primary symbol MED23. The text only mentions "sur-2, a C. elegans homologue of mammalian MED23" but does not directly equate SUR-2 with MED23 or expand it to the full gene name. Therefore, I cannot conclude that SUR-2 is used as an alternate abbreviation for MED23 in this context.
-Here is the JSON output:
+          <t>Based on the provided text, I do not see sufficient evidence to classify SUR-2 as an alternate abbreviation for MED23 (mediator complex subunit 23). The text mentions SUR-2 as a C. elegans homologue of mammalian MED23, but does not explicitly expand the SUR-2 abbreviation to the full gene name. Therefore, my assessment is:
 {
 "pmid": "38987256",
 "alias_symbol": "SUR-2",
@@ -4027,25 +4123,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -4261,25 +4364,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -4338,12 +4448,12 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Based on the provided text, I do not see evidence that the alias symbol "GB3S" is explicitly defined or expanded as an alternate abbreviation for the official gene name "alpha 1,4-galactosyltransferase (P1PK blood group)" or the primary gene symbol "A4GALT". The text discusses globotriaosylceramide (Gb3) glycosphingolipids and their interactions with Shiga toxin, but does not appear to mention the A4GALT gene or use GB3S as an alias. Therefore, I cannot conclude that GB3S is used as an alternate abbreviation in this context.
-Here is the output in the requested JSON format:
+          <t>Based on the provided text, I do not see clear evidence that the alias symbol "GB3S" is an alternate abbreviation for the official gene name "alpha 1,4-galactosyltransferase (P1PK blood group)" or the primary symbol "A4GALT". The text discusses globotriaosylceramide (Gb3) glycosphingolipids, but does not appear to link "GB3S" to the official gene name or symbol. Therefore, I cannot conclude that "GB3S" is an alternate abbreviation in this context.
+Here is the JSON output:
 {
 "pmid": "36279320",
 "alias_symbol": "GB3S",
-"primary_gene_symbol": "A4GALT",
+"primary_gene_symbol": "A4GALT", 
 "name": "alpha 1,4-galactosyltransferase (P1PK blood group)",
 "alternate_abbreviation": "FALSE",
 "evidence": ""
@@ -4489,25 +4599,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -4552,7 +4669,7 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Based on the provided text, I do not see any evidence that the alias symbol ACA36b is explicitly expanded to or linked with the official HGNC gene name "small nucleolar RNA, H/ACA box 36B" or the primary symbol SNORA36B. The text mentions ACA36B as a snoRNA, but does not provide an explicit expansion or link to the full official name. Therefore, I cannot classify it as an alternate abbreviation based solely on this text.
+          <t>Based on the provided text, I do not see evidence that ACA36b is an alternate abbreviation for SNORA36B or small nucleolar RNA, H/ACA box 36B. The text does not contain an expansion of ACA36b to the full gene name. Therefore, I cannot classify it as an alternate abbreviation based solely on this text.
 Here is the JSON output:
 {
 "pmid": "19763159",
@@ -4681,25 +4798,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -4879,25 +5003,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -4940,7 +5071,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Based on the provided text, I cannot confirm that IGB3S is an alternate abbreviation for A3GALT2 (alpha 1,3-galactosyltransferase 2). The text does not explicitly link IGB3S to the official gene name through an expansion. Therefore, my assessment is:
+          <t>Based on the provided text and task description, here is my analysis:
 {
 "pmid": "37426661",
 "alias_symbol": "IGB3S",
@@ -4948,7 +5079,8 @@
 "name": "alpha 1,3-galactosyltransferase 2",
 "alternate_abbreviation": "FALSE",
 "evidence": ""
-}</t>
+}
+Reasoning: The text does not contain any explicit expansion or definition of IGB3S that matches or closely resembles the official HGNC gene name "alpha 1,3-galactosyltransferase 2". While the text does mention iGb3s (isoglobotrihexosylceramide synthase), it does not directly link this to IGB3S or expand it in a way that matches the official gene name. Therefore, there is insufficient evidence to classify IGB3S as an alternate abbreviation for A3GALT2 based on this text.</t>
         </is>
       </c>
     </row>
@@ -5084,25 +5216,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -5144,8 +5283,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Based on the provided text, I cannot determine if the alias symbol HNRNP-G is an alternate abbreviation for the gene RBMXP1 (RBMX pseudogene 1). The text does not contain any explicit mention or expansion of HNRNP-G or RBMXP1. Therefore, I cannot classify this as an alternate abbreviation.
-Here is the output in the requested JSON format:
+          <t>Based on the provided text, I cannot confirm that HNRNP-G is an alternate abbreviation for RBMX pseudogene 1 (RBMXP1). The text does not contain any information linking HNRNP-G to RBMXP1 or expanding it to the official gene name. Therefore, I will classify this as not an alternate abbreviation.
 {
 "pmid": "40448182",
 "alias_symbol": "HNRNP-G",
@@ -5287,25 +5425,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -5517,25 +5662,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -5590,8 +5742,7 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Based on the provided text, I did not find any evidence that the alias symbol ACF65 is explicitly linked to or expanded as the official gene name "APOBEC1 complementation factor" for the gene A1CF. The text does not appear to mention ACF65 or discuss the A1CF gene. Therefore, I cannot confirm that ACF65 is used as an alternate abbreviation for A1CF in this context.
-Here is the output in the requested JSON format:
+          <t>Based on the provided text, there is no evidence that ACF65 is an alternate abbreviation for A1CF (APOBEC1 complementation factor). The text does not mention ACF65 or expand it to the official gene name. Therefore:
 {
 "pmid": "11815617",
 "alias_symbol": "ACF65",
@@ -5743,25 +5894,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -5816,7 +5974,7 @@
 "alternate_abbreviation": "TRUE",
 "evidence": "SerotoninN-acetyltransferase (SNAT.; also named arylakylamineN-acetyltransferase) is the penultimate or final enzyme of melatonin biosynthesis, depending on the substrate, in both animals and plants [1,2]."
 }
-The text explicitly links the alias symbol SNAT to the official gene name aralkylamine N-acetyltransferase through an expansion, indicating it is an alternate abbreviation. The evidence sentence directly states this relationship.</t>
+The text provides evidence that SNAT is an alternate abbreviation for aralkylamine N-acetyltransferase (AANAT). The sentence directly links SNAT to the full name "arylakylamineN-acetyltransferase", which is essentially identical to the official HGNC name "aralkylamine N-acetyltransferase".</t>
         </is>
       </c>
     </row>
@@ -5956,25 +6114,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -6018,7 +6183,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Based on the provided text, I cannot determine if "ABP1" is an alternate abbreviation for the gene with HGNC ID HGNC:80 (AOC1, amine oxidase copper containing 1). The text does not mention ABP1, AOC1, or amine oxidase copper containing 1. The text appears to be about HSP110 and its interactions with chromatin remodeling complexes. Without any relevant information about the gene in question, I cannot classify ABP1 as an alternate abbreviation.
+          <t>Based on the provided text, I cannot find any evidence that the alias symbol ABP1 is an alternate abbreviation for the gene AOC1 (amine oxidase copper containing 1). The text does not mention ABP1 or AOC1 at all. Therefore, I cannot classify this as an alternate abbreviation.
 {
 "pmid": "40498025",
 "alias_symbol": "ABP1",
@@ -6192,25 +6357,32 @@
     Task:
     Determine whether the alias symbol in the given text represents the gene associated with the provided HGNC record ID
     as an alternate abbreviation of the official HGNC gene symbol.
-    Classify the alias symbol as an Alternate Abbreviation only if it is explicitly expanded in the text to the official
+    Classify the alias symbol as an Alternate Abbreviation only if it is expanded in the text to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     The mere presence of both the alias symbol and the official HGNC gene name in the text is not sufficient. 
-    The text must explicitly link the alias symbol to the official gene name through an expansion 
-    (e.g., “ALIAS (Official Gene Name)” or equivalent phrasing).
+    The text must link the alias symbol to the official gene name through an expansion.
     Examples:
     1-
-    Text: “Alpha 1-beta glycoprotein (A1B) was purified to homogeneity from human plasma using a three-step 
-    procedure involving pseudo-ligand affinity chromatography on immobilized Cibacron Blue 3-GA, gel filtration 
-    chromatography on Sephadex G-200 and ion-exchange chromatography on DEAE Affigel Blue.”
-    Alias gene symbol: A1B
-    Official HGNC gene name: alpha-1-B glycoprotein
-    Primary gene symbol: A1BG
+    Text: “A 64-kDa human protein, cloned and identified as either ACF (APOBEC-1complementation factor) (8) or 
+    ASP (APOBEC-1 stimulating protein) (9), together with APOBEC-1 function as a minimal editosome in vitro.”
+    Reasoning: ACF64 and ACF65 are used like this "ACF64/ACF65" in the text and therefore it can be assumed that
+    this sentence is also applicable to ACF65.
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
     2-
     Text: “Editing of apolipoprotein (apo) B mRNA is mediated by an enzyme-complex that consists of the catalytic 
     cytidine deaminase APOBEC-1 and the mRNA binding protein APOBEC-1 complementation factor or APOBEC-1 stimulating protein (ACF/ASP).”
+    Reasoning: ASP is represented by APOBEC-1 stimulating protein where stimulating is a synonym for complementation
     Alias gene symbol: ASP
     Official HGNC gene name: APOBEC1 complementation factor
     Primary gene symbol: A1CF
+    3-
+    Text: In the abbreviations section “α4GnT α1,4-N-acetylglucosaminyltransferase”
+    Reasoning: ALPHA4GNT is the same as A4GNT but with the term alpha spelled out instead of just shortened to an A
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -6265,8 +6437,7 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>Based on my analysis of the provided text, there is no evidence that the alias symbol "GB3S" is explicitly used as an alternate abbreviation for the official gene name "alpha 1,4-galactosyltransferase (P1PK blood group)" or the primary gene symbol "A4GALT". The text discusses Gb3 (globotriaosylceramide) lipids and sphingolipids, but does not mention the A4GALT gene or use GB3S as an abbreviation for it. Therefore, I cannot conclude that GB3S is being used as an alternate abbreviation for A4GALT in this context.
-Here is the JSON output:
+          <t>Based on the provided text, there is no evidence that the alias symbol "GB3S" is an alternate abbreviation for the official gene name "alpha 1,4-galactosyltransferase (P1PK blood group)" or the primary gene symbol "A4GALT". The text discusses Gb3 (globotriaosylceramide) lipids and their interactions with Shiga toxin, but does not mention the A4GALT gene or any alternate abbreviations for it. Therefore, I cannot conclude that GB3S is an alternate abbreviation in this context.
 {
 "pmid": "32948883",
 "alias_symbol": "GB3S",

</xml_diff>